<commit_message>
Atualização automática: emergencias (14/09/2026 13:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="101">
   <si>
     <t>om_emg</t>
   </si>
@@ -244,9 +244,6 @@
     <t>Expedido total</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -281,6 +278,9 @@
   </si>
   <si>
     <t>AWB 12756560825 - volume retirado na loja GOLLOG - BSB por Mateus Oliveira em 10/09. Godoy 10/09/26.</t>
+  </si>
+  <si>
+    <t>Operador informou que o Pn solicitado não se aplica a efetividade da Anv 2702. Godoy 11/09/26.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -764,7 +764,7 @@
         <v>74</v>
       </c>
       <c r="I2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J2" s="1">
         <v>46238</v>
@@ -776,7 +776,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N2" s="1">
         <v>46269</v>
@@ -785,16 +785,16 @@
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="S2" t="s">
+        <v>80</v>
+      </c>
+      <c r="T2" t="s">
         <v>81</v>
-      </c>
-      <c r="T2" t="s">
-        <v>82</v>
       </c>
       <c r="V2" t="s">
         <v>89</v>
@@ -832,7 +832,7 @@
         <v>74</v>
       </c>
       <c r="I3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J3" s="1">
         <v>46251</v>
@@ -844,7 +844,7 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N3" s="1">
         <v>46280</v>
@@ -853,16 +853,16 @@
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R3">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="S3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T3" t="s">
         <v>81</v>
-      </c>
-      <c r="T3" t="s">
-        <v>82</v>
       </c>
       <c r="V3" t="s">
         <v>90</v>
@@ -900,7 +900,7 @@
         <v>74</v>
       </c>
       <c r="I4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J4" s="1">
         <v>46253</v>
@@ -912,22 +912,22 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N4" s="1">
         <v>46283</v>
       </c>
       <c r="Q4">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R4">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="S4" t="s">
+        <v>80</v>
+      </c>
+      <c r="T4" t="s">
         <v>81</v>
-      </c>
-      <c r="T4" t="s">
-        <v>82</v>
       </c>
       <c r="W4" t="s">
         <v>100</v>
@@ -962,7 +962,7 @@
         <v>74</v>
       </c>
       <c r="I5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J5" s="1">
         <v>46254</v>
@@ -974,7 +974,7 @@
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N5" s="1">
         <v>46286</v>
@@ -983,19 +983,19 @@
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R5">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="S5" t="s">
+        <v>80</v>
+      </c>
+      <c r="T5" t="s">
         <v>81</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>82</v>
-      </c>
-      <c r="U5" t="s">
-        <v>83</v>
       </c>
       <c r="V5" t="s">
         <v>91</v>
@@ -1033,7 +1033,7 @@
         <v>74</v>
       </c>
       <c r="I6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J6" s="1">
         <v>46262</v>
@@ -1045,7 +1045,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N6" s="1">
         <v>46269</v>
@@ -1054,19 +1054,19 @@
         <v>46269</v>
       </c>
       <c r="Q6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R6">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="T6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="V6" t="s">
         <v>92</v>
@@ -1104,7 +1104,7 @@
         <v>74</v>
       </c>
       <c r="I7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J7" s="1">
         <v>46262</v>
@@ -1116,7 +1116,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N7" s="1">
         <v>46293</v>
@@ -1125,16 +1125,16 @@
         <v>46293</v>
       </c>
       <c r="Q7">
-        <v>-17</v>
+        <v>-14</v>
       </c>
       <c r="R7">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S7" t="s">
+        <v>80</v>
+      </c>
+      <c r="T7" t="s">
         <v>81</v>
-      </c>
-      <c r="T7" t="s">
-        <v>82</v>
       </c>
       <c r="V7" t="s">
         <v>93</v>
@@ -1172,7 +1172,7 @@
         <v>75</v>
       </c>
       <c r="I8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J8" s="1">
         <v>46265</v>
@@ -1184,7 +1184,7 @@
         <v>5</v>
       </c>
       <c r="M8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N8" s="1">
         <v>46297</v>
@@ -1193,19 +1193,19 @@
         <v>46297</v>
       </c>
       <c r="Q8">
-        <v>-21</v>
+        <v>-18</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="S8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="V8" t="s">
         <v>94</v>
@@ -1243,7 +1243,7 @@
         <v>74</v>
       </c>
       <c r="I9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J9" s="1">
         <v>46269</v>
@@ -1255,7 +1255,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N9" s="1">
         <v>46284</v>
@@ -1264,19 +1264,19 @@
         <v>46277</v>
       </c>
       <c r="Q9">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="V9" t="s">
         <v>95</v>
@@ -1314,7 +1314,7 @@
         <v>75</v>
       </c>
       <c r="I10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J10" s="1">
         <v>46274</v>
@@ -1326,25 +1326,25 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N10" s="1">
         <v>46282</v>
       </c>
       <c r="Q10">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="T10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="V10" t="s">
         <v>96</v>
@@ -1379,10 +1379,10 @@
         <v>2709</v>
       </c>
       <c r="H11" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J11" s="1">
         <v>46274</v>
@@ -1394,7 +1394,7 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N11" s="1">
         <v>46282</v>
@@ -1403,19 +1403,19 @@
         <v>46275</v>
       </c>
       <c r="Q11">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="T11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="V11" t="s">
         <v>97</v>
@@ -1450,10 +1450,10 @@
         <v>2702</v>
       </c>
       <c r="H12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J12" s="1">
         <v>46275</v>
@@ -1465,7 +1465,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N12" s="1">
         <v>46312</v>
@@ -1474,16 +1474,19 @@
         <v>46282</v>
       </c>
       <c r="Q12">
-        <v>-36</v>
+        <v>-33</v>
       </c>
       <c r="R12">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="S12" t="s">
+        <v>80</v>
+      </c>
+      <c r="T12" t="s">
         <v>81</v>
       </c>
-      <c r="T12" t="s">
-        <v>82</v>
+      <c r="U12" t="s">
+        <v>88</v>
       </c>
       <c r="V12" t="s">
         <v>98</v>
@@ -1518,10 +1521,10 @@
         <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J13" s="1">
         <v>46275</v>
@@ -1533,7 +1536,7 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N13" s="1">
         <v>46312</v>
@@ -1542,16 +1545,19 @@
         <v>46282</v>
       </c>
       <c r="Q13">
-        <v>-36</v>
+        <v>-33</v>
       </c>
       <c r="R13">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="S13" t="s">
+        <v>80</v>
+      </c>
+      <c r="T13" t="s">
         <v>81</v>
       </c>
-      <c r="T13" t="s">
-        <v>82</v>
+      <c r="U13" t="s">
+        <v>88</v>
       </c>
       <c r="V13" t="s">
         <v>98</v>
@@ -1586,10 +1592,10 @@
         <v>2729</v>
       </c>
       <c r="H14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="I14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J14" s="1">
         <v>46275</v>
@@ -1601,22 +1607,22 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="N14" s="1">
         <v>46316</v>
       </c>
       <c r="Q14">
-        <v>-40</v>
+        <v>-37</v>
       </c>
       <c r="R14">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="S14" t="s">
+        <v>80</v>
+      </c>
+      <c r="T14" t="s">
         <v>81</v>
-      </c>
-      <c r="T14" t="s">
-        <v>82</v>
       </c>
       <c r="V14" t="s">
         <v>99</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (15/09/2026 08:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -326,8 +326,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -343,7 +351,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -351,12 +359,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -656,85 +682,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -766,10 +792,10 @@
       <c r="I2" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -778,17 +804,17 @@
       <c r="M2" t="s">
         <v>79</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="S2" t="s">
         <v>80</v>
@@ -834,10 +860,10 @@
       <c r="I3" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -846,17 +872,17 @@
       <c r="M3" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R3">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S3" t="s">
         <v>80</v>
@@ -902,10 +928,10 @@
       <c r="I4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -914,14 +940,14 @@
       <c r="M4" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46283</v>
       </c>
       <c r="Q4">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S4" t="s">
         <v>80</v>
@@ -964,10 +990,10 @@
       <c r="I5" t="s">
         <v>76</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -976,17 +1002,17 @@
       <c r="M5" t="s">
         <v>79</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R5">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="S5" t="s">
         <v>80</v>
@@ -1035,10 +1061,10 @@
       <c r="I6" t="s">
         <v>77</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46262</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46262</v>
       </c>
       <c r="L6">
@@ -1047,17 +1073,17 @@
       <c r="M6" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46269</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46269</v>
       </c>
       <c r="Q6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R6">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S6" t="s">
         <v>80</v>
@@ -1106,10 +1132,10 @@
       <c r="I7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46262</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46262</v>
       </c>
       <c r="L7">
@@ -1118,17 +1144,17 @@
       <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46293</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46293</v>
       </c>
       <c r="Q7">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="R7">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S7" t="s">
         <v>80</v>
@@ -1174,10 +1200,10 @@
       <c r="I8" t="s">
         <v>76</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46265</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46266</v>
       </c>
       <c r="L8">
@@ -1186,17 +1212,17 @@
       <c r="M8" t="s">
         <v>79</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46297</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46297</v>
       </c>
       <c r="Q8">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R8">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S8" t="s">
         <v>81</v>
@@ -1245,10 +1271,10 @@
       <c r="I9" t="s">
         <v>78</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46269</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46273</v>
       </c>
       <c r="L9">
@@ -1257,17 +1283,17 @@
       <c r="M9" t="s">
         <v>79</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46284</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46277</v>
       </c>
       <c r="Q9">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>81</v>
@@ -1316,10 +1342,10 @@
       <c r="I10" t="s">
         <v>77</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46274</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46275</v>
       </c>
       <c r="L10">
@@ -1328,14 +1354,14 @@
       <c r="M10" t="s">
         <v>79</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46282</v>
       </c>
       <c r="Q10">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>81</v>
@@ -1384,10 +1410,10 @@
       <c r="I11" t="s">
         <v>77</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46274</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46275</v>
       </c>
       <c r="L11">
@@ -1396,17 +1422,17 @@
       <c r="M11" t="s">
         <v>79</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46282</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="2">
         <v>46275</v>
       </c>
       <c r="Q11">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>80</v>
@@ -1455,10 +1481,10 @@
       <c r="I12" t="s">
         <v>77</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46275</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46305</v>
       </c>
       <c r="L12">
@@ -1467,17 +1493,17 @@
       <c r="M12" t="s">
         <v>79</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46312</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="2">
         <v>46282</v>
       </c>
       <c r="Q12">
-        <v>-33</v>
+        <v>-32</v>
       </c>
       <c r="R12">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="S12" t="s">
         <v>80</v>
@@ -1526,10 +1552,10 @@
       <c r="I13" t="s">
         <v>77</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46275</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46305</v>
       </c>
       <c r="L13">
@@ -1538,17 +1564,17 @@
       <c r="M13" t="s">
         <v>79</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46312</v>
       </c>
-      <c r="O13" s="1">
+      <c r="O13" s="2">
         <v>46282</v>
       </c>
       <c r="Q13">
-        <v>-33</v>
+        <v>-32</v>
       </c>
       <c r="R13">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="S13" t="s">
         <v>80</v>
@@ -1597,10 +1623,10 @@
       <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46275</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46305</v>
       </c>
       <c r="L14">
@@ -1609,14 +1635,14 @@
       <c r="M14" t="s">
         <v>79</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46316</v>
       </c>
       <c r="Q14">
-        <v>-37</v>
+        <v>-36</v>
       </c>
       <c r="R14">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="S14" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (15/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -326,16 +326,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -351,7 +343,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -359,30 +351,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -682,85 +656,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -792,10 +766,10 @@
       <c r="I2" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46238</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -804,10 +778,10 @@
       <c r="M2" t="s">
         <v>79</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46269</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -860,10 +834,10 @@
       <c r="I3" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -872,10 +846,10 @@
       <c r="M3" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -928,10 +902,10 @@
       <c r="I4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46253</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -940,7 +914,7 @@
       <c r="M4" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46283</v>
       </c>
       <c r="Q4">
@@ -990,10 +964,10 @@
       <c r="I5" t="s">
         <v>76</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46254</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -1002,10 +976,10 @@
       <c r="M5" t="s">
         <v>79</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46286</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46258</v>
       </c>
       <c r="Q5">
@@ -1061,10 +1035,10 @@
       <c r="I6" t="s">
         <v>77</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46262</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46262</v>
       </c>
       <c r="L6">
@@ -1073,10 +1047,10 @@
       <c r="M6" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46269</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46269</v>
       </c>
       <c r="Q6">
@@ -1132,10 +1106,10 @@
       <c r="I7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46262</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46262</v>
       </c>
       <c r="L7">
@@ -1144,10 +1118,10 @@
       <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46293</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46293</v>
       </c>
       <c r="Q7">
@@ -1200,10 +1174,10 @@
       <c r="I8" t="s">
         <v>76</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46265</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46266</v>
       </c>
       <c r="L8">
@@ -1212,10 +1186,10 @@
       <c r="M8" t="s">
         <v>79</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46297</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46297</v>
       </c>
       <c r="Q8">
@@ -1271,10 +1245,10 @@
       <c r="I9" t="s">
         <v>78</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46269</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46273</v>
       </c>
       <c r="L9">
@@ -1283,10 +1257,10 @@
       <c r="M9" t="s">
         <v>79</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46284</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46277</v>
       </c>
       <c r="Q9">
@@ -1342,10 +1316,10 @@
       <c r="I10" t="s">
         <v>77</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46274</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46275</v>
       </c>
       <c r="L10">
@@ -1354,7 +1328,7 @@
       <c r="M10" t="s">
         <v>79</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46282</v>
       </c>
       <c r="Q10">
@@ -1410,10 +1384,10 @@
       <c r="I11" t="s">
         <v>77</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46274</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46275</v>
       </c>
       <c r="L11">
@@ -1422,10 +1396,10 @@
       <c r="M11" t="s">
         <v>79</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46282</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11" s="1">
         <v>46275</v>
       </c>
       <c r="Q11">
@@ -1481,10 +1455,10 @@
       <c r="I12" t="s">
         <v>77</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46275</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46305</v>
       </c>
       <c r="L12">
@@ -1493,10 +1467,10 @@
       <c r="M12" t="s">
         <v>79</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46312</v>
       </c>
-      <c r="O12" s="2">
+      <c r="O12" s="1">
         <v>46282</v>
       </c>
       <c r="Q12">
@@ -1552,10 +1526,10 @@
       <c r="I13" t="s">
         <v>77</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46275</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46305</v>
       </c>
       <c r="L13">
@@ -1564,10 +1538,10 @@
       <c r="M13" t="s">
         <v>79</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46312</v>
       </c>
-      <c r="O13" s="2">
+      <c r="O13" s="1">
         <v>46282</v>
       </c>
       <c r="Q13">
@@ -1623,10 +1597,10 @@
       <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46275</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46305</v>
       </c>
       <c r="L14">
@@ -1635,7 +1609,7 @@
       <c r="M14" t="s">
         <v>79</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46316</v>
       </c>
       <c r="Q14">

</xml_diff>

<commit_message>
Atualização automática: emergencias (15/09/2026 13:53)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -326,8 +326,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -343,7 +351,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -351,12 +359,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -656,85 +682,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -766,10 +792,10 @@
       <c r="I2" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -778,10 +804,10 @@
       <c r="M2" t="s">
         <v>79</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -834,10 +860,10 @@
       <c r="I3" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -846,10 +872,10 @@
       <c r="M3" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -902,10 +928,10 @@
       <c r="I4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -914,7 +940,7 @@
       <c r="M4" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46283</v>
       </c>
       <c r="Q4">
@@ -964,10 +990,10 @@
       <c r="I5" t="s">
         <v>76</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -976,10 +1002,10 @@
       <c r="M5" t="s">
         <v>79</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
@@ -1035,10 +1061,10 @@
       <c r="I6" t="s">
         <v>77</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46262</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46262</v>
       </c>
       <c r="L6">
@@ -1047,10 +1073,10 @@
       <c r="M6" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46269</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46269</v>
       </c>
       <c r="Q6">
@@ -1106,10 +1132,10 @@
       <c r="I7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46262</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46262</v>
       </c>
       <c r="L7">
@@ -1118,10 +1144,10 @@
       <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46293</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46293</v>
       </c>
       <c r="Q7">
@@ -1174,10 +1200,10 @@
       <c r="I8" t="s">
         <v>76</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46265</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46266</v>
       </c>
       <c r="L8">
@@ -1186,10 +1212,10 @@
       <c r="M8" t="s">
         <v>79</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46297</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46297</v>
       </c>
       <c r="Q8">
@@ -1245,10 +1271,10 @@
       <c r="I9" t="s">
         <v>78</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46269</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46273</v>
       </c>
       <c r="L9">
@@ -1257,10 +1283,10 @@
       <c r="M9" t="s">
         <v>79</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46284</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46277</v>
       </c>
       <c r="Q9">
@@ -1316,10 +1342,10 @@
       <c r="I10" t="s">
         <v>77</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46274</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46275</v>
       </c>
       <c r="L10">
@@ -1328,7 +1354,7 @@
       <c r="M10" t="s">
         <v>79</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46282</v>
       </c>
       <c r="Q10">
@@ -1384,10 +1410,10 @@
       <c r="I11" t="s">
         <v>77</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46274</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46275</v>
       </c>
       <c r="L11">
@@ -1396,10 +1422,10 @@
       <c r="M11" t="s">
         <v>79</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46282</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="2">
         <v>46275</v>
       </c>
       <c r="Q11">
@@ -1455,10 +1481,10 @@
       <c r="I12" t="s">
         <v>77</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46275</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46305</v>
       </c>
       <c r="L12">
@@ -1467,10 +1493,10 @@
       <c r="M12" t="s">
         <v>79</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46312</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="2">
         <v>46282</v>
       </c>
       <c r="Q12">
@@ -1526,10 +1552,10 @@
       <c r="I13" t="s">
         <v>77</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46275</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46305</v>
       </c>
       <c r="L13">
@@ -1538,10 +1564,10 @@
       <c r="M13" t="s">
         <v>79</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46312</v>
       </c>
-      <c r="O13" s="1">
+      <c r="O13" s="2">
         <v>46282</v>
       </c>
       <c r="Q13">
@@ -1597,10 +1623,10 @@
       <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46275</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46305</v>
       </c>
       <c r="L14">
@@ -1609,7 +1635,7 @@
       <c r="M14" t="s">
         <v>79</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46316</v>
       </c>
       <c r="Q14">

</xml_diff>

<commit_message>
Atualização automática: emergencias (15/09/2026 13:57)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -1485,7 +1485,7 @@
         <v>46275</v>
       </c>
       <c r="K12" s="2">
-        <v>46305</v>
+        <v>46275</v>
       </c>
       <c r="L12">
         <v>1</v>
@@ -1494,16 +1494,16 @@
         <v>79</v>
       </c>
       <c r="N12" s="2">
-        <v>46312</v>
+        <v>46282</v>
       </c>
       <c r="O12" s="2">
         <v>46282</v>
       </c>
       <c r="Q12">
-        <v>-32</v>
+        <v>-2</v>
       </c>
       <c r="R12">
-        <v>-25</v>
+        <v>5</v>
       </c>
       <c r="S12" t="s">
         <v>80</v>
@@ -1556,7 +1556,7 @@
         <v>46275</v>
       </c>
       <c r="K13" s="2">
-        <v>46305</v>
+        <v>46275</v>
       </c>
       <c r="L13">
         <v>1</v>
@@ -1565,16 +1565,16 @@
         <v>79</v>
       </c>
       <c r="N13" s="2">
-        <v>46312</v>
+        <v>46282</v>
       </c>
       <c r="O13" s="2">
         <v>46282</v>
       </c>
       <c r="Q13">
-        <v>-32</v>
+        <v>-2</v>
       </c>
       <c r="R13">
-        <v>-25</v>
+        <v>5</v>
       </c>
       <c r="S13" t="s">
         <v>80</v>
@@ -1627,7 +1627,7 @@
         <v>46275</v>
       </c>
       <c r="K14" s="2">
-        <v>46305</v>
+        <v>46275</v>
       </c>
       <c r="L14">
         <v>1</v>
@@ -1636,13 +1636,13 @@
         <v>79</v>
       </c>
       <c r="N14" s="2">
-        <v>46316</v>
+        <v>46286</v>
       </c>
       <c r="Q14">
-        <v>-36</v>
+        <v>-6</v>
       </c>
       <c r="R14">
-        <v>-25</v>
+        <v>5</v>
       </c>
       <c r="S14" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (16/09/2026 12:24)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="93">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,9 +103,6 @@
     <t>BAMN</t>
   </si>
   <si>
-    <t>BABR</t>
-  </si>
-  <si>
     <t>BACG</t>
   </si>
   <si>
@@ -124,33 +121,33 @@
     <t>313260018713</t>
   </si>
   <si>
-    <t>329260019288</t>
-  </si>
-  <si>
     <t>396260016603</t>
   </si>
   <si>
     <t>690260002556</t>
   </si>
   <si>
-    <t>313260018737</t>
-  </si>
-  <si>
-    <t>690260002566</t>
-  </si>
-  <si>
-    <t>329260019291</t>
-  </si>
-  <si>
-    <t>685260012774</t>
-  </si>
-  <si>
-    <t>685260012773</t>
-  </si>
-  <si>
     <t>685260012775</t>
   </si>
   <si>
+    <t>313260018745</t>
+  </si>
+  <si>
+    <t>313260018746</t>
+  </si>
+  <si>
+    <t>685260012785</t>
+  </si>
+  <si>
+    <t>685260012786</t>
+  </si>
+  <si>
+    <t>685260012787</t>
+  </si>
+  <si>
+    <t>685260012788</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -163,31 +160,31 @@
     <t>2115040-8</t>
   </si>
   <si>
-    <t>C662504-0101</t>
-  </si>
-  <si>
     <t>OD1232-24MB</t>
   </si>
   <si>
     <t>C592001-0206</t>
   </si>
   <si>
-    <t>D210507</t>
-  </si>
-  <si>
-    <t>HM-6C</t>
+    <t>060-0017-00</t>
+  </si>
+  <si>
+    <t>702801-5</t>
   </si>
   <si>
     <t>3244897-4</t>
   </si>
   <si>
-    <t>S3465-2-0132</t>
-  </si>
-  <si>
-    <t>S3465-2-0146</t>
-  </si>
-  <si>
-    <t>060-0017-00</t>
+    <t>S2889-3-0132</t>
+  </si>
+  <si>
+    <t>S2889-3-0146</t>
+  </si>
+  <si>
+    <t>S2889-3-0112</t>
+  </si>
+  <si>
+    <t>S3465-2-0160</t>
   </si>
   <si>
     <t>COMPRESSOR DRIVE ASS</t>
@@ -202,19 +199,16 @@
     <t>CYLINDER GAS S</t>
   </si>
   <si>
-    <t>GAGE VOLT AMME</t>
-  </si>
-  <si>
     <t>DC FAN</t>
   </si>
   <si>
     <t>WICK-STAT DISC</t>
   </si>
   <si>
-    <t>GOVERNOR,OVERSPEED</t>
-  </si>
-  <si>
-    <t>BEARING,PLAIN,ROD EN</t>
+    <t>FLIGHT DIR HOR</t>
+  </si>
+  <si>
+    <t>FUEL PUMP</t>
   </si>
   <si>
     <t>FUEL CONTROL UNIT</t>
@@ -226,7 +220,7 @@
     <t>HOSE ASSY BRAK</t>
   </si>
   <si>
-    <t>FLIGHT DIR HOR</t>
+    <t>HOSE ASSY TEE</t>
   </si>
   <si>
     <t>C</t>
@@ -238,21 +232,27 @@
     <t>R</t>
   </si>
   <si>
+    <t>Providencia tom</t>
+  </si>
+  <si>
     <t>Providência tomada</t>
   </si>
   <si>
     <t>Expedido total</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
+    <t>IPLR</t>
+  </si>
+  <si>
     <t>AIFP</t>
   </si>
   <si>
-    <t>IPLR</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -265,55 +265,31 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>AWB 127-5593 2321 -  volume retirado na loja GOLLOG - BSB por mateus em 10/09 - Godoy 10/09/2026.</t>
-  </si>
-  <si>
     <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026.</t>
   </si>
   <si>
-    <t>ITEM FOI REMOVIDO PARA ATENDER A ANV 2736 POR MOTIVO DE PANE. Godoy 08/09/26.</t>
-  </si>
-  <si>
-    <t>Pedido será atendido pelo estoque FAB pedido n° 18398885 - Godoy 02/09/2026.</t>
-  </si>
-  <si>
-    <t>AWB 12756560825 - volume retirado na loja GOLLOG - BSB por Mateus Oliveira em 10/09. Godoy 10/09/26.</t>
-  </si>
-  <si>
-    <t>Operador informou que o Pn solicitado não se aplica a efetividade da Anv 2702. Godoy 11/09/26.</t>
+    <t>AWB 127-5676 0804 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 11/09 - Godoy 16/09/26.</t>
+  </si>
+  <si>
+    <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de chegada GIG 16/09</t>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de liberação 15/09 (voo 4384)</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
-    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5593 2321- REZ</t>
-  </si>
-  <si>
-    <t>Colocado pedido IJ17699595 - entregue V1 JPA 09/09. Em processo de envio para a base FAB.</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ - Material disponivel para coleta, em contato com a transportadora rc 10/09/2026</t>
-  </si>
-  <si>
-    <t>MATERIAL ENVIADO VIA RECIBO 764/FAB/26 AWB 12756368406 DPE 12/09/2026</t>
-  </si>
-  <si>
-    <t>Será atendido via estoque FAB.</t>
-  </si>
-  <si>
-    <t>MATERIAL ENVIADO VIA RECIBO 769/FAB/26 AWB 12756560825 dpe 10/09/2026 - MATERIAL DISPONIVEL PARA RETIRADA DIA 10/09/2026 11:58 RC 10/09/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido WB0003149512 - envio direto para o Brasil</t>
-  </si>
-  <si>
-    <t>SERÁ ENVIADO DA BASE PAMALS</t>
+    <t>Colocado pedido IJ17699595 - entregue V1 JPA 09/09. Em processo de envio para a base FAB. - MATERIAL ENVIADO VIA RECIBO 775/FAB/26 AWB 12756746104 - material disponivel para retirada 14/09/2026</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ - Material disponivel para coleta, em contato com a transportadora rc 10/09/2026 - material entregue dia 15/09/2026</t>
+  </si>
+  <si>
+    <t>SERÁ ENVIADO DA BASE PAMALS, ITEM ENVIANO DIA 10-09-2026, AWB 127-5676 0804, RECIBO ASSINADO NO DRIVE-CLA-14-09</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -326,16 +302,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -351,7 +319,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -359,30 +327,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -682,85 +632,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -772,30 +722,30 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I2" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46238</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -804,17 +754,17 @@
       <c r="M2" t="s">
         <v>79</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46269</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S2" t="s">
         <v>80</v>
@@ -823,10 +773,10 @@
         <v>81</v>
       </c>
       <c r="V2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="W2" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -840,30 +790,30 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I3" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -872,17 +822,17 @@
       <c r="M3" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R3">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S3" t="s">
         <v>80</v>
@@ -891,10 +841,10 @@
         <v>81</v>
       </c>
       <c r="V3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="W3" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -908,30 +858,30 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46253</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -940,14 +890,14 @@
       <c r="M4" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46283</v>
       </c>
       <c r="Q4">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R4">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S4" t="s">
         <v>80</v>
@@ -956,7 +906,7 @@
         <v>81</v>
       </c>
       <c r="W4" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -970,30 +920,30 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I5" t="s">
         <v>76</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46254</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -1002,17 +952,17 @@
       <c r="M5" t="s">
         <v>79</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46286</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S5" t="s">
         <v>80</v>
@@ -1024,10 +974,10 @@
         <v>82</v>
       </c>
       <c r="V5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="W5" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1035,36 +985,36 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G6">
+        <v>2733</v>
+      </c>
+      <c r="H6" t="s">
         <v>72</v>
       </c>
-      <c r="G6">
-        <v>2721</v>
-      </c>
-      <c r="H6" t="s">
-        <v>74</v>
-      </c>
       <c r="I6" t="s">
-        <v>77</v>
-      </c>
-      <c r="J6" s="2">
+        <v>76</v>
+      </c>
+      <c r="J6" s="1">
         <v>46262</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46262</v>
       </c>
       <c r="L6">
@@ -1073,32 +1023,29 @@
       <c r="M6" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="2">
-        <v>46269</v>
-      </c>
-      <c r="O6" s="2">
-        <v>46269</v>
+      <c r="N6" s="1">
+        <v>46293</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46280</v>
       </c>
       <c r="Q6">
-        <v>11</v>
+        <v>-12</v>
       </c>
       <c r="R6">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S6" t="s">
         <v>80</v>
       </c>
       <c r="T6" t="s">
-        <v>80</v>
-      </c>
-      <c r="U6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="V6" t="s">
+        <v>89</v>
+      </c>
+      <c r="W6" t="s">
         <v>92</v>
-      </c>
-      <c r="W6" t="s">
-        <v>100</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1106,25 +1053,25 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>396</v>
+        <v>690</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G7">
-        <v>2733</v>
+        <v>2727</v>
       </c>
       <c r="H7" t="s">
         <v>74</v>
@@ -1132,41 +1079,44 @@
       <c r="I7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="2">
-        <v>46262</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46262</v>
+      <c r="J7" s="1">
+        <v>46265</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46266</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="N7" s="2">
-        <v>46293</v>
-      </c>
-      <c r="O7" s="2">
-        <v>46293</v>
+      <c r="N7" s="1">
+        <v>46297</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46280</v>
       </c>
       <c r="Q7">
-        <v>-13</v>
+        <v>-16</v>
       </c>
       <c r="R7">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="S7" t="s">
+        <v>81</v>
+      </c>
+      <c r="T7" t="s">
         <v>80</v>
       </c>
-      <c r="T7" t="s">
-        <v>81</v>
+      <c r="U7" t="s">
+        <v>83</v>
       </c>
       <c r="V7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="W7" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1174,70 +1124,67 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="B8" t="s">
         <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F8" t="s">
         <v>71</v>
       </c>
       <c r="G8">
-        <v>2727</v>
+        <v>2729</v>
       </c>
       <c r="H8" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I8" t="s">
-        <v>76</v>
-      </c>
-      <c r="J8" s="2">
-        <v>46265</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46266</v>
+        <v>77</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46275</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46275</v>
       </c>
       <c r="L8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M8" t="s">
         <v>79</v>
       </c>
-      <c r="N8" s="2">
-        <v>46297</v>
-      </c>
-      <c r="O8" s="2">
-        <v>46297</v>
+      <c r="N8" s="1">
+        <v>46286</v>
       </c>
       <c r="Q8">
-        <v>-17</v>
+        <v>-5</v>
       </c>
       <c r="R8">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
+        <v>80</v>
+      </c>
+      <c r="T8" t="s">
         <v>81</v>
-      </c>
-      <c r="T8" t="s">
-        <v>80</v>
       </c>
       <c r="U8" t="s">
         <v>84</v>
       </c>
       <c r="V8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="W8" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1251,31 +1198,31 @@
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G9">
-        <v>2730</v>
+        <v>2732</v>
       </c>
       <c r="H9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I9" t="s">
-        <v>78</v>
-      </c>
-      <c r="J9" s="2">
-        <v>46269</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46273</v>
+        <v>77</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46280</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46281</v>
       </c>
       <c r="L9">
         <v>1</v>
@@ -1283,17 +1230,14 @@
       <c r="M9" t="s">
         <v>79</v>
       </c>
-      <c r="N9" s="2">
-        <v>46284</v>
-      </c>
-      <c r="O9" s="2">
-        <v>46277</v>
+      <c r="N9" s="1">
+        <v>46292</v>
       </c>
       <c r="Q9">
-        <v>-4</v>
+        <v>-11</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S9" t="s">
         <v>81</v>
@@ -1304,11 +1248,8 @@
       <c r="U9" t="s">
         <v>85</v>
       </c>
-      <c r="V9" t="s">
-        <v>95</v>
-      </c>
       <c r="W9" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1316,25 +1257,25 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>690</v>
+        <v>313</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F10" t="s">
         <v>71</v>
       </c>
       <c r="G10">
-        <v>2727</v>
+        <v>2732</v>
       </c>
       <c r="H10" t="s">
         <v>75</v>
@@ -1342,11 +1283,11 @@
       <c r="I10" t="s">
         <v>77</v>
       </c>
-      <c r="J10" s="2">
-        <v>46274</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46275</v>
+      <c r="J10" s="1">
+        <v>46280</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46281</v>
       </c>
       <c r="L10">
         <v>1</v>
@@ -1354,29 +1295,26 @@
       <c r="M10" t="s">
         <v>79</v>
       </c>
-      <c r="N10" s="2">
-        <v>46282</v>
+      <c r="N10" s="1">
+        <v>46292</v>
       </c>
       <c r="Q10">
-        <v>-2</v>
+        <v>-11</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S10" t="s">
+        <v>80</v>
+      </c>
+      <c r="T10" t="s">
         <v>81</v>
       </c>
-      <c r="T10" t="s">
-        <v>80</v>
-      </c>
       <c r="U10" t="s">
-        <v>86</v>
-      </c>
-      <c r="V10" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="W10" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1384,37 +1322,37 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G11">
-        <v>2709</v>
+        <v>2702</v>
       </c>
       <c r="H11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I11" t="s">
-        <v>77</v>
-      </c>
-      <c r="J11" s="2">
-        <v>46274</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46275</v>
+        <v>78</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46281</v>
       </c>
       <c r="L11">
         <v>1</v>
@@ -1422,32 +1360,23 @@
       <c r="M11" t="s">
         <v>79</v>
       </c>
-      <c r="N11" s="2">
-        <v>46282</v>
-      </c>
-      <c r="O11" s="2">
-        <v>46275</v>
+      <c r="N11" s="1">
+        <v>46288</v>
       </c>
       <c r="Q11">
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S11" t="s">
         <v>80</v>
       </c>
       <c r="T11" t="s">
-        <v>80</v>
-      </c>
-      <c r="U11" t="s">
-        <v>87</v>
-      </c>
-      <c r="V11" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="W11" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1458,34 +1387,34 @@
         <v>685</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G12">
         <v>2702</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I12" t="s">
-        <v>77</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46275</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46275</v>
+        <v>78</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46281</v>
       </c>
       <c r="L12">
         <v>1</v>
@@ -1493,17 +1422,14 @@
       <c r="M12" t="s">
         <v>79</v>
       </c>
-      <c r="N12" s="2">
-        <v>46282</v>
-      </c>
-      <c r="O12" s="2">
-        <v>46282</v>
+      <c r="N12" s="1">
+        <v>46288</v>
       </c>
       <c r="Q12">
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="R12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S12" t="s">
         <v>80</v>
@@ -1511,14 +1437,8 @@
       <c r="T12" t="s">
         <v>81</v>
       </c>
-      <c r="U12" t="s">
-        <v>88</v>
-      </c>
-      <c r="V12" t="s">
-        <v>98</v>
-      </c>
       <c r="W12" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1529,34 +1449,34 @@
         <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" t="s">
         <v>69</v>
-      </c>
-      <c r="F13" t="s">
-        <v>71</v>
       </c>
       <c r="G13">
         <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I13" t="s">
-        <v>77</v>
-      </c>
-      <c r="J13" s="2">
-        <v>46275</v>
-      </c>
-      <c r="K13" s="2">
-        <v>46275</v>
+        <v>78</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46281</v>
       </c>
       <c r="L13">
         <v>1</v>
@@ -1564,17 +1484,14 @@
       <c r="M13" t="s">
         <v>79</v>
       </c>
-      <c r="N13" s="2">
-        <v>46282</v>
-      </c>
-      <c r="O13" s="2">
-        <v>46282</v>
+      <c r="N13" s="1">
+        <v>46288</v>
       </c>
       <c r="Q13">
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="R13">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S13" t="s">
         <v>80</v>
@@ -1582,14 +1499,8 @@
       <c r="T13" t="s">
         <v>81</v>
       </c>
-      <c r="U13" t="s">
-        <v>88</v>
-      </c>
-      <c r="V13" t="s">
-        <v>98</v>
-      </c>
       <c r="W13" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1600,34 +1511,34 @@
         <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G14">
-        <v>2729</v>
+        <v>2702</v>
       </c>
       <c r="H14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="2">
-        <v>46275</v>
-      </c>
-      <c r="K14" s="2">
-        <v>46275</v>
+      <c r="J14" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46281</v>
       </c>
       <c r="L14">
         <v>1</v>
@@ -1635,26 +1546,23 @@
       <c r="M14" t="s">
         <v>79</v>
       </c>
-      <c r="N14" s="2">
-        <v>46286</v>
+      <c r="N14" s="1">
+        <v>46288</v>
       </c>
       <c r="Q14">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="R14">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="T14" t="s">
         <v>81</v>
       </c>
-      <c r="V14" t="s">
-        <v>99</v>
-      </c>
       <c r="W14" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (16/09/2026 12:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -302,8 +302,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -319,7 +327,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -327,12 +335,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -632,85 +658,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -742,10 +768,10 @@
       <c r="I2" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -754,10 +780,10 @@
       <c r="M2" t="s">
         <v>79</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -810,10 +836,10 @@
       <c r="I3" t="s">
         <v>76</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -822,10 +848,10 @@
       <c r="M3" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -878,10 +904,10 @@
       <c r="I4" t="s">
         <v>76</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -890,7 +916,7 @@
       <c r="M4" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46283</v>
       </c>
       <c r="Q4">
@@ -940,10 +966,10 @@
       <c r="I5" t="s">
         <v>76</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -952,10 +978,10 @@
       <c r="M5" t="s">
         <v>79</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
@@ -1011,10 +1037,10 @@
       <c r="I6" t="s">
         <v>76</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46262</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46262</v>
       </c>
       <c r="L6">
@@ -1023,10 +1049,10 @@
       <c r="M6" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46293</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46280</v>
       </c>
       <c r="Q6">
@@ -1079,10 +1105,10 @@
       <c r="I7" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46265</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46266</v>
       </c>
       <c r="L7">
@@ -1091,10 +1117,10 @@
       <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46297</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46280</v>
       </c>
       <c r="Q7">
@@ -1150,10 +1176,10 @@
       <c r="I8" t="s">
         <v>77</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46275</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46275</v>
       </c>
       <c r="L8">
@@ -1162,7 +1188,7 @@
       <c r="M8" t="s">
         <v>79</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46286</v>
       </c>
       <c r="Q8">
@@ -1218,10 +1244,10 @@
       <c r="I9" t="s">
         <v>77</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46280</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46281</v>
       </c>
       <c r="L9">
@@ -1230,7 +1256,7 @@
       <c r="M9" t="s">
         <v>79</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46292</v>
       </c>
       <c r="Q9">
@@ -1283,10 +1309,10 @@
       <c r="I10" t="s">
         <v>77</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46280</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46281</v>
       </c>
       <c r="L10">
@@ -1295,7 +1321,7 @@
       <c r="M10" t="s">
         <v>79</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46292</v>
       </c>
       <c r="Q10">
@@ -1348,10 +1374,10 @@
       <c r="I11" t="s">
         <v>78</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46279</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46281</v>
       </c>
       <c r="L11">
@@ -1360,7 +1386,7 @@
       <c r="M11" t="s">
         <v>79</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46288</v>
       </c>
       <c r="Q11">
@@ -1410,10 +1436,10 @@
       <c r="I12" t="s">
         <v>78</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46279</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46281</v>
       </c>
       <c r="L12">
@@ -1422,7 +1448,7 @@
       <c r="M12" t="s">
         <v>79</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46288</v>
       </c>
       <c r="Q12">
@@ -1472,10 +1498,10 @@
       <c r="I13" t="s">
         <v>78</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46279</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46281</v>
       </c>
       <c r="L13">
@@ -1484,7 +1510,7 @@
       <c r="M13" t="s">
         <v>79</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46288</v>
       </c>
       <c r="Q13">
@@ -1534,10 +1560,10 @@
       <c r="I14" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46279</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46281</v>
       </c>
       <c r="L14">
@@ -1546,7 +1572,7 @@
       <c r="M14" t="s">
         <v>79</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46288</v>
       </c>
       <c r="Q14">

</xml_diff>

<commit_message>
Atualização automática: emergencias (17/09/2026 12:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="98">
   <si>
     <t>om_emg</t>
   </si>
@@ -232,18 +232,12 @@
     <t>R</t>
   </si>
   <si>
-    <t>Providencia tom</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
     <t>Expedido total</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -265,15 +259,24 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026.</t>
+    <t>AWB 12756746104 - volume retirado na loja GOLLOG - BEL por mmarlos bispo em 15/09. Godoy 17/09/26.</t>
+  </si>
+  <si>
+    <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026. AWB 127-5594 5035 - volume retirado na loja GOLLOG - CGR por givanildo em 14/09. Godoy 17/09/26.</t>
   </si>
   <si>
     <t>AWB 127-5676 0804 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 11/09 - Godoy 16/09/26.</t>
   </si>
   <si>
+    <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737. será atendido pelo estoque FAB pedido n° 18443495. Godoy 16/09/26</t>
+  </si>
+  <si>
     <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737.</t>
   </si>
   <si>
+    <t>será atendido pelo estoque FAB pedido n° 18422910. Godoy 16/09/26</t>
+  </si>
+  <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
@@ -290,6 +293,18 @@
   </si>
   <si>
     <t>SERÁ ENVIADO DA BASE PAMALS, ITEM ENVIANO DIA 10-09-2026, AWB 127-5676 0804, RECIBO ASSINADO NO DRIVE-CLA-14-09</t>
+  </si>
+  <si>
+    <t>MATERIAL POSSUI NO ESTOQUE FAB, AGUARDANDO LIBERAÇÃO PARA ATENDIMENTO DE EMERGENCIA RC 16/09/2026</t>
+  </si>
+  <si>
+    <t>MATERIAL EM TRANSITO - RECIBO 796/FAB/26 AWB A SER GERADA PELA GOLLOG, DPE 19/09/2026 RC 16/09/2026</t>
+  </si>
+  <si>
+    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0146 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026</t>
+  </si>
+  <si>
+    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0132 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -302,16 +317,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -327,7 +334,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -335,30 +342,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -658,85 +647,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -766,43 +755,43 @@
         <v>72</v>
       </c>
       <c r="I2" t="s">
-        <v>76</v>
-      </c>
-      <c r="J2" s="2">
+        <v>74</v>
+      </c>
+      <c r="J2" s="1">
         <v>46238</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46238</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N2" s="1">
+        <v>46269</v>
+      </c>
+      <c r="O2" s="1">
+        <v>46269</v>
+      </c>
+      <c r="Q2">
+        <v>13</v>
+      </c>
+      <c r="R2">
+        <v>44</v>
+      </c>
+      <c r="S2" t="s">
+        <v>78</v>
+      </c>
+      <c r="T2" t="s">
         <v>79</v>
       </c>
-      <c r="N2" s="2">
-        <v>46269</v>
-      </c>
-      <c r="O2" s="2">
-        <v>46269</v>
-      </c>
-      <c r="Q2">
-        <v>12</v>
-      </c>
-      <c r="R2">
-        <v>43</v>
-      </c>
-      <c r="S2" t="s">
-        <v>80</v>
-      </c>
-      <c r="T2" t="s">
-        <v>81</v>
-      </c>
       <c r="V2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="W2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -834,43 +823,43 @@
         <v>72</v>
       </c>
       <c r="I3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J3" s="2">
+        <v>74</v>
+      </c>
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
+        <v>77</v>
+      </c>
+      <c r="N3" s="1">
+        <v>46280</v>
+      </c>
+      <c r="O3" s="1">
+        <v>46280</v>
+      </c>
+      <c r="Q3">
+        <v>2</v>
+      </c>
+      <c r="R3">
+        <v>33</v>
+      </c>
+      <c r="S3" t="s">
+        <v>78</v>
+      </c>
+      <c r="T3" t="s">
         <v>79</v>
       </c>
-      <c r="N3" s="2">
-        <v>46280</v>
-      </c>
-      <c r="O3" s="2">
-        <v>46280</v>
-      </c>
-      <c r="Q3">
-        <v>1</v>
-      </c>
-      <c r="R3">
-        <v>32</v>
-      </c>
-      <c r="S3" t="s">
-        <v>80</v>
-      </c>
-      <c r="T3" t="s">
-        <v>81</v>
-      </c>
       <c r="V3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="W3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -902,37 +891,37 @@
         <v>72</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
-      </c>
-      <c r="J4" s="2">
+        <v>74</v>
+      </c>
+      <c r="J4" s="1">
         <v>46253</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46252</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
+        <v>77</v>
+      </c>
+      <c r="N4" s="1">
+        <v>46283</v>
+      </c>
+      <c r="Q4">
+        <v>-1</v>
+      </c>
+      <c r="R4">
+        <v>30</v>
+      </c>
+      <c r="S4" t="s">
+        <v>78</v>
+      </c>
+      <c r="T4" t="s">
         <v>79</v>
       </c>
-      <c r="N4" s="2">
-        <v>46283</v>
-      </c>
-      <c r="Q4">
-        <v>-2</v>
-      </c>
-      <c r="R4">
-        <v>29</v>
-      </c>
-      <c r="S4" t="s">
-        <v>80</v>
-      </c>
-      <c r="T4" t="s">
-        <v>81</v>
-      </c>
       <c r="W4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -961,49 +950,49 @@
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I5" t="s">
-        <v>76</v>
-      </c>
-      <c r="J5" s="2">
+        <v>74</v>
+      </c>
+      <c r="J5" s="1">
         <v>46254</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46255</v>
       </c>
       <c r="L5">
         <v>2</v>
       </c>
       <c r="M5" t="s">
+        <v>77</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46286</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46258</v>
+      </c>
+      <c r="Q5">
+        <v>-4</v>
+      </c>
+      <c r="R5">
+        <v>27</v>
+      </c>
+      <c r="S5" t="s">
+        <v>78</v>
+      </c>
+      <c r="T5" t="s">
         <v>79</v>
       </c>
-      <c r="N5" s="2">
-        <v>46286</v>
-      </c>
-      <c r="O5" s="2">
-        <v>46258</v>
-      </c>
-      <c r="Q5">
-        <v>-5</v>
-      </c>
-      <c r="R5">
-        <v>26</v>
-      </c>
-      <c r="S5" t="s">
+      <c r="U5" t="s">
         <v>80</v>
       </c>
-      <c r="T5" t="s">
-        <v>81</v>
-      </c>
-      <c r="U5" t="s">
-        <v>82</v>
-      </c>
       <c r="V5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W5" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1035,43 +1024,46 @@
         <v>72</v>
       </c>
       <c r="I6" t="s">
-        <v>76</v>
-      </c>
-      <c r="J6" s="2">
+        <v>74</v>
+      </c>
+      <c r="J6" s="1">
         <v>46262</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46262</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
+        <v>77</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46293</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46280</v>
+      </c>
+      <c r="Q6">
+        <v>-11</v>
+      </c>
+      <c r="R6">
+        <v>20</v>
+      </c>
+      <c r="S6" t="s">
+        <v>78</v>
+      </c>
+      <c r="T6" t="s">
         <v>79</v>
       </c>
-      <c r="N6" s="2">
-        <v>46293</v>
-      </c>
-      <c r="O6" s="2">
-        <v>46280</v>
-      </c>
-      <c r="Q6">
-        <v>-12</v>
-      </c>
-      <c r="R6">
-        <v>19</v>
-      </c>
-      <c r="S6" t="s">
-        <v>80</v>
-      </c>
-      <c r="T6" t="s">
+      <c r="U6" t="s">
         <v>81</v>
       </c>
       <c r="V6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="W6" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1100,49 +1092,49 @@
         <v>2727</v>
       </c>
       <c r="H7" t="s">
+        <v>73</v>
+      </c>
+      <c r="I7" t="s">
         <v>74</v>
       </c>
-      <c r="I7" t="s">
-        <v>76</v>
-      </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46265</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46266</v>
       </c>
       <c r="L7">
         <v>5</v>
       </c>
       <c r="M7" t="s">
+        <v>77</v>
+      </c>
+      <c r="N7" s="1">
+        <v>46297</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46280</v>
+      </c>
+      <c r="Q7">
+        <v>-15</v>
+      </c>
+      <c r="R7">
+        <v>16</v>
+      </c>
+      <c r="S7" t="s">
         <v>79</v>
       </c>
-      <c r="N7" s="2">
-        <v>46297</v>
-      </c>
-      <c r="O7" s="2">
-        <v>46280</v>
-      </c>
-      <c r="Q7">
-        <v>-16</v>
-      </c>
-      <c r="R7">
-        <v>15</v>
-      </c>
-      <c r="S7" t="s">
-        <v>81</v>
-      </c>
       <c r="T7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="U7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="V7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="W7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1174,43 +1166,43 @@
         <v>72</v>
       </c>
       <c r="I8" t="s">
+        <v>75</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46275</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46275</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
         <v>77</v>
       </c>
-      <c r="J8" s="2">
-        <v>46275</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46275</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
+      <c r="N8" s="1">
+        <v>46286</v>
+      </c>
+      <c r="Q8">
+        <v>-4</v>
+      </c>
+      <c r="R8">
+        <v>7</v>
+      </c>
+      <c r="S8" t="s">
+        <v>78</v>
+      </c>
+      <c r="T8" t="s">
         <v>79</v>
       </c>
-      <c r="N8" s="2">
-        <v>46286</v>
-      </c>
-      <c r="Q8">
-        <v>-5</v>
-      </c>
-      <c r="R8">
-        <v>6</v>
-      </c>
-      <c r="S8" t="s">
-        <v>80</v>
-      </c>
-      <c r="T8" t="s">
-        <v>81</v>
-      </c>
       <c r="U8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="V8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="W8" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1239,43 +1231,46 @@
         <v>2732</v>
       </c>
       <c r="H9" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" t="s">
         <v>75</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" s="1">
+        <v>46280</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
         <v>77</v>
       </c>
-      <c r="J9" s="2">
-        <v>46280</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
+      <c r="N9" s="1">
+        <v>46292</v>
+      </c>
+      <c r="Q9">
+        <v>-10</v>
+      </c>
+      <c r="R9">
+        <v>1</v>
+      </c>
+      <c r="S9" t="s">
         <v>79</v>
       </c>
-      <c r="N9" s="2">
-        <v>46292</v>
-      </c>
-      <c r="Q9">
-        <v>-11</v>
-      </c>
-      <c r="R9">
-        <v>0</v>
-      </c>
-      <c r="S9" t="s">
-        <v>81</v>
-      </c>
       <c r="T9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="U9" t="s">
-        <v>85</v>
+        <v>84</v>
+      </c>
+      <c r="V9" t="s">
+        <v>93</v>
       </c>
       <c r="W9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1304,43 +1299,46 @@
         <v>2732</v>
       </c>
       <c r="H10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" t="s">
         <v>75</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" s="1">
+        <v>46280</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
         <v>77</v>
       </c>
-      <c r="J10" s="2">
-        <v>46280</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
+      <c r="N10" s="1">
+        <v>46292</v>
+      </c>
+      <c r="Q10">
+        <v>-10</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+      <c r="S10" t="s">
+        <v>78</v>
+      </c>
+      <c r="T10" t="s">
         <v>79</v>
-      </c>
-      <c r="N10" s="2">
-        <v>46292</v>
-      </c>
-      <c r="Q10">
-        <v>-11</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10" t="s">
-        <v>80</v>
-      </c>
-      <c r="T10" t="s">
-        <v>81</v>
       </c>
       <c r="U10" t="s">
         <v>85</v>
       </c>
+      <c r="V10" t="s">
+        <v>94</v>
+      </c>
       <c r="W10" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1369,40 +1367,43 @@
         <v>2702</v>
       </c>
       <c r="H11" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I11" t="s">
+        <v>76</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>77</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46288</v>
+      </c>
+      <c r="Q11">
+        <v>-6</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+      <c r="S11" t="s">
         <v>78</v>
       </c>
-      <c r="J11" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
+      <c r="T11" t="s">
         <v>79</v>
       </c>
-      <c r="N11" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q11">
-        <v>-7</v>
-      </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11" t="s">
-        <v>80</v>
-      </c>
-      <c r="T11" t="s">
-        <v>81</v>
+      <c r="V11" t="s">
+        <v>95</v>
       </c>
       <c r="W11" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1431,40 +1432,43 @@
         <v>2702</v>
       </c>
       <c r="H12" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I12" t="s">
+        <v>76</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>77</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46288</v>
+      </c>
+      <c r="Q12">
+        <v>-6</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12" t="s">
         <v>78</v>
       </c>
-      <c r="J12" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
+      <c r="T12" t="s">
         <v>79</v>
       </c>
-      <c r="N12" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q12">
-        <v>-7</v>
-      </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12" t="s">
-        <v>80</v>
-      </c>
-      <c r="T12" t="s">
-        <v>81</v>
+      <c r="V12" t="s">
+        <v>96</v>
       </c>
       <c r="W12" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1493,40 +1497,40 @@
         <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I13" t="s">
+        <v>76</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>77</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46288</v>
+      </c>
+      <c r="Q13">
+        <v>-6</v>
+      </c>
+      <c r="R13">
+        <v>1</v>
+      </c>
+      <c r="S13" t="s">
         <v>78</v>
       </c>
-      <c r="J13" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K13" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
+      <c r="T13" t="s">
         <v>79</v>
       </c>
-      <c r="N13" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q13">
-        <v>-7</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13" t="s">
-        <v>80</v>
-      </c>
-      <c r="T13" t="s">
-        <v>81</v>
-      </c>
       <c r="W13" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1555,40 +1559,46 @@
         <v>2702</v>
       </c>
       <c r="H14" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>78</v>
-      </c>
-      <c r="J14" s="2">
+        <v>76</v>
+      </c>
+      <c r="J14" s="1">
         <v>46279</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46281</v>
       </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
+        <v>77</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46288</v>
+      </c>
+      <c r="Q14">
+        <v>-6</v>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+      <c r="S14" t="s">
         <v>79</v>
       </c>
-      <c r="N14" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q14">
-        <v>-7</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14" t="s">
-        <v>81</v>
-      </c>
       <c r="T14" t="s">
-        <v>81</v>
+        <v>79</v>
+      </c>
+      <c r="U14" t="s">
+        <v>86</v>
+      </c>
+      <c r="V14" t="s">
+        <v>93</v>
       </c>
       <c r="W14" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (17/09/2026 12:58)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -317,8 +317,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -334,7 +342,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -342,12 +350,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -647,85 +673,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -757,10 +783,10 @@
       <c r="I2" t="s">
         <v>74</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -769,10 +795,10 @@
       <c r="M2" t="s">
         <v>77</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -825,10 +851,10 @@
       <c r="I3" t="s">
         <v>74</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -837,10 +863,10 @@
       <c r="M3" t="s">
         <v>77</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -893,10 +919,10 @@
       <c r="I4" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -905,7 +931,7 @@
       <c r="M4" t="s">
         <v>77</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46283</v>
       </c>
       <c r="Q4">
@@ -955,10 +981,10 @@
       <c r="I5" t="s">
         <v>74</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -967,10 +993,10 @@
       <c r="M5" t="s">
         <v>77</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
@@ -1026,10 +1052,10 @@
       <c r="I6" t="s">
         <v>74</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46262</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46262</v>
       </c>
       <c r="L6">
@@ -1038,10 +1064,10 @@
       <c r="M6" t="s">
         <v>77</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46293</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46280</v>
       </c>
       <c r="Q6">
@@ -1097,10 +1123,10 @@
       <c r="I7" t="s">
         <v>74</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46265</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46266</v>
       </c>
       <c r="L7">
@@ -1109,10 +1135,10 @@
       <c r="M7" t="s">
         <v>77</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46297</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46280</v>
       </c>
       <c r="Q7">
@@ -1168,10 +1194,10 @@
       <c r="I8" t="s">
         <v>75</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46275</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46275</v>
       </c>
       <c r="L8">
@@ -1180,7 +1206,7 @@
       <c r="M8" t="s">
         <v>77</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46286</v>
       </c>
       <c r="Q8">
@@ -1236,10 +1262,10 @@
       <c r="I9" t="s">
         <v>75</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46280</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46281</v>
       </c>
       <c r="L9">
@@ -1248,7 +1274,7 @@
       <c r="M9" t="s">
         <v>77</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46292</v>
       </c>
       <c r="Q9">
@@ -1304,10 +1330,10 @@
       <c r="I10" t="s">
         <v>75</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46280</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46281</v>
       </c>
       <c r="L10">
@@ -1316,7 +1342,7 @@
       <c r="M10" t="s">
         <v>77</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46292</v>
       </c>
       <c r="Q10">
@@ -1372,10 +1398,10 @@
       <c r="I11" t="s">
         <v>76</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46279</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46281</v>
       </c>
       <c r="L11">
@@ -1384,7 +1410,7 @@
       <c r="M11" t="s">
         <v>77</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46288</v>
       </c>
       <c r="Q11">
@@ -1437,10 +1463,10 @@
       <c r="I12" t="s">
         <v>76</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46279</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46281</v>
       </c>
       <c r="L12">
@@ -1449,7 +1475,7 @@
       <c r="M12" t="s">
         <v>77</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46288</v>
       </c>
       <c r="Q12">
@@ -1502,10 +1528,10 @@
       <c r="I13" t="s">
         <v>76</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46279</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46281</v>
       </c>
       <c r="L13">
@@ -1514,7 +1540,7 @@
       <c r="M13" t="s">
         <v>77</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46288</v>
       </c>
       <c r="Q13">
@@ -1564,10 +1590,10 @@
       <c r="I14" t="s">
         <v>76</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46279</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46281</v>
       </c>
       <c r="L14">
@@ -1576,7 +1602,7 @@
       <c r="M14" t="s">
         <v>77</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46288</v>
       </c>
       <c r="Q14">

</xml_diff>

<commit_message>
Atualização automática: emergencias (18/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="92">
   <si>
     <t>om_emg</t>
   </si>
@@ -121,9 +121,6 @@
     <t>313260018713</t>
   </si>
   <si>
-    <t>396260016603</t>
-  </si>
-  <si>
     <t>690260002556</t>
   </si>
   <si>
@@ -145,9 +142,6 @@
     <t>685260012787</t>
   </si>
   <si>
-    <t>685260012788</t>
-  </si>
-  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -160,9 +154,6 @@
     <t>2115040-8</t>
   </si>
   <si>
-    <t>OD1232-24MB</t>
-  </si>
-  <si>
     <t>C592001-0206</t>
   </si>
   <si>
@@ -184,9 +175,6 @@
     <t>S2889-3-0112</t>
   </si>
   <si>
-    <t>S3465-2-0160</t>
-  </si>
-  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -199,9 +187,6 @@
     <t>CYLINDER GAS S</t>
   </si>
   <si>
-    <t>DC FAN</t>
-  </si>
-  <si>
     <t>WICK-STAT DISC</t>
   </si>
   <si>
@@ -259,9 +244,6 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>AWB 12756746104 - volume retirado na loja GOLLOG - BEL por mmarlos bispo em 15/09. Godoy 17/09/26.</t>
-  </si>
-  <si>
     <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026. AWB 127-5594 5035 - volume retirado na loja GOLLOG - CGR por givanildo em 14/09. Godoy 17/09/26.</t>
   </si>
   <si>
@@ -274,37 +256,37 @@
     <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737.</t>
   </si>
   <si>
-    <t>será atendido pelo estoque FAB pedido n° 18422910. Godoy 16/09/26</t>
+    <t>Operador pediu para fornecer o PN informado. Godoy 18/09/26.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - previsão de liberação 15/09 (voo 4384)</t>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - entregue em Campinas 16/09</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
-    <t>Colocado pedido IJ17699595 - entregue V1 JPA 09/09. Em processo de envio para a base FAB. - MATERIAL ENVIADO VIA RECIBO 775/FAB/26 AWB 12756746104 - material disponivel para retirada 14/09/2026</t>
-  </si>
-  <si>
     <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ - Material disponivel para coleta, em contato com a transportadora rc 10/09/2026 - material entregue dia 15/09/2026</t>
   </si>
   <si>
     <t>SERÁ ENVIADO DA BASE PAMALS, ITEM ENVIANO DIA 10-09-2026, AWB 127-5676 0804, RECIBO ASSINADO NO DRIVE-CLA-14-09</t>
   </si>
   <si>
-    <t>MATERIAL POSSUI NO ESTOQUE FAB, AGUARDANDO LIBERAÇÃO PARA ATENDIMENTO DE EMERGENCIA RC 16/09/2026</t>
-  </si>
-  <si>
-    <t>MATERIAL EM TRANSITO - RECIBO 796/FAB/26 AWB A SER GERADA PELA GOLLOG, DPE 19/09/2026 RC 16/09/2026</t>
+    <t>MATERIAL POSSUI NO ESTOQUE FAB, AGUARDANDO LIBERAÇÃO PARA ATENDIMENTO DE EMERGENCIA RC 16/09/2026 - item foi envado no dia 16-09-26 AWB 127-5790 1454 -CLA 16-09</t>
+  </si>
+  <si>
+    <t>MATERIAL EM TRANSITO - RECIBO 796/FAB/26 AWB 12757879883, DPE 19/09/2026 RC 16/09/2026</t>
   </si>
   <si>
     <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0146 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026</t>
   </si>
   <si>
     <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0132 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003156622 - será enviado direto para o Brasil</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -317,16 +299,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -342,7 +316,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -350,30 +324,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -669,89 +625,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -766,58 +722,58 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K2" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
         <v>72</v>
       </c>
-      <c r="I2" t="s">
+      <c r="N2" s="1">
+        <v>46269</v>
+      </c>
+      <c r="O2" s="1">
+        <v>46269</v>
+      </c>
+      <c r="Q2">
+        <v>14</v>
+      </c>
+      <c r="R2">
+        <v>45</v>
+      </c>
+      <c r="S2" t="s">
+        <v>73</v>
+      </c>
+      <c r="T2" t="s">
         <v>74</v>
       </c>
-      <c r="J2" s="2">
-        <v>46238</v>
-      </c>
-      <c r="K2" s="2">
-        <v>46238</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2" t="s">
-        <v>77</v>
-      </c>
-      <c r="N2" s="2">
-        <v>46269</v>
-      </c>
-      <c r="O2" s="2">
-        <v>46269</v>
-      </c>
-      <c r="Q2">
-        <v>13</v>
-      </c>
-      <c r="R2">
-        <v>44</v>
-      </c>
-      <c r="S2" t="s">
-        <v>78</v>
-      </c>
-      <c r="T2" t="s">
-        <v>79</v>
-      </c>
       <c r="V2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="W2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -834,58 +790,58 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>74</v>
-      </c>
-      <c r="J3" s="2">
+        <v>69</v>
+      </c>
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>77</v>
-      </c>
-      <c r="N3" s="2">
+        <v>72</v>
+      </c>
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R3">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="T3" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="V3" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="W3" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -902,52 +858,52 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" t="s">
+        <v>70</v>
+      </c>
+      <c r="J4" s="1">
+        <v>46253</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46252</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
         <v>72</v>
       </c>
-      <c r="I4" t="s">
+      <c r="N4" s="1">
+        <v>46263</v>
+      </c>
+      <c r="Q4">
+        <v>20</v>
+      </c>
+      <c r="R4">
+        <v>31</v>
+      </c>
+      <c r="S4" t="s">
+        <v>73</v>
+      </c>
+      <c r="T4" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="2">
-        <v>46253</v>
-      </c>
-      <c r="K4" s="2">
-        <v>46252</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4" t="s">
-        <v>77</v>
-      </c>
-      <c r="N4" s="2">
-        <v>46283</v>
-      </c>
-      <c r="Q4">
-        <v>-1</v>
-      </c>
-      <c r="R4">
-        <v>30</v>
-      </c>
-      <c r="S4" t="s">
-        <v>78</v>
-      </c>
-      <c r="T4" t="s">
-        <v>79</v>
-      </c>
       <c r="W4" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -964,61 +920,61 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>74</v>
-      </c>
-      <c r="J5" s="2">
+        <v>69</v>
+      </c>
+      <c r="J5" s="1">
         <v>46254</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46255</v>
       </c>
       <c r="L5">
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>77</v>
-      </c>
-      <c r="N5" s="2">
+        <v>72</v>
+      </c>
+      <c r="N5" s="1">
         <v>46286</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R5">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S5" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="T5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="U5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="V5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="W5" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1026,70 +982,70 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>396</v>
+        <v>690</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6">
+        <v>2727</v>
+      </c>
+      <c r="H6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I6" t="s">
         <v>69</v>
       </c>
-      <c r="G6">
-        <v>2733</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="J6" s="1">
+        <v>46265</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46266</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6" t="s">
         <v>72</v>
       </c>
-      <c r="I6" t="s">
+      <c r="N6" s="1">
+        <v>46297</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46280</v>
+      </c>
+      <c r="Q6">
+        <v>-14</v>
+      </c>
+      <c r="R6">
+        <v>17</v>
+      </c>
+      <c r="S6" t="s">
         <v>74</v>
       </c>
-      <c r="J6" s="2">
-        <v>46262</v>
-      </c>
-      <c r="K6" s="2">
-        <v>46262</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>77</v>
-      </c>
-      <c r="N6" s="2">
-        <v>46293</v>
-      </c>
-      <c r="O6" s="2">
-        <v>46280</v>
-      </c>
-      <c r="Q6">
-        <v>-11</v>
-      </c>
-      <c r="R6">
-        <v>20</v>
-      </c>
-      <c r="S6" t="s">
-        <v>78</v>
-      </c>
       <c r="T6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="U6" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="V6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="W6" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1097,70 +1053,67 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G7">
-        <v>2727</v>
+        <v>2729</v>
       </c>
       <c r="H7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" t="s">
+        <v>70</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46275</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46275</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>72</v>
+      </c>
+      <c r="N7" s="1">
+        <v>46286</v>
+      </c>
+      <c r="Q7">
+        <v>-3</v>
+      </c>
+      <c r="R7">
+        <v>8</v>
+      </c>
+      <c r="S7" t="s">
         <v>73</v>
       </c>
-      <c r="I7" t="s">
+      <c r="T7" t="s">
         <v>74</v>
       </c>
-      <c r="J7" s="2">
-        <v>46265</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46266</v>
-      </c>
-      <c r="L7">
-        <v>5</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="U7" t="s">
         <v>77</v>
       </c>
-      <c r="N7" s="2">
-        <v>46297</v>
-      </c>
-      <c r="O7" s="2">
-        <v>46280</v>
-      </c>
-      <c r="Q7">
-        <v>-15</v>
-      </c>
-      <c r="R7">
-        <v>16</v>
-      </c>
-      <c r="S7" t="s">
-        <v>79</v>
-      </c>
-      <c r="T7" t="s">
-        <v>78</v>
-      </c>
-      <c r="U7" t="s">
-        <v>82</v>
-      </c>
       <c r="V7" t="s">
+        <v>85</v>
+      </c>
+      <c r="W7" t="s">
         <v>91</v>
-      </c>
-      <c r="W7" t="s">
-        <v>97</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1168,67 +1121,70 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="G8">
-        <v>2729</v>
+        <v>2732</v>
       </c>
       <c r="H8" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" t="s">
+        <v>70</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46280</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
         <v>72</v>
       </c>
-      <c r="I8" t="s">
-        <v>75</v>
-      </c>
-      <c r="J8" s="2">
-        <v>46275</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46275</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>77</v>
-      </c>
-      <c r="N8" s="2">
-        <v>46286</v>
+      <c r="N8" s="1">
+        <v>46292</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46283</v>
       </c>
       <c r="Q8">
-        <v>-4</v>
+        <v>-9</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S8" t="s">
+        <v>74</v>
+      </c>
+      <c r="T8" t="s">
+        <v>74</v>
+      </c>
+      <c r="U8" t="s">
         <v>78</v>
       </c>
-      <c r="T8" t="s">
-        <v>79</v>
-      </c>
-      <c r="U8" t="s">
-        <v>83</v>
-      </c>
       <c r="V8" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="W8" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1245,58 +1201,61 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="G9">
         <v>2732</v>
       </c>
       <c r="H9" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46280</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>72</v>
+      </c>
+      <c r="N9" s="1">
+        <v>46292</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46284</v>
+      </c>
+      <c r="Q9">
+        <v>-9</v>
+      </c>
+      <c r="R9">
+        <v>2</v>
+      </c>
+      <c r="S9" t="s">
         <v>73</v>
       </c>
-      <c r="I9" t="s">
-        <v>75</v>
-      </c>
-      <c r="J9" s="2">
-        <v>46280</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>77</v>
-      </c>
-      <c r="N9" s="2">
-        <v>46292</v>
-      </c>
-      <c r="Q9">
-        <v>-10</v>
-      </c>
-      <c r="R9">
-        <v>1</v>
-      </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
+        <v>74</v>
+      </c>
+      <c r="U9" t="s">
         <v>79</v>
       </c>
-      <c r="T9" t="s">
-        <v>79</v>
-      </c>
-      <c r="U9" t="s">
-        <v>84</v>
-      </c>
       <c r="V9" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="W9" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1304,67 +1263,70 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10">
+        <v>2702</v>
+      </c>
+      <c r="H10" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" t="s">
         <v>71</v>
       </c>
-      <c r="G10">
-        <v>2732</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="J10" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
         <v>72</v>
       </c>
-      <c r="I10" t="s">
-        <v>75</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46280</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>77</v>
-      </c>
-      <c r="N10" s="2">
-        <v>46292</v>
+      <c r="N10" s="1">
+        <v>46288</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46288</v>
       </c>
       <c r="Q10">
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="T10" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="U10" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="V10" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="W10" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1381,55 +1343,61 @@
         <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F11" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G11">
         <v>2702</v>
       </c>
       <c r="H11" t="s">
+        <v>67</v>
+      </c>
+      <c r="I11" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
         <v>72</v>
       </c>
-      <c r="I11" t="s">
-        <v>76</v>
-      </c>
-      <c r="J11" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>77</v>
-      </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46288</v>
       </c>
+      <c r="O11" s="1">
+        <v>46288</v>
+      </c>
       <c r="Q11">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="T11" t="s">
-        <v>79</v>
+        <v>74</v>
+      </c>
+      <c r="U11" t="s">
+        <v>80</v>
       </c>
       <c r="V11" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="W11" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1446,187 +1414,60 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G12">
         <v>2702</v>
       </c>
       <c r="H12" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" t="s">
+        <v>71</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
         <v>72</v>
       </c>
-      <c r="I12" t="s">
-        <v>76</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>77</v>
-      </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46288</v>
       </c>
+      <c r="O12" s="1">
+        <v>46288</v>
+      </c>
       <c r="Q12">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="T12" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="V12" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="W12" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="AA12" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27">
-      <c r="A13">
-        <v>685</v>
-      </c>
-      <c r="B13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" t="s">
-        <v>68</v>
-      </c>
-      <c r="F13" t="s">
-        <v>69</v>
-      </c>
-      <c r="G13">
-        <v>2702</v>
-      </c>
-      <c r="H13" t="s">
-        <v>72</v>
-      </c>
-      <c r="I13" t="s">
-        <v>76</v>
-      </c>
-      <c r="J13" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K13" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
-        <v>77</v>
-      </c>
-      <c r="N13" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q13">
-        <v>-6</v>
-      </c>
-      <c r="R13">
-        <v>1</v>
-      </c>
-      <c r="S13" t="s">
-        <v>78</v>
-      </c>
-      <c r="T13" t="s">
-        <v>79</v>
-      </c>
-      <c r="W13" t="s">
-        <v>97</v>
-      </c>
-      <c r="AA13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27">
-      <c r="A14">
-        <v>685</v>
-      </c>
-      <c r="B14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F14" t="s">
-        <v>69</v>
-      </c>
-      <c r="G14">
-        <v>2702</v>
-      </c>
-      <c r="H14" t="s">
-        <v>73</v>
-      </c>
-      <c r="I14" t="s">
-        <v>76</v>
-      </c>
-      <c r="J14" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K14" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L14">
-        <v>1</v>
-      </c>
-      <c r="M14" t="s">
-        <v>77</v>
-      </c>
-      <c r="N14" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q14">
-        <v>-6</v>
-      </c>
-      <c r="R14">
-        <v>1</v>
-      </c>
-      <c r="S14" t="s">
-        <v>79</v>
-      </c>
-      <c r="T14" t="s">
-        <v>79</v>
-      </c>
-      <c r="U14" t="s">
-        <v>86</v>
-      </c>
-      <c r="V14" t="s">
-        <v>93</v>
-      </c>
-      <c r="W14" t="s">
-        <v>97</v>
-      </c>
-      <c r="AA14" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (18/09/2026 16:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="91">
   <si>
     <t>om_emg</t>
   </si>
@@ -227,9 +227,6 @@
   </si>
   <si>
     <t>IPLR</t>
-  </si>
-  <si>
-    <t>AIFP</t>
   </si>
   <si>
     <t>EA</t>
@@ -299,8 +296,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -316,7 +321,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -324,12 +329,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -629,85 +652,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -739,22 +762,22 @@
       <c r="I2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>72</v>
-      </c>
-      <c r="N2" s="1">
+        <v>71</v>
+      </c>
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -764,16 +787,16 @@
         <v>45</v>
       </c>
       <c r="S2" t="s">
+        <v>72</v>
+      </c>
+      <c r="T2" t="s">
         <v>73</v>
       </c>
-      <c r="T2" t="s">
-        <v>74</v>
-      </c>
       <c r="V2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="W2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -807,22 +830,22 @@
       <c r="I3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>72</v>
-      </c>
-      <c r="N3" s="1">
+        <v>71</v>
+      </c>
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -832,16 +855,16 @@
         <v>34</v>
       </c>
       <c r="S3" t="s">
+        <v>72</v>
+      </c>
+      <c r="T3" t="s">
         <v>73</v>
       </c>
-      <c r="T3" t="s">
-        <v>74</v>
-      </c>
       <c r="V3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="W3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -875,19 +898,19 @@
       <c r="I4" t="s">
         <v>70</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46252</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>72</v>
-      </c>
-      <c r="N4" s="1">
+        <v>71</v>
+      </c>
+      <c r="N4" s="2">
         <v>46263</v>
       </c>
       <c r="Q4">
@@ -897,13 +920,13 @@
         <v>31</v>
       </c>
       <c r="S4" t="s">
+        <v>72</v>
+      </c>
+      <c r="T4" t="s">
         <v>73</v>
       </c>
-      <c r="T4" t="s">
-        <v>74</v>
-      </c>
       <c r="W4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -937,22 +960,22 @@
       <c r="I5" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>72</v>
-      </c>
-      <c r="N5" s="1">
+        <v>71</v>
+      </c>
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
@@ -962,19 +985,19 @@
         <v>28</v>
       </c>
       <c r="S5" t="s">
+        <v>72</v>
+      </c>
+      <c r="T5" t="s">
         <v>73</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>74</v>
       </c>
-      <c r="U5" t="s">
-        <v>75</v>
-      </c>
       <c r="V5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="W5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1008,22 +1031,22 @@
       <c r="I6" t="s">
         <v>69</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46265</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46266</v>
       </c>
       <c r="L6">
         <v>5</v>
       </c>
       <c r="M6" t="s">
-        <v>72</v>
-      </c>
-      <c r="N6" s="1">
+        <v>71</v>
+      </c>
+      <c r="N6" s="2">
         <v>46297</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46280</v>
       </c>
       <c r="Q6">
@@ -1033,19 +1056,19 @@
         <v>17</v>
       </c>
       <c r="S6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="T6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="U6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="W6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1079,19 +1102,19 @@
       <c r="I7" t="s">
         <v>70</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46275</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46275</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>72</v>
-      </c>
-      <c r="N7" s="1">
+        <v>71</v>
+      </c>
+      <c r="N7" s="2">
         <v>46286</v>
       </c>
       <c r="Q7">
@@ -1101,19 +1124,19 @@
         <v>8</v>
       </c>
       <c r="S7" t="s">
+        <v>72</v>
+      </c>
+      <c r="T7" t="s">
         <v>73</v>
       </c>
-      <c r="T7" t="s">
-        <v>74</v>
-      </c>
       <c r="U7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="V7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="W7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1147,22 +1170,22 @@
       <c r="I8" t="s">
         <v>70</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46280</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46281</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>72</v>
-      </c>
-      <c r="N8" s="1">
+        <v>71</v>
+      </c>
+      <c r="N8" s="2">
         <v>46292</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46283</v>
       </c>
       <c r="Q8">
@@ -1172,19 +1195,19 @@
         <v>2</v>
       </c>
       <c r="S8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="T8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="U8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="V8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="W8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1218,22 +1241,22 @@
       <c r="I9" t="s">
         <v>70</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46280</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46281</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>72</v>
-      </c>
-      <c r="N9" s="1">
+        <v>71</v>
+      </c>
+      <c r="N9" s="2">
         <v>46292</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46284</v>
       </c>
       <c r="Q9">
@@ -1243,19 +1266,19 @@
         <v>2</v>
       </c>
       <c r="S9" t="s">
+        <v>72</v>
+      </c>
+      <c r="T9" t="s">
         <v>73</v>
       </c>
-      <c r="T9" t="s">
-        <v>74</v>
-      </c>
       <c r="U9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="V9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="W9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1287,46 +1310,46 @@
         <v>67</v>
       </c>
       <c r="I10" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46279</v>
+      </c>
+      <c r="K10" s="2">
+        <v>46281</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="1">
-        <v>46279</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46281</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>72</v>
-      </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
+        <v>46312</v>
+      </c>
+      <c r="O10" s="2">
         <v>46288</v>
       </c>
-      <c r="O10" s="1">
-        <v>46288</v>
-      </c>
       <c r="Q10">
-        <v>-5</v>
+        <v>-29</v>
       </c>
       <c r="R10">
         <v>2</v>
       </c>
       <c r="S10" t="s">
+        <v>72</v>
+      </c>
+      <c r="T10" t="s">
         <v>73</v>
       </c>
-      <c r="T10" t="s">
-        <v>74</v>
-      </c>
       <c r="U10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="V10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="W10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1358,46 +1381,46 @@
         <v>67</v>
       </c>
       <c r="I11" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46279</v>
+      </c>
+      <c r="K11" s="2">
+        <v>46281</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="J11" s="1">
-        <v>46279</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46281</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>72</v>
-      </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
+        <v>46312</v>
+      </c>
+      <c r="O11" s="2">
         <v>46288</v>
       </c>
-      <c r="O11" s="1">
-        <v>46288</v>
-      </c>
       <c r="Q11">
-        <v>-5</v>
+        <v>-29</v>
       </c>
       <c r="R11">
         <v>2</v>
       </c>
       <c r="S11" t="s">
+        <v>72</v>
+      </c>
+      <c r="T11" t="s">
         <v>73</v>
       </c>
-      <c r="T11" t="s">
-        <v>74</v>
-      </c>
       <c r="U11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="V11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="W11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1429,43 +1452,43 @@
         <v>67</v>
       </c>
       <c r="I12" t="s">
+        <v>69</v>
+      </c>
+      <c r="J12" s="2">
+        <v>46279</v>
+      </c>
+      <c r="K12" s="2">
+        <v>46281</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
         <v>71</v>
       </c>
-      <c r="J12" s="1">
-        <v>46279</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46281</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>72</v>
-      </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
+        <v>46312</v>
+      </c>
+      <c r="O12" s="2">
         <v>46288</v>
       </c>
-      <c r="O12" s="1">
-        <v>46288</v>
-      </c>
       <c r="Q12">
-        <v>-5</v>
+        <v>-29</v>
       </c>
       <c r="R12">
         <v>2</v>
       </c>
       <c r="S12" t="s">
+        <v>72</v>
+      </c>
+      <c r="T12" t="s">
         <v>73</v>
       </c>
-      <c r="T12" t="s">
-        <v>74</v>
-      </c>
       <c r="V12" t="s">
+        <v>89</v>
+      </c>
+      <c r="W12" t="s">
         <v>90</v>
-      </c>
-      <c r="W12" t="s">
-        <v>91</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/09/2026 13:59)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -277,13 +277,13 @@
     <t>MATERIAL EM TRANSITO - RECIBO 796/FAB/26 AWB 12757879883, DPE 19/09/2026 RC 16/09/2026</t>
   </si>
   <si>
-    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0146 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026</t>
-  </si>
-  <si>
-    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0132 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003156622 - será enviado direto para o Brasil</t>
+    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0146 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026 / MATERIAL ENVIADO VIA RECIBO 804//FAB/26. AWB - 12758218764. DPE 19/09/26. Lucas 18/09/26</t>
+  </si>
+  <si>
+    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0132 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026 / MATERIAL ENVIADO VIA RECIBO 804//FAB/26. AWB - 12758218764. DPE 19/09/26. Lucas 18/09/26</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -296,16 +296,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -321,7 +313,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -329,30 +321,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -652,85 +626,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -762,10 +736,10 @@
       <c r="I2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46238</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -774,17 +748,17 @@
       <c r="M2" t="s">
         <v>71</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46269</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="R2">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="S2" t="s">
         <v>72</v>
@@ -830,10 +804,10 @@
       <c r="I3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -842,17 +816,17 @@
       <c r="M3" t="s">
         <v>71</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R3">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="S3" t="s">
         <v>72</v>
@@ -896,12 +870,12 @@
         <v>67</v>
       </c>
       <c r="I4" t="s">
-        <v>70</v>
-      </c>
-      <c r="J4" s="2">
+        <v>69</v>
+      </c>
+      <c r="J4" s="1">
         <v>46253</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -910,14 +884,14 @@
       <c r="M4" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="2">
-        <v>46263</v>
+      <c r="N4" s="1">
+        <v>46283</v>
       </c>
       <c r="Q4">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="R4">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S4" t="s">
         <v>72</v>
@@ -960,10 +934,10 @@
       <c r="I5" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46254</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -972,17 +946,17 @@
       <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46286</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="R5">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="S5" t="s">
         <v>72</v>
@@ -1031,10 +1005,10 @@
       <c r="I6" t="s">
         <v>69</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46265</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46266</v>
       </c>
       <c r="L6">
@@ -1043,17 +1017,17 @@
       <c r="M6" t="s">
         <v>71</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46297</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46280</v>
       </c>
       <c r="Q6">
-        <v>-14</v>
+        <v>-11</v>
       </c>
       <c r="R6">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="S6" t="s">
         <v>73</v>
@@ -1102,10 +1076,10 @@
       <c r="I7" t="s">
         <v>70</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46275</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46275</v>
       </c>
       <c r="L7">
@@ -1114,14 +1088,14 @@
       <c r="M7" t="s">
         <v>71</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46286</v>
       </c>
       <c r="Q7">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="R7">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
         <v>72</v>
@@ -1170,10 +1144,10 @@
       <c r="I8" t="s">
         <v>70</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46280</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46281</v>
       </c>
       <c r="L8">
@@ -1182,17 +1156,17 @@
       <c r="M8" t="s">
         <v>71</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46292</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46283</v>
       </c>
       <c r="Q8">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S8" t="s">
         <v>73</v>
@@ -1241,10 +1215,10 @@
       <c r="I9" t="s">
         <v>70</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46280</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46281</v>
       </c>
       <c r="L9">
@@ -1253,17 +1227,17 @@
       <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46292</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46284</v>
       </c>
       <c r="Q9">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
         <v>72</v>
@@ -1312,10 +1286,10 @@
       <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46279</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46281</v>
       </c>
       <c r="L10">
@@ -1324,17 +1298,17 @@
       <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46312</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10" s="1">
         <v>46288</v>
       </c>
       <c r="Q10">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>72</v>
@@ -1383,10 +1357,10 @@
       <c r="I11" t="s">
         <v>69</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46279</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46281</v>
       </c>
       <c r="L11">
@@ -1395,17 +1369,17 @@
       <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46312</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11" s="1">
         <v>46288</v>
       </c>
       <c r="Q11">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>72</v>
@@ -1454,10 +1428,10 @@
       <c r="I12" t="s">
         <v>69</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46279</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46281</v>
       </c>
       <c r="L12">
@@ -1466,17 +1440,17 @@
       <c r="M12" t="s">
         <v>71</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46312</v>
       </c>
-      <c r="O12" s="2">
+      <c r="O12" s="1">
         <v>46288</v>
       </c>
       <c r="Q12">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/09/2026 14:29)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -296,8 +296,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -313,7 +321,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -321,12 +329,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -626,85 +652,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -736,10 +762,10 @@
       <c r="I2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -748,10 +774,10 @@
       <c r="M2" t="s">
         <v>71</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -804,10 +830,10 @@
       <c r="I3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -816,10 +842,10 @@
       <c r="M3" t="s">
         <v>71</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -872,10 +898,10 @@
       <c r="I4" t="s">
         <v>69</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46252</v>
       </c>
       <c r="L4">
@@ -884,7 +910,7 @@
       <c r="M4" t="s">
         <v>71</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46283</v>
       </c>
       <c r="Q4">
@@ -934,10 +960,10 @@
       <c r="I5" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -946,10 +972,10 @@
       <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
@@ -1005,10 +1031,10 @@
       <c r="I6" t="s">
         <v>69</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46265</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46266</v>
       </c>
       <c r="L6">
@@ -1017,10 +1043,10 @@
       <c r="M6" t="s">
         <v>71</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46297</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46280</v>
       </c>
       <c r="Q6">
@@ -1076,10 +1102,10 @@
       <c r="I7" t="s">
         <v>70</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46275</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46275</v>
       </c>
       <c r="L7">
@@ -1088,7 +1114,7 @@
       <c r="M7" t="s">
         <v>71</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46286</v>
       </c>
       <c r="Q7">
@@ -1144,10 +1170,10 @@
       <c r="I8" t="s">
         <v>70</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46280</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46281</v>
       </c>
       <c r="L8">
@@ -1156,10 +1182,10 @@
       <c r="M8" t="s">
         <v>71</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46292</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46283</v>
       </c>
       <c r="Q8">
@@ -1215,10 +1241,10 @@
       <c r="I9" t="s">
         <v>70</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46280</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46281</v>
       </c>
       <c r="L9">
@@ -1227,10 +1253,10 @@
       <c r="M9" t="s">
         <v>71</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46292</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46284</v>
       </c>
       <c r="Q9">
@@ -1286,10 +1312,10 @@
       <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46279</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46281</v>
       </c>
       <c r="L10">
@@ -1298,10 +1324,10 @@
       <c r="M10" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46312</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="2">
         <v>46288</v>
       </c>
       <c r="Q10">
@@ -1357,10 +1383,10 @@
       <c r="I11" t="s">
         <v>69</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46279</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46281</v>
       </c>
       <c r="L11">
@@ -1369,10 +1395,10 @@
       <c r="M11" t="s">
         <v>71</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46312</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="2">
         <v>46288</v>
       </c>
       <c r="Q11">
@@ -1428,10 +1454,10 @@
       <c r="I12" t="s">
         <v>69</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46279</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46281</v>
       </c>
       <c r="L12">
@@ -1440,10 +1466,10 @@
       <c r="M12" t="s">
         <v>71</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46312</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="2">
         <v>46288</v>
       </c>
       <c r="Q12">

</xml_diff>

<commit_message>
Atualização automática: emergencias (22/09/2026 12:30)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="82">
   <si>
     <t>om_emg</t>
   </si>
@@ -124,15 +124,9 @@
     <t>690260002556</t>
   </si>
   <si>
-    <t>685260012775</t>
-  </si>
-  <si>
     <t>313260018745</t>
   </si>
   <si>
-    <t>313260018746</t>
-  </si>
-  <si>
     <t>685260012785</t>
   </si>
   <si>
@@ -157,15 +151,9 @@
     <t>C592001-0206</t>
   </si>
   <si>
-    <t>060-0017-00</t>
-  </si>
-  <si>
     <t>702801-5</t>
   </si>
   <si>
-    <t>3244897-4</t>
-  </si>
-  <si>
     <t>S2889-3-0132</t>
   </si>
   <si>
@@ -190,15 +178,9 @@
     <t>WICK-STAT DISC</t>
   </si>
   <si>
-    <t>FLIGHT DIR HOR</t>
-  </si>
-  <si>
     <t>FUEL PUMP</t>
   </si>
   <si>
-    <t>FUEL CONTROL UNIT</t>
-  </si>
-  <si>
     <t>HOSE ASSY BRAKE CYL</t>
   </si>
   <si>
@@ -226,7 +208,7 @@
     <t>ANCE</t>
   </si>
   <si>
-    <t>IPLR</t>
+    <t>AIFP</t>
   </si>
   <si>
     <t>EA</t>
@@ -238,19 +220,16 @@
     <t>Sim</t>
   </si>
   <si>
+    <t>Emg aberta equivocadamente como ANCE. Alterado para AIFP e será contabilizado assim a partir do dia 22/09. Ramon 21/09/26</t>
+  </si>
+  <si>
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
     <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026. AWB 127-5594 5035 - volume retirado na loja GOLLOG - CGR por givanildo em 14/09. Godoy 17/09/26.</t>
   </si>
   <si>
-    <t>AWB 127-5676 0804 -  volume retirado na loja GOLLOG - NAT por Teodoro silva em 11/09 - Godoy 16/09/26.</t>
-  </si>
-  <si>
-    <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737. será atendido pelo estoque FAB pedido n° 18443495. Godoy 16/09/26</t>
-  </si>
-  <si>
-    <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737.</t>
+    <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737. será atendido pelo estoque FAB pedido n° 18443495. Godoy 16/09/26 AWB 127-5790 1454 liberado para retirada em 18/09. Ramon 21/09/26</t>
   </si>
   <si>
     <t>Operador pediu para fornecer o PN informado. Godoy 18/09/26.</t>
@@ -268,13 +247,7 @@
     <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ - Material disponivel para coleta, em contato com a transportadora rc 10/09/2026 - material entregue dia 15/09/2026</t>
   </si>
   <si>
-    <t>SERÁ ENVIADO DA BASE PAMALS, ITEM ENVIANO DIA 10-09-2026, AWB 127-5676 0804, RECIBO ASSINADO NO DRIVE-CLA-14-09</t>
-  </si>
-  <si>
     <t>MATERIAL POSSUI NO ESTOQUE FAB, AGUARDANDO LIBERAÇÃO PARA ATENDIMENTO DE EMERGENCIA RC 16/09/2026 - item foi envado no dia 16-09-26 AWB 127-5790 1454 -CLA 16-09</t>
-  </si>
-  <si>
-    <t>MATERIAL EM TRANSITO - RECIBO 796/FAB/26 AWB 12757879883, DPE 19/09/2026 RC 16/09/2026</t>
   </si>
   <si>
     <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0146 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026 / MATERIAL ENVIADO VIA RECIBO 804//FAB/26. AWB - 12758218764. DPE 19/09/26. Lucas 18/09/26</t>
@@ -296,16 +269,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -321,7 +286,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -329,30 +294,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -648,89 +595,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -745,58 +692,58 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J2" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K2" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N2" s="1">
+        <v>46269</v>
+      </c>
+      <c r="O2" s="1">
+        <v>46269</v>
+      </c>
+      <c r="Q2">
+        <v>18</v>
+      </c>
+      <c r="R2">
+        <v>49</v>
+      </c>
+      <c r="S2" t="s">
+        <v>66</v>
+      </c>
+      <c r="T2" t="s">
         <v>67</v>
       </c>
-      <c r="I2" t="s">
-        <v>69</v>
-      </c>
-      <c r="J2" s="2">
-        <v>46238</v>
-      </c>
-      <c r="K2" s="2">
-        <v>46238</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2" t="s">
-        <v>71</v>
-      </c>
-      <c r="N2" s="2">
-        <v>46269</v>
-      </c>
-      <c r="O2" s="2">
-        <v>46269</v>
-      </c>
-      <c r="Q2">
-        <v>17</v>
-      </c>
-      <c r="R2">
-        <v>48</v>
-      </c>
-      <c r="S2" t="s">
-        <v>72</v>
-      </c>
-      <c r="T2" t="s">
+      <c r="V2" t="s">
         <v>73</v>
       </c>
-      <c r="V2" t="s">
-        <v>80</v>
-      </c>
       <c r="W2" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -813,58 +760,58 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
-      </c>
-      <c r="J3" s="2">
+        <v>63</v>
+      </c>
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>71</v>
-      </c>
-      <c r="N3" s="2">
+        <v>65</v>
+      </c>
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R3">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="S3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="T3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="V3" t="s">
+        <v>74</v>
+      </c>
+      <c r="W3" t="s">
         <v>81</v>
-      </c>
-      <c r="W3" t="s">
-        <v>90</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -881,52 +828,55 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J4" s="1">
+        <v>46253</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46287</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
+        <v>65</v>
+      </c>
+      <c r="N4" s="1">
+        <v>46294</v>
+      </c>
+      <c r="Q4">
+        <v>-7</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4" t="s">
+        <v>66</v>
+      </c>
+      <c r="T4" t="s">
         <v>67</v>
       </c>
-      <c r="I4" t="s">
-        <v>69</v>
-      </c>
-      <c r="J4" s="2">
-        <v>46253</v>
-      </c>
-      <c r="K4" s="2">
-        <v>46252</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4" t="s">
-        <v>71</v>
-      </c>
-      <c r="N4" s="2">
-        <v>46283</v>
-      </c>
-      <c r="Q4">
-        <v>3</v>
-      </c>
-      <c r="R4">
-        <v>34</v>
-      </c>
-      <c r="S4" t="s">
-        <v>72</v>
-      </c>
-      <c r="T4" t="s">
-        <v>73</v>
+      <c r="U4" t="s">
+        <v>68</v>
       </c>
       <c r="W4" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -943,61 +893,61 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="I5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J5" s="2">
+        <v>63</v>
+      </c>
+      <c r="J5" s="1">
         <v>46254</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46255</v>
       </c>
       <c r="L5">
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>71</v>
-      </c>
-      <c r="N5" s="2">
+        <v>65</v>
+      </c>
+      <c r="N5" s="1">
         <v>46286</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="T5" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U5" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="V5" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="W5" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1014,61 +964,61 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G6">
         <v>2727</v>
       </c>
       <c r="H6" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I6" t="s">
-        <v>69</v>
-      </c>
-      <c r="J6" s="2">
+        <v>63</v>
+      </c>
+      <c r="J6" s="1">
         <v>46265</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46266</v>
       </c>
       <c r="L6">
         <v>5</v>
       </c>
       <c r="M6" t="s">
-        <v>71</v>
-      </c>
-      <c r="N6" s="2">
+        <v>65</v>
+      </c>
+      <c r="N6" s="1">
         <v>46297</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46280</v>
       </c>
       <c r="Q6">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S6" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="T6" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="U6" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="V6" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="W6" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1076,67 +1026,70 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="G7">
-        <v>2729</v>
+        <v>2732</v>
       </c>
       <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7" t="s">
+        <v>64</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46280</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>65</v>
+      </c>
+      <c r="N7" s="1">
+        <v>46288</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46283</v>
+      </c>
+      <c r="Q7">
+        <v>-1</v>
+      </c>
+      <c r="R7">
+        <v>6</v>
+      </c>
+      <c r="S7" t="s">
         <v>67</v>
       </c>
-      <c r="I7" t="s">
-        <v>70</v>
-      </c>
-      <c r="J7" s="2">
-        <v>46275</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46275</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="T7" t="s">
+        <v>67</v>
+      </c>
+      <c r="U7" t="s">
         <v>71</v>
       </c>
-      <c r="N7" s="2">
-        <v>46286</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>11</v>
-      </c>
-      <c r="S7" t="s">
-        <v>72</v>
-      </c>
-      <c r="T7" t="s">
-        <v>73</v>
-      </c>
-      <c r="U7" t="s">
-        <v>76</v>
-      </c>
       <c r="V7" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="W7" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1144,70 +1097,70 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F8" t="s">
+        <v>58</v>
+      </c>
+      <c r="G8">
+        <v>2702</v>
+      </c>
+      <c r="H8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>65</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46312</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46288</v>
+      </c>
+      <c r="Q8">
+        <v>-25</v>
+      </c>
+      <c r="R8">
+        <v>6</v>
+      </c>
+      <c r="S8" t="s">
         <v>66</v>
       </c>
-      <c r="G8">
-        <v>2732</v>
-      </c>
-      <c r="H8" t="s">
-        <v>68</v>
-      </c>
-      <c r="I8" t="s">
-        <v>70</v>
-      </c>
-      <c r="J8" s="2">
-        <v>46280</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>71</v>
-      </c>
-      <c r="N8" s="2">
-        <v>46292</v>
-      </c>
-      <c r="O8" s="2">
-        <v>46283</v>
-      </c>
-      <c r="Q8">
-        <v>-6</v>
-      </c>
-      <c r="R8">
-        <v>5</v>
-      </c>
-      <c r="S8" t="s">
-        <v>73</v>
-      </c>
       <c r="T8" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="U8" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="V8" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="W8" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1215,70 +1168,70 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9">
+        <v>2702</v>
+      </c>
+      <c r="H9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" t="s">
+        <v>63</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>65</v>
+      </c>
+      <c r="N9" s="1">
+        <v>46312</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46288</v>
+      </c>
+      <c r="Q9">
+        <v>-25</v>
+      </c>
+      <c r="R9">
+        <v>6</v>
+      </c>
+      <c r="S9" t="s">
         <v>66</v>
       </c>
-      <c r="G9">
-        <v>2732</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="T9" t="s">
         <v>67</v>
       </c>
-      <c r="I9" t="s">
-        <v>70</v>
-      </c>
-      <c r="J9" s="2">
-        <v>46280</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>71</v>
-      </c>
-      <c r="N9" s="2">
-        <v>46292</v>
-      </c>
-      <c r="O9" s="2">
-        <v>46284</v>
-      </c>
-      <c r="Q9">
-        <v>-6</v>
-      </c>
-      <c r="R9">
-        <v>5</v>
-      </c>
-      <c r="S9" t="s">
+      <c r="U9" t="s">
         <v>72</v>
       </c>
-      <c r="T9" t="s">
-        <v>73</v>
-      </c>
-      <c r="U9" t="s">
-        <v>78</v>
-      </c>
       <c r="V9" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="W9" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1295,202 +1248,60 @@
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G10">
         <v>2702</v>
       </c>
       <c r="H10" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" t="s">
+        <v>63</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>65</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46312</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46288</v>
+      </c>
+      <c r="Q10">
+        <v>-25</v>
+      </c>
+      <c r="R10">
+        <v>6</v>
+      </c>
+      <c r="S10" t="s">
+        <v>66</v>
+      </c>
+      <c r="T10" t="s">
         <v>67</v>
       </c>
-      <c r="I10" t="s">
-        <v>69</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>71</v>
-      </c>
-      <c r="N10" s="2">
-        <v>46312</v>
-      </c>
-      <c r="O10" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q10">
-        <v>-26</v>
-      </c>
-      <c r="R10">
-        <v>5</v>
-      </c>
-      <c r="S10" t="s">
-        <v>72</v>
-      </c>
-      <c r="T10" t="s">
-        <v>73</v>
-      </c>
-      <c r="U10" t="s">
-        <v>79</v>
-      </c>
       <c r="V10" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="W10" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27">
-      <c r="A11">
-        <v>685</v>
-      </c>
-      <c r="B11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G11">
-        <v>2702</v>
-      </c>
-      <c r="H11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I11" t="s">
-        <v>69</v>
-      </c>
-      <c r="J11" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>71</v>
-      </c>
-      <c r="N11" s="2">
-        <v>46312</v>
-      </c>
-      <c r="O11" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q11">
-        <v>-26</v>
-      </c>
-      <c r="R11">
-        <v>5</v>
-      </c>
-      <c r="S11" t="s">
-        <v>72</v>
-      </c>
-      <c r="T11" t="s">
-        <v>73</v>
-      </c>
-      <c r="U11" t="s">
-        <v>79</v>
-      </c>
-      <c r="V11" t="s">
-        <v>88</v>
-      </c>
-      <c r="W11" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27">
-      <c r="A12">
-        <v>685</v>
-      </c>
-      <c r="B12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" t="s">
-        <v>64</v>
-      </c>
-      <c r="G12">
-        <v>2702</v>
-      </c>
-      <c r="H12" t="s">
-        <v>67</v>
-      </c>
-      <c r="I12" t="s">
-        <v>69</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>71</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46312</v>
-      </c>
-      <c r="O12" s="2">
-        <v>46288</v>
-      </c>
-      <c r="Q12">
-        <v>-26</v>
-      </c>
-      <c r="R12">
-        <v>5</v>
-      </c>
-      <c r="S12" t="s">
-        <v>72</v>
-      </c>
-      <c r="T12" t="s">
-        <v>73</v>
-      </c>
-      <c r="V12" t="s">
-        <v>89</v>
-      </c>
-      <c r="W12" t="s">
-        <v>90</v>
-      </c>
-      <c r="AA12" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/09/2026 10:01)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="69">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,9 +103,6 @@
     <t>BAMN</t>
   </si>
   <si>
-    <t>BACG</t>
-  </si>
-  <si>
     <t>BANT</t>
   </si>
   <si>
@@ -121,12 +118,6 @@
     <t>313260018713</t>
   </si>
   <si>
-    <t>690260002556</t>
-  </si>
-  <si>
-    <t>313260018745</t>
-  </si>
-  <si>
     <t>685260012785</t>
   </si>
   <si>
@@ -148,12 +139,6 @@
     <t>2115040-8</t>
   </si>
   <si>
-    <t>C592001-0206</t>
-  </si>
-  <si>
-    <t>702801-5</t>
-  </si>
-  <si>
     <t>S2889-3-0132</t>
   </si>
   <si>
@@ -175,12 +160,6 @@
     <t>CYLINDER GAS S</t>
   </si>
   <si>
-    <t>WICK-STAT DISC</t>
-  </si>
-  <si>
-    <t>FUEL PUMP</t>
-  </si>
-  <si>
     <t>HOSE ASSY BRAKE CYL</t>
   </si>
   <si>
@@ -196,15 +175,9 @@
     <t>T</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Expedido total</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -220,19 +193,13 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>Emg aberta equivocadamente como ANCE. Alterado para AIFP e será contabilizado assim a partir do dia 22/09. Ramon 21/09/26</t>
+    <t>EMG aberta equivocadamente como ANCE. Alterada para AIFP e será contabilizada dessa forma a partir do dia 22/09. Ramon – 21/09/2026.  Conforme apresentado na Carta nº 016/MNT-C98/2026, de 21/09/2026, a empresa informou impeditivos técnicos para a recuperação da PASSENGER DOOR, P/N 2698010-7, especialmente quanto à ausência de escopo homologado e de literatura técnica específica que permita respaldar e certificar o reparo. A contratada também se colocou à disposição para buscar solução em cooperação com os meios técnicos da FAB. Diante da manifestação apresentada, o Fiscal analisará o conteúdo e os argumentos técnicos encaminhados e, durante essa análise, não será aplicada avaliação negativa à empresa quanto a essa ocorrência. Após a conclusão da análise, será emitida resposta formal à contratada. Wallace – 22/09/2026.</t>
   </si>
   <si>
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>Pedido será atendido pelo estoque FAB pedido n° 18353156- Godoy 02/09/2026. AWB 127-5594 5035 - volume retirado na loja GOLLOG - CGR por givanildo em 14/09. Godoy 17/09/26.</t>
-  </si>
-  <si>
-    <t>ITEM DESTA ANV FOI REMOVIDO PARA ATENDER A ANV 2737. será atendido pelo estoque FAB pedido n° 18443495. Godoy 16/09/26 AWB 127-5790 1454 liberado para retirada em 18/09. Ramon 21/09/26</t>
-  </si>
-  <si>
-    <t>Operador pediu para fornecer o PN informado. Godoy 18/09/26.</t>
+    <t>Operador pediu para fornecer o PN informado. Godoy 18/09/26. AWB 12758218764 -  volume retirado na loja GOLLOG - NAT por teodoro silva no dia 21/09. Godoy 22/09/26.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -242,12 +209,6 @@
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador dia 03/09/26 - AWB 127-5594 5035- REZ - Material disponivel para coleta, em contato com a transportadora rc 10/09/2026 - material entregue dia 15/09/2026</t>
-  </si>
-  <si>
-    <t>MATERIAL POSSUI NO ESTOQUE FAB, AGUARDANDO LIBERAÇÃO PARA ATENDIMENTO DE EMERGENCIA RC 16/09/2026 - item foi envado no dia 16-09-26 AWB 127-5790 1454 -CLA 16-09</t>
   </si>
   <si>
     <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0146 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026 / MATERIAL ENVIADO VIA RECIBO 804//FAB/26. AWB - 12758218764. DPE 19/09/26. Lucas 18/09/26</t>
@@ -269,8 +230,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -286,7 +255,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -294,12 +263,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -595,89 +582,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -689,61 +676,61 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="I2" t="s">
-        <v>63</v>
-      </c>
-      <c r="J2" s="1">
+        <v>54</v>
+      </c>
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>65</v>
-      </c>
-      <c r="N2" s="1">
+        <v>56</v>
+      </c>
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="S2" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="T2" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="V2" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="W2" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -757,61 +744,61 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="I3" t="s">
-        <v>63</v>
-      </c>
-      <c r="J3" s="1">
+        <v>54</v>
+      </c>
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>65</v>
-      </c>
-      <c r="N3" s="1">
+        <v>56</v>
+      </c>
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R3">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S3" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="T3" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="V3" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="W3" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -825,58 +812,58 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="I4" t="s">
-        <v>64</v>
-      </c>
-      <c r="J4" s="1">
+        <v>55</v>
+      </c>
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46287</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>65</v>
-      </c>
-      <c r="N4" s="1">
+        <v>56</v>
+      </c>
+      <c r="N4" s="2">
         <v>46294</v>
       </c>
       <c r="Q4">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S4" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="T4" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="U4" t="s">
+        <v>59</v>
+      </c>
+      <c r="W4" t="s">
         <v>68</v>
-      </c>
-      <c r="W4" t="s">
-        <v>81</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -890,64 +877,64 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="I5" t="s">
-        <v>63</v>
-      </c>
-      <c r="J5" s="1">
+        <v>54</v>
+      </c>
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>65</v>
-      </c>
-      <c r="N5" s="1">
+        <v>56</v>
+      </c>
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R5">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S5" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="T5" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="U5" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="V5" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="W5" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -955,70 +942,70 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6">
+        <v>2702</v>
+      </c>
+      <c r="H6" t="s">
         <v>53</v>
       </c>
-      <c r="F6" t="s">
+      <c r="I6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" s="2">
+        <v>46279</v>
+      </c>
+      <c r="K6" s="2">
+        <v>46281</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
+        <v>56</v>
+      </c>
+      <c r="N6" s="2">
+        <v>46312</v>
+      </c>
+      <c r="O6" s="2">
+        <v>46288</v>
+      </c>
+      <c r="Q6">
+        <v>-24</v>
+      </c>
+      <c r="R6">
+        <v>7</v>
+      </c>
+      <c r="S6" t="s">
+        <v>57</v>
+      </c>
+      <c r="T6" t="s">
         <v>58</v>
       </c>
-      <c r="G6">
-        <v>2727</v>
-      </c>
-      <c r="H6" t="s">
-        <v>62</v>
-      </c>
-      <c r="I6" t="s">
-        <v>63</v>
-      </c>
-      <c r="J6" s="1">
-        <v>46265</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46266</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6" t="s">
+      <c r="U6" t="s">
+        <v>61</v>
+      </c>
+      <c r="V6" t="s">
         <v>65</v>
       </c>
-      <c r="N6" s="1">
-        <v>46297</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46280</v>
-      </c>
-      <c r="Q6">
-        <v>-10</v>
-      </c>
-      <c r="R6">
-        <v>21</v>
-      </c>
-      <c r="S6" t="s">
-        <v>67</v>
-      </c>
-      <c r="T6" t="s">
-        <v>66</v>
-      </c>
-      <c r="U6" t="s">
-        <v>70</v>
-      </c>
-      <c r="V6" t="s">
-        <v>76</v>
-      </c>
       <c r="W6" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1026,70 +1013,70 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7">
+        <v>2702</v>
+      </c>
+      <c r="H7" t="s">
+        <v>53</v>
+      </c>
+      <c r="I7" t="s">
         <v>54</v>
       </c>
-      <c r="F7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G7">
-        <v>2732</v>
-      </c>
-      <c r="H7" t="s">
-        <v>62</v>
-      </c>
-      <c r="I7" t="s">
-        <v>64</v>
-      </c>
-      <c r="J7" s="1">
-        <v>46280</v>
-      </c>
-      <c r="K7" s="1">
+      <c r="J7" s="2">
+        <v>46279</v>
+      </c>
+      <c r="K7" s="2">
         <v>46281</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>65</v>
-      </c>
-      <c r="N7" s="1">
+        <v>56</v>
+      </c>
+      <c r="N7" s="2">
+        <v>46312</v>
+      </c>
+      <c r="O7" s="2">
         <v>46288</v>
       </c>
-      <c r="O7" s="1">
-        <v>46283</v>
-      </c>
       <c r="Q7">
-        <v>-1</v>
+        <v>-24</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="T7" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="U7" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="V7" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="W7" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1100,208 +1087,66 @@
         <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="G8">
         <v>2702</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="I8" t="s">
-        <v>63</v>
-      </c>
-      <c r="J8" s="1">
+        <v>54</v>
+      </c>
+      <c r="J8" s="2">
         <v>46279</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46281</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>65</v>
-      </c>
-      <c r="N8" s="1">
+        <v>56</v>
+      </c>
+      <c r="N8" s="2">
         <v>46312</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46288</v>
       </c>
       <c r="Q8">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="T8" t="s">
+        <v>58</v>
+      </c>
+      <c r="V8" t="s">
         <v>67</v>
       </c>
-      <c r="U8" t="s">
-        <v>72</v>
-      </c>
-      <c r="V8" t="s">
-        <v>78</v>
-      </c>
       <c r="W8" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="AA8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27">
-      <c r="A9">
-        <v>685</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" t="s">
-        <v>58</v>
-      </c>
-      <c r="G9">
-        <v>2702</v>
-      </c>
-      <c r="H9" t="s">
-        <v>61</v>
-      </c>
-      <c r="I9" t="s">
-        <v>63</v>
-      </c>
-      <c r="J9" s="1">
-        <v>46279</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46281</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>65</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46312</v>
-      </c>
-      <c r="O9" s="1">
-        <v>46288</v>
-      </c>
-      <c r="Q9">
-        <v>-25</v>
-      </c>
-      <c r="R9">
-        <v>6</v>
-      </c>
-      <c r="S9" t="s">
-        <v>66</v>
-      </c>
-      <c r="T9" t="s">
-        <v>67</v>
-      </c>
-      <c r="U9" t="s">
-        <v>72</v>
-      </c>
-      <c r="V9" t="s">
-        <v>79</v>
-      </c>
-      <c r="W9" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27">
-      <c r="A10">
-        <v>685</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10">
-        <v>2702</v>
-      </c>
-      <c r="H10" t="s">
-        <v>61</v>
-      </c>
-      <c r="I10" t="s">
-        <v>63</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46279</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46281</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>65</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46312</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46288</v>
-      </c>
-      <c r="Q10">
-        <v>-25</v>
-      </c>
-      <c r="R10">
-        <v>6</v>
-      </c>
-      <c r="S10" t="s">
-        <v>66</v>
-      </c>
-      <c r="T10" t="s">
-        <v>67</v>
-      </c>
-      <c r="V10" t="s">
-        <v>80</v>
-      </c>
-      <c r="W10" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA10" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/09/2026 12:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -230,16 +230,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -255,7 +247,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -263,30 +255,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -586,85 +560,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -696,10 +670,10 @@
       <c r="I2" t="s">
         <v>54</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46238</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -708,10 +682,10 @@
       <c r="M2" t="s">
         <v>56</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46269</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -764,10 +738,10 @@
       <c r="I3" t="s">
         <v>54</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -776,10 +750,10 @@
       <c r="M3" t="s">
         <v>56</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -832,10 +806,10 @@
       <c r="I4" t="s">
         <v>55</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46253</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46287</v>
       </c>
       <c r="L4">
@@ -844,7 +818,7 @@
       <c r="M4" t="s">
         <v>56</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46294</v>
       </c>
       <c r="Q4">
@@ -897,10 +871,10 @@
       <c r="I5" t="s">
         <v>54</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46254</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46255</v>
       </c>
       <c r="L5">
@@ -909,10 +883,10 @@
       <c r="M5" t="s">
         <v>56</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46286</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46258</v>
       </c>
       <c r="Q5">
@@ -968,10 +942,10 @@
       <c r="I6" t="s">
         <v>54</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46279</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46281</v>
       </c>
       <c r="L6">
@@ -980,10 +954,10 @@
       <c r="M6" t="s">
         <v>56</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46312</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46288</v>
       </c>
       <c r="Q6">
@@ -1039,10 +1013,10 @@
       <c r="I7" t="s">
         <v>54</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46279</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46281</v>
       </c>
       <c r="L7">
@@ -1051,10 +1025,10 @@
       <c r="M7" t="s">
         <v>56</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46312</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46288</v>
       </c>
       <c r="Q7">
@@ -1110,10 +1084,10 @@
       <c r="I8" t="s">
         <v>54</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46279</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46281</v>
       </c>
       <c r="L8">
@@ -1122,10 +1096,10 @@
       <c r="M8" t="s">
         <v>56</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46312</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46288</v>
       </c>
       <c r="Q8">

</xml_diff>

<commit_message>
Atualização automática: emergencias (24/09/2026 12:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -689,10 +689,10 @@
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="S2" t="s">
         <v>57</v>
@@ -757,10 +757,10 @@
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="R3">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="S3" t="s">
         <v>57</v>
@@ -822,10 +822,10 @@
         <v>46294</v>
       </c>
       <c r="Q4">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S4" t="s">
         <v>57</v>
@@ -890,10 +890,10 @@
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S5" t="s">
         <v>57</v>
@@ -961,10 +961,10 @@
         <v>46288</v>
       </c>
       <c r="Q6">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s">
         <v>57</v>
@@ -1032,10 +1032,10 @@
         <v>46288</v>
       </c>
       <c r="Q7">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S7" t="s">
         <v>57</v>
@@ -1103,10 +1103,10 @@
         <v>46288</v>
       </c>
       <c r="Q8">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S8" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (25/09/2026 12:49)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="71">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,6 +106,9 @@
     <t>BANT</t>
   </si>
   <si>
+    <t>CLA</t>
+  </si>
+  <si>
     <t>396260016580</t>
   </si>
   <si>
@@ -118,15 +121,15 @@
     <t>313260018713</t>
   </si>
   <si>
-    <t>685260012785</t>
-  </si>
-  <si>
-    <t>685260012786</t>
-  </si>
-  <si>
     <t>685260012787</t>
   </si>
   <si>
+    <t>419260000560</t>
+  </si>
+  <si>
+    <t>685260012831</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -139,15 +142,15 @@
     <t>2115040-8</t>
   </si>
   <si>
-    <t>S2889-3-0132</t>
-  </si>
-  <si>
-    <t>S2889-3-0146</t>
-  </si>
-  <si>
     <t>S2889-3-0112</t>
   </si>
   <si>
+    <t>065-0042-03</t>
+  </si>
+  <si>
+    <t>2641008-200</t>
+  </si>
+  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -160,21 +163,24 @@
     <t>CYLINDER GAS S</t>
   </si>
   <si>
-    <t>HOSE ASSY BRAKE CYL</t>
-  </si>
-  <si>
-    <t>HOSE ASSY BRAK</t>
-  </si>
-  <si>
     <t>HOSE ASSY TEE</t>
   </si>
   <si>
+    <t>COMPUTER PA</t>
+  </si>
+  <si>
+    <t>PIN-MAIN GEAR ATTACH</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
     <t>T</t>
   </si>
   <si>
+    <t>R</t>
+  </si>
+  <si>
     <t>Providência tomada</t>
   </si>
   <si>
@@ -184,6 +190,9 @@
     <t>AIFP</t>
   </si>
   <si>
+    <t>IPLR</t>
+  </si>
+  <si>
     <t>EA</t>
   </si>
   <si>
@@ -199,22 +208,19 @@
     <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
   </si>
   <si>
-    <t>Operador pediu para fornecer o PN informado. Godoy 18/09/26. AWB 12758218764 -  volume retirado na loja GOLLOG - NAT por teodoro silva no dia 21/09. Godoy 22/09/26.</t>
+    <t>O atendimento deve ser do PN 065-0042-03. Ramon 25/09/26</t>
+  </si>
+  <si>
+    <t>Emergência aberta como IPLR e lançado errado na planilha. Ramon 25/09/26</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - entregue em Campinas 16/09</t>
+    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - entregue em Campinas 16/09 - MATERIAL SENDO ENVIADO DIA 22/09/2026, ESTAVAMOS CONFIRMANDO O PN COM O FORNECEDOR, RECEBEMOS O PN 040-0046 AWB 12759015025 dpe 26/09/2026</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
-  </si>
-  <si>
-    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0146 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026 / MATERIAL ENVIADO VIA RECIBO 804//FAB/26. AWB - 12758218764. DPE 19/09/26. Lucas 18/09/26</t>
-  </si>
-  <si>
-    <t>POR FAVOR, PODERIAM CONFIRMAR SE O PN AE3663231B0132 SERIA COMPATÍVEL COM A AERONAVE, PARA ATENDIMENTO A EMERGENCIA RC 16/09/2026 / MATERIAL ENVIADO VIA RECIBO 804//FAB/26. AWB - 12758218764. DPE 19/09/26. Lucas 18/09/26</t>
   </si>
   <si>
     <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09</t>
@@ -650,25 +656,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J2" s="1">
         <v>46238</v>
@@ -680,7 +686,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N2" s="1">
         <v>46269</v>
@@ -689,22 +695,22 @@
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="S2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="T2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="V2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="W2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -718,25 +724,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J3" s="1">
         <v>46251</v>
@@ -748,7 +754,7 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N3" s="1">
         <v>46280</v>
@@ -757,22 +763,22 @@
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R3">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="S3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="T3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="V3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="W3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -786,25 +792,25 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J4" s="1">
         <v>46253</v>
@@ -816,28 +822,28 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N4" s="1">
         <v>46294</v>
       </c>
       <c r="Q4">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="T4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="U4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="W4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -851,25 +857,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J5" s="1">
         <v>46254</v>
@@ -881,7 +887,7 @@
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N5" s="1">
         <v>46286</v>
@@ -890,25 +896,25 @@
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R5">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="S5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="T5" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="U5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="V5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="W5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -922,25 +928,25 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G6">
         <v>2702</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J6" s="1">
         <v>46279</v>
@@ -952,7 +958,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N6" s="1">
         <v>46312</v>
@@ -961,25 +967,22 @@
         <v>46288</v>
       </c>
       <c r="Q6">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="T6" t="s">
-        <v>58</v>
-      </c>
-      <c r="U6" t="s">
         <v>61</v>
       </c>
       <c r="V6" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="W6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -987,70 +990,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G7">
-        <v>2702</v>
+        <v>2723</v>
       </c>
       <c r="H7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J7" s="1">
-        <v>46279</v>
+        <v>46289</v>
       </c>
       <c r="K7" s="1">
-        <v>46281</v>
+        <v>46289</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N7" s="1">
-        <v>46312</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46288</v>
+        <v>46320</v>
       </c>
       <c r="Q7">
-        <v>-23</v>
+        <v>-30</v>
       </c>
       <c r="R7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="S7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="T7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="U7" t="s">
-        <v>61</v>
-      </c>
-      <c r="V7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="W7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1064,61 +1061,58 @@
         <v>29</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G8">
-        <v>2702</v>
+        <v>2703</v>
       </c>
       <c r="H8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I8" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="J8" s="1">
-        <v>46279</v>
+        <v>46289</v>
       </c>
       <c r="K8" s="1">
-        <v>46281</v>
+        <v>46290</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N8" s="1">
-        <v>46312</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46288</v>
+        <v>46301</v>
       </c>
       <c r="Q8">
-        <v>-23</v>
+        <v>-11</v>
       </c>
       <c r="R8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="T8" t="s">
-        <v>58</v>
-      </c>
-      <c r="V8" t="s">
-        <v>67</v>
+        <v>61</v>
+      </c>
+      <c r="U8" t="s">
+        <v>65</v>
       </c>
       <c r="W8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/09/2026 13:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="88">
   <si>
     <t>om_emg</t>
   </si>
@@ -130,6 +130,18 @@
     <t>685260012831</t>
   </si>
   <si>
+    <t>313260018904</t>
+  </si>
+  <si>
+    <t>313260018905</t>
+  </si>
+  <si>
+    <t>685260012858</t>
+  </si>
+  <si>
+    <t>685260012859</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -151,6 +163,18 @@
     <t>2641008-200</t>
   </si>
   <si>
+    <t>2652022-18</t>
+  </si>
+  <si>
+    <t>2651031-1</t>
+  </si>
+  <si>
+    <t>AS5178W03</t>
+  </si>
+  <si>
+    <t>2643031-7</t>
+  </si>
+  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -172,6 +196,18 @@
     <t>PIN-MAIN GEAR ATTACH</t>
   </si>
   <si>
+    <t>TUBE ASSY</t>
+  </si>
+  <si>
+    <t>LEVER FUEL CON</t>
+  </si>
+  <si>
+    <t>NUT BRAKE SYSTEM</t>
+  </si>
+  <si>
+    <t>FORK ASSY,NOSE GEAR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -184,6 +220,9 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -202,6 +241,9 @@
     <t>Sim</t>
   </si>
   <si>
+    <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26.</t>
+  </si>
+  <si>
     <t>EMG aberta equivocadamente como ANCE. Alterada para AIFP e será contabilizada dessa forma a partir do dia 22/09. Ramon – 21/09/2026.  Conforme apresentado na Carta nº 016/MNT-C98/2026, de 21/09/2026, a empresa informou impeditivos técnicos para a recuperação da PASSENGER DOOR, P/N 2698010-7, especialmente quanto à ausência de escopo homologado e de literatura técnica específica que permita respaldar e certificar o reparo. A contratada também se colocou à disposição para buscar solução em cooperação com os meios técnicos da FAB. Diante da manifestação apresentada, o Fiscal analisará o conteúdo e os argumentos técnicos encaminhados e, durante essa análise, não será aplicada avaliação negativa à empresa quanto a essa ocorrência. Após a conclusão da análise, será emitida resposta formal à contratada. Wallace – 22/09/2026.</t>
   </si>
   <si>
@@ -211,7 +253,13 @@
     <t>O atendimento deve ser do PN 065-0042-03. Ramon 25/09/26</t>
   </si>
   <si>
-    <t>Emergência aberta como IPLR e lançado errado na planilha. Ramon 25/09/26</t>
+    <t>Emergência aberta como IPLR e lançado errado na planilha. Ramon 25/09/26. AWB 12759552135 - volume retirado na loja GOLLOG - NAT por teodoro silva em 25/09. Godoy 28/09/26.</t>
+  </si>
+  <si>
+    <t>Cedeu o item para o 2736. Ramon 28/09/26</t>
+  </si>
+  <si>
+    <t>Estoque do Pn AN924-3D (alternado). Godoy 28/09/26.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -224,6 +272,9 @@
   </si>
   <si>
     <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO DIA 24/09/2026 AWB 12759552135 DPE 25/09/2026 RECIBO 821/FAB/26</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -236,8 +287,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -253,7 +312,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -261,12 +320,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -562,89 +639,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA8"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -659,58 +736,58 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" s="2">
+        <v>46238</v>
+      </c>
+      <c r="K2" s="2">
+        <v>46238</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>72</v>
+      </c>
+      <c r="N2" s="2">
+        <v>46269</v>
+      </c>
+      <c r="O2" s="2">
+        <v>46269</v>
+      </c>
+      <c r="Q2">
+        <v>24</v>
+      </c>
+      <c r="R2">
         <v>55</v>
       </c>
-      <c r="I2" t="s">
-        <v>56</v>
-      </c>
-      <c r="J2" s="1">
-        <v>46238</v>
-      </c>
-      <c r="K2" s="1">
-        <v>46238</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2" t="s">
-        <v>59</v>
-      </c>
-      <c r="N2" s="1">
-        <v>46269</v>
-      </c>
-      <c r="O2" s="1">
-        <v>46269</v>
-      </c>
-      <c r="Q2">
-        <v>21</v>
-      </c>
-      <c r="R2">
-        <v>52</v>
-      </c>
       <c r="S2" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="T2" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="V2" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="W2" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -727,58 +804,61 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>56</v>
-      </c>
-      <c r="J3" s="1">
+        <v>69</v>
+      </c>
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>59</v>
-      </c>
-      <c r="N3" s="1">
+        <v>72</v>
+      </c>
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
-        <v>46280</v>
+      <c r="O3" s="2">
+        <v>46291</v>
       </c>
       <c r="Q3">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="R3">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="S3" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="T3" t="s">
-        <v>61</v>
+        <v>74</v>
+      </c>
+      <c r="U3" t="s">
+        <v>75</v>
       </c>
       <c r="V3" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="W3" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -795,55 +875,55 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="F4" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="I4" t="s">
-        <v>57</v>
-      </c>
-      <c r="J4" s="1">
+        <v>70</v>
+      </c>
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46287</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>59</v>
-      </c>
-      <c r="N4" s="1">
+        <v>72</v>
+      </c>
+      <c r="N4" s="2">
         <v>46294</v>
       </c>
       <c r="Q4">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R4">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S4" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="T4" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="U4" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="W4" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -860,61 +940,61 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="G5">
         <v>2737</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>56</v>
-      </c>
-      <c r="J5" s="1">
+        <v>69</v>
+      </c>
+      <c r="J5" s="2">
         <v>46254</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46255</v>
       </c>
       <c r="L5">
         <v>2</v>
       </c>
       <c r="M5" t="s">
-        <v>59</v>
-      </c>
-      <c r="N5" s="1">
+        <v>72</v>
+      </c>
+      <c r="N5" s="2">
         <v>46286</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46258</v>
       </c>
       <c r="Q5">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="R5">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="S5" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="T5" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="U5" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="V5" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="W5" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -931,58 +1011,58 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="G6">
         <v>2702</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="I6" t="s">
-        <v>56</v>
-      </c>
-      <c r="J6" s="1">
+        <v>69</v>
+      </c>
+      <c r="J6" s="2">
         <v>46279</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46281</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>59</v>
-      </c>
-      <c r="N6" s="1">
+        <v>72</v>
+      </c>
+      <c r="N6" s="2">
         <v>46312</v>
       </c>
-      <c r="O6" s="1">
-        <v>46288</v>
+      <c r="O6" s="2">
+        <v>46312</v>
       </c>
       <c r="Q6">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="R6">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S6" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="T6" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="V6" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="W6" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -999,55 +1079,55 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G7">
         <v>2723</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="I7" t="s">
-        <v>56</v>
-      </c>
-      <c r="J7" s="1">
+        <v>69</v>
+      </c>
+      <c r="J7" s="2">
         <v>46289</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46289</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>59</v>
-      </c>
-      <c r="N7" s="1">
+        <v>72</v>
+      </c>
+      <c r="N7" s="2">
         <v>46320</v>
       </c>
       <c r="Q7">
-        <v>-30</v>
+        <v>-27</v>
       </c>
       <c r="R7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S7" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="T7" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="U7" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="W7" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1064,57 +1144,320 @@
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="G8">
         <v>2703</v>
       </c>
       <c r="H8" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>58</v>
-      </c>
-      <c r="J8" s="1">
+        <v>71</v>
+      </c>
+      <c r="J8" s="2">
         <v>46289</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46290</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>59</v>
-      </c>
-      <c r="N8" s="1">
+        <v>72</v>
+      </c>
+      <c r="N8" s="2">
         <v>46301</v>
       </c>
+      <c r="O8" s="2">
+        <v>46290</v>
+      </c>
       <c r="Q8">
+        <v>-8</v>
+      </c>
+      <c r="R8">
+        <v>3</v>
+      </c>
+      <c r="S8" t="s">
+        <v>74</v>
+      </c>
+      <c r="T8" t="s">
+        <v>74</v>
+      </c>
+      <c r="U8" t="s">
+        <v>79</v>
+      </c>
+      <c r="V8" t="s">
+        <v>86</v>
+      </c>
+      <c r="W8" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27">
+      <c r="A9">
+        <v>313</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9">
+        <v>2734</v>
+      </c>
+      <c r="H9" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" t="s">
+        <v>71</v>
+      </c>
+      <c r="J9" s="2">
+        <v>46290</v>
+      </c>
+      <c r="K9" s="2">
+        <v>46293</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>72</v>
+      </c>
+      <c r="N9" s="2">
+        <v>46304</v>
+      </c>
+      <c r="Q9">
         <v>-11</v>
       </c>
-      <c r="R8">
+      <c r="R9">
         <v>0</v>
       </c>
-      <c r="S8" t="s">
+      <c r="S9" t="s">
+        <v>73</v>
+      </c>
+      <c r="T9" t="s">
+        <v>74</v>
+      </c>
+      <c r="U9" t="s">
+        <v>80</v>
+      </c>
+      <c r="W9" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27">
+      <c r="A10">
+        <v>313</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" t="s">
         <v>61</v>
       </c>
-      <c r="T8" t="s">
-        <v>61</v>
-      </c>
-      <c r="U8" t="s">
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10">
+        <v>2734</v>
+      </c>
+      <c r="H10" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="2">
+        <v>46290</v>
+      </c>
+      <c r="K10" s="2">
+        <v>46293</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>72</v>
+      </c>
+      <c r="N10" s="2">
+        <v>46304</v>
+      </c>
+      <c r="Q10">
+        <v>-11</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10" t="s">
+        <v>73</v>
+      </c>
+      <c r="T10" t="s">
+        <v>74</v>
+      </c>
+      <c r="U10" t="s">
+        <v>80</v>
+      </c>
+      <c r="W10" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="A11">
+        <v>685</v>
+      </c>
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11">
+        <v>2729</v>
+      </c>
+      <c r="H11" t="s">
+        <v>68</v>
+      </c>
+      <c r="I11" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46293</v>
+      </c>
+      <c r="K11" s="2">
+        <v>46293</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>72</v>
+      </c>
+      <c r="N11" s="2">
+        <v>46304</v>
+      </c>
+      <c r="Q11">
+        <v>-11</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11" t="s">
+        <v>74</v>
+      </c>
+      <c r="T11" t="s">
+        <v>74</v>
+      </c>
+      <c r="U11" t="s">
+        <v>81</v>
+      </c>
+      <c r="W11" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="A12">
+        <v>685</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12" t="s">
         <v>65</v>
       </c>
-      <c r="W8" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA8" t="b">
+      <c r="G12">
+        <v>2703</v>
+      </c>
+      <c r="H12" t="s">
+        <v>68</v>
+      </c>
+      <c r="I12" t="s">
+        <v>71</v>
+      </c>
+      <c r="J12" s="2">
+        <v>46293</v>
+      </c>
+      <c r="K12" s="2">
+        <v>46293</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>72</v>
+      </c>
+      <c r="N12" s="2">
+        <v>46304</v>
+      </c>
+      <c r="Q12">
+        <v>-11</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12" t="s">
+        <v>73</v>
+      </c>
+      <c r="T12" t="s">
+        <v>74</v>
+      </c>
+      <c r="W12" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA12" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/09/2026 15:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="83">
   <si>
     <t>om_emg</t>
   </si>
@@ -118,9 +118,6 @@
     <t>313260018708</t>
   </si>
   <si>
-    <t>313260018713</t>
-  </si>
-  <si>
     <t>685260012787</t>
   </si>
   <si>
@@ -151,9 +148,6 @@
     <t>2698010-7</t>
   </si>
   <si>
-    <t>2115040-8</t>
-  </si>
-  <si>
     <t>S2889-3-0112</t>
   </si>
   <si>
@@ -184,9 +178,6 @@
     <t>PASSENGER DOOR - LOW</t>
   </si>
   <si>
-    <t>CYLINDER GAS S</t>
-  </si>
-  <si>
     <t>HOSE ASSY TEE</t>
   </si>
   <si>
@@ -241,15 +232,12 @@
     <t>Sim</t>
   </si>
   <si>
-    <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26.</t>
+    <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
     <t>EMG aberta equivocadamente como ANCE. Alterada para AIFP e será contabilizada dessa forma a partir do dia 22/09. Ramon – 21/09/2026.  Conforme apresentado na Carta nº 016/MNT-C98/2026, de 21/09/2026, a empresa informou impeditivos técnicos para a recuperação da PASSENGER DOOR, P/N 2698010-7, especialmente quanto à ausência de escopo homologado e de literatura técnica específica que permita respaldar e certificar o reparo. A contratada também se colocou à disposição para buscar solução em cooperação com os meios técnicos da FAB. Diante da manifestação apresentada, o Fiscal analisará o conteúdo e os argumentos técnicos encaminhados e, durante essa análise, não será aplicada avaliação negativa à empresa quanto a essa ocorrência. Após a conclusão da análise, será emitida resposta formal à contratada. Wallace – 22/09/2026.</t>
   </si>
   <si>
-    <t>Emergência transformada em ANCE em 24/08. Aguardaremos atendimento com item da Vee One. Ramon 24/08/26.</t>
-  </si>
-  <si>
     <t>O atendimento deve ser do PN 065-0042-03. Ramon 25/09/26</t>
   </si>
   <si>
@@ -259,16 +247,13 @@
     <t>Cedeu o item para o 2736. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>Estoque do Pn AN924-3D (alternado). Godoy 28/09/26.</t>
+    <t>Estoque do Pn AN924-3D (alternado). Godoy 28/09/26. Emerg será atendida pelo estoque FAB pedido 18530012. Godoy 28/09.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
     <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - entregue em Campinas 16/09 - MATERIAL SENDO ENVIADO DIA 22/09/2026, ESTAVAMOS CONFIRMANDO O PN COM O FORNECEDOR, RECEBEMOS O PN 040-0046 AWB 12759015025 dpe 26/09/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido no fornecedor I823285 - entregue em Miami 21/08 - TEMOS 3 EA NO ESTOQUE DA BANT. Material seguiu via awb 12754249845. Recebido por Kleyton em 24/08. Atl Ges.</t>
   </si>
   <si>
     <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09</t>
@@ -287,16 +272,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -312,7 +289,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -320,30 +297,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -639,89 +598,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -736,39 +695,39 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="1">
+        <v>46238</v>
+      </c>
+      <c r="K2" s="1">
+        <v>46238</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="2">
-        <v>46238</v>
-      </c>
-      <c r="K2" s="2">
-        <v>46238</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2" t="s">
-        <v>72</v>
-      </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46269</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -778,16 +737,16 @@
         <v>55</v>
       </c>
       <c r="S2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="T2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="V2" t="s">
+        <v>78</v>
+      </c>
+      <c r="W2" t="s">
         <v>82</v>
-      </c>
-      <c r="W2" t="s">
-        <v>87</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -804,39 +763,39 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
-      </c>
-      <c r="J3" s="2">
+        <v>66</v>
+      </c>
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>72</v>
-      </c>
-      <c r="N3" s="2">
+        <v>69</v>
+      </c>
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46291</v>
       </c>
       <c r="Q3">
@@ -846,19 +805,19 @@
         <v>44</v>
       </c>
       <c r="S3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="T3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="U3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="W3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -875,36 +834,36 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
+        <v>64</v>
+      </c>
+      <c r="I4" t="s">
         <v>67</v>
       </c>
-      <c r="I4" t="s">
-        <v>70</v>
-      </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46253</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46287</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>72</v>
-      </c>
-      <c r="N4" s="2">
+        <v>69</v>
+      </c>
+      <c r="N4" s="1">
         <v>46294</v>
       </c>
       <c r="Q4">
@@ -914,16 +873,16 @@
         <v>6</v>
       </c>
       <c r="S4" t="s">
+        <v>70</v>
+      </c>
+      <c r="T4" t="s">
+        <v>71</v>
+      </c>
+      <c r="U4" t="s">
         <v>73</v>
       </c>
-      <c r="T4" t="s">
-        <v>74</v>
-      </c>
-      <c r="U4" t="s">
-        <v>76</v>
-      </c>
       <c r="W4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -931,70 +890,67 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5">
+        <v>2702</v>
+      </c>
+      <c r="H5" t="s">
         <v>64</v>
       </c>
-      <c r="G5">
-        <v>2737</v>
-      </c>
-      <c r="H5" t="s">
-        <v>67</v>
-      </c>
       <c r="I5" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46281</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
         <v>69</v>
       </c>
-      <c r="J5" s="2">
-        <v>46254</v>
-      </c>
-      <c r="K5" s="2">
-        <v>46255</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5" t="s">
-        <v>72</v>
-      </c>
-      <c r="N5" s="2">
-        <v>46286</v>
-      </c>
-      <c r="O5" s="2">
-        <v>46258</v>
+      <c r="N5" s="1">
+        <v>46312</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46312</v>
       </c>
       <c r="Q5">
-        <v>7</v>
+        <v>-19</v>
       </c>
       <c r="R5">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="S5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="T5" t="s">
-        <v>74</v>
-      </c>
-      <c r="U5" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="V5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="W5" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1002,67 +958,64 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6">
+        <v>2723</v>
+      </c>
+      <c r="H6" t="s">
         <v>64</v>
       </c>
-      <c r="G6">
-        <v>2702</v>
-      </c>
-      <c r="H6" t="s">
-        <v>67</v>
-      </c>
       <c r="I6" t="s">
+        <v>66</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46289</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46289</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
         <v>69</v>
       </c>
-      <c r="J6" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K6" s="2">
-        <v>46281</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>72</v>
-      </c>
-      <c r="N6" s="2">
-        <v>46312</v>
-      </c>
-      <c r="O6" s="2">
-        <v>46312</v>
+      <c r="N6" s="1">
+        <v>46320</v>
       </c>
       <c r="Q6">
-        <v>-19</v>
+        <v>-27</v>
       </c>
       <c r="R6">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="S6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="T6" t="s">
+        <v>70</v>
+      </c>
+      <c r="U6" t="s">
         <v>74</v>
       </c>
-      <c r="V6" t="s">
-        <v>85</v>
-      </c>
       <c r="W6" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1070,64 +1023,70 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F7" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G7">
-        <v>2723</v>
+        <v>2703</v>
       </c>
       <c r="H7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46289</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46290</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>69</v>
       </c>
-      <c r="J7" s="2">
-        <v>46289</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46289</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>72</v>
-      </c>
-      <c r="N7" s="2">
-        <v>46320</v>
+      <c r="N7" s="1">
+        <v>46301</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46290</v>
       </c>
       <c r="Q7">
-        <v>-27</v>
+        <v>-8</v>
       </c>
       <c r="R7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="T7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="U7" t="s">
-        <v>78</v>
+        <v>75</v>
+      </c>
+      <c r="V7" t="s">
+        <v>81</v>
       </c>
       <c r="W7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1135,70 +1094,64 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G8">
-        <v>2703</v>
+        <v>2734</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46290</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46293</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>69</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46304</v>
+      </c>
+      <c r="Q8">
+        <v>-11</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8" t="s">
+        <v>70</v>
+      </c>
+      <c r="T8" t="s">
         <v>71</v>
       </c>
-      <c r="J8" s="2">
-        <v>46289</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46290</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>72</v>
-      </c>
-      <c r="N8" s="2">
-        <v>46301</v>
-      </c>
-      <c r="O8" s="2">
-        <v>46290</v>
-      </c>
-      <c r="Q8">
-        <v>-8</v>
-      </c>
-      <c r="R8">
-        <v>3</v>
-      </c>
-      <c r="S8" t="s">
-        <v>74</v>
-      </c>
-      <c r="T8" t="s">
-        <v>74</v>
-      </c>
       <c r="U8" t="s">
-        <v>79</v>
-      </c>
-      <c r="V8" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="W8" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1215,36 +1168,36 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G9">
         <v>2734</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>71</v>
-      </c>
-      <c r="J9" s="2">
+        <v>68</v>
+      </c>
+      <c r="J9" s="1">
         <v>46290</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46293</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>72</v>
-      </c>
-      <c r="N9" s="2">
+        <v>69</v>
+      </c>
+      <c r="N9" s="1">
         <v>46304</v>
       </c>
       <c r="Q9">
@@ -1254,16 +1207,16 @@
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="T9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="U9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="W9" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1271,45 +1224,45 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" t="s">
         <v>61</v>
       </c>
-      <c r="F10" t="s">
-        <v>64</v>
-      </c>
       <c r="G10">
-        <v>2734</v>
+        <v>2729</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I10" t="s">
-        <v>71</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46290</v>
-      </c>
-      <c r="K10" s="2">
+        <v>68</v>
+      </c>
+      <c r="J10" s="1">
         <v>46293</v>
       </c>
+      <c r="K10" s="1">
+        <v>46293</v>
+      </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>72</v>
-      </c>
-      <c r="N10" s="2">
+        <v>69</v>
+      </c>
+      <c r="N10" s="1">
         <v>46304</v>
       </c>
       <c r="Q10">
@@ -1319,16 +1272,16 @@
         <v>0</v>
       </c>
       <c r="S10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="T10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="U10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="W10" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1345,36 +1298,36 @@
         <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" t="s">
         <v>62</v>
       </c>
-      <c r="F11" t="s">
-        <v>64</v>
-      </c>
       <c r="G11">
-        <v>2729</v>
+        <v>2703</v>
       </c>
       <c r="H11" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" t="s">
         <v>68</v>
       </c>
-      <c r="I11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46293</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46293</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>72</v>
-      </c>
-      <c r="N11" s="2">
+        <v>69</v>
+      </c>
+      <c r="N11" s="1">
         <v>46304</v>
       </c>
       <c r="Q11">
@@ -1384,80 +1337,15 @@
         <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="T11" t="s">
-        <v>74</v>
-      </c>
-      <c r="U11" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="W11" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="AA11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27">
-      <c r="A12">
-        <v>685</v>
-      </c>
-      <c r="B12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G12">
-        <v>2703</v>
-      </c>
-      <c r="H12" t="s">
-        <v>68</v>
-      </c>
-      <c r="I12" t="s">
-        <v>71</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46293</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46293</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>72</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46304</v>
-      </c>
-      <c r="Q12">
-        <v>-11</v>
-      </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12" t="s">
-        <v>73</v>
-      </c>
-      <c r="T12" t="s">
-        <v>74</v>
-      </c>
-      <c r="W12" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA12" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (29/09/2026 13:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="88">
   <si>
     <t>om_emg</t>
   </si>
@@ -139,6 +139,9 @@
     <t>685260012859</t>
   </si>
   <si>
+    <t>685260012864</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -169,6 +172,9 @@
     <t>2643031-7</t>
   </si>
   <si>
+    <t>MS24462-5</t>
+  </si>
+  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -199,6 +205,9 @@
     <t>FORK ASSY,NOSE GEAR</t>
   </si>
   <si>
+    <t>BEARING,ROLLER,NEEDL</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -211,6 +220,9 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
@@ -248,6 +260,9 @@
   </si>
   <si>
     <t>Estoque do Pn AN924-3D (alternado). Godoy 28/09/26. Emerg será atendida pelo estoque FAB pedido 18530012. Godoy 28/09.</t>
+  </si>
+  <si>
+    <t>Emerg será atendida pelo estoque FAB pedido 18540739. Godoy 29/09.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -598,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -695,22 +710,22 @@
         <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J2" s="1">
         <v>46238</v>
@@ -722,7 +737,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N2" s="1">
         <v>46269</v>
@@ -731,22 +746,22 @@
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="S2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="T2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="V2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="W2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -763,22 +778,22 @@
         <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J3" s="1">
         <v>46251</v>
@@ -790,7 +805,7 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N3" s="1">
         <v>46280</v>
@@ -799,25 +814,25 @@
         <v>46291</v>
       </c>
       <c r="Q3">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R3">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="S3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="T3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="U3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="V3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="W3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -834,22 +849,22 @@
         <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="I4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="J4" s="1">
         <v>46253</v>
@@ -861,28 +876,28 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N4" s="1">
         <v>46294</v>
       </c>
       <c r="Q4">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="T4" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="U4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="W4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -899,22 +914,22 @@
         <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G5">
         <v>2702</v>
       </c>
       <c r="H5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J5" s="1">
         <v>46279</v>
@@ -926,7 +941,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N5" s="1">
         <v>46312</v>
@@ -935,22 +950,22 @@
         <v>46312</v>
       </c>
       <c r="Q5">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="T5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="V5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="W5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -967,22 +982,22 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G6">
         <v>2723</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J6" s="1">
         <v>46289</v>
@@ -994,28 +1009,28 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N6" s="1">
         <v>46320</v>
       </c>
       <c r="Q6">
-        <v>-27</v>
+        <v>-26</v>
       </c>
       <c r="R6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="T6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="U6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="W6" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1032,22 +1047,22 @@
         <v>36</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G7">
         <v>2703</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I7" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J7" s="1">
         <v>46289</v>
@@ -1059,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N7" s="1">
         <v>46301</v>
@@ -1068,25 +1083,25 @@
         <v>46290</v>
       </c>
       <c r="Q7">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="T7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="U7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="V7" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="W7" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1103,22 +1118,22 @@
         <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G8">
         <v>2734</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J8" s="1">
         <v>46290</v>
@@ -1130,28 +1145,28 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N8" s="1">
         <v>46304</v>
       </c>
       <c r="Q8">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="T8" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="U8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="W8" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1168,22 +1183,22 @@
         <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G9">
         <v>2734</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J9" s="1">
         <v>46290</v>
@@ -1195,28 +1210,28 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N9" s="1">
         <v>46304</v>
       </c>
       <c r="Q9">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="T9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="U9" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="W9" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1233,22 +1248,22 @@
         <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G10">
         <v>2729</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J10" s="1">
         <v>46293</v>
@@ -1260,28 +1275,28 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N10" s="1">
         <v>46304</v>
       </c>
       <c r="Q10">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="T10" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="U10" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="W10" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1298,22 +1313,22 @@
         <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G11">
         <v>2703</v>
       </c>
       <c r="H11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I11" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="J11" s="1">
         <v>46293</v>
@@ -1325,27 +1340,92 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="N11" s="1">
         <v>46304</v>
       </c>
       <c r="Q11">
+        <v>-10</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+      <c r="S11" t="s">
+        <v>74</v>
+      </c>
+      <c r="T11" t="s">
+        <v>75</v>
+      </c>
+      <c r="W11" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="A12">
+        <v>685</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12">
+        <v>2703</v>
+      </c>
+      <c r="H12" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" t="s">
+        <v>72</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46293</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46294</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>73</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46305</v>
+      </c>
+      <c r="Q12">
         <v>-11</v>
       </c>
-      <c r="R11">
+      <c r="R12">
         <v>0</v>
       </c>
-      <c r="S11" t="s">
-        <v>70</v>
-      </c>
-      <c r="T11" t="s">
-        <v>71</v>
-      </c>
-      <c r="W11" t="s">
+      <c r="S12" t="s">
+        <v>75</v>
+      </c>
+      <c r="T12" t="s">
+        <v>75</v>
+      </c>
+      <c r="U12" t="s">
         <v>82</v>
       </c>
-      <c r="AA11" t="b">
+      <c r="W12" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA12" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (29/09/2026 19:53)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -287,8 +287,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -304,7 +312,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -312,12 +320,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -617,85 +643,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -727,10 +753,10 @@
       <c r="I2" t="s">
         <v>70</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -739,10 +765,10 @@
       <c r="M2" t="s">
         <v>73</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -795,10 +821,10 @@
       <c r="I3" t="s">
         <v>70</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -807,10 +833,10 @@
       <c r="M3" t="s">
         <v>73</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46291</v>
       </c>
       <c r="Q3">
@@ -866,10 +892,10 @@
       <c r="I4" t="s">
         <v>71</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46287</v>
       </c>
       <c r="L4">
@@ -878,7 +904,7 @@
       <c r="M4" t="s">
         <v>73</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46294</v>
       </c>
       <c r="Q4">
@@ -931,10 +957,10 @@
       <c r="I5" t="s">
         <v>70</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46279</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46281</v>
       </c>
       <c r="L5">
@@ -943,10 +969,10 @@
       <c r="M5" t="s">
         <v>73</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46312</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46312</v>
       </c>
       <c r="Q5">
@@ -999,10 +1025,10 @@
       <c r="I6" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46289</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46289</v>
       </c>
       <c r="L6">
@@ -1011,7 +1037,7 @@
       <c r="M6" t="s">
         <v>73</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46320</v>
       </c>
       <c r="Q6">
@@ -1064,10 +1090,10 @@
       <c r="I7" t="s">
         <v>72</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46289</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46290</v>
       </c>
       <c r="L7">
@@ -1076,10 +1102,10 @@
       <c r="M7" t="s">
         <v>73</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46301</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46290</v>
       </c>
       <c r="Q7">
@@ -1135,10 +1161,10 @@
       <c r="I8" t="s">
         <v>72</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46290</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46293</v>
       </c>
       <c r="L8">
@@ -1147,7 +1173,7 @@
       <c r="M8" t="s">
         <v>73</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46304</v>
       </c>
       <c r="Q8">
@@ -1200,10 +1226,10 @@
       <c r="I9" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46290</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46293</v>
       </c>
       <c r="L9">
@@ -1212,7 +1238,7 @@
       <c r="M9" t="s">
         <v>73</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46304</v>
       </c>
       <c r="Q9">
@@ -1265,10 +1291,10 @@
       <c r="I10" t="s">
         <v>72</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46293</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46293</v>
       </c>
       <c r="L10">
@@ -1277,7 +1303,7 @@
       <c r="M10" t="s">
         <v>73</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46304</v>
       </c>
       <c r="Q10">
@@ -1330,10 +1356,10 @@
       <c r="I11" t="s">
         <v>72</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46293</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46293</v>
       </c>
       <c r="L11">
@@ -1342,7 +1368,7 @@
       <c r="M11" t="s">
         <v>73</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46304</v>
       </c>
       <c r="Q11">
@@ -1392,10 +1418,10 @@
       <c r="I12" t="s">
         <v>72</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46293</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46294</v>
       </c>
       <c r="L12">
@@ -1404,7 +1430,7 @@
       <c r="M12" t="s">
         <v>73</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46305</v>
       </c>
       <c r="Q12">

</xml_diff>

<commit_message>
Atualização automática: emergencias (30/09/2026 13:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="113">
   <si>
     <t>om_emg</t>
   </si>
@@ -109,6 +109,9 @@
     <t>CLA</t>
   </si>
   <si>
+    <t>BABR</t>
+  </si>
+  <si>
     <t>396260016580</t>
   </si>
   <si>
@@ -142,6 +145,24 @@
     <t>685260012864</t>
   </si>
   <si>
+    <t>329260019299</t>
+  </si>
+  <si>
+    <t>396260016626</t>
+  </si>
+  <si>
+    <t>396260016627</t>
+  </si>
+  <si>
+    <t>685260012893</t>
+  </si>
+  <si>
+    <t>685260012894</t>
+  </si>
+  <si>
+    <t>685260012897</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -175,6 +196,24 @@
     <t>MS24462-5</t>
   </si>
   <si>
+    <t>066-3046-07</t>
+  </si>
+  <si>
+    <t>2643084-1</t>
+  </si>
+  <si>
+    <t>431-0101-01</t>
+  </si>
+  <si>
+    <t>065-0042-15</t>
+  </si>
+  <si>
+    <t>065-0065-01</t>
+  </si>
+  <si>
+    <t>2643062-1</t>
+  </si>
+  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -208,6 +247,24 @@
     <t>BEARING,ROLLER,NEEDL</t>
   </si>
   <si>
+    <t>CONTROL,INDICATOR</t>
+  </si>
+  <si>
+    <t>TORQUE LINK ASSY-UPP</t>
+  </si>
+  <si>
+    <t>SWITCH,PROXIMITY</t>
+  </si>
+  <si>
+    <t>AUTOPILOT COMPUTER</t>
+  </si>
+  <si>
+    <t>SELECTOR ALT</t>
+  </si>
+  <si>
+    <t>SPRING NOSE GEAR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -223,9 +280,6 @@
     <t>Expedido total</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -265,16 +319,37 @@
     <t>Emerg será atendida pelo estoque FAB pedido 18540739. Godoy 29/09.</t>
   </si>
   <si>
+    <t>Emerg será atendida pelo estoque FAB pedido 18553814. Godoy 30/09.</t>
+  </si>
+  <si>
+    <t>Emerg será atendida pelo estoque FAB pedido 18556805 . Godoy 30/09.</t>
+  </si>
+  <si>
+    <t>Emerg será atendida pelo estoque FAB pedido 18556904 . Godoy 30/09.</t>
+  </si>
+  <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
   </si>
   <si>
-    <t>Colocado pedido no fornecedor WAGA INTERNATIONAL INV26-00008 - tracking 876324334524 - entregue em Campinas 16/09 - MATERIAL SENDO ENVIADO DIA 22/09/2026, ESTAVAMOS CONFIRMANDO O PN COM O FORNECEDOR, RECEBEMOS O PN 040-0046 AWB 12759015025 dpe 26/09/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09</t>
-  </si>
-  <si>
-    <t>MATERIAL ENVIADO DIA 24/09/2026 AWB 12759552135 DPE 25/09/2026 RECIBO 821/FAB/26</t>
+    <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO DO PAMA-LS, REPARADO PELO PARQUE, ENVIADO VIA AWB 12760434076, DPE 30/09/2026</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO VIA RECIBO 821/FAB/26, MATERIAL ENTREGUE DIA 25/09/2026, ASSINADO POR JÕAO VITOR</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003167445 - tracking 542505808925 - previsão de entrega V1 RJ 01/10</t>
+  </si>
+  <si>
+    <t>Atendido via estoque FAB. Em processo de compra para reposição - ITEM ENVIADO DO ESTOQUE FAB, AWB 12760433586, DPE 30/09/2026</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO VIA RECIBO: 842/FAB/26, AWB:127-6050-8125 - DPE 01/10/26.atlz Lucas (30/09/26)</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003168062 - em processo de envio - tracking 542505817838 - ESSE ITEM ESTÁ LIGADO AO PN 2643031-7, POR SER O BEARING DO MESMO.</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -287,16 +362,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -312,7 +379,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -320,30 +387,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -639,89 +688,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -733,61 +782,61 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I2" t="s">
-        <v>70</v>
-      </c>
-      <c r="J2" s="2">
+        <v>88</v>
+      </c>
+      <c r="J2" s="1">
         <v>46238</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46238</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>73</v>
-      </c>
-      <c r="N2" s="2">
+        <v>91</v>
+      </c>
+      <c r="N2" s="1">
         <v>46269</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="R2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="S2" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T2" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="V2" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="W2" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -801,64 +850,61 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I3" t="s">
-        <v>70</v>
-      </c>
-      <c r="J3" s="2">
+        <v>88</v>
+      </c>
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>73</v>
-      </c>
-      <c r="N3" s="2">
+        <v>91</v>
+      </c>
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
-      <c r="O3" s="2">
-        <v>46291</v>
-      </c>
       <c r="Q3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R3">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="S3" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T3" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="U3" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="V3" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="W3" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -872,58 +918,64 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="G4">
         <v>2741</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="I4" t="s">
-        <v>71</v>
-      </c>
-      <c r="J4" s="2">
+        <v>89</v>
+      </c>
+      <c r="J4" s="1">
         <v>46253</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46287</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N4" s="2">
+        <v>91</v>
+      </c>
+      <c r="N4" s="1">
         <v>46294</v>
       </c>
+      <c r="O4" s="1">
+        <v>46295</v>
+      </c>
       <c r="Q4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S4" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T4" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="U4" t="s">
-        <v>77</v>
+        <v>95</v>
+      </c>
+      <c r="V4" t="s">
+        <v>106</v>
       </c>
       <c r="W4" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -937,61 +989,58 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="G5">
         <v>2702</v>
       </c>
       <c r="H5" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I5" t="s">
-        <v>70</v>
-      </c>
-      <c r="J5" s="2">
+        <v>88</v>
+      </c>
+      <c r="J5" s="1">
         <v>46279</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46281</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>73</v>
-      </c>
-      <c r="N5" s="2">
+        <v>91</v>
+      </c>
+      <c r="N5" s="1">
         <v>46312</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46312</v>
       </c>
       <c r="Q5">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T5" t="s">
-        <v>75</v>
-      </c>
-      <c r="V5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="W5" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1005,58 +1054,61 @@
         <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="F6" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="G6">
         <v>2723</v>
       </c>
       <c r="H6" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I6" t="s">
-        <v>70</v>
-      </c>
-      <c r="J6" s="2">
+        <v>88</v>
+      </c>
+      <c r="J6" s="1">
         <v>46289</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46289</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>73</v>
-      </c>
-      <c r="N6" s="2">
+        <v>91</v>
+      </c>
+      <c r="N6" s="1">
         <v>46320</v>
       </c>
+      <c r="O6" s="1">
+        <v>46320</v>
+      </c>
       <c r="Q6">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S6" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T6" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="U6" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="W6" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1070,64 +1122,64 @@
         <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="F7" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="G7">
         <v>2703</v>
       </c>
       <c r="H7" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I7" t="s">
-        <v>72</v>
-      </c>
-      <c r="J7" s="2">
+        <v>90</v>
+      </c>
+      <c r="J7" s="1">
         <v>46289</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46290</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>73</v>
-      </c>
-      <c r="N7" s="2">
+        <v>91</v>
+      </c>
+      <c r="N7" s="1">
         <v>46301</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46290</v>
       </c>
       <c r="Q7">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S7" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="T7" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="U7" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="V7" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="W7" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1141,58 +1193,64 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="F8" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="G8">
         <v>2734</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I8" t="s">
-        <v>72</v>
-      </c>
-      <c r="J8" s="2">
+        <v>90</v>
+      </c>
+      <c r="J8" s="1">
         <v>46290</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46293</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>73</v>
-      </c>
-      <c r="N8" s="2">
+        <v>91</v>
+      </c>
+      <c r="N8" s="1">
         <v>46304</v>
       </c>
+      <c r="O8" s="1">
+        <v>46304</v>
+      </c>
       <c r="Q8">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S8" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T8" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="U8" t="s">
-        <v>80</v>
+        <v>98</v>
+      </c>
+      <c r="V8" t="s">
+        <v>108</v>
       </c>
       <c r="W8" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1206,58 +1264,64 @@
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="G9">
         <v>2734</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="2">
+        <v>90</v>
+      </c>
+      <c r="J9" s="1">
         <v>46290</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46293</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>73</v>
-      </c>
-      <c r="N9" s="2">
+        <v>91</v>
+      </c>
+      <c r="N9" s="1">
         <v>46304</v>
       </c>
+      <c r="O9" s="1">
+        <v>46304</v>
+      </c>
       <c r="Q9">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T9" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="U9" t="s">
-        <v>80</v>
+        <v>98</v>
+      </c>
+      <c r="V9" t="s">
+        <v>108</v>
       </c>
       <c r="W9" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1271,58 +1335,64 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="G10">
         <v>2729</v>
       </c>
       <c r="H10" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="I10" t="s">
-        <v>72</v>
-      </c>
-      <c r="J10" s="2">
+        <v>90</v>
+      </c>
+      <c r="J10" s="1">
         <v>46293</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46293</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>73</v>
-      </c>
-      <c r="N10" s="2">
+        <v>91</v>
+      </c>
+      <c r="N10" s="1">
         <v>46304</v>
       </c>
+      <c r="O10" s="1">
+        <v>46295</v>
+      </c>
       <c r="Q10">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="T10" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="U10" t="s">
-        <v>81</v>
+        <v>99</v>
+      </c>
+      <c r="V10" t="s">
+        <v>109</v>
       </c>
       <c r="W10" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1336,55 +1406,61 @@
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="G11">
         <v>2703</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="I11" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" s="2">
+        <v>90</v>
+      </c>
+      <c r="J11" s="1">
         <v>46293</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46293</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>73</v>
-      </c>
-      <c r="N11" s="2">
+        <v>91</v>
+      </c>
+      <c r="N11" s="1">
         <v>46304</v>
       </c>
+      <c r="O11" s="1">
+        <v>46296</v>
+      </c>
       <c r="Q11">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="T11" t="s">
-        <v>75</v>
+        <v>93</v>
+      </c>
+      <c r="V11" t="s">
+        <v>110</v>
       </c>
       <c r="W11" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1398,60 +1474,447 @@
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="F12" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="G12">
         <v>2703</v>
       </c>
       <c r="H12" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="I12" t="s">
-        <v>72</v>
-      </c>
-      <c r="J12" s="2">
+        <v>90</v>
+      </c>
+      <c r="J12" s="1">
         <v>46293</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46294</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>73</v>
-      </c>
-      <c r="N12" s="2">
+        <v>91</v>
+      </c>
+      <c r="N12" s="1">
         <v>46305</v>
       </c>
+      <c r="O12" s="1">
+        <v>46296</v>
+      </c>
       <c r="Q12">
+        <v>-10</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12" t="s">
+        <v>93</v>
+      </c>
+      <c r="T12" t="s">
+        <v>93</v>
+      </c>
+      <c r="U12" t="s">
+        <v>100</v>
+      </c>
+      <c r="V12" t="s">
+        <v>111</v>
+      </c>
+      <c r="W12" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13">
+        <v>329</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13">
+        <v>2721</v>
+      </c>
+      <c r="H13" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" t="s">
+        <v>89</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>91</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46302</v>
+      </c>
+      <c r="Q13">
+        <v>-7</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s">
+        <v>92</v>
+      </c>
+      <c r="T13" t="s">
+        <v>92</v>
+      </c>
+      <c r="W13" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27">
+      <c r="A14">
+        <v>396</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" t="s">
+        <v>83</v>
+      </c>
+      <c r="G14">
+        <v>2739</v>
+      </c>
+      <c r="H14" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" t="s">
+        <v>90</v>
+      </c>
+      <c r="J14" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>91</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46306</v>
+      </c>
+      <c r="Q14">
         <v>-11</v>
       </c>
-      <c r="R12">
+      <c r="R14">
         <v>0</v>
       </c>
-      <c r="S12" t="s">
-        <v>75</v>
-      </c>
-      <c r="T12" t="s">
-        <v>75</v>
-      </c>
-      <c r="U12" t="s">
+      <c r="S14" t="s">
+        <v>93</v>
+      </c>
+      <c r="T14" t="s">
+        <v>93</v>
+      </c>
+      <c r="U14" t="s">
+        <v>101</v>
+      </c>
+      <c r="W14" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27">
+      <c r="A15">
+        <v>396</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" t="s">
+        <v>83</v>
+      </c>
+      <c r="G15">
+        <v>2739</v>
+      </c>
+      <c r="H15" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" t="s">
+        <v>90</v>
+      </c>
+      <c r="J15" s="1">
+        <v>46295</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>91</v>
+      </c>
+      <c r="N15" s="1">
+        <v>46306</v>
+      </c>
+      <c r="Q15">
+        <v>-11</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15" t="s">
+        <v>93</v>
+      </c>
+      <c r="T15" t="s">
+        <v>93</v>
+      </c>
+      <c r="U15" t="s">
+        <v>102</v>
+      </c>
+      <c r="W15" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27">
+      <c r="A16">
+        <v>685</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" t="s">
+        <v>85</v>
+      </c>
+      <c r="G16">
+        <v>2703</v>
+      </c>
+      <c r="H16" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" t="s">
+        <v>88</v>
+      </c>
+      <c r="J16" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
+        <v>91</v>
+      </c>
+      <c r="N16" s="1">
+        <v>46326</v>
+      </c>
+      <c r="Q16">
+        <v>-31</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16" t="s">
+        <v>92</v>
+      </c>
+      <c r="T16" t="s">
+        <v>93</v>
+      </c>
+      <c r="W16" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27">
+      <c r="A17">
+        <v>685</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" t="s">
+        <v>81</v>
+      </c>
+      <c r="F17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G17">
+        <v>2703</v>
+      </c>
+      <c r="H17" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" t="s">
+        <v>88</v>
+      </c>
+      <c r="J17" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17" t="s">
+        <v>91</v>
+      </c>
+      <c r="N17" s="1">
+        <v>46326</v>
+      </c>
+      <c r="Q17">
+        <v>-31</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17" t="s">
+        <v>92</v>
+      </c>
+      <c r="T17" t="s">
+        <v>93</v>
+      </c>
+      <c r="W17" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27">
+      <c r="A18">
+        <v>685</v>
+      </c>
+      <c r="B18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" t="s">
         <v>82</v>
       </c>
-      <c r="W12" t="s">
-        <v>87</v>
-      </c>
-      <c r="AA12" t="b">
+      <c r="F18" t="s">
+        <v>84</v>
+      </c>
+      <c r="G18">
+        <v>2703</v>
+      </c>
+      <c r="H18" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" t="s">
+        <v>90</v>
+      </c>
+      <c r="J18" s="1">
+        <v>46295</v>
+      </c>
+      <c r="K18" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18" t="s">
+        <v>91</v>
+      </c>
+      <c r="N18" s="1">
+        <v>46306</v>
+      </c>
+      <c r="Q18">
+        <v>-11</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18" t="s">
+        <v>93</v>
+      </c>
+      <c r="T18" t="s">
+        <v>93</v>
+      </c>
+      <c r="U18" t="s">
+        <v>103</v>
+      </c>
+      <c r="W18" t="s">
+        <v>112</v>
+      </c>
+      <c r="AA18" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (01/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="116">
   <si>
     <t>om_emg</t>
   </si>
@@ -136,9 +136,6 @@
     <t>313260018905</t>
   </si>
   <si>
-    <t>685260012858</t>
-  </si>
-  <si>
     <t>685260012859</t>
   </si>
   <si>
@@ -163,6 +160,9 @@
     <t>685260012897</t>
   </si>
   <si>
+    <t>419260000561</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
@@ -187,9 +187,6 @@
     <t>2651031-1</t>
   </si>
   <si>
-    <t>AS5178W03</t>
-  </si>
-  <si>
     <t>2643031-7</t>
   </si>
   <si>
@@ -214,6 +211,9 @@
     <t>2643062-1</t>
   </si>
   <si>
+    <t>SD5H14C4527</t>
+  </si>
+  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
@@ -238,9 +238,6 @@
     <t>LEVER FUEL CON</t>
   </si>
   <si>
-    <t>NUT BRAKE SYSTEM</t>
-  </si>
-  <si>
     <t>FORK ASSY,NOSE GEAR</t>
   </si>
   <si>
@@ -265,6 +262,9 @@
     <t>SPRING NOSE GEAR</t>
   </si>
   <si>
+    <t>AIR COMPRESSOR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -280,6 +280,9 @@
     <t>Expedido total</t>
   </si>
   <si>
+    <t>Aguardando solução</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -313,9 +316,6 @@
     <t>Cedeu o item para o 2736. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>Estoque do Pn AN924-3D (alternado). Godoy 28/09/26. Emerg será atendida pelo estoque FAB pedido 18530012. Godoy 28/09.</t>
-  </si>
-  <si>
     <t>Emerg será atendida pelo estoque FAB pedido 18540739. Godoy 29/09.</t>
   </si>
   <si>
@@ -334,7 +334,10 @@
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
   </si>
   <si>
-    <t>MATERIAL ENVIADO DO PAMA-LS, REPARADO PELO PARQUE, ENVIADO VIA AWB 12760434076, DPE 30/09/2026</t>
+    <t>MATERIAL ENVIADO DO PAMA-LS, REPARADO PELO PARQUE, ENVIADO VIA AWB 12760434076, DPE 01/10/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17740209 - entregue V1 RJ 24/09</t>
   </si>
   <si>
     <t>MATERIAL ENVIADO VIA RECIBO 821/FAB/26, MATERIAL ENTREGUE DIA 25/09/2026, ASSINADO POR JÕAO VITOR</t>
@@ -343,13 +346,19 @@
     <t>Colocado pedido Textron WB0003167445 - tracking 542505808925 - previsão de entrega V1 RJ 01/10</t>
   </si>
   <si>
-    <t>Atendido via estoque FAB. Em processo de compra para reposição - ITEM ENVIADO DO ESTOQUE FAB, AWB 12760433586, DPE 30/09/2026</t>
-  </si>
-  <si>
-    <t>MATERIAL ENVIADO VIA RECIBO: 842/FAB/26, AWB:127-6050-8125 - DPE 01/10/26.atlz Lucas (30/09/26)</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003168062 - em processo de envio - tracking 542505817838 - ESSE ITEM ESTÁ LIGADO AO PN 2643031-7, POR SER O BEARING DO MESMO.</t>
+    <t>MATERIAL ENVIADO VIA RECIBO: 842/FAB/26, AWB:127-6050-8125 - DPE 01/10/26.atlz Lucas (30/09/26) - material entregue dia 30/09/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003168062 - em processo de envio - tracking 542505817838 - ESSE ITEM ESTÁ LIGADO AO PN 2643031-7, POR SER O BEARING DO MESMO. FOI ENVIADO COM STK FAB AWB 127-6070 1421 DIA 30-09-26 - CLA-01-10</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO PELA AWB 12760704954 DPE 02/10/2026</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO PELA AWB 12760678343 DPE 03/10/2026</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO PELA AWB 12760701421 DPE 02/10/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -800,7 +809,7 @@
         <v>86</v>
       </c>
       <c r="I2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J2" s="1">
         <v>46238</v>
@@ -812,7 +821,7 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N2" s="1">
         <v>46269</v>
@@ -821,22 +830,22 @@
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="S2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="V2" t="s">
         <v>104</v>
       </c>
       <c r="W2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -868,7 +877,7 @@
         <v>86</v>
       </c>
       <c r="I3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J3" s="1">
         <v>46251</v>
@@ -880,31 +889,31 @@
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R3">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="S3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="V3" t="s">
         <v>105</v>
       </c>
       <c r="W3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -936,7 +945,7 @@
         <v>87</v>
       </c>
       <c r="I4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J4" s="1">
         <v>46253</v>
@@ -948,34 +957,34 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N4" s="1">
         <v>46294</v>
       </c>
       <c r="O4" s="1">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="Q4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="V4" t="s">
         <v>106</v>
       </c>
       <c r="W4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1007,7 +1016,7 @@
         <v>86</v>
       </c>
       <c r="I5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J5" s="1">
         <v>46279</v>
@@ -1019,7 +1028,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N5" s="1">
         <v>46312</v>
@@ -1028,19 +1037,22 @@
         <v>46312</v>
       </c>
       <c r="Q5">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T5" t="s">
-        <v>93</v>
+        <v>94</v>
+      </c>
+      <c r="V5" t="s">
+        <v>107</v>
       </c>
       <c r="W5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1072,7 +1084,7 @@
         <v>86</v>
       </c>
       <c r="I6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J6" s="1">
         <v>46289</v>
@@ -1084,7 +1096,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N6" s="1">
         <v>46320</v>
@@ -1093,22 +1105,22 @@
         <v>46320</v>
       </c>
       <c r="Q6">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="U6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="W6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1140,7 +1152,7 @@
         <v>86</v>
       </c>
       <c r="I7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J7" s="1">
         <v>46289</v>
@@ -1152,7 +1164,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N7" s="1">
         <v>46301</v>
@@ -1161,25 +1173,25 @@
         <v>46290</v>
       </c>
       <c r="Q7">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="T7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="V7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="W7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1211,7 +1223,7 @@
         <v>86</v>
       </c>
       <c r="I8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J8" s="1">
         <v>46290</v>
@@ -1223,7 +1235,7 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N8" s="1">
         <v>46304</v>
@@ -1232,25 +1244,25 @@
         <v>46304</v>
       </c>
       <c r="Q8">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="V8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="W8" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1282,7 +1294,7 @@
         <v>86</v>
       </c>
       <c r="I9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J9" s="1">
         <v>46290</v>
@@ -1294,7 +1306,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N9" s="1">
         <v>46304</v>
@@ -1303,25 +1315,25 @@
         <v>46304</v>
       </c>
       <c r="Q9">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="V9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="W9" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1344,16 +1356,16 @@
         <v>74</v>
       </c>
       <c r="F10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G10">
-        <v>2729</v>
+        <v>2703</v>
       </c>
       <c r="H10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J10" s="1">
         <v>46293</v>
@@ -1365,7 +1377,7 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N10" s="1">
         <v>46304</v>
@@ -1374,25 +1386,22 @@
         <v>46295</v>
       </c>
       <c r="Q10">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S10" t="s">
         <v>93</v>
       </c>
       <c r="T10" t="s">
-        <v>93</v>
-      </c>
-      <c r="U10" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="V10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="W10" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1415,7 +1424,7 @@
         <v>75</v>
       </c>
       <c r="F11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G11">
         <v>2703</v>
@@ -1424,22 +1433,22 @@
         <v>86</v>
       </c>
       <c r="I11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J11" s="1">
         <v>46293</v>
       </c>
       <c r="K11" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N11" s="1">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="O11" s="1">
         <v>46296</v>
@@ -1451,16 +1460,19 @@
         <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="T11" t="s">
-        <v>93</v>
+        <v>94</v>
+      </c>
+      <c r="U11" t="s">
+        <v>100</v>
       </c>
       <c r="V11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="W11" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1468,10 +1480,10 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
         <v>42</v>
@@ -1483,37 +1495,37 @@
         <v>76</v>
       </c>
       <c r="F12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G12">
-        <v>2703</v>
+        <v>2721</v>
       </c>
       <c r="H12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I12" t="s">
         <v>90</v>
       </c>
       <c r="J12" s="1">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="K12" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N12" s="1">
-        <v>46305</v>
+        <v>46302</v>
       </c>
       <c r="O12" s="1">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="Q12">
-        <v>-10</v>
+        <v>-6</v>
       </c>
       <c r="R12">
         <v>1</v>
@@ -1524,14 +1536,11 @@
       <c r="T12" t="s">
         <v>93</v>
       </c>
-      <c r="U12" t="s">
-        <v>100</v>
-      </c>
       <c r="V12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="W12" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1539,10 +1548,10 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1554,16 +1563,16 @@
         <v>77</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G13">
-        <v>2721</v>
+        <v>2739</v>
       </c>
       <c r="H13" t="s">
         <v>86</v>
       </c>
       <c r="I13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="J13" s="1">
         <v>46294</v>
@@ -1575,25 +1584,34 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N13" s="1">
-        <v>46302</v>
+        <v>46306</v>
+      </c>
+      <c r="O13" s="1">
+        <v>46298</v>
       </c>
       <c r="Q13">
-        <v>-7</v>
+        <v>-10</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="T13" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="U13" t="s">
+        <v>101</v>
+      </c>
+      <c r="V13" t="s">
+        <v>113</v>
       </c>
       <c r="W13" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1625,10 +1643,10 @@
         <v>86</v>
       </c>
       <c r="I14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="J14" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="K14" s="1">
         <v>46295</v>
@@ -1637,28 +1655,34 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N14" s="1">
         <v>46306</v>
       </c>
+      <c r="O14" s="1">
+        <v>46298</v>
+      </c>
       <c r="Q14">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="T14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="U14" t="s">
-        <v>101</v>
+        <v>102</v>
+      </c>
+      <c r="V14" t="s">
+        <v>113</v>
       </c>
       <c r="W14" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1666,10 +1690,10 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
         <v>45</v>
@@ -1681,19 +1705,19 @@
         <v>79</v>
       </c>
       <c r="F15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G15">
-        <v>2739</v>
+        <v>2703</v>
       </c>
       <c r="H15" t="s">
         <v>86</v>
       </c>
       <c r="I15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J15" s="1">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="K15" s="1">
         <v>46295</v>
@@ -1702,28 +1726,25 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N15" s="1">
-        <v>46306</v>
+        <v>46326</v>
       </c>
       <c r="Q15">
-        <v>-11</v>
+        <v>-30</v>
       </c>
       <c r="R15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="s">
         <v>93</v>
       </c>
       <c r="T15" t="s">
-        <v>93</v>
-      </c>
-      <c r="U15" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="W15" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1746,7 +1767,7 @@
         <v>80</v>
       </c>
       <c r="F16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G16">
         <v>2703</v>
@@ -1755,7 +1776,7 @@
         <v>86</v>
       </c>
       <c r="I16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J16" s="1">
         <v>46294</v>
@@ -1767,25 +1788,25 @@
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N16" s="1">
         <v>46326</v>
       </c>
       <c r="Q16">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="T16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="W16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1814,13 +1835,13 @@
         <v>2703</v>
       </c>
       <c r="H17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I17" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="J17" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="K17" s="1">
         <v>46295</v>
@@ -1829,25 +1850,34 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N17" s="1">
-        <v>46326</v>
+        <v>46306</v>
+      </c>
+      <c r="O17" s="1">
+        <v>46297</v>
       </c>
       <c r="Q17">
-        <v>-31</v>
+        <v>-10</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="T17" t="s">
-        <v>93</v>
+        <v>94</v>
+      </c>
+      <c r="U17" t="s">
+        <v>103</v>
+      </c>
+      <c r="V17" t="s">
+        <v>114</v>
       </c>
       <c r="W17" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1855,10 +1885,10 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
         <v>48</v>
@@ -1870,34 +1900,34 @@
         <v>82</v>
       </c>
       <c r="F18" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G18">
-        <v>2703</v>
+        <v>2723</v>
       </c>
       <c r="H18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J18" s="1">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="K18" s="1">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L18">
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="N18" s="1">
-        <v>46306</v>
+        <v>46327</v>
       </c>
       <c r="Q18">
-        <v>-11</v>
+        <v>-31</v>
       </c>
       <c r="R18">
         <v>0</v>
@@ -1908,11 +1938,8 @@
       <c r="T18" t="s">
         <v>93</v>
       </c>
-      <c r="U18" t="s">
-        <v>103</v>
-      </c>
       <c r="W18" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (02/10/2026 09:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="118">
   <si>
     <t>om_emg</t>
   </si>
@@ -304,7 +304,7 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>EMG aberta equivocadamente como ANCE. Alterada para AIFP e será contabilizada dessa forma a partir do dia 22/09. Ramon – 21/09/2026.  Conforme apresentado na Carta nº 016/MNT-C98/2026, de 21/09/2026, a empresa informou impeditivos técnicos para a recuperação da PASSENGER DOOR, P/N 2698010-7, especialmente quanto à ausência de escopo homologado e de literatura técnica específica que permita respaldar e certificar o reparo. A contratada também se colocou à disposição para buscar solução em cooperação com os meios técnicos da FAB. Diante da manifestação apresentada, o Fiscal analisará o conteúdo e os argumentos técnicos encaminhados e, durante essa análise, não será aplicada avaliação negativa à empresa quanto a essa ocorrência. Após a conclusão da análise, será emitida resposta formal à contratada. Wallace – 22/09/2026.</t>
+    <t>EMG aberta equivocadamente como ANCE. Alterada para AIFP e será contabilizada dessa forma a partir do dia 22/09. Ramon – 21/09/2026.  Conforme apresentado na Carta nº 016/MNT-C98/2026, de 21/09/2026, a empresa informou impeditivos técnicos para a recuperação da PASSENGER DOOR, P/N 2698010-7, especialmente quanto à ausência de escopo homologado e de literatura técnica específica que permita respaldar e certificar o reparo. A contratada também se colocou à disposição para buscar solução em cooperação com os meios técnicos da FAB. Diante da manifestação apresentada, o Fiscal analisará o conteúdo e os argumentos técnicos encaminhados e, durante essa análise, não será aplicada avaliação negativa à empresa quanto a essa ocorrência. Após a conclusão da análise, será emitida resposta formal à contratada. Wallace – 22/09/2026. AWB 12760434076 - volume retirado na loja GOLLOG - QMA por Kleyton em 01/10. Godoy 02/10/26.</t>
   </si>
   <si>
     <t>O atendimento deve ser do PN 065-0042-03. Ramon 25/09/26</t>
@@ -316,6 +316,9 @@
     <t>Cedeu o item para o 2736. Ramon 28/09/26</t>
   </si>
   <si>
+    <t>AWB 127-6050-8125 - volume retirado na loja GOLLOG - NAT por teodoro silva em 30/09. Godoy 02/10/26.</t>
+  </si>
+  <si>
     <t>Emerg será atendida pelo estoque FAB pedido 18540739. Godoy 29/09.</t>
   </si>
   <si>
@@ -337,7 +340,10 @@
     <t>MATERIAL ENVIADO DO PAMA-LS, REPARADO PELO PARQUE, ENVIADO VIA AWB 12760434076, DPE 01/10/2026</t>
   </si>
   <si>
-    <t>Colocado pedido Textron IJ17740209 - entregue V1 RJ 24/09</t>
+    <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09 - MATERIAL ENVIADO VIA RECIBO 822/FAB/26 AWB 12759588944 DPE 25/09/2026 - MATERIAL JÁ ENTREGUE NO SUPRIMENTOS BANT DIA 25/09/2026</t>
+  </si>
+  <si>
+    <t>ENVIADO DI A 30-09-26 AWB 127-6046 3314 - CLA-01-10</t>
   </si>
   <si>
     <t>MATERIAL ENVIADO VIA RECIBO 821/FAB/26, MATERIAL ENTREGUE DIA 25/09/2026, ASSINADO POR JÕAO VITOR</t>
@@ -371,8 +377,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -388,7 +402,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -396,12 +410,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -701,85 +733,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -811,10 +843,10 @@
       <c r="I2" t="s">
         <v>89</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -823,17 +855,17 @@
       <c r="M2" t="s">
         <v>92</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S2" t="s">
         <v>93</v>
@@ -842,10 +874,10 @@
         <v>94</v>
       </c>
       <c r="V2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="W2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -879,10 +911,10 @@
       <c r="I3" t="s">
         <v>89</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -891,14 +923,14 @@
       <c r="M3" t="s">
         <v>92</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R3">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="S3" t="s">
         <v>93</v>
@@ -910,10 +942,10 @@
         <v>95</v>
       </c>
       <c r="V3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="W3" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -947,10 +979,10 @@
       <c r="I4" t="s">
         <v>90</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46253</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46287</v>
       </c>
       <c r="L4">
@@ -959,17 +991,17 @@
       <c r="M4" t="s">
         <v>92</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46294</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46296</v>
       </c>
       <c r="Q4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S4" t="s">
         <v>93</v>
@@ -981,10 +1013,10 @@
         <v>96</v>
       </c>
       <c r="V4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="W4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1018,10 +1050,10 @@
       <c r="I5" t="s">
         <v>89</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46279</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46281</v>
       </c>
       <c r="L5">
@@ -1030,17 +1062,17 @@
       <c r="M5" t="s">
         <v>92</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46312</v>
       </c>
-      <c r="O5" s="1">
-        <v>46312</v>
+      <c r="O5" s="2">
+        <v>46290</v>
       </c>
       <c r="Q5">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S5" t="s">
         <v>93</v>
@@ -1049,10 +1081,10 @@
         <v>94</v>
       </c>
       <c r="V5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="W5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1086,10 +1118,10 @@
       <c r="I6" t="s">
         <v>89</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46289</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46289</v>
       </c>
       <c r="L6">
@@ -1098,17 +1130,17 @@
       <c r="M6" t="s">
         <v>92</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46320</v>
       </c>
-      <c r="O6" s="1">
-        <v>46320</v>
+      <c r="O6" s="2">
+        <v>46063</v>
       </c>
       <c r="Q6">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s">
         <v>93</v>
@@ -1119,8 +1151,11 @@
       <c r="U6" t="s">
         <v>97</v>
       </c>
+      <c r="V6" t="s">
+        <v>109</v>
+      </c>
       <c r="W6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1154,10 +1189,10 @@
       <c r="I7" t="s">
         <v>91</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46289</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46290</v>
       </c>
       <c r="L7">
@@ -1166,17 +1201,17 @@
       <c r="M7" t="s">
         <v>92</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46301</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46290</v>
       </c>
       <c r="Q7">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
         <v>94</v>
@@ -1188,10 +1223,10 @@
         <v>98</v>
       </c>
       <c r="V7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="W7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1225,10 +1260,10 @@
       <c r="I8" t="s">
         <v>91</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46290</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46293</v>
       </c>
       <c r="L8">
@@ -1237,17 +1272,17 @@
       <c r="M8" t="s">
         <v>92</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46304</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46304</v>
       </c>
       <c r="Q8">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S8" t="s">
         <v>93</v>
@@ -1259,10 +1294,10 @@
         <v>99</v>
       </c>
       <c r="V8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="W8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1296,10 +1331,10 @@
       <c r="I9" t="s">
         <v>91</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46290</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46293</v>
       </c>
       <c r="L9">
@@ -1308,17 +1343,17 @@
       <c r="M9" t="s">
         <v>92</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46304</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46304</v>
       </c>
       <c r="Q9">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S9" t="s">
         <v>93</v>
@@ -1330,10 +1365,10 @@
         <v>99</v>
       </c>
       <c r="V9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="W9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1367,10 +1402,10 @@
       <c r="I10" t="s">
         <v>91</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46293</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46293</v>
       </c>
       <c r="L10">
@@ -1379,17 +1414,17 @@
       <c r="M10" t="s">
         <v>92</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46304</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="2">
         <v>46295</v>
       </c>
       <c r="Q10">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S10" t="s">
         <v>93</v>
@@ -1397,11 +1432,14 @@
       <c r="T10" t="s">
         <v>94</v>
       </c>
+      <c r="U10" t="s">
+        <v>100</v>
+      </c>
       <c r="V10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="W10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1435,10 +1473,10 @@
       <c r="I11" t="s">
         <v>91</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46293</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46294</v>
       </c>
       <c r="L11">
@@ -1447,17 +1485,17 @@
       <c r="M11" t="s">
         <v>92</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46305</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="2">
         <v>46296</v>
       </c>
       <c r="Q11">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S11" t="s">
         <v>94</v>
@@ -1466,13 +1504,13 @@
         <v>94</v>
       </c>
       <c r="U11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="V11" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="W11" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1506,10 +1544,10 @@
       <c r="I12" t="s">
         <v>90</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46294</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46295</v>
       </c>
       <c r="L12">
@@ -1518,17 +1556,17 @@
       <c r="M12" t="s">
         <v>92</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46302</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="2">
         <v>46297</v>
       </c>
       <c r="Q12">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
         <v>93</v>
@@ -1537,10 +1575,10 @@
         <v>93</v>
       </c>
       <c r="V12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="W12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1574,10 +1612,10 @@
       <c r="I13" t="s">
         <v>91</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46294</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46295</v>
       </c>
       <c r="L13">
@@ -1586,17 +1624,17 @@
       <c r="M13" t="s">
         <v>92</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46306</v>
       </c>
-      <c r="O13" s="1">
+      <c r="O13" s="2">
         <v>46298</v>
       </c>
       <c r="Q13">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" t="s">
         <v>94</v>
@@ -1605,13 +1643,13 @@
         <v>94</v>
       </c>
       <c r="U13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="V13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W13" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1645,10 +1683,10 @@
       <c r="I14" t="s">
         <v>91</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46295</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46295</v>
       </c>
       <c r="L14">
@@ -1657,17 +1695,17 @@
       <c r="M14" t="s">
         <v>92</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46306</v>
       </c>
-      <c r="O14" s="1">
+      <c r="O14" s="2">
         <v>46298</v>
       </c>
       <c r="Q14">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" t="s">
         <v>94</v>
@@ -1676,13 +1714,13 @@
         <v>94</v>
       </c>
       <c r="U14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="V14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="W14" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1716,10 +1754,10 @@
       <c r="I15" t="s">
         <v>89</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46294</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46295</v>
       </c>
       <c r="L15">
@@ -1728,14 +1766,14 @@
       <c r="M15" t="s">
         <v>92</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46326</v>
       </c>
       <c r="Q15">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S15" t="s">
         <v>93</v>
@@ -1744,7 +1782,7 @@
         <v>94</v>
       </c>
       <c r="W15" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1778,10 +1816,10 @@
       <c r="I16" t="s">
         <v>89</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46294</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46295</v>
       </c>
       <c r="L16">
@@ -1790,14 +1828,14 @@
       <c r="M16" t="s">
         <v>92</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46326</v>
       </c>
       <c r="Q16">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S16" t="s">
         <v>93</v>
@@ -1806,7 +1844,7 @@
         <v>94</v>
       </c>
       <c r="W16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1840,10 +1878,10 @@
       <c r="I17" t="s">
         <v>91</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46295</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46295</v>
       </c>
       <c r="L17">
@@ -1852,17 +1890,17 @@
       <c r="M17" t="s">
         <v>92</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46306</v>
       </c>
-      <c r="O17" s="1">
+      <c r="O17" s="2">
         <v>46297</v>
       </c>
       <c r="Q17">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S17" t="s">
         <v>94</v>
@@ -1871,13 +1909,13 @@
         <v>94</v>
       </c>
       <c r="U17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="V17" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="W17" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1911,10 +1949,10 @@
       <c r="I18" t="s">
         <v>89</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46296</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46296</v>
       </c>
       <c r="L18">
@@ -1923,14 +1961,14 @@
       <c r="M18" t="s">
         <v>92</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46327</v>
       </c>
       <c r="Q18">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" t="s">
         <v>93</v>
@@ -1939,7 +1977,7 @@
         <v>93</v>
       </c>
       <c r="W18" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (02/10/2026 13:36)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="121">
   <si>
     <t>om_emg</t>
   </si>
@@ -118,9 +118,6 @@
     <t>313260018702</t>
   </si>
   <si>
-    <t>313260018708</t>
-  </si>
-  <si>
     <t>685260012787</t>
   </si>
   <si>
@@ -139,9 +136,6 @@
     <t>685260012859</t>
   </si>
   <si>
-    <t>685260012864</t>
-  </si>
-  <si>
     <t>329260019299</t>
   </si>
   <si>
@@ -157,21 +151,33 @@
     <t>685260012894</t>
   </si>
   <si>
-    <t>685260012897</t>
-  </si>
-  <si>
     <t>419260000561</t>
   </si>
   <si>
+    <t>329260019303</t>
+  </si>
+  <si>
+    <t>329260019304</t>
+  </si>
+  <si>
+    <t>329260019305</t>
+  </si>
+  <si>
+    <t>329260019306</t>
+  </si>
+  <si>
+    <t>396260016629</t>
+  </si>
+  <si>
+    <t>685260012904</t>
+  </si>
+  <si>
     <t>2601188-204</t>
   </si>
   <si>
     <t>040-0043</t>
   </si>
   <si>
-    <t>2698010-7</t>
-  </si>
-  <si>
     <t>S2889-3-0112</t>
   </si>
   <si>
@@ -190,9 +196,6 @@
     <t>2643031-7</t>
   </si>
   <si>
-    <t>MS24462-5</t>
-  </si>
-  <si>
     <t>066-3046-07</t>
   </si>
   <si>
@@ -208,21 +211,33 @@
     <t>065-0065-01</t>
   </si>
   <si>
-    <t>2643062-1</t>
-  </si>
-  <si>
     <t>SD5H14C4527</t>
   </si>
   <si>
+    <t>AN921-3D</t>
+  </si>
+  <si>
+    <t>MS20822-3D</t>
+  </si>
+  <si>
+    <t>MS28778-3</t>
+  </si>
+  <si>
+    <t>200SGL119Q-2</t>
+  </si>
+  <si>
+    <t>2643100-201</t>
+  </si>
+  <si>
+    <t>80-0583-3</t>
+  </si>
+  <si>
     <t>COMPRESSOR DRIVE ASS</t>
   </si>
   <si>
     <t>STROB TUB</t>
   </si>
   <si>
-    <t>PASSENGER DOOR - LOW</t>
-  </si>
-  <si>
     <t>HOSE ASSY TEE</t>
   </si>
   <si>
@@ -241,9 +256,6 @@
     <t>FORK ASSY,NOSE GEAR</t>
   </si>
   <si>
-    <t>BEARING,ROLLER,NEEDL</t>
-  </si>
-  <si>
     <t>CONTROL,INDICATOR</t>
   </si>
   <si>
@@ -259,39 +271,51 @@
     <t>SELECTOR ALT</t>
   </si>
   <si>
-    <t>SPRING NOSE GEAR</t>
-  </si>
-  <si>
     <t>AIR COMPRESSOR</t>
   </si>
   <si>
+    <t>ELBOW</t>
+  </si>
+  <si>
+    <t>ELBOW,PIPE TO</t>
+  </si>
+  <si>
+    <t>ANEL-O</t>
+  </si>
+  <si>
+    <t>STARTER GENERATOR</t>
+  </si>
+  <si>
+    <t>NOSE GEAR STRUT ASSY</t>
+  </si>
+  <si>
+    <t>ANNUNCIATOR PA</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
+    <t>R</t>
+  </si>
+  <si>
     <t>T</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Expedido total</t>
-  </si>
-  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
     <t>ANCE</t>
   </si>
   <si>
+    <t>IPLR</t>
+  </si>
+  <si>
     <t>AIFP</t>
   </si>
   <si>
-    <t>IPLR</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -304,9 +328,6 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>EMG aberta equivocadamente como ANCE. Alterada para AIFP e será contabilizada dessa forma a partir do dia 22/09. Ramon – 21/09/2026.  Conforme apresentado na Carta nº 016/MNT-C98/2026, de 21/09/2026, a empresa informou impeditivos técnicos para a recuperação da PASSENGER DOOR, P/N 2698010-7, especialmente quanto à ausência de escopo homologado e de literatura técnica específica que permita respaldar e certificar o reparo. A contratada também se colocou à disposição para buscar solução em cooperação com os meios técnicos da FAB. Diante da manifestação apresentada, o Fiscal analisará o conteúdo e os argumentos técnicos encaminhados e, durante essa análise, não será aplicada avaliação negativa à empresa quanto a essa ocorrência. Após a conclusão da análise, será emitida resposta formal à contratada. Wallace – 22/09/2026. AWB 12760434076 - volume retirado na loja GOLLOG - QMA por Kleyton em 01/10. Godoy 02/10/26.</t>
-  </si>
-  <si>
     <t>O atendimento deve ser do PN 065-0042-03. Ramon 25/09/26</t>
   </si>
   <si>
@@ -319,16 +340,13 @@
     <t>AWB 127-6050-8125 - volume retirado na loja GOLLOG - NAT por teodoro silva em 30/09. Godoy 02/10/26.</t>
   </si>
   <si>
-    <t>Emerg será atendida pelo estoque FAB pedido 18540739. Godoy 29/09.</t>
-  </si>
-  <si>
     <t>Emerg será atendida pelo estoque FAB pedido 18553814. Godoy 30/09.</t>
   </si>
   <si>
     <t>Emerg será atendida pelo estoque FAB pedido 18556805 . Godoy 30/09.</t>
   </si>
   <si>
-    <t>Emerg será atendida pelo estoque FAB pedido 18556904 . Godoy 30/09.</t>
+    <t>Emerg será atendida pelo estoque FAB pedido 18568180. Godoy 02/10/26.</t>
   </si>
   <si>
     <t>PEDIDO NO EPM E-C98-26060 - CLA-05-08 , por gentileza, me confirme se está correto a data da informação e prazo de entrega do item.O item solicitado não atende a pane do sistema ARCOND,pôs a pane é de 18/11/2024, anterior ao contrato vigente ,desta forma deve ser feito toda analise do sistema ,devido muito tempo inoperante e sem o item. SO R1 Bispo VEE-ONE-BE em 06/08/26</t>
@@ -337,9 +355,6 @@
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
   </si>
   <si>
-    <t>MATERIAL ENVIADO DO PAMA-LS, REPARADO PELO PARQUE, ENVIADO VIA AWB 12760434076, DPE 01/10/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09 - MATERIAL ENVIADO VIA RECIBO 822/FAB/26 AWB 12759588944 DPE 25/09/2026 - MATERIAL JÁ ENTREGUE NO SUPRIMENTOS BANT DIA 25/09/2026</t>
   </si>
   <si>
@@ -355,16 +370,10 @@
     <t>MATERIAL ENVIADO VIA RECIBO: 842/FAB/26, AWB:127-6050-8125 - DPE 01/10/26.atlz Lucas (30/09/26) - material entregue dia 30/09/2026</t>
   </si>
   <si>
-    <t>Colocado pedido Textron WB0003168062 - em processo de envio - tracking 542505817838 - ESSE ITEM ESTÁ LIGADO AO PN 2643031-7, POR SER O BEARING DO MESMO. FOI ENVIADO COM STK FAB AWB 127-6070 1421 DIA 30-09-26 - CLA-01-10</t>
-  </si>
-  <si>
     <t>MATERIAL ENVIADO PELA AWB 12760704954 DPE 02/10/2026</t>
   </si>
   <si>
     <t>MATERIAL ENVIADO PELA AWB 12760678343 DPE 03/10/2026</t>
-  </si>
-  <si>
-    <t>MATERIAL ENVIADO PELA AWB 12760701421 DPE 02/10/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -377,16 +386,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -402,7 +403,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -410,30 +411,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -729,89 +712,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA18"/>
+  <dimension ref="A1:AA21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -826,39 +809,39 @@
         <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F2" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="G2">
         <v>2733</v>
       </c>
       <c r="H2" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I2" t="s">
-        <v>89</v>
-      </c>
-      <c r="J2" s="2">
+        <v>97</v>
+      </c>
+      <c r="J2" s="1">
         <v>46238</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46238</v>
       </c>
       <c r="L2">
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>92</v>
-      </c>
-      <c r="N2" s="2">
+        <v>100</v>
+      </c>
+      <c r="N2" s="1">
         <v>46269</v>
       </c>
-      <c r="O2" s="2">
+      <c r="O2" s="1">
         <v>46269</v>
       </c>
       <c r="Q2">
@@ -868,16 +851,16 @@
         <v>59</v>
       </c>
       <c r="S2" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="V2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="W2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -894,36 +877,36 @@
         <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="F3" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="G3">
         <v>2741</v>
       </c>
       <c r="H3" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I3" t="s">
-        <v>89</v>
-      </c>
-      <c r="J3" s="2">
+        <v>97</v>
+      </c>
+      <c r="J3" s="1">
         <v>46251</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46249</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3" t="s">
-        <v>92</v>
-      </c>
-      <c r="N3" s="2">
+        <v>100</v>
+      </c>
+      <c r="N3" s="1">
         <v>46280</v>
       </c>
       <c r="Q3">
@@ -933,19 +916,19 @@
         <v>48</v>
       </c>
       <c r="S3" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T3" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="U3" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="V3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="W3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -953,70 +936,67 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F4" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G4">
-        <v>2741</v>
+        <v>2702</v>
       </c>
       <c r="H4" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="I4" t="s">
-        <v>90</v>
-      </c>
-      <c r="J4" s="2">
-        <v>46253</v>
-      </c>
-      <c r="K4" s="2">
-        <v>46287</v>
+        <v>97</v>
+      </c>
+      <c r="J4" s="1">
+        <v>46279</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46281</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>92</v>
-      </c>
-      <c r="N4" s="2">
-        <v>46294</v>
-      </c>
-      <c r="O4" s="2">
-        <v>46296</v>
+        <v>100</v>
+      </c>
+      <c r="N4" s="1">
+        <v>46312</v>
+      </c>
+      <c r="O4" s="1">
+        <v>46290</v>
       </c>
       <c r="Q4">
-        <v>3</v>
+        <v>-15</v>
       </c>
       <c r="R4">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="S4" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T4" t="s">
-        <v>94</v>
-      </c>
-      <c r="U4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="V4" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="W4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1024,67 +1004,70 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="F5" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G5">
-        <v>2702</v>
+        <v>2723</v>
       </c>
       <c r="H5" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I5" t="s">
-        <v>89</v>
-      </c>
-      <c r="J5" s="2">
-        <v>46279</v>
-      </c>
-      <c r="K5" s="2">
-        <v>46281</v>
+        <v>97</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46289</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46289</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>92</v>
-      </c>
-      <c r="N5" s="2">
-        <v>46312</v>
-      </c>
-      <c r="O5" s="2">
-        <v>46290</v>
+        <v>100</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46320</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46063</v>
       </c>
       <c r="Q5">
-        <v>-15</v>
+        <v>-23</v>
       </c>
       <c r="R5">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="S5" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T5" t="s">
-        <v>94</v>
+        <v>101</v>
+      </c>
+      <c r="U5" t="s">
+        <v>104</v>
       </c>
       <c r="V5" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="W5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1092,70 +1075,70 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="F6" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="G6">
-        <v>2723</v>
+        <v>2703</v>
       </c>
       <c r="H6" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I6" t="s">
-        <v>89</v>
-      </c>
-      <c r="J6" s="2">
+        <v>98</v>
+      </c>
+      <c r="J6" s="1">
         <v>46289</v>
       </c>
-      <c r="K6" s="2">
-        <v>46289</v>
+      <c r="K6" s="1">
+        <v>46290</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>92</v>
-      </c>
-      <c r="N6" s="2">
-        <v>46320</v>
-      </c>
-      <c r="O6" s="2">
-        <v>46063</v>
+        <v>100</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46301</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46290</v>
       </c>
       <c r="Q6">
-        <v>-23</v>
+        <v>-4</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S6" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="T6" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="U6" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="V6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="W6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1163,70 +1146,70 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
         <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E7" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F7" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G7">
-        <v>2703</v>
+        <v>2734</v>
       </c>
       <c r="H7" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I7" t="s">
-        <v>91</v>
-      </c>
-      <c r="J7" s="2">
-        <v>46289</v>
-      </c>
-      <c r="K7" s="2">
+        <v>98</v>
+      </c>
+      <c r="J7" s="1">
         <v>46290</v>
       </c>
+      <c r="K7" s="1">
+        <v>46293</v>
+      </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>92</v>
-      </c>
-      <c r="N7" s="2">
-        <v>46301</v>
-      </c>
-      <c r="O7" s="2">
-        <v>46290</v>
+        <v>100</v>
+      </c>
+      <c r="N7" s="1">
+        <v>46304</v>
+      </c>
+      <c r="O7" s="1">
+        <v>46304</v>
       </c>
       <c r="Q7">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="R7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S7" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="T7" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="U7" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="V7" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="W7" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1243,39 +1226,39 @@
         <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="G8">
         <v>2734</v>
       </c>
       <c r="H8" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I8" t="s">
-        <v>91</v>
-      </c>
-      <c r="J8" s="2">
+        <v>98</v>
+      </c>
+      <c r="J8" s="1">
         <v>46290</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46293</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>92</v>
-      </c>
-      <c r="N8" s="2">
+        <v>100</v>
+      </c>
+      <c r="N8" s="1">
         <v>46304</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46304</v>
       </c>
       <c r="Q8">
@@ -1285,19 +1268,19 @@
         <v>4</v>
       </c>
       <c r="S8" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T8" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="U8" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="V8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="W8" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1305,49 +1288,49 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="F9" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="G9">
-        <v>2734</v>
+        <v>2703</v>
       </c>
       <c r="H9" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I9" t="s">
-        <v>91</v>
-      </c>
-      <c r="J9" s="2">
-        <v>46290</v>
-      </c>
-      <c r="K9" s="2">
+        <v>98</v>
+      </c>
+      <c r="J9" s="1">
         <v>46293</v>
       </c>
+      <c r="K9" s="1">
+        <v>46293</v>
+      </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>92</v>
-      </c>
-      <c r="N9" s="2">
+        <v>100</v>
+      </c>
+      <c r="N9" s="1">
         <v>46304</v>
       </c>
-      <c r="O9" s="2">
-        <v>46304</v>
+      <c r="O9" s="1">
+        <v>46295</v>
       </c>
       <c r="Q9">
         <v>-7</v>
@@ -1356,19 +1339,19 @@
         <v>4</v>
       </c>
       <c r="S9" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T9" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="U9" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="V9" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="W9" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1376,70 +1359,67 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
         <v>40</v>
       </c>
       <c r="D10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E10" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="G10">
-        <v>2703</v>
+        <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I10" t="s">
-        <v>91</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46293</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46293</v>
+        <v>99</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46295</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>92</v>
-      </c>
-      <c r="N10" s="2">
-        <v>46304</v>
-      </c>
-      <c r="O10" s="2">
-        <v>46295</v>
+        <v>100</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46302</v>
+      </c>
+      <c r="O10" s="1">
+        <v>46297</v>
       </c>
       <c r="Q10">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T10" t="s">
-        <v>94</v>
-      </c>
-      <c r="U10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="V10" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="W10" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1447,70 +1427,70 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F11" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="G11">
-        <v>2703</v>
+        <v>2739</v>
       </c>
       <c r="H11" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I11" t="s">
-        <v>91</v>
-      </c>
-      <c r="J11" s="2">
-        <v>46293</v>
-      </c>
-      <c r="K11" s="2">
+        <v>98</v>
+      </c>
+      <c r="J11" s="1">
         <v>46294</v>
       </c>
+      <c r="K11" s="1">
+        <v>46295</v>
+      </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>92</v>
-      </c>
-      <c r="N11" s="2">
-        <v>46305</v>
-      </c>
-      <c r="O11" s="2">
-        <v>46296</v>
+        <v>100</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46306</v>
+      </c>
+      <c r="O11" s="1">
+        <v>46298</v>
       </c>
       <c r="Q11">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="R11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="T11" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="U11" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="V11" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="W11" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1518,67 +1498,70 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
         <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="F12" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="G12">
-        <v>2721</v>
+        <v>2739</v>
       </c>
       <c r="H12" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I12" t="s">
-        <v>90</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46294</v>
-      </c>
-      <c r="K12" s="2">
+        <v>98</v>
+      </c>
+      <c r="J12" s="1">
         <v>46295</v>
       </c>
+      <c r="K12" s="1">
+        <v>46295</v>
+      </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>92</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46302</v>
-      </c>
-      <c r="O12" s="2">
-        <v>46297</v>
+        <v>100</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46306</v>
+      </c>
+      <c r="O12" s="1">
+        <v>46298</v>
       </c>
       <c r="Q12">
-        <v>-5</v>
+        <v>-9</v>
       </c>
       <c r="R12">
         <v>2</v>
       </c>
       <c r="S12" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="T12" t="s">
-        <v>93</v>
+        <v>102</v>
+      </c>
+      <c r="U12" t="s">
+        <v>109</v>
       </c>
       <c r="V12" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="W12" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1586,70 +1569,61 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E13" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F13" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="G13">
-        <v>2739</v>
+        <v>2703</v>
       </c>
       <c r="H13" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I13" t="s">
-        <v>91</v>
-      </c>
-      <c r="J13" s="2">
+        <v>97</v>
+      </c>
+      <c r="J13" s="1">
         <v>46294</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46295</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>92</v>
-      </c>
-      <c r="N13" s="2">
-        <v>46306</v>
-      </c>
-      <c r="O13" s="2">
-        <v>46298</v>
+        <v>100</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46326</v>
       </c>
       <c r="Q13">
-        <v>-9</v>
+        <v>-29</v>
       </c>
       <c r="R13">
         <v>2</v>
       </c>
       <c r="S13" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="T13" t="s">
-        <v>94</v>
-      </c>
-      <c r="U13" t="s">
         <v>102</v>
       </c>
-      <c r="V13" t="s">
-        <v>115</v>
-      </c>
       <c r="W13" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1657,70 +1631,61 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E14" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F14" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="G14">
-        <v>2739</v>
+        <v>2703</v>
       </c>
       <c r="H14" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="I14" t="s">
-        <v>91</v>
-      </c>
-      <c r="J14" s="2">
+        <v>97</v>
+      </c>
+      <c r="J14" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K14" s="1">
         <v>46295</v>
       </c>
-      <c r="K14" s="2">
-        <v>46295</v>
-      </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>92</v>
-      </c>
-      <c r="N14" s="2">
-        <v>46306</v>
-      </c>
-      <c r="O14" s="2">
-        <v>46298</v>
+        <v>100</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46326</v>
       </c>
       <c r="Q14">
-        <v>-9</v>
+        <v>-29</v>
       </c>
       <c r="R14">
         <v>2</v>
       </c>
       <c r="S14" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="T14" t="s">
-        <v>94</v>
-      </c>
-      <c r="U14" t="s">
-        <v>103</v>
-      </c>
-      <c r="V14" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="W14" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1728,61 +1693,61 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
         <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="G15">
-        <v>2703</v>
+        <v>2723</v>
       </c>
       <c r="H15" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="I15" t="s">
-        <v>89</v>
-      </c>
-      <c r="J15" s="2">
-        <v>46294</v>
-      </c>
-      <c r="K15" s="2">
-        <v>46295</v>
+        <v>97</v>
+      </c>
+      <c r="J15" s="1">
+        <v>46296</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46296</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>92</v>
-      </c>
-      <c r="N15" s="2">
-        <v>46326</v>
+        <v>100</v>
+      </c>
+      <c r="N15" s="1">
+        <v>46327</v>
       </c>
       <c r="Q15">
-        <v>-29</v>
+        <v>-30</v>
       </c>
       <c r="R15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S15" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="T15" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="W15" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1790,61 +1755,61 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
         <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E16" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F16" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G16">
-        <v>2703</v>
+        <v>2721</v>
       </c>
       <c r="H16" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="I16" t="s">
-        <v>89</v>
-      </c>
-      <c r="J16" s="2">
-        <v>46294</v>
-      </c>
-      <c r="K16" s="2">
-        <v>46295</v>
+        <v>99</v>
+      </c>
+      <c r="J16" s="1">
+        <v>46296</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46297</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M16" t="s">
-        <v>92</v>
-      </c>
-      <c r="N16" s="2">
-        <v>46326</v>
+        <v>100</v>
+      </c>
+      <c r="N16" s="1">
+        <v>46304</v>
       </c>
       <c r="Q16">
-        <v>-29</v>
+        <v>-7</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S16" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="T16" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="W16" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1852,70 +1817,61 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E17" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F17" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="G17">
-        <v>2703</v>
+        <v>2721</v>
       </c>
       <c r="H17" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="I17" t="s">
-        <v>91</v>
-      </c>
-      <c r="J17" s="2">
-        <v>46295</v>
-      </c>
-      <c r="K17" s="2">
-        <v>46295</v>
+        <v>99</v>
+      </c>
+      <c r="J17" s="1">
+        <v>46296</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46297</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M17" t="s">
-        <v>92</v>
-      </c>
-      <c r="N17" s="2">
-        <v>46306</v>
-      </c>
-      <c r="O17" s="2">
-        <v>46297</v>
+        <v>100</v>
+      </c>
+      <c r="N17" s="1">
+        <v>46304</v>
       </c>
       <c r="Q17">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="R17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S17" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="T17" t="s">
-        <v>94</v>
-      </c>
-      <c r="U17" t="s">
-        <v>104</v>
-      </c>
-      <c r="V17" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="W17" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1923,63 +1879,252 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>419</v>
+        <v>329</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
         <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F18" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="G18">
-        <v>2723</v>
+        <v>2721</v>
       </c>
       <c r="H18" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="I18" t="s">
+        <v>99</v>
+      </c>
+      <c r="J18" s="1">
+        <v>46296</v>
+      </c>
+      <c r="K18" s="1">
+        <v>46297</v>
+      </c>
+      <c r="L18">
+        <v>4</v>
+      </c>
+      <c r="M18" t="s">
+        <v>100</v>
+      </c>
+      <c r="N18" s="1">
+        <v>46304</v>
+      </c>
+      <c r="Q18">
+        <v>-7</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18" t="s">
+        <v>101</v>
+      </c>
+      <c r="T18" t="s">
+        <v>101</v>
+      </c>
+      <c r="W18" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27">
+      <c r="A19">
+        <v>329</v>
+      </c>
+      <c r="B19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" t="s">
+        <v>69</v>
+      </c>
+      <c r="E19" t="s">
         <v>89</v>
       </c>
-      <c r="J18" s="2">
+      <c r="F19" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19">
+        <v>2721</v>
+      </c>
+      <c r="H19" t="s">
+        <v>96</v>
+      </c>
+      <c r="I19" t="s">
+        <v>98</v>
+      </c>
+      <c r="J19" s="1">
         <v>46296</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K19" s="1">
+        <v>46297</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19" t="s">
+        <v>100</v>
+      </c>
+      <c r="N19" s="1">
+        <v>46308</v>
+      </c>
+      <c r="Q19">
+        <v>-11</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19" t="s">
+        <v>101</v>
+      </c>
+      <c r="T19" t="s">
+        <v>101</v>
+      </c>
+      <c r="W19" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27">
+      <c r="A20">
+        <v>396</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20">
+        <v>2739</v>
+      </c>
+      <c r="H20" t="s">
+        <v>96</v>
+      </c>
+      <c r="I20" t="s">
+        <v>98</v>
+      </c>
+      <c r="J20" s="1">
         <v>46296</v>
       </c>
-      <c r="L18">
-        <v>1</v>
-      </c>
-      <c r="M18" t="s">
-        <v>92</v>
-      </c>
-      <c r="N18" s="2">
-        <v>46327</v>
-      </c>
-      <c r="Q18">
-        <v>-30</v>
-      </c>
-      <c r="R18">
-        <v>1</v>
-      </c>
-      <c r="S18" t="s">
-        <v>93</v>
-      </c>
-      <c r="T18" t="s">
-        <v>93</v>
-      </c>
-      <c r="W18" t="s">
-        <v>117</v>
-      </c>
-      <c r="AA18" t="b">
+      <c r="K20" s="1">
+        <v>46297</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20" t="s">
+        <v>100</v>
+      </c>
+      <c r="N20" s="1">
+        <v>46308</v>
+      </c>
+      <c r="Q20">
+        <v>-11</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20" t="s">
+        <v>101</v>
+      </c>
+      <c r="T20" t="s">
+        <v>102</v>
+      </c>
+      <c r="W20" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27">
+      <c r="A21">
+        <v>685</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E21" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" t="s">
+        <v>94</v>
+      </c>
+      <c r="G21">
+        <v>2703</v>
+      </c>
+      <c r="H21" t="s">
+        <v>96</v>
+      </c>
+      <c r="I21" t="s">
+        <v>98</v>
+      </c>
+      <c r="J21" s="1">
+        <v>46296</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46297</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21" t="s">
+        <v>100</v>
+      </c>
+      <c r="N21" s="1">
+        <v>46308</v>
+      </c>
+      <c r="Q21">
+        <v>-11</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21" t="s">
+        <v>102</v>
+      </c>
+      <c r="T21" t="s">
+        <v>102</v>
+      </c>
+      <c r="U21" t="s">
+        <v>110</v>
+      </c>
+      <c r="W21" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA21" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (05/10/2026 08:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -386,8 +386,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -403,7 +411,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -411,12 +419,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -716,85 +742,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -826,10 +852,10 @@
       <c r="I2" t="s">
         <v>97</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46238</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46238</v>
       </c>
       <c r="L2">
@@ -838,17 +864,17 @@
       <c r="M2" t="s">
         <v>100</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46269</v>
       </c>
-      <c r="O2" s="1">
+      <c r="O2" s="2">
         <v>46269</v>
       </c>
       <c r="Q2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="R2">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="S2" t="s">
         <v>101</v>
@@ -894,10 +920,10 @@
       <c r="I3" t="s">
         <v>97</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46251</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46249</v>
       </c>
       <c r="L3">
@@ -906,14 +932,14 @@
       <c r="M3" t="s">
         <v>100</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46280</v>
       </c>
       <c r="Q3">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="R3">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="S3" t="s">
         <v>101</v>
@@ -962,10 +988,10 @@
       <c r="I4" t="s">
         <v>97</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46279</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46281</v>
       </c>
       <c r="L4">
@@ -974,17 +1000,17 @@
       <c r="M4" t="s">
         <v>100</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46312</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46290</v>
       </c>
       <c r="Q4">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="R4">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S4" t="s">
         <v>101</v>
@@ -1030,10 +1056,10 @@
       <c r="I5" t="s">
         <v>97</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46289</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46289</v>
       </c>
       <c r="L5">
@@ -1042,17 +1068,17 @@
       <c r="M5" t="s">
         <v>100</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46320</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46063</v>
       </c>
       <c r="Q5">
-        <v>-23</v>
+        <v>-20</v>
       </c>
       <c r="R5">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S5" t="s">
         <v>101</v>
@@ -1101,10 +1127,10 @@
       <c r="I6" t="s">
         <v>98</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46289</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46290</v>
       </c>
       <c r="L6">
@@ -1113,17 +1139,17 @@
       <c r="M6" t="s">
         <v>100</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46301</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46290</v>
       </c>
       <c r="Q6">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S6" t="s">
         <v>102</v>
@@ -1172,10 +1198,10 @@
       <c r="I7" t="s">
         <v>98</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46290</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46293</v>
       </c>
       <c r="L7">
@@ -1184,17 +1210,17 @@
       <c r="M7" t="s">
         <v>100</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46304</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46304</v>
       </c>
       <c r="Q7">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R7">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
         <v>101</v>
@@ -1243,10 +1269,10 @@
       <c r="I8" t="s">
         <v>98</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46290</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46293</v>
       </c>
       <c r="L8">
@@ -1255,17 +1281,17 @@
       <c r="M8" t="s">
         <v>100</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46304</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46304</v>
       </c>
       <c r="Q8">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
         <v>101</v>
@@ -1314,10 +1340,10 @@
       <c r="I9" t="s">
         <v>98</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46293</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46293</v>
       </c>
       <c r="L9">
@@ -1326,17 +1352,17 @@
       <c r="M9" t="s">
         <v>100</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46304</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46295</v>
       </c>
       <c r="Q9">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R9">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>101</v>
@@ -1385,10 +1411,10 @@
       <c r="I10" t="s">
         <v>99</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46294</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46295</v>
       </c>
       <c r="L10">
@@ -1397,17 +1423,17 @@
       <c r="M10" t="s">
         <v>100</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46302</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="2">
         <v>46297</v>
       </c>
       <c r="Q10">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>101</v>
@@ -1453,10 +1479,10 @@
       <c r="I11" t="s">
         <v>98</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46294</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46295</v>
       </c>
       <c r="L11">
@@ -1465,17 +1491,17 @@
       <c r="M11" t="s">
         <v>100</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46306</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="2">
         <v>46298</v>
       </c>
       <c r="Q11">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>102</v>
@@ -1524,10 +1550,10 @@
       <c r="I12" t="s">
         <v>98</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46295</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46295</v>
       </c>
       <c r="L12">
@@ -1536,17 +1562,17 @@
       <c r="M12" t="s">
         <v>100</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46306</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="2">
         <v>46298</v>
       </c>
       <c r="Q12">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12" t="s">
         <v>102</v>
@@ -1595,10 +1621,10 @@
       <c r="I13" t="s">
         <v>97</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46294</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46295</v>
       </c>
       <c r="L13">
@@ -1607,14 +1633,14 @@
       <c r="M13" t="s">
         <v>100</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46326</v>
       </c>
       <c r="Q13">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S13" t="s">
         <v>101</v>
@@ -1657,10 +1683,10 @@
       <c r="I14" t="s">
         <v>97</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46294</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46295</v>
       </c>
       <c r="L14">
@@ -1669,14 +1695,14 @@
       <c r="M14" t="s">
         <v>100</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46326</v>
       </c>
       <c r="Q14">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S14" t="s">
         <v>101</v>
@@ -1719,10 +1745,10 @@
       <c r="I15" t="s">
         <v>97</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46296</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46296</v>
       </c>
       <c r="L15">
@@ -1731,14 +1757,14 @@
       <c r="M15" t="s">
         <v>100</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46327</v>
       </c>
       <c r="Q15">
-        <v>-30</v>
+        <v>-27</v>
       </c>
       <c r="R15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S15" t="s">
         <v>101</v>
@@ -1781,10 +1807,10 @@
       <c r="I16" t="s">
         <v>99</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46296</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46297</v>
       </c>
       <c r="L16">
@@ -1793,14 +1819,14 @@
       <c r="M16" t="s">
         <v>100</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46304</v>
       </c>
       <c r="Q16">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S16" t="s">
         <v>102</v>
@@ -1843,10 +1869,10 @@
       <c r="I17" t="s">
         <v>99</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46296</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46297</v>
       </c>
       <c r="L17">
@@ -1855,14 +1881,14 @@
       <c r="M17" t="s">
         <v>100</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46304</v>
       </c>
       <c r="Q17">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S17" t="s">
         <v>101</v>
@@ -1905,10 +1931,10 @@
       <c r="I18" t="s">
         <v>99</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46296</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46297</v>
       </c>
       <c r="L18">
@@ -1917,14 +1943,14 @@
       <c r="M18" t="s">
         <v>100</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46304</v>
       </c>
       <c r="Q18">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R18">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S18" t="s">
         <v>101</v>
@@ -1967,10 +1993,10 @@
       <c r="I19" t="s">
         <v>98</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46296</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46297</v>
       </c>
       <c r="L19">
@@ -1979,14 +2005,14 @@
       <c r="M19" t="s">
         <v>100</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46308</v>
       </c>
       <c r="Q19">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S19" t="s">
         <v>101</v>
@@ -2029,10 +2055,10 @@
       <c r="I20" t="s">
         <v>98</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46296</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46297</v>
       </c>
       <c r="L20">
@@ -2041,14 +2067,14 @@
       <c r="M20" t="s">
         <v>100</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46308</v>
       </c>
       <c r="Q20">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S20" t="s">
         <v>101</v>
@@ -2091,10 +2117,10 @@
       <c r="I21" t="s">
         <v>98</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46296</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46297</v>
       </c>
       <c r="L21">
@@ -2103,14 +2129,14 @@
       <c r="M21" t="s">
         <v>100</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46308</v>
       </c>
       <c r="Q21">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S21" t="s">
         <v>102</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (06/10/2026 14:09)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -290,16 +290,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -315,7 +307,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -323,30 +315,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -646,85 +620,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -756,10 +730,10 @@
       <c r="I2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -768,7 +742,7 @@
       <c r="M2" t="s">
         <v>72</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -824,10 +798,10 @@
       <c r="I3" t="s">
         <v>69</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46279</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46281</v>
       </c>
       <c r="L3">
@@ -836,10 +810,10 @@
       <c r="M3" t="s">
         <v>72</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46312</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46290</v>
       </c>
       <c r="Q3">
@@ -895,10 +869,10 @@
       <c r="I4" t="s">
         <v>69</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46289</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46289</v>
       </c>
       <c r="L4">
@@ -907,10 +881,10 @@
       <c r="M4" t="s">
         <v>72</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46320</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46063</v>
       </c>
       <c r="Q4">
@@ -966,10 +940,10 @@
       <c r="I5" t="s">
         <v>70</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46290</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46293</v>
       </c>
       <c r="L5">
@@ -978,10 +952,10 @@
       <c r="M5" t="s">
         <v>72</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46304</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46304</v>
       </c>
       <c r="Q5">
@@ -1037,10 +1011,10 @@
       <c r="I6" t="s">
         <v>70</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46290</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46293</v>
       </c>
       <c r="L6">
@@ -1049,10 +1023,10 @@
       <c r="M6" t="s">
         <v>72</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46304</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46304</v>
       </c>
       <c r="Q6">
@@ -1108,10 +1082,10 @@
       <c r="I7" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46294</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46295</v>
       </c>
       <c r="L7">
@@ -1120,10 +1094,10 @@
       <c r="M7" t="s">
         <v>72</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46302</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46300</v>
       </c>
       <c r="Q7">
@@ -1179,10 +1153,10 @@
       <c r="I8" t="s">
         <v>69</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46294</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46295</v>
       </c>
       <c r="L8">
@@ -1191,7 +1165,7 @@
       <c r="M8" t="s">
         <v>72</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46326</v>
       </c>
       <c r="Q8">
@@ -1244,10 +1218,10 @@
       <c r="I9" t="s">
         <v>69</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46294</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46295</v>
       </c>
       <c r="L9">
@@ -1256,7 +1230,7 @@
       <c r="M9" t="s">
         <v>72</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46326</v>
       </c>
       <c r="Q9">
@@ -1309,10 +1283,10 @@
       <c r="I10" t="s">
         <v>69</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46296</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46296</v>
       </c>
       <c r="L10">
@@ -1321,7 +1295,7 @@
       <c r="M10" t="s">
         <v>72</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46327</v>
       </c>
       <c r="Q10">
@@ -1371,10 +1345,10 @@
       <c r="I11" t="s">
         <v>70</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46296</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46297</v>
       </c>
       <c r="L11">
@@ -1383,7 +1357,7 @@
       <c r="M11" t="s">
         <v>72</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46308</v>
       </c>
       <c r="Q11">
@@ -1436,10 +1410,10 @@
       <c r="I12" t="s">
         <v>69</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46301</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46301</v>
       </c>
       <c r="L12">
@@ -1448,7 +1422,7 @@
       <c r="M12" t="s">
         <v>72</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46332</v>
       </c>
       <c r="Q12">

</xml_diff>

<commit_message>
Atualização automática: emergencias (07/10/2026 11:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="99">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,10 +103,16 @@
     <t>BANT</t>
   </si>
   <si>
+    <t>BABR</t>
+  </si>
+  <si>
     <t>CLA</t>
   </si>
   <si>
-    <t>BABR</t>
+    <t>DACTA II</t>
+  </si>
+  <si>
+    <t>BABE</t>
   </si>
   <si>
     <t>313260018702</t>
@@ -115,9 +121,6 @@
     <t>685260012787</t>
   </si>
   <si>
-    <t>419260000560</t>
-  </si>
-  <si>
     <t>313260018904</t>
   </si>
   <si>
@@ -139,7 +142,22 @@
     <t>329260019306</t>
   </si>
   <si>
-    <t>419260000562</t>
+    <t>685260012943</t>
+  </si>
+  <si>
+    <t>685260012944</t>
+  </si>
+  <si>
+    <t>384260009403</t>
+  </si>
+  <si>
+    <t>396260016636</t>
+  </si>
+  <si>
+    <t>685260012947</t>
+  </si>
+  <si>
+    <t>685260012948</t>
   </si>
   <si>
     <t>040-0043</t>
@@ -148,31 +166,40 @@
     <t>S2889-3-0112</t>
   </si>
   <si>
+    <t>2652022-18</t>
+  </si>
+  <si>
+    <t>2651031-1</t>
+  </si>
+  <si>
+    <t>066-3046-07</t>
+  </si>
+  <si>
+    <t>065-0042-15</t>
+  </si>
+  <si>
+    <t>065-0065-01</t>
+  </si>
+  <si>
+    <t>SD5H14C4527</t>
+  </si>
+  <si>
+    <t>200SGL119Q-2</t>
+  </si>
+  <si>
     <t>065-0042-03</t>
   </si>
   <si>
-    <t>2652022-18</t>
-  </si>
-  <si>
-    <t>2651031-1</t>
-  </si>
-  <si>
-    <t>066-3046-07</t>
-  </si>
-  <si>
-    <t>065-0042-15</t>
-  </si>
-  <si>
-    <t>065-0065-01</t>
-  </si>
-  <si>
-    <t>SD5H14C4527</t>
-  </si>
-  <si>
-    <t>200SGL119Q-2</t>
-  </si>
-  <si>
-    <t>3122678-04</t>
+    <t>066-1055-00</t>
+  </si>
+  <si>
+    <t>9514A-1</t>
+  </si>
+  <si>
+    <t>2651022-20-1</t>
+  </si>
+  <si>
+    <t>2618510-10</t>
   </si>
   <si>
     <t>STROB TUB</t>
@@ -181,31 +208,40 @@
     <t>HOSE ASSY TEE</t>
   </si>
   <si>
+    <t>TUBE ASSY</t>
+  </si>
+  <si>
+    <t>LEVER FUEL CON</t>
+  </si>
+  <si>
+    <t>CONTROL,INDICATOR</t>
+  </si>
+  <si>
+    <t>AUTOPILOT COMPUTER</t>
+  </si>
+  <si>
+    <t>SELECTOR ALT</t>
+  </si>
+  <si>
+    <t>AIR COMPRESSOR</t>
+  </si>
+  <si>
+    <t>STARTER GENERATOR</t>
+  </si>
+  <si>
     <t>COMPUTER PA</t>
   </si>
   <si>
-    <t>TUBE ASSY</t>
-  </si>
-  <si>
-    <t>LEVER FUEL CON</t>
-  </si>
-  <si>
-    <t>CONTROL,INDICATOR</t>
-  </si>
-  <si>
-    <t>AUTOPILOT COMPUTER</t>
-  </si>
-  <si>
-    <t>SELECTOR ALT</t>
-  </si>
-  <si>
-    <t>AIR COMPRESSOR</t>
-  </si>
-  <si>
-    <t>STARTER GENERATOR</t>
-  </si>
-  <si>
-    <t>FUEL CONTROL UNIT</t>
+    <t>AUDIO CONTROL PANEL</t>
+  </si>
+  <si>
+    <t>PUMP ASSY</t>
+  </si>
+  <si>
+    <t>RING AY-ENGINE MOUNT</t>
+  </si>
+  <si>
+    <t>ALTERNATOR CONTROL U</t>
   </si>
   <si>
     <t>C</t>
@@ -247,9 +283,6 @@
     <t>AWB 12759588944 - volume retirado na loja GOLLOG - NAT por teodoro silva em 25/09. Godoy 06/10/26.</t>
   </si>
   <si>
-    <t>O atendimento deve ser do PN 065-0042-03. Ramon 25/09/26. AWB 127-6046 3314 - volume retirado na loja GOLLOG - SLZ por CARLOS FERNANDO em 02/10. Godoy 06/10/26.</t>
-  </si>
-  <si>
     <t>Cedeu o item para o 2736. Ramon 28/09/26</t>
   </si>
   <si>
@@ -262,22 +295,19 @@
     <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09 - MATERIAL ENVIADO VIA RECIBO 822/FAB/26 AWB 12759588944 DPE 25/09/2026 - MATERIAL JÁ ENTREGUE NO SUPRIMENTOS BANT DIA 25/09/2026</t>
   </si>
   <si>
-    <t>ENVIADO DI A 30-09-26 AWB 127-6046 3314 - CLA-01-10</t>
-  </si>
-  <si>
     <t>Colocado pedido Textron WB0003167445 - tracking 542505808925 - previsão de entrega V1 RJ 01/10 - MATERIAL ENVIADO PELA AWB 12761197990 dpe 08/10/2026</t>
   </si>
   <si>
     <t>MATERIAL ENVIADO PELA AWB 12760704954 DPE 02/10/2026 - MATERIAL RETIRADO DIA 05/10/26 POR SGT KÉSIA</t>
   </si>
   <si>
-    <t>AGD ABERTURA DE OS- REZ</t>
+    <t>AGD ABERTURA DE OS- REZ , email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26</t>
   </si>
   <si>
     <t>RECEBIDO 01 EA, REPARADO , DA WILLIAM EM 05/10/26. SERÁ ATD ESTA EMERG - REZ (06/10/26)</t>
   </si>
   <si>
-    <t>DPE 09/10/26 - REZ(06-10-26)</t>
+    <t>DPE 09/10/26 - REZ(06-10-26), email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -290,8 +320,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -307,7 +345,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -315,12 +353,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -616,89 +672,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -710,61 +766,61 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="F2" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I2" t="s">
-        <v>69</v>
-      </c>
-      <c r="J2" s="1">
+        <v>81</v>
+      </c>
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>72</v>
-      </c>
-      <c r="N2" s="1">
+        <v>84</v>
+      </c>
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="S2" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T2" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="U2" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="V2" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="W2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -778,64 +834,64 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="G3">
         <v>2702</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I3" t="s">
-        <v>69</v>
-      </c>
-      <c r="J3" s="1">
+        <v>81</v>
+      </c>
+      <c r="J3" s="2">
         <v>46279</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46281</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>72</v>
-      </c>
-      <c r="N3" s="1">
+        <v>84</v>
+      </c>
+      <c r="N3" s="2">
         <v>46312</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46290</v>
       </c>
       <c r="Q3">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S3" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T3" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="U3" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="V3" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="W3" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -843,70 +899,70 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>419</v>
+        <v>313</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E4" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="G4">
-        <v>2723</v>
+        <v>2734</v>
       </c>
       <c r="H4" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I4" t="s">
-        <v>69</v>
-      </c>
-      <c r="J4" s="1">
-        <v>46289</v>
-      </c>
-      <c r="K4" s="1">
-        <v>46289</v>
+        <v>82</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46290</v>
+      </c>
+      <c r="K4" s="2">
+        <v>46293</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>72</v>
-      </c>
-      <c r="N4" s="1">
-        <v>46320</v>
-      </c>
-      <c r="O4" s="1">
-        <v>46063</v>
+        <v>84</v>
+      </c>
+      <c r="N4" s="2">
+        <v>46304</v>
+      </c>
+      <c r="O4" s="2">
+        <v>46304</v>
       </c>
       <c r="Q4">
-        <v>-19</v>
+        <v>-2</v>
       </c>
       <c r="R4">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="S4" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T4" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="U4" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="V4" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="W4" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -920,64 +976,64 @@
         <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="G5">
         <v>2734</v>
       </c>
       <c r="H5" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I5" t="s">
-        <v>70</v>
-      </c>
-      <c r="J5" s="1">
+        <v>82</v>
+      </c>
+      <c r="J5" s="2">
         <v>46290</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46293</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>72</v>
-      </c>
-      <c r="N5" s="1">
+        <v>84</v>
+      </c>
+      <c r="N5" s="2">
         <v>46304</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46304</v>
       </c>
       <c r="Q5">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S5" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T5" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="U5" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="V5" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="W5" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -985,70 +1041,70 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="G6">
-        <v>2734</v>
+        <v>2721</v>
       </c>
       <c r="H6" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I6" t="s">
-        <v>70</v>
-      </c>
-      <c r="J6" s="1">
-        <v>46290</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46293</v>
+        <v>83</v>
+      </c>
+      <c r="J6" s="2">
+        <v>46294</v>
+      </c>
+      <c r="K6" s="2">
+        <v>46295</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>72</v>
-      </c>
-      <c r="N6" s="1">
-        <v>46304</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46304</v>
+        <v>84</v>
+      </c>
+      <c r="N6" s="2">
+        <v>46302</v>
+      </c>
+      <c r="O6" s="2">
+        <v>46297</v>
       </c>
       <c r="Q6">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S6" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T6" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="U6" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="V6" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="W6" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1056,70 +1112,67 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="F7" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="G7">
-        <v>2721</v>
+        <v>2703</v>
       </c>
       <c r="H7" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I7" t="s">
-        <v>71</v>
-      </c>
-      <c r="J7" s="1">
+        <v>81</v>
+      </c>
+      <c r="J7" s="2">
         <v>46294</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46295</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>72</v>
-      </c>
-      <c r="N7" s="1">
-        <v>46302</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46300</v>
+        <v>84</v>
+      </c>
+      <c r="N7" s="2">
+        <v>46326</v>
+      </c>
+      <c r="O7" s="2">
+        <v>46326</v>
       </c>
       <c r="Q7">
-        <v>-1</v>
+        <v>-24</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T7" t="s">
-        <v>73</v>
-      </c>
-      <c r="U7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="V7" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="W7" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1133,58 +1186,61 @@
         <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="F8" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="G8">
         <v>2703</v>
       </c>
       <c r="H8" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I8" t="s">
-        <v>69</v>
-      </c>
-      <c r="J8" s="1">
+        <v>81</v>
+      </c>
+      <c r="J8" s="2">
         <v>46294</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46295</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>72</v>
-      </c>
-      <c r="N8" s="1">
+        <v>84</v>
+      </c>
+      <c r="N8" s="2">
         <v>46326</v>
       </c>
+      <c r="O8" s="2">
+        <v>46326</v>
+      </c>
       <c r="Q8">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T8" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="V8" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="W8" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1192,46 +1248,46 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="F9" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="G9">
-        <v>2703</v>
+        <v>2723</v>
       </c>
       <c r="H9" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
-        <v>69</v>
-      </c>
-      <c r="J9" s="1">
-        <v>46294</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46295</v>
+        <v>81</v>
+      </c>
+      <c r="J9" s="2">
+        <v>46296</v>
+      </c>
+      <c r="K9" s="2">
+        <v>46296</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>72</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46326</v>
+        <v>84</v>
+      </c>
+      <c r="N9" s="2">
+        <v>46327</v>
       </c>
       <c r="Q9">
         <v>-25</v>
@@ -1240,16 +1296,13 @@
         <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T9" t="s">
-        <v>74</v>
-      </c>
-      <c r="V9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="W9" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1257,61 +1310,67 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>419</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="G10">
-        <v>2723</v>
+        <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="I10" t="s">
-        <v>69</v>
-      </c>
-      <c r="J10" s="1">
+        <v>83</v>
+      </c>
+      <c r="J10" s="2">
         <v>46296</v>
       </c>
-      <c r="K10" s="1">
-        <v>46296</v>
+      <c r="K10" s="2">
+        <v>46297</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>72</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46327</v>
+        <v>84</v>
+      </c>
+      <c r="N10" s="2">
+        <v>46304</v>
+      </c>
+      <c r="O10" s="2">
+        <v>46308</v>
       </c>
       <c r="Q10">
-        <v>-26</v>
+        <v>-2</v>
       </c>
       <c r="R10">
         <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T10" t="s">
-        <v>73</v>
+        <v>85</v>
+      </c>
+      <c r="V10" t="s">
+        <v>97</v>
       </c>
       <c r="W10" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1319,64 +1378,61 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="G11">
-        <v>2721</v>
+        <v>2708</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="I11" t="s">
-        <v>70</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46296</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46297</v>
+        <v>81</v>
+      </c>
+      <c r="J11" s="2">
+        <v>46301</v>
+      </c>
+      <c r="K11" s="2">
+        <v>46302</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>72</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46308</v>
+        <v>84</v>
+      </c>
+      <c r="N11" s="2">
+        <v>46333</v>
       </c>
       <c r="Q11">
-        <v>-7</v>
+        <v>-31</v>
       </c>
       <c r="R11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S11" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="T11" t="s">
-        <v>73</v>
-      </c>
-      <c r="V11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="W11" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1384,63 +1440,311 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="G12">
-        <v>2723</v>
+        <v>2702</v>
       </c>
       <c r="H12" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="I12" t="s">
-        <v>69</v>
-      </c>
-      <c r="J12" s="1">
+        <v>82</v>
+      </c>
+      <c r="J12" s="2">
         <v>46301</v>
       </c>
-      <c r="K12" s="1">
-        <v>46301</v>
+      <c r="K12" s="2">
+        <v>46302</v>
       </c>
       <c r="L12">
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>72</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46332</v>
+        <v>84</v>
+      </c>
+      <c r="N12" s="2">
+        <v>46313</v>
       </c>
       <c r="Q12">
-        <v>-31</v>
+        <v>-11</v>
       </c>
       <c r="R12">
         <v>0</v>
       </c>
       <c r="S12" t="s">
+        <v>86</v>
+      </c>
+      <c r="T12" t="s">
+        <v>86</v>
+      </c>
+      <c r="W12" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="A13">
+        <v>384</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="s">
         <v>73</v>
       </c>
-      <c r="T12" t="s">
-        <v>73</v>
-      </c>
-      <c r="W12" t="s">
-        <v>88</v>
-      </c>
-      <c r="AA12" t="b">
+      <c r="F13" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13">
+        <v>2742</v>
+      </c>
+      <c r="H13" t="s">
+        <v>80</v>
+      </c>
+      <c r="I13" t="s">
+        <v>81</v>
+      </c>
+      <c r="J13" s="2">
+        <v>46302</v>
+      </c>
+      <c r="K13" s="2">
+        <v>46302</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
+        <v>84</v>
+      </c>
+      <c r="N13" s="2">
+        <v>46333</v>
+      </c>
+      <c r="Q13">
+        <v>-31</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s">
+        <v>85</v>
+      </c>
+      <c r="T13" t="s">
+        <v>85</v>
+      </c>
+      <c r="W13" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27">
+      <c r="A14">
+        <v>396</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14">
+        <v>2731</v>
+      </c>
+      <c r="H14" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" t="s">
+        <v>82</v>
+      </c>
+      <c r="J14" s="2">
+        <v>46302</v>
+      </c>
+      <c r="K14" s="2">
+        <v>46302</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>84</v>
+      </c>
+      <c r="N14" s="2">
+        <v>46313</v>
+      </c>
+      <c r="Q14">
+        <v>-11</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14" t="s">
+        <v>86</v>
+      </c>
+      <c r="T14" t="s">
+        <v>86</v>
+      </c>
+      <c r="W14" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27">
+      <c r="A15">
+        <v>685</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15">
+        <v>2702</v>
+      </c>
+      <c r="H15" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" t="s">
+        <v>82</v>
+      </c>
+      <c r="J15" s="2">
+        <v>46302</v>
+      </c>
+      <c r="K15" s="2">
+        <v>46302</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>84</v>
+      </c>
+      <c r="N15" s="2">
+        <v>46313</v>
+      </c>
+      <c r="Q15">
+        <v>-11</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15" t="s">
+        <v>85</v>
+      </c>
+      <c r="T15" t="s">
+        <v>86</v>
+      </c>
+      <c r="W15" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27">
+      <c r="A16">
+        <v>685</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G16">
+        <v>2729</v>
+      </c>
+      <c r="H16" t="s">
+        <v>80</v>
+      </c>
+      <c r="I16" t="s">
+        <v>82</v>
+      </c>
+      <c r="J16" s="2">
+        <v>46302</v>
+      </c>
+      <c r="K16" s="2">
+        <v>46302</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
+        <v>84</v>
+      </c>
+      <c r="N16" s="2">
+        <v>46313</v>
+      </c>
+      <c r="Q16">
+        <v>-11</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16" t="s">
+        <v>85</v>
+      </c>
+      <c r="T16" t="s">
+        <v>86</v>
+      </c>
+      <c r="W16" t="s">
+        <v>98</v>
+      </c>
+      <c r="AA16" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (07/10/2026 14:46)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -320,16 +320,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -345,7 +337,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -353,30 +345,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -676,85 +650,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -786,10 +760,10 @@
       <c r="I2" t="s">
         <v>81</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -798,7 +772,7 @@
       <c r="M2" t="s">
         <v>84</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -854,10 +828,10 @@
       <c r="I3" t="s">
         <v>81</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46279</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46281</v>
       </c>
       <c r="L3">
@@ -866,10 +840,10 @@
       <c r="M3" t="s">
         <v>84</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46312</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46290</v>
       </c>
       <c r="Q3">
@@ -925,10 +899,10 @@
       <c r="I4" t="s">
         <v>82</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46290</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46293</v>
       </c>
       <c r="L4">
@@ -937,10 +911,10 @@
       <c r="M4" t="s">
         <v>84</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46304</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46304</v>
       </c>
       <c r="Q4">
@@ -996,10 +970,10 @@
       <c r="I5" t="s">
         <v>82</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46290</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46293</v>
       </c>
       <c r="L5">
@@ -1008,10 +982,10 @@
       <c r="M5" t="s">
         <v>84</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46304</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="1">
         <v>46304</v>
       </c>
       <c r="Q5">
@@ -1067,10 +1041,10 @@
       <c r="I6" t="s">
         <v>83</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46294</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46295</v>
       </c>
       <c r="L6">
@@ -1079,10 +1053,10 @@
       <c r="M6" t="s">
         <v>84</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46302</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46297</v>
       </c>
       <c r="Q6">
@@ -1138,10 +1112,10 @@
       <c r="I7" t="s">
         <v>81</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46294</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46295</v>
       </c>
       <c r="L7">
@@ -1150,10 +1124,10 @@
       <c r="M7" t="s">
         <v>84</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46326</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46326</v>
       </c>
       <c r="Q7">
@@ -1206,10 +1180,10 @@
       <c r="I8" t="s">
         <v>81</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46294</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46295</v>
       </c>
       <c r="L8">
@@ -1218,10 +1192,10 @@
       <c r="M8" t="s">
         <v>84</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46326</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8" s="1">
         <v>46326</v>
       </c>
       <c r="Q8">
@@ -1274,10 +1248,10 @@
       <c r="I9" t="s">
         <v>81</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46296</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46296</v>
       </c>
       <c r="L9">
@@ -1286,7 +1260,7 @@
       <c r="M9" t="s">
         <v>84</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46327</v>
       </c>
       <c r="Q9">
@@ -1336,10 +1310,10 @@
       <c r="I10" t="s">
         <v>83</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46296</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46297</v>
       </c>
       <c r="L10">
@@ -1348,10 +1322,10 @@
       <c r="M10" t="s">
         <v>84</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46304</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10" s="1">
         <v>46308</v>
       </c>
       <c r="Q10">
@@ -1404,10 +1378,10 @@
       <c r="I11" t="s">
         <v>81</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46301</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46302</v>
       </c>
       <c r="L11">
@@ -1416,7 +1390,7 @@
       <c r="M11" t="s">
         <v>84</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46333</v>
       </c>
       <c r="Q11">
@@ -1466,10 +1440,10 @@
       <c r="I12" t="s">
         <v>82</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46301</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46302</v>
       </c>
       <c r="L12">
@@ -1478,7 +1452,7 @@
       <c r="M12" t="s">
         <v>84</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46313</v>
       </c>
       <c r="Q12">
@@ -1528,10 +1502,10 @@
       <c r="I13" t="s">
         <v>81</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46302</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46302</v>
       </c>
       <c r="L13">
@@ -1540,7 +1514,7 @@
       <c r="M13" t="s">
         <v>84</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46333</v>
       </c>
       <c r="Q13">
@@ -1590,10 +1564,10 @@
       <c r="I14" t="s">
         <v>82</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46302</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46302</v>
       </c>
       <c r="L14">
@@ -1602,7 +1576,7 @@
       <c r="M14" t="s">
         <v>84</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46313</v>
       </c>
       <c r="Q14">
@@ -1652,10 +1626,10 @@
       <c r="I15" t="s">
         <v>82</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46302</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46302</v>
       </c>
       <c r="L15">
@@ -1664,7 +1638,7 @@
       <c r="M15" t="s">
         <v>84</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46313</v>
       </c>
       <c r="Q15">
@@ -1714,10 +1688,10 @@
       <c r="I16" t="s">
         <v>82</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46302</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46302</v>
       </c>
       <c r="L16">
@@ -1726,7 +1700,7 @@
       <c r="M16" t="s">
         <v>84</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46313</v>
       </c>
       <c r="Q16">

</xml_diff>

<commit_message>
Atualização automática: emergencias (08/10/2026 14:50)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="92">
   <si>
     <t>om_emg</t>
   </si>
@@ -103,12 +103,12 @@
     <t>BANT</t>
   </si>
   <si>
+    <t>CLA</t>
+  </si>
+  <si>
     <t>BABR</t>
   </si>
   <si>
-    <t>CLA</t>
-  </si>
-  <si>
     <t>DACTA II</t>
   </si>
   <si>
@@ -118,18 +118,12 @@
     <t>313260018702</t>
   </si>
   <si>
-    <t>685260012787</t>
-  </si>
-  <si>
     <t>313260018904</t>
   </si>
   <si>
     <t>313260018905</t>
   </si>
   <si>
-    <t>329260019299</t>
-  </si>
-  <si>
     <t>685260012893</t>
   </si>
   <si>
@@ -163,18 +157,12 @@
     <t>040-0043</t>
   </si>
   <si>
-    <t>S2889-3-0112</t>
-  </si>
-  <si>
     <t>2652022-18</t>
   </si>
   <si>
     <t>2651031-1</t>
   </si>
   <si>
-    <t>066-3046-07</t>
-  </si>
-  <si>
     <t>065-0042-15</t>
   </si>
   <si>
@@ -205,18 +193,12 @@
     <t>STROB TUB</t>
   </si>
   <si>
-    <t>HOSE ASSY TEE</t>
-  </si>
-  <si>
     <t>TUBE ASSY</t>
   </si>
   <si>
     <t>LEVER FUEL CON</t>
   </si>
   <si>
-    <t>CONTROL,INDICATOR</t>
-  </si>
-  <si>
     <t>AUTOPILOT COMPUTER</t>
   </si>
   <si>
@@ -280,34 +262,31 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>AWB 12759588944 - volume retirado na loja GOLLOG - NAT por teodoro silva em 25/09. Godoy 06/10/26.</t>
-  </si>
-  <si>
     <t>Cedeu o item para o 2736. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>AWB 12760704954 - volume retirado na loja GOLLOG - BSB por Kesia de Sousa. Godoy 06/10/2026</t>
+    <t>Atendido com esoque local em 08/10. Ramon 08/10/26.</t>
   </si>
   <si>
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
   </si>
   <si>
-    <t>Colocado pedido Textron IJ17740209 - tracking 539575366041 - previsão de entrega V1 RJ 23/09 - MATERIAL ENVIADO VIA RECIBO 822/FAB/26 AWB 12759588944 DPE 25/09/2026 - MATERIAL JÁ ENTREGUE NO SUPRIMENTOS BANT DIA 25/09/2026</t>
-  </si>
-  <si>
     <t>Colocado pedido Textron WB0003167445 - tracking 542505808925 - previsão de entrega V1 RJ 01/10 - MATERIAL ENVIADO PELA AWB 12761197990 dpe 08/10/2026</t>
   </si>
   <si>
-    <t>MATERIAL ENVIADO PELA AWB 12760704954 DPE 02/10/2026 - MATERIAL RETIRADO DIA 05/10/26 POR SGT KÉSIA</t>
-  </si>
-  <si>
     <t>AGD ABERTURA DE OS- REZ , email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26</t>
   </si>
   <si>
     <t>RECEBIDO 01 EA, REPARADO , DA WILLIAM EM 05/10/26. SERÁ ATD ESTA EMERG - REZ (06/10/26)</t>
   </si>
   <si>
+    <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26</t>
+  </si>
+  <si>
     <t>DPE 09/10/26 - REZ(06-10-26), email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26</t>
+  </si>
+  <si>
+    <t>Em cotação no mercado. ATZ 07/10</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -646,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA16"/>
+  <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -743,22 +722,22 @@
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -770,31 +749,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="S2" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="T2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="U2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="V2" t="s">
+        <v>84</v>
+      </c>
+      <c r="W2" t="s">
         <v>91</v>
-      </c>
-      <c r="W2" t="s">
-        <v>98</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -802,70 +781,70 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
         <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3">
+        <v>2734</v>
+      </c>
+      <c r="H3" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" t="s">
         <v>76</v>
       </c>
-      <c r="G3">
-        <v>2702</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="J3" s="1">
+        <v>46290</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46293</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>78</v>
+      </c>
+      <c r="N3" s="1">
+        <v>46304</v>
+      </c>
+      <c r="O3" s="1">
+        <v>46304</v>
+      </c>
+      <c r="Q3">
+        <v>-1</v>
+      </c>
+      <c r="R3">
+        <v>10</v>
+      </c>
+      <c r="S3" t="s">
         <v>79</v>
       </c>
-      <c r="I3" t="s">
-        <v>81</v>
-      </c>
-      <c r="J3" s="1">
-        <v>46279</v>
-      </c>
-      <c r="K3" s="1">
-        <v>46281</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3" t="s">
-        <v>84</v>
-      </c>
-      <c r="N3" s="1">
-        <v>46312</v>
-      </c>
-      <c r="O3" s="1">
-        <v>46290</v>
-      </c>
-      <c r="Q3">
-        <v>-10</v>
-      </c>
-      <c r="R3">
-        <v>21</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
+        <v>80</v>
+      </c>
+      <c r="U3" t="s">
+        <v>82</v>
+      </c>
+      <c r="V3" t="s">
         <v>85</v>
       </c>
-      <c r="T3" t="s">
-        <v>86</v>
-      </c>
-      <c r="U3" t="s">
-        <v>88</v>
-      </c>
-      <c r="V3" t="s">
-        <v>92</v>
-      </c>
       <c r="W3" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -882,22 +861,22 @@
         <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G4">
         <v>2734</v>
       </c>
       <c r="H4" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="J4" s="1">
         <v>46290</v>
@@ -909,7 +888,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N4" s="1">
         <v>46304</v>
@@ -918,25 +897,25 @@
         <v>46304</v>
       </c>
       <c r="Q4">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S4" t="s">
+        <v>79</v>
+      </c>
+      <c r="T4" t="s">
+        <v>80</v>
+      </c>
+      <c r="U4" t="s">
+        <v>82</v>
+      </c>
+      <c r="V4" t="s">
         <v>85</v>
       </c>
-      <c r="T4" t="s">
-        <v>86</v>
-      </c>
-      <c r="U4" t="s">
-        <v>89</v>
-      </c>
-      <c r="V4" t="s">
-        <v>93</v>
-      </c>
       <c r="W4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -944,70 +923,67 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="G5">
-        <v>2734</v>
+        <v>2703</v>
       </c>
       <c r="H5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I5" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>78</v>
+      </c>
+      <c r="N5" s="1">
+        <v>46326</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46326</v>
+      </c>
+      <c r="Q5">
+        <v>-23</v>
+      </c>
+      <c r="R5">
+        <v>8</v>
+      </c>
+      <c r="S5" t="s">
         <v>79</v>
       </c>
-      <c r="I5" t="s">
-        <v>82</v>
-      </c>
-      <c r="J5" s="1">
-        <v>46290</v>
-      </c>
-      <c r="K5" s="1">
-        <v>46293</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>84</v>
-      </c>
-      <c r="N5" s="1">
-        <v>46304</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46304</v>
-      </c>
-      <c r="Q5">
-        <v>-2</v>
-      </c>
-      <c r="R5">
-        <v>9</v>
-      </c>
-      <c r="S5" t="s">
-        <v>85</v>
-      </c>
       <c r="T5" t="s">
+        <v>80</v>
+      </c>
+      <c r="V5" t="s">
         <v>86</v>
       </c>
-      <c r="U5" t="s">
-        <v>89</v>
-      </c>
-      <c r="V5" t="s">
-        <v>93</v>
-      </c>
       <c r="W5" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1015,31 +991,31 @@
     </row>
     <row r="6" spans="1:27">
       <c r="A6">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="G6">
-        <v>2721</v>
+        <v>2703</v>
       </c>
       <c r="H6" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I6" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="J6" s="1">
         <v>46294</v>
@@ -1051,34 +1027,31 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N6" s="1">
-        <v>46302</v>
+        <v>46326</v>
       </c>
       <c r="O6" s="1">
-        <v>46297</v>
+        <v>46326</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>-23</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="T6" t="s">
-        <v>85</v>
-      </c>
-      <c r="U6" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="V6" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="W6" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1086,49 +1059,46 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G7">
-        <v>2703</v>
+        <v>2723</v>
       </c>
       <c r="H7" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I7" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="J7" s="1">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K7" s="1">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N7" s="1">
-        <v>46326</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46326</v>
+        <v>46327</v>
       </c>
       <c r="Q7">
         <v>-24</v>
@@ -1137,16 +1107,16 @@
         <v>7</v>
       </c>
       <c r="S7" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="T7" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="V7" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="W7" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1154,67 +1124,67 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8">
+        <v>2721</v>
+      </c>
+      <c r="H8" t="s">
+        <v>73</v>
+      </c>
+      <c r="I8" t="s">
+        <v>77</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46296</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46297</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
         <v>78</v>
       </c>
-      <c r="G8">
-        <v>2703</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="N8" s="1">
+        <v>46304</v>
+      </c>
+      <c r="O8" s="1">
+        <v>46308</v>
+      </c>
+      <c r="Q8">
+        <v>-1</v>
+      </c>
+      <c r="R8">
+        <v>6</v>
+      </c>
+      <c r="S8" t="s">
         <v>79</v>
       </c>
-      <c r="I8" t="s">
-        <v>81</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46294</v>
-      </c>
-      <c r="K8" s="1">
-        <v>46295</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>84</v>
-      </c>
-      <c r="N8" s="1">
-        <v>46326</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46326</v>
-      </c>
-      <c r="Q8">
-        <v>-24</v>
-      </c>
-      <c r="R8">
-        <v>7</v>
-      </c>
-      <c r="S8" t="s">
-        <v>85</v>
-      </c>
       <c r="T8" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="V8" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="W8" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1222,61 +1192,61 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G9">
-        <v>2723</v>
+        <v>2708</v>
       </c>
       <c r="H9" t="s">
+        <v>74</v>
+      </c>
+      <c r="I9" t="s">
+        <v>75</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46301</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46302</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>78</v>
+      </c>
+      <c r="N9" s="1">
+        <v>46333</v>
+      </c>
+      <c r="Q9">
+        <v>-30</v>
+      </c>
+      <c r="R9">
+        <v>1</v>
+      </c>
+      <c r="S9" t="s">
         <v>79</v>
       </c>
-      <c r="I9" t="s">
-        <v>81</v>
-      </c>
-      <c r="J9" s="1">
-        <v>46296</v>
-      </c>
-      <c r="K9" s="1">
-        <v>46296</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>84</v>
-      </c>
-      <c r="N9" s="1">
-        <v>46327</v>
-      </c>
-      <c r="Q9">
-        <v>-25</v>
-      </c>
-      <c r="R9">
-        <v>6</v>
-      </c>
-      <c r="S9" t="s">
-        <v>85</v>
-      </c>
       <c r="T9" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="W9" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1284,67 +1254,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G10">
-        <v>2721</v>
+        <v>2702</v>
       </c>
       <c r="H10" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46301</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46302</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+      <c r="M10" t="s">
+        <v>78</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46313</v>
+      </c>
+      <c r="Q10">
+        <v>-10</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+      <c r="S10" t="s">
+        <v>80</v>
+      </c>
+      <c r="T10" t="s">
+        <v>80</v>
+      </c>
+      <c r="U10" t="s">
         <v>83</v>
       </c>
-      <c r="J10" s="1">
-        <v>46296</v>
-      </c>
-      <c r="K10" s="1">
-        <v>46297</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10" t="s">
-        <v>84</v>
-      </c>
-      <c r="N10" s="1">
-        <v>46304</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46308</v>
-      </c>
-      <c r="Q10">
-        <v>-2</v>
-      </c>
-      <c r="R10">
-        <v>5</v>
-      </c>
-      <c r="S10" t="s">
-        <v>85</v>
-      </c>
-      <c r="T10" t="s">
-        <v>85</v>
-      </c>
-      <c r="V10" t="s">
-        <v>97</v>
-      </c>
       <c r="W10" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1352,34 +1319,34 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>685</v>
+        <v>384</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="G11">
-        <v>2708</v>
+        <v>2742</v>
       </c>
       <c r="H11" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="I11" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="J11" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K11" s="1">
         <v>46302</v>
@@ -1388,25 +1355,28 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N11" s="1">
         <v>46333</v>
       </c>
       <c r="Q11">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="T11" t="s">
-        <v>86</v>
+        <v>79</v>
+      </c>
+      <c r="V11" t="s">
+        <v>90</v>
       </c>
       <c r="W11" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1414,34 +1384,34 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
         <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" t="s">
         <v>72</v>
       </c>
-      <c r="F12" t="s">
-        <v>77</v>
-      </c>
       <c r="G12">
-        <v>2702</v>
+        <v>2731</v>
       </c>
       <c r="H12" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="I12" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="J12" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K12" s="1">
         <v>46302</v>
@@ -1450,25 +1420,28 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N12" s="1">
         <v>46313</v>
       </c>
       <c r="Q12">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="T12" t="s">
-        <v>86</v>
+        <v>80</v>
+      </c>
+      <c r="U12" t="s">
+        <v>83</v>
       </c>
       <c r="W12" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1476,31 +1449,31 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>384</v>
+        <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13">
+        <v>2702</v>
+      </c>
+      <c r="H13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" t="s">
         <v>76</v>
-      </c>
-      <c r="G13">
-        <v>2742</v>
-      </c>
-      <c r="H13" t="s">
-        <v>80</v>
-      </c>
-      <c r="I13" t="s">
-        <v>81</v>
       </c>
       <c r="J13" s="1">
         <v>46302</v>
@@ -1512,25 +1485,25 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N13" s="1">
-        <v>46333</v>
+        <v>46313</v>
       </c>
       <c r="Q13">
-        <v>-31</v>
+        <v>-10</v>
       </c>
       <c r="R13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="T13" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="W13" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1538,31 +1511,31 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14">
+        <v>2729</v>
+      </c>
+      <c r="H14" t="s">
         <v>74</v>
       </c>
-      <c r="F14" t="s">
-        <v>78</v>
-      </c>
-      <c r="G14">
-        <v>2731</v>
-      </c>
-      <c r="H14" t="s">
-        <v>80</v>
-      </c>
       <c r="I14" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="J14" s="1">
         <v>46302</v>
@@ -1574,151 +1547,27 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N14" s="1">
         <v>46313</v>
       </c>
       <c r="Q14">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S14" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="T14" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="W14" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="AA14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27">
-      <c r="A15">
-        <v>685</v>
-      </c>
-      <c r="B15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" t="s">
-        <v>78</v>
-      </c>
-      <c r="G15">
-        <v>2702</v>
-      </c>
-      <c r="H15" t="s">
-        <v>80</v>
-      </c>
-      <c r="I15" t="s">
-        <v>82</v>
-      </c>
-      <c r="J15" s="1">
-        <v>46302</v>
-      </c>
-      <c r="K15" s="1">
-        <v>46302</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15" t="s">
-        <v>84</v>
-      </c>
-      <c r="N15" s="1">
-        <v>46313</v>
-      </c>
-      <c r="Q15">
-        <v>-11</v>
-      </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15" t="s">
-        <v>85</v>
-      </c>
-      <c r="T15" t="s">
-        <v>86</v>
-      </c>
-      <c r="W15" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27">
-      <c r="A16">
-        <v>685</v>
-      </c>
-      <c r="B16" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" t="s">
-        <v>61</v>
-      </c>
-      <c r="E16" t="s">
-        <v>75</v>
-      </c>
-      <c r="F16" t="s">
-        <v>78</v>
-      </c>
-      <c r="G16">
-        <v>2729</v>
-      </c>
-      <c r="H16" t="s">
-        <v>80</v>
-      </c>
-      <c r="I16" t="s">
-        <v>82</v>
-      </c>
-      <c r="J16" s="1">
-        <v>46302</v>
-      </c>
-      <c r="K16" s="1">
-        <v>46302</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16" t="s">
-        <v>84</v>
-      </c>
-      <c r="N16" s="1">
-        <v>46313</v>
-      </c>
-      <c r="Q16">
-        <v>-11</v>
-      </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16" t="s">
-        <v>85</v>
-      </c>
-      <c r="T16" t="s">
-        <v>86</v>
-      </c>
-      <c r="W16" t="s">
-        <v>98</v>
-      </c>
-      <c r="AA16" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (09/10/2026 14:25)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="128">
   <si>
     <t>om_emg</t>
   </si>
@@ -115,6 +115,9 @@
     <t>BABE</t>
   </si>
   <si>
+    <t>BACG</t>
+  </si>
+  <si>
     <t>313260018702</t>
   </si>
   <si>
@@ -154,6 +157,42 @@
     <t>685260012948</t>
   </si>
   <si>
+    <t>329260019312</t>
+  </si>
+  <si>
+    <t>329260019313</t>
+  </si>
+  <si>
+    <t>396260016638</t>
+  </si>
+  <si>
+    <t>685260012964</t>
+  </si>
+  <si>
+    <t>690260002674</t>
+  </si>
+  <si>
+    <t>690260002675</t>
+  </si>
+  <si>
+    <t>690260002676</t>
+  </si>
+  <si>
+    <t>690260002677</t>
+  </si>
+  <si>
+    <t>690260002678</t>
+  </si>
+  <si>
+    <t>690260002679</t>
+  </si>
+  <si>
+    <t>690260002680</t>
+  </si>
+  <si>
+    <t>690260002681</t>
+  </si>
+  <si>
     <t>040-0043</t>
   </si>
   <si>
@@ -190,6 +229,39 @@
     <t>2618510-10</t>
   </si>
   <si>
+    <t>9910338-6</t>
+  </si>
+  <si>
+    <t>MS28773-05</t>
+  </si>
+  <si>
+    <t>2601266-2</t>
+  </si>
+  <si>
+    <t>103-20400</t>
+  </si>
+  <si>
+    <t>3244897-4</t>
+  </si>
+  <si>
+    <t>MS29512-5</t>
+  </si>
+  <si>
+    <t>3014223</t>
+  </si>
+  <si>
+    <t>3034792</t>
+  </si>
+  <si>
+    <t>3004085</t>
+  </si>
+  <si>
+    <t>M83248/1-029</t>
+  </si>
+  <si>
+    <t>3022375</t>
+  </si>
+  <si>
     <t>STROB TUB</t>
   </si>
   <si>
@@ -226,6 +298,36 @@
     <t>ALTERNATOR CONTROL U</t>
   </si>
   <si>
+    <t>TRANSMITTER,RATE OF</t>
+  </si>
+  <si>
+    <t>RETAINER,PACKING</t>
+  </si>
+  <si>
+    <t>COUPLING-SPLINED</t>
+  </si>
+  <si>
+    <t>BOLT,MACHINE</t>
+  </si>
+  <si>
+    <t>FUEL CONTROL UNIT</t>
+  </si>
+  <si>
+    <t>ANEL-O</t>
+  </si>
+  <si>
+    <t>PACKING,PREFORMED</t>
+  </si>
+  <si>
+    <t>BOMBA DE COMBUSTÍVEL</t>
+  </si>
+  <si>
+    <t>SEAL</t>
+  </si>
+  <si>
+    <t>SEAL,PLAIN</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -238,7 +340,7 @@
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Aguardando solução</t>
+    <t>Expedido total</t>
   </si>
   <si>
     <t>ANCE</t>
@@ -266,6 +368,12 @@
   </si>
   <si>
     <t>Atendido com esoque local em 08/10. Ramon 08/10/26.</t>
+  </si>
+  <si>
+    <t>Estoque com o Pn DCN4-3807 (Alternado). Godoy 09/10/26.</t>
+  </si>
+  <si>
+    <t>Atendido com estoque local em 09/10. Ramon 09/10/26</t>
   </si>
   <si>
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
@@ -625,7 +733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AA26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -719,25 +827,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="E2" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I2" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -749,31 +857,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="S2" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T2" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="U2" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="V2" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
       <c r="W2" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -787,25 +895,25 @@
         <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="G3">
         <v>2734</v>
       </c>
       <c r="H3" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I3" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="J3" s="1">
         <v>46290</v>
@@ -817,7 +925,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N3" s="1">
         <v>46304</v>
@@ -826,25 +934,25 @@
         <v>46304</v>
       </c>
       <c r="Q3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S3" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T3" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="U3" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="V3" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="W3" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -858,25 +966,25 @@
         <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="G4">
         <v>2734</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I4" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="J4" s="1">
         <v>46290</v>
@@ -888,7 +996,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N4" s="1">
         <v>46304</v>
@@ -897,25 +1005,25 @@
         <v>46304</v>
       </c>
       <c r="Q4">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S4" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T4" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="U4" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="V4" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="W4" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -929,25 +1037,25 @@
         <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="E5" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
       <c r="G5">
         <v>2703</v>
       </c>
       <c r="H5" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I5" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="J5" s="1">
         <v>46294</v>
@@ -959,7 +1067,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N5" s="1">
         <v>46326</v>
@@ -968,22 +1076,22 @@
         <v>46326</v>
       </c>
       <c r="Q5">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S5" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T5" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="V5" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
       <c r="W5" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -997,25 +1105,25 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="F6" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="G6">
         <v>2703</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I6" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="J6" s="1">
         <v>46294</v>
@@ -1027,7 +1135,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N6" s="1">
         <v>46326</v>
@@ -1036,22 +1144,22 @@
         <v>46326</v>
       </c>
       <c r="Q6">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S6" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T6" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="V6" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
       <c r="W6" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1065,25 +1173,25 @@
         <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
       <c r="G7">
         <v>2723</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I7" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="J7" s="1">
         <v>46296</v>
@@ -1095,28 +1203,28 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N7" s="1">
         <v>46327</v>
       </c>
       <c r="Q7">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S7" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T7" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="V7" t="s">
-        <v>88</v>
+        <v>124</v>
       </c>
       <c r="W7" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1130,25 +1238,25 @@
         <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="F8" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
       <c r="G8">
         <v>2721</v>
       </c>
       <c r="H8" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="I8" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="J8" s="1">
         <v>46296</v>
@@ -1160,31 +1268,31 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N8" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="O8" s="1">
         <v>46308</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T8" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="V8" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="W8" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1198,25 +1306,25 @@
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
       <c r="G9">
         <v>2708</v>
       </c>
       <c r="H9" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="I9" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="J9" s="1">
         <v>46301</v>
@@ -1228,25 +1336,25 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N9" s="1">
         <v>46333</v>
       </c>
       <c r="Q9">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S9" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T9" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="W9" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1260,25 +1368,25 @@
         <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="E10" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="F10" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
       <c r="G10">
         <v>2702</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="J10" s="1">
         <v>46301</v>
@@ -1290,28 +1398,28 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N10" s="1">
-        <v>46313</v>
+        <v>46333</v>
       </c>
       <c r="Q10">
-        <v>-10</v>
+        <v>-29</v>
       </c>
       <c r="R10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S10" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="T10" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="U10" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="W10" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1325,25 +1433,25 @@
         <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
       <c r="G11">
         <v>2742</v>
       </c>
       <c r="H11" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="I11" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="J11" s="1">
         <v>46302</v>
@@ -1355,28 +1463,28 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N11" s="1">
         <v>46333</v>
       </c>
       <c r="Q11">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S11" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T11" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="V11" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="W11" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1390,25 +1498,25 @@
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="F12" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="G12">
         <v>2731</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="I12" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="J12" s="1">
         <v>46302</v>
@@ -1420,28 +1528,28 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N12" s="1">
-        <v>46313</v>
+        <v>46309</v>
       </c>
       <c r="Q12">
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S12" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="T12" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="U12" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="W12" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1455,25 +1563,25 @@
         <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="F13" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="G13">
         <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="I13" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="J13" s="1">
         <v>46302</v>
@@ -1485,25 +1593,25 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N13" s="1">
-        <v>46313</v>
+        <v>46333</v>
       </c>
       <c r="Q13">
-        <v>-10</v>
+        <v>-29</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S13" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="T13" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="W13" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1517,25 +1625,25 @@
         <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>106</v>
       </c>
       <c r="G14">
         <v>2729</v>
       </c>
       <c r="H14" t="s">
-        <v>74</v>
+        <v>107</v>
       </c>
       <c r="I14" t="s">
-        <v>76</v>
+        <v>110</v>
       </c>
       <c r="J14" s="1">
         <v>46302</v>
@@ -1547,27 +1655,780 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="N14" s="1">
         <v>46313</v>
       </c>
       <c r="Q14">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S14" t="s">
+        <v>113</v>
+      </c>
+      <c r="T14" t="s">
+        <v>114</v>
+      </c>
+      <c r="W14" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27">
+      <c r="A15">
+        <v>329</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" t="s">
+        <v>94</v>
+      </c>
+      <c r="F15" t="s">
+        <v>105</v>
+      </c>
+      <c r="G15">
+        <v>2721</v>
+      </c>
+      <c r="H15" t="s">
+        <v>107</v>
+      </c>
+      <c r="I15" t="s">
+        <v>110</v>
+      </c>
+      <c r="J15" s="1">
+        <v>46304</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+      <c r="M15" t="s">
+        <v>112</v>
+      </c>
+      <c r="N15" s="1">
+        <v>46315</v>
+      </c>
+      <c r="Q15">
+        <v>-11</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15" t="s">
+        <v>113</v>
+      </c>
+      <c r="T15" t="s">
+        <v>113</v>
+      </c>
+      <c r="W15" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27">
+      <c r="A16">
+        <v>329</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" t="s">
+        <v>104</v>
+      </c>
+      <c r="G16">
+        <v>2721</v>
+      </c>
+      <c r="H16" t="s">
+        <v>107</v>
+      </c>
+      <c r="I16" t="s">
+        <v>111</v>
+      </c>
+      <c r="J16" s="1">
+        <v>46304</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16" t="s">
+        <v>112</v>
+      </c>
+      <c r="N16" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q16">
+        <v>-7</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16" t="s">
+        <v>113</v>
+      </c>
+      <c r="T16" t="s">
+        <v>113</v>
+      </c>
+      <c r="W16" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27">
+      <c r="A17">
+        <v>396</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" t="s">
+        <v>73</v>
+      </c>
+      <c r="E17" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17" t="s">
+        <v>104</v>
+      </c>
+      <c r="G17">
+        <v>2731</v>
+      </c>
+      <c r="H17" t="s">
+        <v>107</v>
+      </c>
+      <c r="I17" t="s">
+        <v>111</v>
+      </c>
+      <c r="J17" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17" t="s">
+        <v>112</v>
+      </c>
+      <c r="N17" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q17">
+        <v>-7</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17" t="s">
+        <v>113</v>
+      </c>
+      <c r="T17" t="s">
+        <v>114</v>
+      </c>
+      <c r="W17" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27">
+      <c r="A18">
+        <v>685</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18">
+        <v>2729</v>
+      </c>
+      <c r="H18" t="s">
+        <v>107</v>
+      </c>
+      <c r="I18" t="s">
+        <v>110</v>
+      </c>
+      <c r="J18" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K18" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L18">
+        <v>12</v>
+      </c>
+      <c r="M18" t="s">
+        <v>112</v>
+      </c>
+      <c r="N18" s="1">
+        <v>46315</v>
+      </c>
+      <c r="Q18">
+        <v>-11</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18" t="s">
+        <v>113</v>
+      </c>
+      <c r="T18" t="s">
+        <v>114</v>
+      </c>
+      <c r="W18" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27">
+      <c r="A19">
+        <v>690</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" t="s">
+        <v>98</v>
+      </c>
+      <c r="F19" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19">
+        <v>2727</v>
+      </c>
+      <c r="H19" t="s">
+        <v>107</v>
+      </c>
+      <c r="I19" t="s">
+        <v>111</v>
+      </c>
+      <c r="J19" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K19" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19" t="s">
+        <v>112</v>
+      </c>
+      <c r="N19" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q19">
+        <v>-7</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19" t="s">
+        <v>113</v>
+      </c>
+      <c r="T19" t="s">
+        <v>113</v>
+      </c>
+      <c r="W19" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27">
+      <c r="A20">
+        <v>690</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" t="s">
+        <v>95</v>
+      </c>
+      <c r="F20" t="s">
+        <v>104</v>
+      </c>
+      <c r="G20">
+        <v>2727</v>
+      </c>
+      <c r="H20" t="s">
+        <v>107</v>
+      </c>
+      <c r="I20" t="s">
+        <v>111</v>
+      </c>
+      <c r="J20" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K20" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L20">
+        <v>2</v>
+      </c>
+      <c r="M20" t="s">
+        <v>112</v>
+      </c>
+      <c r="N20" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q20">
+        <v>-7</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20" t="s">
+        <v>113</v>
+      </c>
+      <c r="T20" t="s">
+        <v>113</v>
+      </c>
+      <c r="W20" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27">
+      <c r="A21">
+        <v>690</v>
+      </c>
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" t="s">
+        <v>99</v>
+      </c>
+      <c r="F21" t="s">
+        <v>104</v>
+      </c>
+      <c r="G21">
+        <v>2727</v>
+      </c>
+      <c r="H21" t="s">
+        <v>107</v>
+      </c>
+      <c r="I21" t="s">
+        <v>111</v>
+      </c>
+      <c r="J21" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L21">
+        <v>2</v>
+      </c>
+      <c r="M21" t="s">
+        <v>112</v>
+      </c>
+      <c r="N21" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q21">
+        <v>-7</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21" t="s">
+        <v>114</v>
+      </c>
+      <c r="T21" t="s">
+        <v>113</v>
+      </c>
+      <c r="U21" t="s">
+        <v>118</v>
+      </c>
+      <c r="W21" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27">
+      <c r="A22">
+        <v>690</v>
+      </c>
+      <c r="B22" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" t="s">
+        <v>77</v>
+      </c>
+      <c r="E22" t="s">
+        <v>100</v>
+      </c>
+      <c r="F22" t="s">
+        <v>104</v>
+      </c>
+      <c r="G22">
+        <v>2727</v>
+      </c>
+      <c r="H22" t="s">
+        <v>107</v>
+      </c>
+      <c r="I22" t="s">
+        <v>111</v>
+      </c>
+      <c r="J22" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K22" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22" t="s">
+        <v>112</v>
+      </c>
+      <c r="N22" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q22">
+        <v>-7</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22" t="s">
+        <v>113</v>
+      </c>
+      <c r="T22" t="s">
+        <v>113</v>
+      </c>
+      <c r="W22" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27">
+      <c r="A23">
+        <v>690</v>
+      </c>
+      <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" t="s">
+        <v>78</v>
+      </c>
+      <c r="E23" t="s">
+        <v>101</v>
+      </c>
+      <c r="F23" t="s">
+        <v>105</v>
+      </c>
+      <c r="G23">
+        <v>2727</v>
+      </c>
+      <c r="H23" t="s">
+        <v>107</v>
+      </c>
+      <c r="I23" t="s">
+        <v>111</v>
+      </c>
+      <c r="J23" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K23" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23" t="s">
+        <v>112</v>
+      </c>
+      <c r="N23" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q23">
+        <v>-7</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23" t="s">
+        <v>114</v>
+      </c>
+      <c r="T23" t="s">
+        <v>113</v>
+      </c>
+      <c r="U23" t="s">
+        <v>119</v>
+      </c>
+      <c r="W23" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27">
+      <c r="A24">
+        <v>690</v>
+      </c>
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" t="s">
         <v>79</v>
       </c>
-      <c r="T14" t="s">
+      <c r="E24" t="s">
+        <v>102</v>
+      </c>
+      <c r="F24" t="s">
+        <v>104</v>
+      </c>
+      <c r="G24">
+        <v>2727</v>
+      </c>
+      <c r="H24" t="s">
+        <v>107</v>
+      </c>
+      <c r="I24" t="s">
+        <v>111</v>
+      </c>
+      <c r="J24" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K24" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L24">
+        <v>1</v>
+      </c>
+      <c r="M24" t="s">
+        <v>112</v>
+      </c>
+      <c r="N24" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q24">
+        <v>-7</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24" t="s">
+        <v>114</v>
+      </c>
+      <c r="T24" t="s">
+        <v>113</v>
+      </c>
+      <c r="W24" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27">
+      <c r="A25">
+        <v>690</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" t="s">
         <v>80</v>
       </c>
-      <c r="W14" t="s">
-        <v>91</v>
-      </c>
-      <c r="AA14" t="b">
+      <c r="E25" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" t="s">
+        <v>104</v>
+      </c>
+      <c r="G25">
+        <v>2727</v>
+      </c>
+      <c r="H25" t="s">
+        <v>107</v>
+      </c>
+      <c r="I25" t="s">
+        <v>111</v>
+      </c>
+      <c r="J25" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K25" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L25">
+        <v>1</v>
+      </c>
+      <c r="M25" t="s">
+        <v>112</v>
+      </c>
+      <c r="N25" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q25">
+        <v>-7</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25" t="s">
+        <v>114</v>
+      </c>
+      <c r="T25" t="s">
+        <v>113</v>
+      </c>
+      <c r="U25" t="s">
+        <v>119</v>
+      </c>
+      <c r="W25" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27">
+      <c r="A26">
+        <v>690</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" t="s">
+        <v>104</v>
+      </c>
+      <c r="G26">
+        <v>2727</v>
+      </c>
+      <c r="H26" t="s">
+        <v>107</v>
+      </c>
+      <c r="I26" t="s">
+        <v>111</v>
+      </c>
+      <c r="J26" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K26" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="M26" t="s">
+        <v>112</v>
+      </c>
+      <c r="N26" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q26">
+        <v>-7</v>
+      </c>
+      <c r="R26">
+        <v>0</v>
+      </c>
+      <c r="S26" t="s">
+        <v>113</v>
+      </c>
+      <c r="T26" t="s">
+        <v>113</v>
+      </c>
+      <c r="W26" t="s">
+        <v>127</v>
+      </c>
+      <c r="AA26" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (12/10/2026 17:14)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -863,10 +863,10 @@
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="R2">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="S2" t="s">
         <v>113</v>
@@ -934,10 +934,10 @@
         <v>46304</v>
       </c>
       <c r="Q3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R3">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="S3" t="s">
         <v>113</v>
@@ -1005,10 +1005,10 @@
         <v>46304</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R4">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="S4" t="s">
         <v>113</v>
@@ -1076,10 +1076,10 @@
         <v>46326</v>
       </c>
       <c r="Q5">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="R5">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S5" t="s">
         <v>113</v>
@@ -1144,10 +1144,10 @@
         <v>46326</v>
       </c>
       <c r="Q6">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="R6">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S6" t="s">
         <v>113</v>
@@ -1209,10 +1209,10 @@
         <v>46327</v>
       </c>
       <c r="Q7">
-        <v>-23</v>
+        <v>-20</v>
       </c>
       <c r="R7">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="S7" t="s">
         <v>113</v>
@@ -1277,10 +1277,10 @@
         <v>46308</v>
       </c>
       <c r="Q8">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
         <v>113</v>
@@ -1342,10 +1342,10 @@
         <v>46333</v>
       </c>
       <c r="Q9">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
         <v>113</v>
@@ -1404,10 +1404,10 @@
         <v>46333</v>
       </c>
       <c r="Q10">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
         <v>114</v>
@@ -1469,10 +1469,10 @@
         <v>46333</v>
       </c>
       <c r="Q11">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
         <v>113</v>
@@ -1534,10 +1534,10 @@
         <v>46309</v>
       </c>
       <c r="Q12">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="R12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S12" t="s">
         <v>114</v>
@@ -1599,10 +1599,10 @@
         <v>46333</v>
       </c>
       <c r="Q13">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S13" t="s">
         <v>113</v>
@@ -1661,10 +1661,10 @@
         <v>46313</v>
       </c>
       <c r="Q14">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S14" t="s">
         <v>113</v>
@@ -1723,10 +1723,10 @@
         <v>46315</v>
       </c>
       <c r="Q15">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S15" t="s">
         <v>113</v>
@@ -1785,10 +1785,10 @@
         <v>46311</v>
       </c>
       <c r="Q16">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S16" t="s">
         <v>113</v>
@@ -1847,10 +1847,10 @@
         <v>46311</v>
       </c>
       <c r="Q17">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S17" t="s">
         <v>113</v>
@@ -1909,10 +1909,10 @@
         <v>46315</v>
       </c>
       <c r="Q18">
-        <v>-11</v>
+        <v>-8</v>
       </c>
       <c r="R18">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S18" t="s">
         <v>113</v>
@@ -1971,10 +1971,10 @@
         <v>46311</v>
       </c>
       <c r="Q19">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S19" t="s">
         <v>113</v>
@@ -2033,10 +2033,10 @@
         <v>46311</v>
       </c>
       <c r="Q20">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S20" t="s">
         <v>113</v>
@@ -2095,10 +2095,10 @@
         <v>46311</v>
       </c>
       <c r="Q21">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S21" t="s">
         <v>114</v>
@@ -2160,10 +2160,10 @@
         <v>46311</v>
       </c>
       <c r="Q22">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S22" t="s">
         <v>113</v>
@@ -2222,10 +2222,10 @@
         <v>46311</v>
       </c>
       <c r="Q23">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S23" t="s">
         <v>114</v>
@@ -2287,10 +2287,10 @@
         <v>46311</v>
       </c>
       <c r="Q24">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R24">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S24" t="s">
         <v>114</v>
@@ -2349,10 +2349,10 @@
         <v>46311</v>
       </c>
       <c r="Q25">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S25" t="s">
         <v>114</v>
@@ -2414,10 +2414,10 @@
         <v>46311</v>
       </c>
       <c r="Q26">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="R26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S26" t="s">
         <v>113</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (13/10/2026 10:13)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -407,8 +407,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -424,7 +432,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -432,12 +440,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -737,85 +763,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -847,10 +873,10 @@
       <c r="I2" t="s">
         <v>109</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -859,14 +885,14 @@
       <c r="M2" t="s">
         <v>112</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S2" t="s">
         <v>113</v>
@@ -915,10 +941,10 @@
       <c r="I3" t="s">
         <v>110</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46290</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46293</v>
       </c>
       <c r="L3">
@@ -927,17 +953,17 @@
       <c r="M3" t="s">
         <v>112</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46304</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46304</v>
       </c>
       <c r="Q3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S3" t="s">
         <v>113</v>
@@ -986,10 +1012,10 @@
       <c r="I4" t="s">
         <v>110</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46290</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46293</v>
       </c>
       <c r="L4">
@@ -998,17 +1024,17 @@
       <c r="M4" t="s">
         <v>112</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46304</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46304</v>
       </c>
       <c r="Q4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S4" t="s">
         <v>113</v>
@@ -1057,10 +1083,10 @@
       <c r="I5" t="s">
         <v>109</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46294</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46295</v>
       </c>
       <c r="L5">
@@ -1069,17 +1095,17 @@
       <c r="M5" t="s">
         <v>112</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46326</v>
       </c>
-      <c r="O5" s="1">
+      <c r="O5" s="2">
         <v>46326</v>
       </c>
       <c r="Q5">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S5" t="s">
         <v>113</v>
@@ -1125,10 +1151,10 @@
       <c r="I6" t="s">
         <v>109</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46294</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46295</v>
       </c>
       <c r="L6">
@@ -1137,17 +1163,17 @@
       <c r="M6" t="s">
         <v>112</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46326</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46326</v>
       </c>
       <c r="Q6">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R6">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
         <v>113</v>
@@ -1193,10 +1219,10 @@
       <c r="I7" t="s">
         <v>109</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46296</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46296</v>
       </c>
       <c r="L7">
@@ -1205,14 +1231,14 @@
       <c r="M7" t="s">
         <v>112</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46327</v>
       </c>
       <c r="Q7">
-        <v>-20</v>
+        <v>-19</v>
       </c>
       <c r="R7">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S7" t="s">
         <v>113</v>
@@ -1258,10 +1284,10 @@
       <c r="I8" t="s">
         <v>110</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46296</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46297</v>
       </c>
       <c r="L8">
@@ -1270,17 +1296,17 @@
       <c r="M8" t="s">
         <v>112</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46308</v>
       </c>
-      <c r="O8" s="1">
+      <c r="O8" s="2">
         <v>46308</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S8" t="s">
         <v>113</v>
@@ -1326,10 +1352,10 @@
       <c r="I9" t="s">
         <v>109</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46301</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46302</v>
       </c>
       <c r="L9">
@@ -1338,14 +1364,14 @@
       <c r="M9" t="s">
         <v>112</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46333</v>
       </c>
       <c r="Q9">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
         <v>113</v>
@@ -1388,10 +1414,10 @@
       <c r="I10" t="s">
         <v>109</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46301</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46302</v>
       </c>
       <c r="L10">
@@ -1400,14 +1426,14 @@
       <c r="M10" t="s">
         <v>112</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46333</v>
       </c>
       <c r="Q10">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>114</v>
@@ -1453,10 +1479,10 @@
       <c r="I11" t="s">
         <v>109</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46302</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46302</v>
       </c>
       <c r="L11">
@@ -1465,14 +1491,14 @@
       <c r="M11" t="s">
         <v>112</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46333</v>
       </c>
       <c r="Q11">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S11" t="s">
         <v>113</v>
@@ -1518,10 +1544,10 @@
       <c r="I12" t="s">
         <v>111</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46302</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46302</v>
       </c>
       <c r="L12">
@@ -1530,14 +1556,14 @@
       <c r="M12" t="s">
         <v>112</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46309</v>
       </c>
       <c r="Q12">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S12" t="s">
         <v>114</v>
@@ -1583,10 +1609,10 @@
       <c r="I13" t="s">
         <v>109</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46302</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46302</v>
       </c>
       <c r="L13">
@@ -1595,14 +1621,14 @@
       <c r="M13" t="s">
         <v>112</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46333</v>
       </c>
       <c r="Q13">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S13" t="s">
         <v>113</v>
@@ -1645,10 +1671,10 @@
       <c r="I14" t="s">
         <v>110</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46302</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46302</v>
       </c>
       <c r="L14">
@@ -1657,14 +1683,14 @@
       <c r="M14" t="s">
         <v>112</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46313</v>
       </c>
       <c r="Q14">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S14" t="s">
         <v>113</v>
@@ -1707,10 +1733,10 @@
       <c r="I15" t="s">
         <v>110</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46304</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1719,14 +1745,14 @@
       <c r="M15" t="s">
         <v>112</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46315</v>
       </c>
       <c r="Q15">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S15" t="s">
         <v>113</v>
@@ -1769,10 +1795,10 @@
       <c r="I16" t="s">
         <v>111</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46304</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1781,14 +1807,14 @@
       <c r="M16" t="s">
         <v>112</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46311</v>
       </c>
       <c r="Q16">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S16" t="s">
         <v>113</v>
@@ -1831,10 +1857,10 @@
       <c r="I17" t="s">
         <v>111</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46303</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1843,14 +1869,14 @@
       <c r="M17" t="s">
         <v>112</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46311</v>
       </c>
       <c r="Q17">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S17" t="s">
         <v>113</v>
@@ -1893,10 +1919,10 @@
       <c r="I18" t="s">
         <v>110</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46303</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1905,14 +1931,14 @@
       <c r="M18" t="s">
         <v>112</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46315</v>
       </c>
       <c r="Q18">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="R18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S18" t="s">
         <v>113</v>
@@ -1955,10 +1981,10 @@
       <c r="I19" t="s">
         <v>111</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46303</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1967,14 +1993,14 @@
       <c r="M19" t="s">
         <v>112</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46311</v>
       </c>
       <c r="Q19">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S19" t="s">
         <v>113</v>
@@ -2017,10 +2043,10 @@
       <c r="I20" t="s">
         <v>111</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46303</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46304</v>
       </c>
       <c r="L20">
@@ -2029,14 +2055,14 @@
       <c r="M20" t="s">
         <v>112</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46311</v>
       </c>
       <c r="Q20">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S20" t="s">
         <v>113</v>
@@ -2079,10 +2105,10 @@
       <c r="I21" t="s">
         <v>111</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46303</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46304</v>
       </c>
       <c r="L21">
@@ -2091,14 +2117,14 @@
       <c r="M21" t="s">
         <v>112</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46311</v>
       </c>
       <c r="Q21">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S21" t="s">
         <v>114</v>
@@ -2144,10 +2170,10 @@
       <c r="I22" t="s">
         <v>111</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46303</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>46304</v>
       </c>
       <c r="L22">
@@ -2156,14 +2182,14 @@
       <c r="M22" t="s">
         <v>112</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <v>46311</v>
       </c>
       <c r="Q22">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S22" t="s">
         <v>113</v>
@@ -2206,10 +2232,10 @@
       <c r="I23" t="s">
         <v>111</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46303</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>46304</v>
       </c>
       <c r="L23">
@@ -2218,14 +2244,14 @@
       <c r="M23" t="s">
         <v>112</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <v>46311</v>
       </c>
       <c r="Q23">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S23" t="s">
         <v>114</v>
@@ -2271,10 +2297,10 @@
       <c r="I24" t="s">
         <v>111</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46303</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>46304</v>
       </c>
       <c r="L24">
@@ -2283,14 +2309,14 @@
       <c r="M24" t="s">
         <v>112</v>
       </c>
-      <c r="N24" s="1">
+      <c r="N24" s="2">
         <v>46311</v>
       </c>
       <c r="Q24">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S24" t="s">
         <v>114</v>
@@ -2333,10 +2359,10 @@
       <c r="I25" t="s">
         <v>111</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46303</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>46304</v>
       </c>
       <c r="L25">
@@ -2345,14 +2371,14 @@
       <c r="M25" t="s">
         <v>112</v>
       </c>
-      <c r="N25" s="1">
+      <c r="N25" s="2">
         <v>46311</v>
       </c>
       <c r="Q25">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S25" t="s">
         <v>114</v>
@@ -2398,10 +2424,10 @@
       <c r="I26" t="s">
         <v>111</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46303</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>46304</v>
       </c>
       <c r="L26">
@@ -2410,14 +2436,14 @@
       <c r="M26" t="s">
         <v>112</v>
       </c>
-      <c r="N26" s="1">
+      <c r="N26" s="2">
         <v>46311</v>
       </c>
       <c r="Q26">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S26" t="s">
         <v>113</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (13/10/2026 11:07)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="112">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,27 +106,21 @@
     <t>CLA</t>
   </si>
   <si>
+    <t>DACTA II</t>
+  </si>
+  <si>
+    <t>BABE</t>
+  </si>
+  <si>
     <t>BABR</t>
   </si>
   <si>
-    <t>DACTA II</t>
-  </si>
-  <si>
-    <t>BABE</t>
-  </si>
-  <si>
     <t>BACG</t>
   </si>
   <si>
     <t>313260018702</t>
   </si>
   <si>
-    <t>313260018904</t>
-  </si>
-  <si>
-    <t>313260018905</t>
-  </si>
-  <si>
     <t>685260012893</t>
   </si>
   <si>
@@ -136,9 +130,6 @@
     <t>419260000561</t>
   </si>
   <si>
-    <t>329260019306</t>
-  </si>
-  <si>
     <t>685260012943</t>
   </si>
   <si>
@@ -151,12 +142,6 @@
     <t>396260016636</t>
   </si>
   <si>
-    <t>685260012947</t>
-  </si>
-  <si>
-    <t>685260012948</t>
-  </si>
-  <si>
     <t>329260019312</t>
   </si>
   <si>
@@ -196,12 +181,6 @@
     <t>040-0043</t>
   </si>
   <si>
-    <t>2652022-18</t>
-  </si>
-  <si>
-    <t>2651031-1</t>
-  </si>
-  <si>
     <t>065-0042-15</t>
   </si>
   <si>
@@ -211,9 +190,6 @@
     <t>SD5H14C4527</t>
   </si>
   <si>
-    <t>200SGL119Q-2</t>
-  </si>
-  <si>
     <t>065-0042-03</t>
   </si>
   <si>
@@ -226,9 +202,6 @@
     <t>2651022-20-1</t>
   </si>
   <si>
-    <t>2618510-10</t>
-  </si>
-  <si>
     <t>9910338-6</t>
   </si>
   <si>
@@ -265,12 +238,6 @@
     <t>STROB TUB</t>
   </si>
   <si>
-    <t>TUBE ASSY</t>
-  </si>
-  <si>
-    <t>LEVER FUEL CON</t>
-  </si>
-  <si>
     <t>AUTOPILOT COMPUTER</t>
   </si>
   <si>
@@ -280,9 +247,6 @@
     <t>AIR COMPRESSOR</t>
   </si>
   <si>
-    <t>STARTER GENERATOR</t>
-  </si>
-  <si>
     <t>COMPUTER PA</t>
   </si>
   <si>
@@ -295,9 +259,6 @@
     <t>RING AY-ENGINE MOUNT</t>
   </si>
   <si>
-    <t>ALTERNATOR CONTROL U</t>
-  </si>
-  <si>
     <t>TRANSMITTER,RATE OF</t>
   </si>
   <si>
@@ -346,12 +307,12 @@
     <t>ANCE</t>
   </si>
   <si>
+    <t>AIFP</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -364,9 +325,6 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>Cedeu o item para o 2736. Ramon 28/09/26</t>
-  </si>
-  <si>
     <t>Atendido com esoque local em 08/10. Ramon 08/10/26.</t>
   </si>
   <si>
@@ -379,9 +337,6 @@
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
   </si>
   <si>
-    <t>Colocado pedido Textron WB0003167445 - tracking 542505808925 - previsão de entrega V1 RJ 01/10 - MATERIAL ENVIADO PELA AWB 12761197990 dpe 08/10/2026</t>
-  </si>
-  <si>
     <t>AGD ABERTURA DE OS- REZ , email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26</t>
   </si>
   <si>
@@ -389,9 +344,6 @@
   </si>
   <si>
     <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26</t>
-  </si>
-  <si>
-    <t>DPE 09/10/26 - REZ(06-10-26), email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26</t>
   </si>
   <si>
     <t>Em cotação no mercado. ATZ 07/10</t>
@@ -759,7 +711,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA26"/>
+  <dimension ref="A1:AA21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -856,22 +808,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I2" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="J2" s="2">
         <v>46251</v>
@@ -883,7 +835,7 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N2" s="2">
         <v>46280</v>
@@ -895,19 +847,19 @@
         <v>59</v>
       </c>
       <c r="S2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T2" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="U2" t="s">
-        <v>115</v>
+        <v>102</v>
       </c>
       <c r="V2" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="W2" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -915,70 +867,67 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="G3">
-        <v>2734</v>
+        <v>2703</v>
       </c>
       <c r="H3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J3" s="2">
+        <v>46294</v>
+      </c>
+      <c r="K3" s="2">
+        <v>46295</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>99</v>
+      </c>
+      <c r="N3" s="2">
+        <v>46326</v>
+      </c>
+      <c r="O3" s="2">
+        <v>46326</v>
+      </c>
+      <c r="Q3">
+        <v>-18</v>
+      </c>
+      <c r="R3">
+        <v>13</v>
+      </c>
+      <c r="S3" t="s">
+        <v>100</v>
+      </c>
+      <c r="T3" t="s">
+        <v>101</v>
+      </c>
+      <c r="V3" t="s">
         <v>107</v>
       </c>
-      <c r="I3" t="s">
-        <v>110</v>
-      </c>
-      <c r="J3" s="2">
-        <v>46290</v>
-      </c>
-      <c r="K3" s="2">
-        <v>46293</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3" t="s">
-        <v>112</v>
-      </c>
-      <c r="N3" s="2">
-        <v>46304</v>
-      </c>
-      <c r="O3" s="2">
-        <v>46304</v>
-      </c>
-      <c r="Q3">
-        <v>4</v>
-      </c>
-      <c r="R3">
-        <v>15</v>
-      </c>
-      <c r="S3" t="s">
-        <v>113</v>
-      </c>
-      <c r="T3" t="s">
-        <v>114</v>
-      </c>
-      <c r="U3" t="s">
-        <v>116</v>
-      </c>
-      <c r="V3" t="s">
-        <v>121</v>
-      </c>
       <c r="W3" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -986,70 +935,67 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="G4">
-        <v>2734</v>
+        <v>2703</v>
       </c>
       <c r="H4" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I4" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="J4" s="2">
-        <v>46290</v>
+        <v>46294</v>
       </c>
       <c r="K4" s="2">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N4" s="2">
-        <v>46304</v>
+        <v>46326</v>
       </c>
       <c r="O4" s="2">
-        <v>46304</v>
+        <v>46326</v>
       </c>
       <c r="Q4">
-        <v>4</v>
+        <v>-18</v>
       </c>
       <c r="R4">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="S4" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T4" t="s">
-        <v>114</v>
-      </c>
-      <c r="U4" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="V4" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="W4" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1057,67 +1003,64 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="F5" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G5">
-        <v>2703</v>
+        <v>2723</v>
       </c>
       <c r="H5" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I5" t="s">
+        <v>96</v>
+      </c>
+      <c r="J5" s="2">
+        <v>46296</v>
+      </c>
+      <c r="K5" s="2">
+        <v>46296</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>99</v>
+      </c>
+      <c r="N5" s="2">
+        <v>46327</v>
+      </c>
+      <c r="Q5">
+        <v>-19</v>
+      </c>
+      <c r="R5">
+        <v>12</v>
+      </c>
+      <c r="S5" t="s">
+        <v>100</v>
+      </c>
+      <c r="T5" t="s">
+        <v>100</v>
+      </c>
+      <c r="V5" t="s">
         <v>109</v>
       </c>
-      <c r="J5" s="2">
-        <v>46294</v>
-      </c>
-      <c r="K5" s="2">
-        <v>46295</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>112</v>
-      </c>
-      <c r="N5" s="2">
-        <v>46326</v>
-      </c>
-      <c r="O5" s="2">
-        <v>46326</v>
-      </c>
-      <c r="Q5">
-        <v>-18</v>
-      </c>
-      <c r="R5">
-        <v>13</v>
-      </c>
-      <c r="S5" t="s">
-        <v>113</v>
-      </c>
-      <c r="T5" t="s">
-        <v>114</v>
-      </c>
-      <c r="V5" t="s">
-        <v>122</v>
-      </c>
       <c r="W5" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1134,58 +1077,52 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="F6" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="G6">
-        <v>2703</v>
+        <v>2708</v>
       </c>
       <c r="H6" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I6" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="J6" s="2">
-        <v>46294</v>
+        <v>46301</v>
       </c>
       <c r="K6" s="2">
-        <v>46295</v>
+        <v>46302</v>
       </c>
       <c r="L6">
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N6" s="2">
-        <v>46326</v>
-      </c>
-      <c r="O6" s="2">
-        <v>46326</v>
+        <v>46333</v>
       </c>
       <c r="Q6">
-        <v>-18</v>
+        <v>-25</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="S6" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T6" t="s">
-        <v>114</v>
-      </c>
-      <c r="V6" t="s">
-        <v>123</v>
+        <v>101</v>
       </c>
       <c r="W6" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1193,64 +1130,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="E7" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G7">
-        <v>2723</v>
+        <v>2702</v>
       </c>
       <c r="H7" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="I7" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="J7" s="2">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K7" s="2">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N7" s="2">
-        <v>46327</v>
+        <v>46333</v>
       </c>
       <c r="Q7">
-        <v>-19</v>
+        <v>-25</v>
       </c>
       <c r="R7">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="S7" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="T7" t="s">
-        <v>113</v>
-      </c>
-      <c r="V7" t="s">
-        <v>124</v>
+        <v>101</v>
+      </c>
+      <c r="U7" t="s">
+        <v>103</v>
       </c>
       <c r="W7" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1258,7 +1195,7 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>329</v>
+        <v>384</v>
       </c>
       <c r="B8" t="s">
         <v>30</v>
@@ -1267,58 +1204,55 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="G8">
-        <v>2721</v>
+        <v>2742</v>
       </c>
       <c r="H8" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I8" t="s">
+        <v>96</v>
+      </c>
+      <c r="J8" s="2">
+        <v>46302</v>
+      </c>
+      <c r="K8" s="2">
+        <v>46302</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>99</v>
+      </c>
+      <c r="N8" s="2">
+        <v>46333</v>
+      </c>
+      <c r="Q8">
+        <v>-25</v>
+      </c>
+      <c r="R8">
+        <v>6</v>
+      </c>
+      <c r="S8" t="s">
+        <v>100</v>
+      </c>
+      <c r="T8" t="s">
+        <v>100</v>
+      </c>
+      <c r="V8" t="s">
         <v>110</v>
       </c>
-      <c r="J8" s="2">
-        <v>46296</v>
-      </c>
-      <c r="K8" s="2">
-        <v>46297</v>
-      </c>
-      <c r="L8">
-        <v>1</v>
-      </c>
-      <c r="M8" t="s">
-        <v>112</v>
-      </c>
-      <c r="N8" s="2">
-        <v>46308</v>
-      </c>
-      <c r="O8" s="2">
-        <v>46308</v>
-      </c>
-      <c r="Q8">
-        <v>0</v>
-      </c>
-      <c r="R8">
-        <v>11</v>
-      </c>
-      <c r="S8" t="s">
-        <v>113</v>
-      </c>
-      <c r="T8" t="s">
-        <v>113</v>
-      </c>
-      <c r="V8" t="s">
-        <v>125</v>
-      </c>
       <c r="W8" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1326,34 +1260,34 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="G9">
-        <v>2708</v>
+        <v>2731</v>
       </c>
       <c r="H9" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="I9" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="J9" s="2">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K9" s="2">
         <v>46302</v>
@@ -1362,25 +1296,28 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N9" s="2">
-        <v>46333</v>
+        <v>46309</v>
       </c>
       <c r="Q9">
-        <v>-25</v>
+        <v>-1</v>
       </c>
       <c r="R9">
         <v>6</v>
       </c>
       <c r="S9" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="T9" t="s">
-        <v>114</v>
+        <v>101</v>
+      </c>
+      <c r="U9" t="s">
+        <v>103</v>
       </c>
       <c r="W9" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1388,64 +1325,61 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E10" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="G10">
-        <v>2702</v>
+        <v>2721</v>
       </c>
       <c r="H10" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="I10" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="J10" s="2">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="K10" s="2">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N10" s="2">
-        <v>46333</v>
+        <v>46315</v>
       </c>
       <c r="Q10">
-        <v>-25</v>
+        <v>-7</v>
       </c>
       <c r="R10">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S10" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="T10" t="s">
-        <v>114</v>
-      </c>
-      <c r="U10" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="W10" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1453,64 +1387,61 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" t="s">
         <v>91</v>
       </c>
-      <c r="F11" t="s">
-        <v>104</v>
-      </c>
       <c r="G11">
-        <v>2742</v>
+        <v>2721</v>
       </c>
       <c r="H11" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I11" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="J11" s="2">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="K11" s="2">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N11" s="2">
-        <v>46333</v>
+        <v>46311</v>
       </c>
       <c r="Q11">
-        <v>-25</v>
+        <v>-3</v>
       </c>
       <c r="R11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S11" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T11" t="s">
-        <v>113</v>
-      </c>
-      <c r="V11" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="W11" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1521,61 +1452,58 @@
         <v>396</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="G12">
         <v>2731</v>
       </c>
       <c r="H12" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="I12" t="s">
+        <v>97</v>
+      </c>
+      <c r="J12" s="2">
+        <v>46303</v>
+      </c>
+      <c r="K12" s="2">
+        <v>46304</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>99</v>
+      </c>
+      <c r="N12" s="2">
+        <v>46311</v>
+      </c>
+      <c r="Q12">
+        <v>-3</v>
+      </c>
+      <c r="R12">
+        <v>4</v>
+      </c>
+      <c r="S12" t="s">
+        <v>100</v>
+      </c>
+      <c r="T12" t="s">
+        <v>101</v>
+      </c>
+      <c r="W12" t="s">
         <v>111</v>
-      </c>
-      <c r="J12" s="2">
-        <v>46302</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46302</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>112</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46309</v>
-      </c>
-      <c r="Q12">
-        <v>-1</v>
-      </c>
-      <c r="R12">
-        <v>6</v>
-      </c>
-      <c r="S12" t="s">
-        <v>114</v>
-      </c>
-      <c r="T12" t="s">
-        <v>114</v>
-      </c>
-      <c r="U12" t="s">
-        <v>117</v>
-      </c>
-      <c r="W12" t="s">
-        <v>127</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1592,52 +1520,52 @@
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="G13">
-        <v>2702</v>
+        <v>2729</v>
       </c>
       <c r="H13" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I13" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="J13" s="2">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="K13" s="2">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="L13">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M13" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N13" s="2">
-        <v>46333</v>
+        <v>46315</v>
       </c>
       <c r="Q13">
-        <v>-25</v>
+        <v>-7</v>
       </c>
       <c r="R13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S13" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T13" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="W13" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1645,61 +1573,61 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="G14">
-        <v>2729</v>
+        <v>2727</v>
       </c>
       <c r="H14" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I14" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="J14" s="2">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="K14" s="2">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N14" s="2">
-        <v>46313</v>
+        <v>46311</v>
       </c>
       <c r="Q14">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="R14">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S14" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T14" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="W14" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1707,61 +1635,61 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>329</v>
+        <v>690</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="E15" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" t="s">
+        <v>91</v>
+      </c>
+      <c r="G15">
+        <v>2727</v>
+      </c>
+      <c r="H15" t="s">
         <v>94</v>
       </c>
-      <c r="F15" t="s">
-        <v>105</v>
-      </c>
-      <c r="G15">
-        <v>2721</v>
-      </c>
-      <c r="H15" t="s">
-        <v>107</v>
-      </c>
       <c r="I15" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="J15" s="2">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K15" s="2">
         <v>46304</v>
       </c>
       <c r="L15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M15" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N15" s="2">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="Q15">
-        <v>-7</v>
+        <v>-3</v>
       </c>
       <c r="R15">
         <v>4</v>
       </c>
       <c r="S15" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T15" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="W15" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1769,43 +1697,43 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16">
-        <v>329</v>
+        <v>690</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
         <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E16" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="F16" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G16">
-        <v>2721</v>
+        <v>2727</v>
       </c>
       <c r="H16" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I16" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="J16" s="2">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K16" s="2">
         <v>46304</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M16" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N16" s="2">
         <v>46311</v>
@@ -1817,13 +1745,16 @@
         <v>4</v>
       </c>
       <c r="S16" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="T16" t="s">
-        <v>113</v>
+        <v>100</v>
+      </c>
+      <c r="U16" t="s">
+        <v>104</v>
       </c>
       <c r="W16" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1831,31 +1762,31 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>396</v>
+        <v>690</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
         <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="F17" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G17">
-        <v>2731</v>
+        <v>2727</v>
       </c>
       <c r="H17" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I17" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="J17" s="2">
         <v>46303</v>
@@ -1867,7 +1798,7 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N17" s="2">
         <v>46311</v>
@@ -1879,13 +1810,13 @@
         <v>4</v>
       </c>
       <c r="S17" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="T17" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="W17" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1893,31 +1824,31 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
         <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E18" t="s">
+        <v>88</v>
+      </c>
+      <c r="F18" t="s">
+        <v>92</v>
+      </c>
+      <c r="G18">
+        <v>2727</v>
+      </c>
+      <c r="H18" t="s">
+        <v>94</v>
+      </c>
+      <c r="I18" t="s">
         <v>97</v>
-      </c>
-      <c r="F18" t="s">
-        <v>104</v>
-      </c>
-      <c r="G18">
-        <v>2729</v>
-      </c>
-      <c r="H18" t="s">
-        <v>107</v>
-      </c>
-      <c r="I18" t="s">
-        <v>110</v>
       </c>
       <c r="J18" s="2">
         <v>46303</v>
@@ -1926,28 +1857,31 @@
         <v>46304</v>
       </c>
       <c r="L18">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N18" s="2">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="Q18">
-        <v>-7</v>
+        <v>-3</v>
       </c>
       <c r="R18">
         <v>4</v>
       </c>
       <c r="S18" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="T18" t="s">
-        <v>114</v>
+        <v>100</v>
+      </c>
+      <c r="U18" t="s">
+        <v>105</v>
       </c>
       <c r="W18" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1964,22 +1898,22 @@
         <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="F19" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="G19">
         <v>2727</v>
       </c>
       <c r="H19" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I19" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="J19" s="2">
         <v>46303</v>
@@ -1991,7 +1925,7 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N19" s="2">
         <v>46311</v>
@@ -2003,13 +1937,13 @@
         <v>4</v>
       </c>
       <c r="S19" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="T19" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="W19" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2026,22 +1960,22 @@
         <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E20" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="F20" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G20">
         <v>2727</v>
       </c>
       <c r="H20" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I20" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="J20" s="2">
         <v>46303</v>
@@ -2050,10 +1984,10 @@
         <v>46304</v>
       </c>
       <c r="L20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N20" s="2">
         <v>46311</v>
@@ -2065,13 +1999,16 @@
         <v>4</v>
       </c>
       <c r="S20" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="T20" t="s">
-        <v>113</v>
+        <v>100</v>
+      </c>
+      <c r="U20" t="s">
+        <v>105</v>
       </c>
       <c r="W20" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2088,22 +2025,22 @@
         <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E21" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="F21" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="G21">
         <v>2727</v>
       </c>
       <c r="H21" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="I21" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="J21" s="2">
         <v>46303</v>
@@ -2112,10 +2049,10 @@
         <v>46304</v>
       </c>
       <c r="L21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="N21" s="2">
         <v>46311</v>
@@ -2127,334 +2064,15 @@
         <v>4</v>
       </c>
       <c r="S21" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="T21" t="s">
-        <v>113</v>
-      </c>
-      <c r="U21" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="W21" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="AA21" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:27">
-      <c r="A22">
-        <v>690</v>
-      </c>
-      <c r="B22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C22" t="s">
-        <v>54</v>
-      </c>
-      <c r="D22" t="s">
-        <v>77</v>
-      </c>
-      <c r="E22" t="s">
-        <v>100</v>
-      </c>
-      <c r="F22" t="s">
-        <v>104</v>
-      </c>
-      <c r="G22">
-        <v>2727</v>
-      </c>
-      <c r="H22" t="s">
-        <v>107</v>
-      </c>
-      <c r="I22" t="s">
-        <v>111</v>
-      </c>
-      <c r="J22" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K22" s="2">
-        <v>46304</v>
-      </c>
-      <c r="L22">
-        <v>1</v>
-      </c>
-      <c r="M22" t="s">
-        <v>112</v>
-      </c>
-      <c r="N22" s="2">
-        <v>46311</v>
-      </c>
-      <c r="Q22">
-        <v>-3</v>
-      </c>
-      <c r="R22">
-        <v>4</v>
-      </c>
-      <c r="S22" t="s">
-        <v>113</v>
-      </c>
-      <c r="T22" t="s">
-        <v>113</v>
-      </c>
-      <c r="W22" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA22" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:27">
-      <c r="A23">
-        <v>690</v>
-      </c>
-      <c r="B23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" t="s">
-        <v>55</v>
-      </c>
-      <c r="D23" t="s">
-        <v>78</v>
-      </c>
-      <c r="E23" t="s">
-        <v>101</v>
-      </c>
-      <c r="F23" t="s">
-        <v>105</v>
-      </c>
-      <c r="G23">
-        <v>2727</v>
-      </c>
-      <c r="H23" t="s">
-        <v>107</v>
-      </c>
-      <c r="I23" t="s">
-        <v>111</v>
-      </c>
-      <c r="J23" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K23" s="2">
-        <v>46304</v>
-      </c>
-      <c r="L23">
-        <v>1</v>
-      </c>
-      <c r="M23" t="s">
-        <v>112</v>
-      </c>
-      <c r="N23" s="2">
-        <v>46311</v>
-      </c>
-      <c r="Q23">
-        <v>-3</v>
-      </c>
-      <c r="R23">
-        <v>4</v>
-      </c>
-      <c r="S23" t="s">
-        <v>114</v>
-      </c>
-      <c r="T23" t="s">
-        <v>113</v>
-      </c>
-      <c r="U23" t="s">
-        <v>119</v>
-      </c>
-      <c r="W23" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:27">
-      <c r="A24">
-        <v>690</v>
-      </c>
-      <c r="B24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" t="s">
-        <v>56</v>
-      </c>
-      <c r="D24" t="s">
-        <v>79</v>
-      </c>
-      <c r="E24" t="s">
-        <v>102</v>
-      </c>
-      <c r="F24" t="s">
-        <v>104</v>
-      </c>
-      <c r="G24">
-        <v>2727</v>
-      </c>
-      <c r="H24" t="s">
-        <v>107</v>
-      </c>
-      <c r="I24" t="s">
-        <v>111</v>
-      </c>
-      <c r="J24" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K24" s="2">
-        <v>46304</v>
-      </c>
-      <c r="L24">
-        <v>1</v>
-      </c>
-      <c r="M24" t="s">
-        <v>112</v>
-      </c>
-      <c r="N24" s="2">
-        <v>46311</v>
-      </c>
-      <c r="Q24">
-        <v>-3</v>
-      </c>
-      <c r="R24">
-        <v>4</v>
-      </c>
-      <c r="S24" t="s">
-        <v>114</v>
-      </c>
-      <c r="T24" t="s">
-        <v>113</v>
-      </c>
-      <c r="W24" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:27">
-      <c r="A25">
-        <v>690</v>
-      </c>
-      <c r="B25" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" t="s">
-        <v>80</v>
-      </c>
-      <c r="E25" t="s">
-        <v>99</v>
-      </c>
-      <c r="F25" t="s">
-        <v>104</v>
-      </c>
-      <c r="G25">
-        <v>2727</v>
-      </c>
-      <c r="H25" t="s">
-        <v>107</v>
-      </c>
-      <c r="I25" t="s">
-        <v>111</v>
-      </c>
-      <c r="J25" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K25" s="2">
-        <v>46304</v>
-      </c>
-      <c r="L25">
-        <v>1</v>
-      </c>
-      <c r="M25" t="s">
-        <v>112</v>
-      </c>
-      <c r="N25" s="2">
-        <v>46311</v>
-      </c>
-      <c r="Q25">
-        <v>-3</v>
-      </c>
-      <c r="R25">
-        <v>4</v>
-      </c>
-      <c r="S25" t="s">
-        <v>114</v>
-      </c>
-      <c r="T25" t="s">
-        <v>113</v>
-      </c>
-      <c r="U25" t="s">
-        <v>119</v>
-      </c>
-      <c r="W25" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA25" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:27">
-      <c r="A26">
-        <v>690</v>
-      </c>
-      <c r="B26" t="s">
-        <v>33</v>
-      </c>
-      <c r="C26" t="s">
-        <v>58</v>
-      </c>
-      <c r="D26" t="s">
-        <v>81</v>
-      </c>
-      <c r="E26" t="s">
-        <v>103</v>
-      </c>
-      <c r="F26" t="s">
-        <v>104</v>
-      </c>
-      <c r="G26">
-        <v>2727</v>
-      </c>
-      <c r="H26" t="s">
-        <v>107</v>
-      </c>
-      <c r="I26" t="s">
-        <v>111</v>
-      </c>
-      <c r="J26" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K26" s="2">
-        <v>46304</v>
-      </c>
-      <c r="L26">
-        <v>1</v>
-      </c>
-      <c r="M26" t="s">
-        <v>112</v>
-      </c>
-      <c r="N26" s="2">
-        <v>46311</v>
-      </c>
-      <c r="Q26">
-        <v>-3</v>
-      </c>
-      <c r="R26">
-        <v>4</v>
-      </c>
-      <c r="S26" t="s">
-        <v>113</v>
-      </c>
-      <c r="T26" t="s">
-        <v>113</v>
-      </c>
-      <c r="W26" t="s">
-        <v>127</v>
-      </c>
-      <c r="AA26" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (13/10/2026 15:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -359,16 +359,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -384,7 +376,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -392,30 +384,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -715,85 +689,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -825,10 +799,10 @@
       <c r="I2" t="s">
         <v>96</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -837,7 +811,7 @@
       <c r="M2" t="s">
         <v>99</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -893,10 +867,10 @@
       <c r="I3" t="s">
         <v>96</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46294</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -905,10 +879,10 @@
       <c r="M3" t="s">
         <v>99</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46326</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46326</v>
       </c>
       <c r="Q3">
@@ -961,10 +935,10 @@
       <c r="I4" t="s">
         <v>96</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46294</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -973,10 +947,10 @@
       <c r="M4" t="s">
         <v>99</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46326</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46326</v>
       </c>
       <c r="Q4">
@@ -1029,10 +1003,10 @@
       <c r="I5" t="s">
         <v>96</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46296</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1041,7 +1015,7 @@
       <c r="M5" t="s">
         <v>99</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
@@ -1094,10 +1068,10 @@
       <c r="I6" t="s">
         <v>96</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46301</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1106,7 +1080,7 @@
       <c r="M6" t="s">
         <v>99</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46333</v>
       </c>
       <c r="Q6">
@@ -1156,10 +1130,10 @@
       <c r="I7" t="s">
         <v>96</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46301</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1168,7 +1142,7 @@
       <c r="M7" t="s">
         <v>99</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46333</v>
       </c>
       <c r="Q7">
@@ -1221,10 +1195,10 @@
       <c r="I8" t="s">
         <v>96</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46302</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46302</v>
       </c>
       <c r="L8">
@@ -1233,7 +1207,7 @@
       <c r="M8" t="s">
         <v>99</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46333</v>
       </c>
       <c r="Q8">
@@ -1286,10 +1260,10 @@
       <c r="I9" t="s">
         <v>97</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46302</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46302</v>
       </c>
       <c r="L9">
@@ -1298,7 +1272,7 @@
       <c r="M9" t="s">
         <v>99</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46309</v>
       </c>
       <c r="Q9">
@@ -1351,10 +1325,10 @@
       <c r="I10" t="s">
         <v>98</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46304</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1363,7 +1337,7 @@
       <c r="M10" t="s">
         <v>99</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46315</v>
       </c>
       <c r="Q10">
@@ -1413,10 +1387,10 @@
       <c r="I11" t="s">
         <v>97</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46304</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1425,7 +1399,7 @@
       <c r="M11" t="s">
         <v>99</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46311</v>
       </c>
       <c r="Q11">
@@ -1475,10 +1449,10 @@
       <c r="I12" t="s">
         <v>97</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46303</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1487,7 +1461,7 @@
       <c r="M12" t="s">
         <v>99</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46311</v>
       </c>
       <c r="Q12">
@@ -1537,10 +1511,10 @@
       <c r="I13" t="s">
         <v>98</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46303</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1549,7 +1523,7 @@
       <c r="M13" t="s">
         <v>99</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46315</v>
       </c>
       <c r="Q13">
@@ -1599,10 +1573,10 @@
       <c r="I14" t="s">
         <v>97</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46303</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1611,7 +1585,7 @@
       <c r="M14" t="s">
         <v>99</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46311</v>
       </c>
       <c r="Q14">
@@ -1661,10 +1635,10 @@
       <c r="I15" t="s">
         <v>97</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46303</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1673,7 +1647,7 @@
       <c r="M15" t="s">
         <v>99</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46311</v>
       </c>
       <c r="Q15">
@@ -1723,10 +1697,10 @@
       <c r="I16" t="s">
         <v>97</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46303</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1735,7 +1709,7 @@
       <c r="M16" t="s">
         <v>99</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46311</v>
       </c>
       <c r="Q16">
@@ -1788,10 +1762,10 @@
       <c r="I17" t="s">
         <v>97</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46303</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1800,7 +1774,7 @@
       <c r="M17" t="s">
         <v>99</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>46311</v>
       </c>
       <c r="Q17">
@@ -1850,10 +1824,10 @@
       <c r="I18" t="s">
         <v>97</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46303</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1862,7 +1836,7 @@
       <c r="M18" t="s">
         <v>99</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>46311</v>
       </c>
       <c r="Q18">
@@ -1915,10 +1889,10 @@
       <c r="I19" t="s">
         <v>97</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46303</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1927,7 +1901,7 @@
       <c r="M19" t="s">
         <v>99</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19" s="1">
         <v>46311</v>
       </c>
       <c r="Q19">
@@ -1977,10 +1951,10 @@
       <c r="I20" t="s">
         <v>97</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46303</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>46304</v>
       </c>
       <c r="L20">
@@ -1989,7 +1963,7 @@
       <c r="M20" t="s">
         <v>99</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46311</v>
       </c>
       <c r="Q20">
@@ -2042,10 +2016,10 @@
       <c r="I21" t="s">
         <v>97</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46303</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>46304</v>
       </c>
       <c r="L21">
@@ -2054,7 +2028,7 @@
       <c r="M21" t="s">
         <v>99</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46311</v>
       </c>
       <c r="Q21">

</xml_diff>

<commit_message>
Atualização automática: emergencias (14/10/2026 12:48)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="117">
   <si>
     <t>om_emg</t>
   </si>
@@ -109,12 +109,12 @@
     <t>DACTA II</t>
   </si>
   <si>
+    <t>BABR</t>
+  </si>
+  <si>
     <t>BABE</t>
   </si>
   <si>
-    <t>BABR</t>
-  </si>
-  <si>
     <t>BACG</t>
   </si>
   <si>
@@ -133,15 +133,9 @@
     <t>685260012943</t>
   </si>
   <si>
-    <t>685260012944</t>
-  </si>
-  <si>
     <t>384260009403</t>
   </si>
   <si>
-    <t>396260016636</t>
-  </si>
-  <si>
     <t>329260019312</t>
   </si>
   <si>
@@ -178,6 +172,18 @@
     <t>690260002681</t>
   </si>
   <si>
+    <t>329260019318</t>
+  </si>
+  <si>
+    <t>329260019319</t>
+  </si>
+  <si>
+    <t>396260016644</t>
+  </si>
+  <si>
+    <t>685260012971</t>
+  </si>
+  <si>
     <t>040-0043</t>
   </si>
   <si>
@@ -193,15 +199,9 @@
     <t>065-0042-03</t>
   </si>
   <si>
-    <t>066-1055-00</t>
-  </si>
-  <si>
     <t>9514A-1</t>
   </si>
   <si>
-    <t>2651022-20-1</t>
-  </si>
-  <si>
     <t>9910338-6</t>
   </si>
   <si>
@@ -235,6 +235,18 @@
     <t>3022375</t>
   </si>
   <si>
+    <t>9910592-2</t>
+  </si>
+  <si>
+    <t>C611008-0101</t>
+  </si>
+  <si>
+    <t>3244809-4</t>
+  </si>
+  <si>
+    <t>066-3046-01</t>
+  </si>
+  <si>
     <t>STROB TUB</t>
   </si>
   <si>
@@ -250,15 +262,9 @@
     <t>COMPUTER PA</t>
   </si>
   <si>
-    <t>AUDIO CONTROL PANEL</t>
-  </si>
-  <si>
     <t>PUMP ASSY</t>
   </si>
   <si>
-    <t>RING AY-ENGINE MOUNT</t>
-  </si>
-  <si>
     <t>TRANSMITTER,RATE OF</t>
   </si>
   <si>
@@ -289,6 +295,18 @@
     <t>SEAL,PLAIN</t>
   </si>
   <si>
+    <t>ALTERNADOR</t>
+  </si>
+  <si>
+    <t>ALTERNATOR CONTROL U</t>
+  </si>
+  <si>
+    <t>FUEL CONTROL,MAIN,TU</t>
+  </si>
+  <si>
+    <t>CONTROL,INDICATOR</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -301,18 +319,18 @@
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Expedido total</t>
+    <t>Aguardando solução</t>
   </si>
   <si>
     <t>ANCE</t>
   </si>
   <si>
+    <t>IPLR</t>
+  </si>
+  <si>
     <t>AIFP</t>
   </si>
   <si>
-    <t>IPLR</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -325,13 +343,10 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>Atendido com esoque local em 08/10. Ramon 08/10/26.</t>
-  </si>
-  <si>
     <t>Estoque com o Pn DCN4-3807 (Alternado). Godoy 09/10/26.</t>
   </si>
   <si>
-    <t>Atendido com estoque local em 09/10. Ramon 09/10/26</t>
+    <t>Atendido com estoque local em 09/10. Ramon 09/10/26. AWB 127-6253 8910 liberado para retirada em 13/10. Ramon 14/10/26.</t>
   </si>
   <si>
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
@@ -685,7 +700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA21"/>
+  <dimension ref="A1:AA23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -782,22 +797,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -809,31 +824,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="R2">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="S2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="U2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="V2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="W2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -850,22 +865,22 @@
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G3">
         <v>2703</v>
       </c>
       <c r="H3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J3" s="1">
         <v>46294</v>
@@ -877,7 +892,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N3" s="1">
         <v>46326</v>
@@ -886,22 +901,22 @@
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R3">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="V3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="W3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -918,22 +933,22 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F4" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="G4">
         <v>2703</v>
       </c>
       <c r="H4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I4" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J4" s="1">
         <v>46294</v>
@@ -945,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N4" s="1">
         <v>46326</v>
@@ -954,22 +969,22 @@
         <v>46326</v>
       </c>
       <c r="Q4">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S4" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T4" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="V4" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="W4" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -986,22 +1001,22 @@
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G5">
         <v>2723</v>
       </c>
       <c r="H5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J5" s="1">
         <v>46296</v>
@@ -1013,28 +1028,28 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R5">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="V5" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="W5" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1051,22 +1066,22 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G6">
         <v>2708</v>
       </c>
       <c r="H6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I6" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J6" s="1">
         <v>46301</v>
@@ -1078,25 +1093,25 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N6" s="1">
         <v>46333</v>
       </c>
       <c r="Q6">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T6" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="W6" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1104,34 +1119,34 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>685</v>
+        <v>384</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G7">
-        <v>2702</v>
+        <v>2742</v>
       </c>
       <c r="H7" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I7" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="J7" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="K7" s="1">
         <v>46302</v>
@@ -1140,28 +1155,28 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N7" s="1">
         <v>46333</v>
       </c>
       <c r="Q7">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S7" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="T7" t="s">
-        <v>101</v>
-      </c>
-      <c r="U7" t="s">
-        <v>103</v>
+        <v>106</v>
+      </c>
+      <c r="V7" t="s">
+        <v>115</v>
       </c>
       <c r="W7" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1169,64 +1184,61 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>384</v>
+        <v>329</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F8" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="G8">
-        <v>2742</v>
+        <v>2721</v>
       </c>
       <c r="H8" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I8" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J8" s="1">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="K8" s="1">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N8" s="1">
-        <v>46333</v>
+        <v>46315</v>
       </c>
       <c r="Q8">
-        <v>-25</v>
+        <v>-6</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S8" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T8" t="s">
-        <v>100</v>
-      </c>
-      <c r="V8" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="W8" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1234,7 +1246,7 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>396</v>
+        <v>329</v>
       </c>
       <c r="B9" t="s">
         <v>31</v>
@@ -1243,55 +1255,52 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F9" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G9">
-        <v>2731</v>
+        <v>2721</v>
       </c>
       <c r="H9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I9" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J9" s="1">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="K9" s="1">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N9" s="1">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="Q9">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="T9" t="s">
-        <v>101</v>
-      </c>
-      <c r="U9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="W9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1299,7 +1308,7 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B10" t="s">
         <v>32</v>
@@ -1308,25 +1317,25 @@
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E10" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G10">
-        <v>2721</v>
+        <v>2731</v>
       </c>
       <c r="H10" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I10" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="J10" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K10" s="1">
         <v>46304</v>
@@ -1335,25 +1344,25 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N10" s="1">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="Q10">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="R10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T10" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="W10" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1361,61 +1370,61 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F11" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G11">
-        <v>2721</v>
+        <v>2729</v>
       </c>
       <c r="H11" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="J11" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="K11" s="1">
         <v>46304</v>
       </c>
       <c r="L11">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M11" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N11" s="1">
-        <v>46311</v>
+        <v>46315</v>
       </c>
       <c r="Q11">
-        <v>-3</v>
+        <v>-6</v>
       </c>
       <c r="R11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S11" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T11" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="W11" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1423,31 +1432,31 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>396</v>
+        <v>690</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E12" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="G12">
-        <v>2731</v>
+        <v>2727</v>
       </c>
       <c r="H12" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I12" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J12" s="1">
         <v>46303</v>
@@ -1459,25 +1468,25 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N12" s="1">
         <v>46311</v>
       </c>
       <c r="Q12">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S12" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T12" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="W12" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1485,31 +1494,31 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E13" t="s">
         <v>84</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G13">
-        <v>2729</v>
+        <v>2727</v>
       </c>
       <c r="H13" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I13" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="J13" s="1">
         <v>46303</v>
@@ -1518,28 +1527,28 @@
         <v>46304</v>
       </c>
       <c r="L13">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="M13" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N13" s="1">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="Q13">
-        <v>-7</v>
+        <v>-2</v>
       </c>
       <c r="R13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S13" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T13" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="W13" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1556,22 +1565,22 @@
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E14" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F14" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G14">
         <v>2727</v>
       </c>
       <c r="H14" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I14" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J14" s="1">
         <v>46303</v>
@@ -1580,28 +1589,31 @@
         <v>46304</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N14" s="1">
         <v>46311</v>
       </c>
       <c r="Q14">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S14" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="T14" t="s">
-        <v>100</v>
+        <v>106</v>
+      </c>
+      <c r="U14" t="s">
+        <v>109</v>
       </c>
       <c r="W14" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1618,22 +1630,22 @@
         <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G15">
         <v>2727</v>
       </c>
       <c r="H15" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I15" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J15" s="1">
         <v>46303</v>
@@ -1642,28 +1654,28 @@
         <v>46304</v>
       </c>
       <c r="L15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N15" s="1">
         <v>46311</v>
       </c>
       <c r="Q15">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S15" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T15" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="W15" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1680,22 +1692,22 @@
         <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="G16">
         <v>2727</v>
       </c>
       <c r="H16" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I16" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J16" s="1">
         <v>46303</v>
@@ -1704,31 +1716,31 @@
         <v>46304</v>
       </c>
       <c r="L16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N16" s="1">
         <v>46311</v>
       </c>
       <c r="Q16">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S16" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="T16" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="U16" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="W16" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1745,22 +1757,22 @@
         <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G17">
         <v>2727</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I17" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J17" s="1">
         <v>46303</v>
@@ -1772,25 +1784,25 @@
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N17" s="1">
         <v>46311</v>
       </c>
       <c r="Q17">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S17" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="T17" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="W17" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1807,22 +1819,22 @@
         <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E18" t="s">
         <v>88</v>
       </c>
       <c r="F18" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G18">
         <v>2727</v>
       </c>
       <c r="H18" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I18" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J18" s="1">
         <v>46303</v>
@@ -1834,28 +1846,28 @@
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N18" s="1">
         <v>46311</v>
       </c>
       <c r="Q18">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S18" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="T18" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="U18" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="W18" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1872,22 +1884,22 @@
         <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E19" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="G19">
         <v>2727</v>
       </c>
       <c r="H19" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I19" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="J19" s="1">
         <v>46303</v>
@@ -1899,25 +1911,25 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N19" s="1">
         <v>46311</v>
       </c>
       <c r="Q19">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S19" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="T19" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="W19" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -1925,64 +1937,61 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20">
-        <v>690</v>
+        <v>329</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s">
         <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F20" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="G20">
-        <v>2727</v>
+        <v>2721</v>
       </c>
       <c r="H20" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="I20" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="J20" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K20" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L20">
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N20" s="1">
-        <v>46311</v>
+        <v>46320</v>
       </c>
       <c r="Q20">
-        <v>-3</v>
+        <v>-11</v>
       </c>
       <c r="R20">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S20" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="T20" t="s">
-        <v>100</v>
-      </c>
-      <c r="U20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="W20" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -1990,63 +1999,187 @@
     </row>
     <row r="21" spans="1:27">
       <c r="A21">
-        <v>690</v>
+        <v>329</v>
       </c>
       <c r="B21" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s">
         <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E21" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F21" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G21">
-        <v>2727</v>
+        <v>2721</v>
       </c>
       <c r="H21" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="I21" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="J21" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K21" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L21">
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="N21" s="1">
-        <v>46311</v>
+        <v>46320</v>
       </c>
       <c r="Q21">
-        <v>-3</v>
+        <v>-11</v>
       </c>
       <c r="R21">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="T21" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="W21" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="AA21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27">
+      <c r="A22">
+        <v>396</v>
+      </c>
+      <c r="B22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" t="s">
+        <v>75</v>
+      </c>
+      <c r="E22" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" t="s">
+        <v>98</v>
+      </c>
+      <c r="G22">
+        <v>2731</v>
+      </c>
+      <c r="H22" t="s">
+        <v>101</v>
+      </c>
+      <c r="I22" t="s">
+        <v>104</v>
+      </c>
+      <c r="J22" s="1">
+        <v>46309</v>
+      </c>
+      <c r="K22" s="1">
+        <v>46309</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22" t="s">
+        <v>105</v>
+      </c>
+      <c r="N22" s="1">
+        <v>46316</v>
+      </c>
+      <c r="Q22">
+        <v>-7</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22" t="s">
+        <v>106</v>
+      </c>
+      <c r="T22" t="s">
+        <v>107</v>
+      </c>
+      <c r="W22" t="s">
+        <v>116</v>
+      </c>
+      <c r="AA22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27">
+      <c r="A23">
+        <v>685</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23">
+        <v>2703</v>
+      </c>
+      <c r="H23" t="s">
+        <v>101</v>
+      </c>
+      <c r="I23" t="s">
+        <v>102</v>
+      </c>
+      <c r="J23" s="1">
+        <v>46308</v>
+      </c>
+      <c r="K23" s="1">
+        <v>46309</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23" t="s">
+        <v>105</v>
+      </c>
+      <c r="N23" s="1">
+        <v>46340</v>
+      </c>
+      <c r="Q23">
+        <v>-31</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23" t="s">
+        <v>106</v>
+      </c>
+      <c r="T23" t="s">
+        <v>107</v>
+      </c>
+      <c r="W23" t="s">
+        <v>116</v>
+      </c>
+      <c r="AA23" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (14/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,8 +374,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -391,7 +399,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -399,12 +407,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -704,85 +730,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -814,10 +840,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -826,7 +852,7 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -882,10 +908,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46294</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -894,10 +920,10 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46326</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46326</v>
       </c>
       <c r="Q3">
@@ -950,10 +976,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46294</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -962,10 +988,10 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46326</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46326</v>
       </c>
       <c r="Q4">
@@ -1018,10 +1044,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46296</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1030,7 +1056,7 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46327</v>
       </c>
       <c r="Q5">
@@ -1083,10 +1109,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46301</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1095,7 +1121,7 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46333</v>
       </c>
       <c r="Q6">
@@ -1145,10 +1171,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46302</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1157,7 +1183,7 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46333</v>
       </c>
       <c r="Q7">
@@ -1210,10 +1236,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46304</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1222,7 +1248,7 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46315</v>
       </c>
       <c r="Q8">
@@ -1272,10 +1298,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46304</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1284,7 +1310,7 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46311</v>
       </c>
       <c r="Q9">
@@ -1334,10 +1360,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46303</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1346,7 +1372,7 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46311</v>
       </c>
       <c r="Q10">
@@ -1396,10 +1422,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46303</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1408,7 +1434,7 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46315</v>
       </c>
       <c r="Q11">
@@ -1458,10 +1484,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46303</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1470,7 +1496,7 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46311</v>
       </c>
       <c r="Q12">
@@ -1520,10 +1546,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46303</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1532,7 +1558,7 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46311</v>
       </c>
       <c r="Q13">
@@ -1582,10 +1608,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46303</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1594,7 +1620,7 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46311</v>
       </c>
       <c r="Q14">
@@ -1647,10 +1673,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46303</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1659,7 +1685,7 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46311</v>
       </c>
       <c r="Q15">
@@ -1709,10 +1735,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46303</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1721,7 +1747,7 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46311</v>
       </c>
       <c r="Q16">
@@ -1774,10 +1800,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46303</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1786,7 +1812,7 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46311</v>
       </c>
       <c r="Q17">
@@ -1836,10 +1862,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46303</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1848,7 +1874,7 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46311</v>
       </c>
       <c r="Q18">
@@ -1901,10 +1927,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46303</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1913,7 +1939,7 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46311</v>
       </c>
       <c r="Q19">
@@ -1963,10 +1989,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46308</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -1975,7 +2001,7 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46320</v>
       </c>
       <c r="Q20">
@@ -2025,10 +2051,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46308</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2037,7 +2063,7 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46320</v>
       </c>
       <c r="Q21">
@@ -2087,10 +2113,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46309</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2099,7 +2125,7 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <v>46316</v>
       </c>
       <c r="Q22">
@@ -2149,10 +2175,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46308</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2161,7 +2187,7 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <v>46340</v>
       </c>
       <c r="Q23">

</xml_diff>

<commit_message>
Atualização automática: emergencias (15/10/2026 12:34)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,16 +374,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -399,7 +391,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -407,30 +399,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -730,85 +704,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -840,10 +814,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -852,14 +826,14 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R2">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="S2" t="s">
         <v>106</v>
@@ -908,10 +882,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46294</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -920,17 +894,17 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46326</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S3" t="s">
         <v>106</v>
@@ -976,10 +950,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46294</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -988,17 +962,17 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46326</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46326</v>
       </c>
       <c r="Q4">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S4" t="s">
         <v>106</v>
@@ -1044,10 +1018,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46296</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1056,14 +1030,14 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R5">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S5" t="s">
         <v>106</v>
@@ -1109,10 +1083,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46301</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1121,14 +1095,14 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46333</v>
       </c>
       <c r="Q6">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s">
         <v>106</v>
@@ -1171,10 +1145,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46302</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1183,14 +1157,14 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46333</v>
       </c>
       <c r="Q7">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S7" t="s">
         <v>106</v>
@@ -1236,10 +1210,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46304</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1248,14 +1222,14 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46315</v>
       </c>
       <c r="Q8">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S8" t="s">
         <v>106</v>
@@ -1298,10 +1272,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46304</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1310,14 +1284,14 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46311</v>
       </c>
       <c r="Q9">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S9" t="s">
         <v>106</v>
@@ -1360,10 +1334,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46303</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1372,14 +1346,14 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46311</v>
       </c>
       <c r="Q10">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S10" t="s">
         <v>106</v>
@@ -1422,10 +1396,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46303</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1434,14 +1408,14 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46315</v>
       </c>
       <c r="Q11">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S11" t="s">
         <v>106</v>
@@ -1484,10 +1458,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46303</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1496,14 +1470,14 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46311</v>
       </c>
       <c r="Q12">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S12" t="s">
         <v>106</v>
@@ -1546,10 +1520,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46303</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1558,14 +1532,14 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46311</v>
       </c>
       <c r="Q13">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S13" t="s">
         <v>106</v>
@@ -1608,10 +1582,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46303</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1620,14 +1594,14 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46311</v>
       </c>
       <c r="Q14">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S14" t="s">
         <v>107</v>
@@ -1673,10 +1647,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46303</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1685,14 +1659,14 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46311</v>
       </c>
       <c r="Q15">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S15" t="s">
         <v>106</v>
@@ -1735,10 +1709,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46303</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1747,14 +1721,14 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46311</v>
       </c>
       <c r="Q16">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S16" t="s">
         <v>107</v>
@@ -1800,10 +1774,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46303</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1812,14 +1786,14 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>46311</v>
       </c>
       <c r="Q17">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S17" t="s">
         <v>107</v>
@@ -1862,10 +1836,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46303</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1874,14 +1848,14 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>46311</v>
       </c>
       <c r="Q18">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S18" t="s">
         <v>107</v>
@@ -1927,10 +1901,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46303</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1939,14 +1913,14 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19" s="1">
         <v>46311</v>
       </c>
       <c r="Q19">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S19" t="s">
         <v>106</v>
@@ -1989,10 +1963,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46308</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -2001,14 +1975,14 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46320</v>
       </c>
       <c r="Q20">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" t="s">
         <v>106</v>
@@ -2051,10 +2025,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46308</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2063,14 +2037,14 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46320</v>
       </c>
       <c r="Q21">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S21" t="s">
         <v>106</v>
@@ -2113,10 +2087,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46309</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2125,14 +2099,14 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22" s="1">
         <v>46316</v>
       </c>
       <c r="Q22">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" t="s">
         <v>106</v>
@@ -2175,10 +2149,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46308</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2187,14 +2161,14 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23" s="1">
         <v>46340</v>
       </c>
       <c r="Q23">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="s">
         <v>106</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (16/10/2026 12:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,8 +374,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -391,7 +399,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -399,12 +407,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -704,85 +730,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -814,10 +840,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -826,14 +852,14 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R2">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="S2" t="s">
         <v>106</v>
@@ -882,10 +908,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46294</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -894,17 +920,17 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46326</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R3">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S3" t="s">
         <v>106</v>
@@ -950,10 +976,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46294</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -962,17 +988,17 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46326</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46326</v>
       </c>
       <c r="Q4">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S4" t="s">
         <v>106</v>
@@ -1018,10 +1044,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46296</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1030,14 +1056,14 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S5" t="s">
         <v>106</v>
@@ -1083,10 +1109,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46301</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1095,14 +1121,14 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46333</v>
       </c>
       <c r="Q6">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S6" t="s">
         <v>106</v>
@@ -1145,10 +1171,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46302</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1157,14 +1183,14 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46333</v>
       </c>
       <c r="Q7">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S7" t="s">
         <v>106</v>
@@ -1210,10 +1236,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46304</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1222,14 +1248,14 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46315</v>
       </c>
       <c r="Q8">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S8" t="s">
         <v>106</v>
@@ -1272,10 +1298,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46304</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1284,14 +1310,14 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46311</v>
       </c>
       <c r="Q9">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S9" t="s">
         <v>106</v>
@@ -1334,10 +1360,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46303</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1346,14 +1372,14 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46311</v>
       </c>
       <c r="Q10">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S10" t="s">
         <v>106</v>
@@ -1396,10 +1422,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46303</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1408,14 +1434,14 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46315</v>
       </c>
       <c r="Q11">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S11" t="s">
         <v>106</v>
@@ -1458,10 +1484,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46303</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1470,14 +1496,14 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46311</v>
       </c>
       <c r="Q12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R12">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S12" t="s">
         <v>106</v>
@@ -1520,10 +1546,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46303</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1532,14 +1558,14 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46311</v>
       </c>
       <c r="Q13">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S13" t="s">
         <v>106</v>
@@ -1582,10 +1608,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46303</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1594,14 +1620,14 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46311</v>
       </c>
       <c r="Q14">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S14" t="s">
         <v>107</v>
@@ -1647,10 +1673,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46303</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1659,14 +1685,14 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46311</v>
       </c>
       <c r="Q15">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R15">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S15" t="s">
         <v>106</v>
@@ -1709,10 +1735,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46303</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1721,14 +1747,14 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46311</v>
       </c>
       <c r="Q16">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S16" t="s">
         <v>107</v>
@@ -1774,10 +1800,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46303</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1786,14 +1812,14 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46311</v>
       </c>
       <c r="Q17">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S17" t="s">
         <v>107</v>
@@ -1836,10 +1862,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46303</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1848,14 +1874,14 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46311</v>
       </c>
       <c r="Q18">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S18" t="s">
         <v>107</v>
@@ -1901,10 +1927,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46303</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1913,14 +1939,14 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46311</v>
       </c>
       <c r="Q19">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S19" t="s">
         <v>106</v>
@@ -1963,10 +1989,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46308</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -1975,14 +2001,14 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46320</v>
       </c>
       <c r="Q20">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" t="s">
         <v>106</v>
@@ -2025,10 +2051,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46308</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2037,14 +2063,14 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46320</v>
       </c>
       <c r="Q21">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S21" t="s">
         <v>106</v>
@@ -2087,10 +2113,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46309</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2099,14 +2125,14 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <v>46316</v>
       </c>
       <c r="Q22">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S22" t="s">
         <v>106</v>
@@ -2149,10 +2175,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46308</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2161,14 +2187,14 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <v>46340</v>
       </c>
       <c r="Q23">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S23" t="s">
         <v>106</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (16/10/2026 12:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,16 +374,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -399,7 +391,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -407,30 +399,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -730,85 +704,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -840,10 +814,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -852,7 +826,7 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -908,10 +882,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46294</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -920,10 +894,10 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46326</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46326</v>
       </c>
       <c r="Q3">
@@ -976,10 +950,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46294</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -988,10 +962,10 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46326</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46326</v>
       </c>
       <c r="Q4">
@@ -1044,10 +1018,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46296</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1056,7 +1030,7 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
@@ -1109,10 +1083,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46301</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1121,7 +1095,7 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46333</v>
       </c>
       <c r="Q6">
@@ -1171,10 +1145,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46302</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1183,7 +1157,7 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46333</v>
       </c>
       <c r="Q7">
@@ -1236,10 +1210,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46304</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1248,7 +1222,7 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46315</v>
       </c>
       <c r="Q8">
@@ -1298,10 +1272,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46304</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1310,7 +1284,7 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46311</v>
       </c>
       <c r="Q9">
@@ -1360,10 +1334,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46303</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1372,7 +1346,7 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46311</v>
       </c>
       <c r="Q10">
@@ -1422,10 +1396,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46303</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1434,7 +1408,7 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46315</v>
       </c>
       <c r="Q11">
@@ -1484,10 +1458,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46303</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1496,7 +1470,7 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46311</v>
       </c>
       <c r="Q12">
@@ -1546,10 +1520,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46303</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1558,7 +1532,7 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46311</v>
       </c>
       <c r="Q13">
@@ -1608,10 +1582,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46303</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1620,7 +1594,7 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46311</v>
       </c>
       <c r="Q14">
@@ -1673,10 +1647,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46303</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1685,7 +1659,7 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46311</v>
       </c>
       <c r="Q15">
@@ -1735,10 +1709,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46303</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1747,7 +1721,7 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46311</v>
       </c>
       <c r="Q16">
@@ -1800,10 +1774,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46303</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1812,7 +1786,7 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>46311</v>
       </c>
       <c r="Q17">
@@ -1862,10 +1836,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46303</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1874,7 +1848,7 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>46311</v>
       </c>
       <c r="Q18">
@@ -1927,10 +1901,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46303</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1939,7 +1913,7 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19" s="1">
         <v>46311</v>
       </c>
       <c r="Q19">
@@ -1989,10 +1963,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46308</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -2001,7 +1975,7 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46320</v>
       </c>
       <c r="Q20">
@@ -2051,10 +2025,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46308</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2063,7 +2037,7 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46320</v>
       </c>
       <c r="Q21">
@@ -2113,10 +2087,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46309</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2125,7 +2099,7 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22" s="1">
         <v>46316</v>
       </c>
       <c r="Q22">
@@ -2175,10 +2149,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46308</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2187,7 +2161,7 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23" s="1">
         <v>46340</v>
       </c>
       <c r="Q23">

</xml_diff>

<commit_message>
Atualização automática: emergencias (19/10/2026 13:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,8 +374,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -391,7 +399,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -399,12 +407,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -704,85 +730,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -814,10 +840,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -826,14 +852,14 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="R2">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="S2" t="s">
         <v>106</v>
@@ -882,10 +908,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46294</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -894,17 +920,17 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46326</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="R3">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S3" t="s">
         <v>106</v>
@@ -950,10 +976,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46294</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -962,17 +988,17 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46326</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46326</v>
       </c>
       <c r="Q4">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="R4">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S4" t="s">
         <v>106</v>
@@ -1018,10 +1044,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46296</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1030,14 +1056,14 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-16</v>
+        <v>-13</v>
       </c>
       <c r="R5">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="S5" t="s">
         <v>106</v>
@@ -1083,10 +1109,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46301</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1095,14 +1121,14 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46333</v>
       </c>
       <c r="Q6">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="R6">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S6" t="s">
         <v>106</v>
@@ -1145,10 +1171,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46302</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1157,14 +1183,14 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46333</v>
       </c>
       <c r="Q7">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="R7">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S7" t="s">
         <v>106</v>
@@ -1210,10 +1236,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46304</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1222,14 +1248,14 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46315</v>
       </c>
       <c r="Q8">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
         <v>106</v>
@@ -1272,10 +1298,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46304</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1284,14 +1310,14 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46311</v>
       </c>
       <c r="Q9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R9">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S9" t="s">
         <v>106</v>
@@ -1334,10 +1360,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46303</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1346,14 +1372,14 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46311</v>
       </c>
       <c r="Q10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R10">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S10" t="s">
         <v>106</v>
@@ -1396,10 +1422,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46303</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1408,14 +1434,14 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46315</v>
       </c>
       <c r="Q11">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R11">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S11" t="s">
         <v>106</v>
@@ -1458,10 +1484,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46303</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1470,14 +1496,14 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46311</v>
       </c>
       <c r="Q12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R12">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S12" t="s">
         <v>106</v>
@@ -1520,10 +1546,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46303</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1532,14 +1558,14 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46311</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R13">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S13" t="s">
         <v>106</v>
@@ -1582,10 +1608,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46303</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1594,14 +1620,14 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46311</v>
       </c>
       <c r="Q14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R14">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S14" t="s">
         <v>107</v>
@@ -1647,10 +1673,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46303</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1659,14 +1685,14 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46311</v>
       </c>
       <c r="Q15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R15">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S15" t="s">
         <v>106</v>
@@ -1709,10 +1735,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46303</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1721,14 +1747,14 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46311</v>
       </c>
       <c r="Q16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R16">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S16" t="s">
         <v>107</v>
@@ -1774,10 +1800,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46303</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1786,14 +1812,14 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46311</v>
       </c>
       <c r="Q17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R17">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S17" t="s">
         <v>107</v>
@@ -1836,10 +1862,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46303</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1848,14 +1874,14 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46311</v>
       </c>
       <c r="Q18">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R18">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S18" t="s">
         <v>107</v>
@@ -1901,10 +1927,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46303</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1913,14 +1939,14 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46311</v>
       </c>
       <c r="Q19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R19">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="S19" t="s">
         <v>106</v>
@@ -1963,10 +1989,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46308</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -1975,14 +2001,14 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46320</v>
       </c>
       <c r="Q20">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S20" t="s">
         <v>106</v>
@@ -2025,10 +2051,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46308</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2037,14 +2063,14 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46320</v>
       </c>
       <c r="Q21">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R21">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S21" t="s">
         <v>106</v>
@@ -2087,10 +2113,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46309</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2099,14 +2125,14 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <v>46316</v>
       </c>
       <c r="Q22">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="R22">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S22" t="s">
         <v>106</v>
@@ -2149,10 +2175,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46308</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2161,14 +2187,14 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <v>46340</v>
       </c>
       <c r="Q23">
-        <v>-29</v>
+        <v>-26</v>
       </c>
       <c r="R23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S23" t="s">
         <v>106</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (19/10/2026 14:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,16 +374,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -399,7 +391,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -407,30 +399,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -730,85 +704,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -840,10 +814,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -852,7 +826,7 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -908,10 +882,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46294</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -920,10 +894,10 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46326</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46326</v>
       </c>
       <c r="Q3">
@@ -976,10 +950,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46294</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -988,10 +962,10 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46326</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46326</v>
       </c>
       <c r="Q4">
@@ -1044,10 +1018,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46296</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1056,7 +1030,7 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
@@ -1109,10 +1083,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46301</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1121,7 +1095,7 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46333</v>
       </c>
       <c r="Q6">
@@ -1171,10 +1145,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46302</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1183,7 +1157,7 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46333</v>
       </c>
       <c r="Q7">
@@ -1236,10 +1210,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46304</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1248,7 +1222,7 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46315</v>
       </c>
       <c r="Q8">
@@ -1298,10 +1272,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46304</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1310,7 +1284,7 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46311</v>
       </c>
       <c r="Q9">
@@ -1360,10 +1334,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46303</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1372,7 +1346,7 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46311</v>
       </c>
       <c r="Q10">
@@ -1422,10 +1396,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46303</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1434,7 +1408,7 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46315</v>
       </c>
       <c r="Q11">
@@ -1484,10 +1458,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46303</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1496,7 +1470,7 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46311</v>
       </c>
       <c r="Q12">
@@ -1546,10 +1520,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46303</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1558,7 +1532,7 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46311</v>
       </c>
       <c r="Q13">
@@ -1608,10 +1582,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46303</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1620,7 +1594,7 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46311</v>
       </c>
       <c r="Q14">
@@ -1673,10 +1647,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46303</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1685,7 +1659,7 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46311</v>
       </c>
       <c r="Q15">
@@ -1735,10 +1709,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46303</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1747,7 +1721,7 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46311</v>
       </c>
       <c r="Q16">
@@ -1800,10 +1774,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46303</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1812,7 +1786,7 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>46311</v>
       </c>
       <c r="Q17">
@@ -1862,10 +1836,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46303</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1874,7 +1848,7 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>46311</v>
       </c>
       <c r="Q18">
@@ -1927,10 +1901,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46303</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1939,7 +1913,7 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19" s="1">
         <v>46311</v>
       </c>
       <c r="Q19">
@@ -1989,10 +1963,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46308</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -2001,7 +1975,7 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46320</v>
       </c>
       <c r="Q20">
@@ -2051,10 +2025,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46308</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2063,7 +2037,7 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46320</v>
       </c>
       <c r="Q21">
@@ -2113,10 +2087,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46309</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2125,7 +2099,7 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22" s="1">
         <v>46316</v>
       </c>
       <c r="Q22">
@@ -2175,10 +2149,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46308</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2187,7 +2161,7 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23" s="1">
         <v>46340</v>
       </c>
       <c r="Q23">

</xml_diff>

<commit_message>
Atualização automática: emergencias (20/10/2026 12:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,8 +374,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -391,7 +399,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -399,12 +407,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -704,85 +730,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -814,10 +840,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -826,14 +852,14 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="S2" t="s">
         <v>106</v>
@@ -882,10 +908,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46294</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -894,17 +920,17 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46326</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R3">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S3" t="s">
         <v>106</v>
@@ -950,10 +976,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46294</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -962,17 +988,17 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46326</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46326</v>
       </c>
       <c r="Q4">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S4" t="s">
         <v>106</v>
@@ -1018,10 +1044,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46296</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1030,14 +1056,14 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-13</v>
+        <v>-12</v>
       </c>
       <c r="R5">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S5" t="s">
         <v>106</v>
@@ -1083,10 +1109,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46301</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1095,14 +1121,14 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46333</v>
       </c>
       <c r="Q6">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R6">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S6" t="s">
         <v>106</v>
@@ -1145,10 +1171,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46302</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1157,14 +1183,14 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46333</v>
       </c>
       <c r="Q7">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="R7">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S7" t="s">
         <v>106</v>
@@ -1210,10 +1236,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46304</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1222,14 +1248,14 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46315</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S8" t="s">
         <v>106</v>
@@ -1272,10 +1298,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46304</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1284,14 +1310,14 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46311</v>
       </c>
       <c r="Q9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S9" t="s">
         <v>106</v>
@@ -1334,10 +1360,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46303</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1346,14 +1372,14 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46311</v>
       </c>
       <c r="Q10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R10">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S10" t="s">
         <v>106</v>
@@ -1396,10 +1422,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46303</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1408,14 +1434,14 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46315</v>
       </c>
       <c r="Q11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S11" t="s">
         <v>106</v>
@@ -1458,10 +1484,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46303</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1470,14 +1496,14 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46311</v>
       </c>
       <c r="Q12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S12" t="s">
         <v>106</v>
@@ -1520,10 +1546,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46303</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1532,14 +1558,14 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46311</v>
       </c>
       <c r="Q13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R13">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S13" t="s">
         <v>106</v>
@@ -1582,10 +1608,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46303</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1594,14 +1620,14 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46311</v>
       </c>
       <c r="Q14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S14" t="s">
         <v>107</v>
@@ -1647,10 +1673,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46303</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1659,14 +1685,14 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46311</v>
       </c>
       <c r="Q15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R15">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S15" t="s">
         <v>106</v>
@@ -1709,10 +1735,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46303</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1721,14 +1747,14 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46311</v>
       </c>
       <c r="Q16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R16">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S16" t="s">
         <v>107</v>
@@ -1774,10 +1800,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46303</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1786,14 +1812,14 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46311</v>
       </c>
       <c r="Q17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R17">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S17" t="s">
         <v>107</v>
@@ -1836,10 +1862,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46303</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1848,14 +1874,14 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46311</v>
       </c>
       <c r="Q18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R18">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S18" t="s">
         <v>107</v>
@@ -1901,10 +1927,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46303</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1913,14 +1939,14 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46311</v>
       </c>
       <c r="Q19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R19">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S19" t="s">
         <v>106</v>
@@ -1963,10 +1989,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46308</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -1975,14 +2001,14 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46320</v>
       </c>
       <c r="Q20">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S20" t="s">
         <v>106</v>
@@ -2025,10 +2051,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46308</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2037,14 +2063,14 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46320</v>
       </c>
       <c r="Q21">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S21" t="s">
         <v>106</v>
@@ -2087,10 +2113,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46309</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2099,14 +2125,14 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <v>46316</v>
       </c>
       <c r="Q22">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S22" t="s">
         <v>106</v>
@@ -2149,10 +2175,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46308</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2161,14 +2187,14 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <v>46340</v>
       </c>
       <c r="Q23">
-        <v>-26</v>
+        <v>-25</v>
       </c>
       <c r="R23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S23" t="s">
         <v>106</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (20/10/2026 12:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -374,16 +374,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -399,7 +391,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -407,30 +399,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -730,85 +704,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -840,10 +814,10 @@
       <c r="I2" t="s">
         <v>102</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -852,7 +826,7 @@
       <c r="M2" t="s">
         <v>105</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -908,10 +882,10 @@
       <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46294</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -920,10 +894,10 @@
       <c r="M3" t="s">
         <v>105</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46326</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46326</v>
       </c>
       <c r="Q3">
@@ -976,10 +950,10 @@
       <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46294</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -988,10 +962,10 @@
       <c r="M4" t="s">
         <v>105</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46326</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46326</v>
       </c>
       <c r="Q4">
@@ -1044,10 +1018,10 @@
       <c r="I5" t="s">
         <v>102</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46296</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1056,7 +1030,7 @@
       <c r="M5" t="s">
         <v>105</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
@@ -1109,10 +1083,10 @@
       <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46301</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1121,7 +1095,7 @@
       <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46333</v>
       </c>
       <c r="Q6">
@@ -1171,10 +1145,10 @@
       <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46302</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1183,7 +1157,7 @@
       <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46333</v>
       </c>
       <c r="Q7">
@@ -1236,10 +1210,10 @@
       <c r="I8" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46304</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1248,7 +1222,7 @@
       <c r="M8" t="s">
         <v>105</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46315</v>
       </c>
       <c r="Q8">
@@ -1298,10 +1272,10 @@
       <c r="I9" t="s">
         <v>104</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46304</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1310,7 +1284,7 @@
       <c r="M9" t="s">
         <v>105</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46311</v>
       </c>
       <c r="Q9">
@@ -1360,10 +1334,10 @@
       <c r="I10" t="s">
         <v>104</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46303</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1372,7 +1346,7 @@
       <c r="M10" t="s">
         <v>105</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46311</v>
       </c>
       <c r="Q10">
@@ -1422,10 +1396,10 @@
       <c r="I11" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46303</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1434,7 +1408,7 @@
       <c r="M11" t="s">
         <v>105</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46315</v>
       </c>
       <c r="Q11">
@@ -1484,10 +1458,10 @@
       <c r="I12" t="s">
         <v>104</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46303</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1496,7 +1470,7 @@
       <c r="M12" t="s">
         <v>105</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46311</v>
       </c>
       <c r="Q12">
@@ -1546,10 +1520,10 @@
       <c r="I13" t="s">
         <v>104</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46303</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46304</v>
       </c>
       <c r="L13">
@@ -1558,7 +1532,7 @@
       <c r="M13" t="s">
         <v>105</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46311</v>
       </c>
       <c r="Q13">
@@ -1608,10 +1582,10 @@
       <c r="I14" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46303</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46304</v>
       </c>
       <c r="L14">
@@ -1620,7 +1594,7 @@
       <c r="M14" t="s">
         <v>105</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46311</v>
       </c>
       <c r="Q14">
@@ -1673,10 +1647,10 @@
       <c r="I15" t="s">
         <v>104</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46303</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46304</v>
       </c>
       <c r="L15">
@@ -1685,7 +1659,7 @@
       <c r="M15" t="s">
         <v>105</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46311</v>
       </c>
       <c r="Q15">
@@ -1735,10 +1709,10 @@
       <c r="I16" t="s">
         <v>104</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46303</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46304</v>
       </c>
       <c r="L16">
@@ -1747,7 +1721,7 @@
       <c r="M16" t="s">
         <v>105</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46311</v>
       </c>
       <c r="Q16">
@@ -1800,10 +1774,10 @@
       <c r="I17" t="s">
         <v>104</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46303</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46304</v>
       </c>
       <c r="L17">
@@ -1812,7 +1786,7 @@
       <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>46311</v>
       </c>
       <c r="Q17">
@@ -1862,10 +1836,10 @@
       <c r="I18" t="s">
         <v>104</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46303</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>46304</v>
       </c>
       <c r="L18">
@@ -1874,7 +1848,7 @@
       <c r="M18" t="s">
         <v>105</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>46311</v>
       </c>
       <c r="Q18">
@@ -1927,10 +1901,10 @@
       <c r="I19" t="s">
         <v>104</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46303</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>46304</v>
       </c>
       <c r="L19">
@@ -1939,7 +1913,7 @@
       <c r="M19" t="s">
         <v>105</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19" s="1">
         <v>46311</v>
       </c>
       <c r="Q19">
@@ -1989,10 +1963,10 @@
       <c r="I20" t="s">
         <v>103</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46308</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>46309</v>
       </c>
       <c r="L20">
@@ -2001,7 +1975,7 @@
       <c r="M20" t="s">
         <v>105</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46320</v>
       </c>
       <c r="Q20">
@@ -2051,10 +2025,10 @@
       <c r="I21" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46308</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>46309</v>
       </c>
       <c r="L21">
@@ -2063,7 +2037,7 @@
       <c r="M21" t="s">
         <v>105</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46320</v>
       </c>
       <c r="Q21">
@@ -2113,10 +2087,10 @@
       <c r="I22" t="s">
         <v>104</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46309</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>46309</v>
       </c>
       <c r="L22">
@@ -2125,7 +2099,7 @@
       <c r="M22" t="s">
         <v>105</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22" s="1">
         <v>46316</v>
       </c>
       <c r="Q22">
@@ -2175,10 +2149,10 @@
       <c r="I23" t="s">
         <v>102</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46308</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>46309</v>
       </c>
       <c r="L23">
@@ -2187,7 +2161,7 @@
       <c r="M23" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23" s="1">
         <v>46340</v>
       </c>
       <c r="Q23">

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/10/2026 12:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="132">
   <si>
     <t>om_emg</t>
   </si>
@@ -112,12 +112,12 @@
     <t>BABR</t>
   </si>
   <si>
+    <t>BACG</t>
+  </si>
+  <si>
     <t>BABE</t>
   </si>
   <si>
-    <t>BACG</t>
-  </si>
-  <si>
     <t>313260018702</t>
   </si>
   <si>
@@ -142,36 +142,15 @@
     <t>329260019313</t>
   </si>
   <si>
-    <t>396260016638</t>
-  </si>
-  <si>
     <t>685260012964</t>
   </si>
   <si>
-    <t>690260002674</t>
-  </si>
-  <si>
-    <t>690260002675</t>
-  </si>
-  <si>
-    <t>690260002676</t>
-  </si>
-  <si>
-    <t>690260002677</t>
-  </si>
-  <si>
     <t>690260002678</t>
   </si>
   <si>
-    <t>690260002679</t>
-  </si>
-  <si>
     <t>690260002680</t>
   </si>
   <si>
-    <t>690260002681</t>
-  </si>
-  <si>
     <t>329260019318</t>
   </si>
   <si>
@@ -184,6 +163,39 @@
     <t>685260012971</t>
   </si>
   <si>
+    <t>313260019100</t>
+  </si>
+  <si>
+    <t>396260016647</t>
+  </si>
+  <si>
+    <t>396260016648</t>
+  </si>
+  <si>
+    <t>685260012988</t>
+  </si>
+  <si>
+    <t>685260012989</t>
+  </si>
+  <si>
+    <t>685260012993</t>
+  </si>
+  <si>
+    <t>685260012994</t>
+  </si>
+  <si>
+    <t>685260012995</t>
+  </si>
+  <si>
+    <t>685260012996</t>
+  </si>
+  <si>
+    <t>685260012998</t>
+  </si>
+  <si>
+    <t>396260016650</t>
+  </si>
+  <si>
     <t>040-0043</t>
   </si>
   <si>
@@ -208,33 +220,15 @@
     <t>MS28773-05</t>
   </si>
   <si>
-    <t>2601266-2</t>
-  </si>
-  <si>
     <t>103-20400</t>
   </si>
   <si>
-    <t>3244897-4</t>
-  </si>
-  <si>
-    <t>MS29512-5</t>
-  </si>
-  <si>
-    <t>3014223</t>
-  </si>
-  <si>
     <t>3034792</t>
   </si>
   <si>
-    <t>3004085</t>
-  </si>
-  <si>
     <t>M83248/1-029</t>
   </si>
   <si>
-    <t>3022375</t>
-  </si>
-  <si>
     <t>9910592-2</t>
   </si>
   <si>
@@ -247,6 +241,30 @@
     <t>066-3046-01</t>
   </si>
   <si>
+    <t>011-00870-00</t>
+  </si>
+  <si>
+    <t>F2552-070</t>
+  </si>
+  <si>
+    <t>NAS147-84</t>
+  </si>
+  <si>
+    <t>2641014-9</t>
+  </si>
+  <si>
+    <t>2641010-7</t>
+  </si>
+  <si>
+    <t>324843-W020</t>
+  </si>
+  <si>
+    <t>MS21043-3</t>
+  </si>
+  <si>
+    <t>2643100-201</t>
+  </si>
+  <si>
     <t>STROB TUB</t>
   </si>
   <si>
@@ -271,30 +289,15 @@
     <t>RETAINER,PACKING</t>
   </si>
   <si>
-    <t>COUPLING-SPLINED</t>
-  </si>
-  <si>
     <t>BOLT,MACHINE</t>
   </si>
   <si>
-    <t>FUEL CONTROL UNIT</t>
+    <t>BOMBA DE COMBUSTÍVEL</t>
   </si>
   <si>
     <t>ANEL-O</t>
   </si>
   <si>
-    <t>PACKING,PREFORMED</t>
-  </si>
-  <si>
-    <t>BOMBA DE COMBUSTÍVEL</t>
-  </si>
-  <si>
-    <t>SEAL</t>
-  </si>
-  <si>
-    <t>SEAL,PLAIN</t>
-  </si>
-  <si>
     <t>ALTERNADOR</t>
   </si>
   <si>
@@ -307,6 +310,30 @@
     <t>CONTROL,INDICATOR</t>
   </si>
   <si>
+    <t>MAGNETOMETER GMU 44</t>
+  </si>
+  <si>
+    <t>BARREL NUT</t>
+  </si>
+  <si>
+    <t>BOLT,INTERNAL WRENCH</t>
+  </si>
+  <si>
+    <t>SPRING ASSY-MAIN GEA</t>
+  </si>
+  <si>
+    <t>AXLE FITTING</t>
+  </si>
+  <si>
+    <t>HEADSET-MICROPHONE</t>
+  </si>
+  <si>
+    <t>NUT,SELF-LOCKING,EXT</t>
+  </si>
+  <si>
+    <t>NOSE GEAR STRUT ASSY</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -343,25 +370,43 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>Estoque com o Pn DCN4-3807 (Alternado). Godoy 09/10/26.</t>
+    <t>O compressor passou por teste no PAMALS onde foi identificada a pane nesse item. Ramon 21/10/26.</t>
   </si>
   <si>
     <t>Atendido com estoque local em 09/10. Ramon 09/10/26. AWB 127-6253 8910 liberado para retirada em 13/10. Ramon 14/10/26.</t>
   </si>
   <si>
+    <t>Cedeu o item para o C-98 2736. Ramon 21/10.</t>
+  </si>
+  <si>
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
   </si>
   <si>
-    <t>AGD ABERTURA DE OS- REZ , email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26</t>
-  </si>
-  <si>
-    <t>RECEBIDO 01 EA, REPARADO , DA WILLIAM EM 05/10/26. SERÁ ATD ESTA EMERG - REZ (06/10/26)</t>
+    <t>AGD ABERTURA DE OS- REZ , email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26. Abertas OS para 05 ea dia 07/10.Material será coletado dia 09/10 fins reparo - REZ</t>
+  </si>
+  <si>
+    <t>Enviado para o Operador dia 09/10/26 - AWB 127-6186 9835 - REZ - MATERIAL ENTREGUE DIA 10/10/2026 no CAN BANT</t>
   </si>
   <si>
     <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26</t>
   </si>
   <si>
-    <t>Em cotação no mercado. ATZ 07/10</t>
+    <t>Abertas OS para 05 ea dia 07/10.Material será coletado dia 09/10 fins reparo - REZ</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17796997 - entregue em Miami 09/10</t>
+  </si>
+  <si>
+    <t>solicitado abertura de OS de 03 ea em 09/10/2026.REZ</t>
+  </si>
+  <si>
+    <t>MATERIAL EM TRANSITO - RECIBO 884/FAB/26 AWB 12762528605 RC 09/10/2026 - AWB DISPONIVEL PARA RETIRADA 13/10/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003180334 - previsão de entrega no RJ 13/10 - MATERIAL RECEBIDO EM RJ 13/10 - PREPARANDO ENVIO 13/10 - recibo 887/FAB/26 AWB 12763073301 DPE 16/10/2026</t>
+  </si>
+  <si>
+    <t>ATENDIDO VIA ESTOQUE FAB, AWB A SER GERADA GOLLOG 09/10/2026. AWB 127-6253 8910</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -700,7 +745,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA23"/>
+  <dimension ref="A1:AA27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -797,22 +842,22 @@
         <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="F2" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I2" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -824,31 +869,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="S2" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T2" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="U2" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="V2" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="W2" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -865,22 +910,22 @@
         <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="F3" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G3">
         <v>2703</v>
       </c>
       <c r="H3" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I3" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="J3" s="1">
         <v>46294</v>
@@ -892,7 +937,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N3" s="1">
         <v>46326</v>
@@ -901,22 +946,22 @@
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S3" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T3" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="V3" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="W3" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -933,22 +978,22 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="G4">
         <v>2703</v>
       </c>
       <c r="H4" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I4" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="J4" s="1">
         <v>46294</v>
@@ -960,31 +1005,31 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N4" s="1">
         <v>46326</v>
       </c>
       <c r="O4" s="1">
-        <v>46326</v>
+        <v>46305</v>
       </c>
       <c r="Q4">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R4">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S4" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T4" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="V4" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="W4" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1001,22 +1046,22 @@
         <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="F5" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G5">
         <v>2723</v>
       </c>
       <c r="H5" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I5" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="J5" s="1">
         <v>46296</v>
@@ -1028,28 +1073,31 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R5">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S5" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T5" t="s">
-        <v>106</v>
+        <v>115</v>
+      </c>
+      <c r="U5" t="s">
+        <v>118</v>
       </c>
       <c r="V5" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="W5" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1066,22 +1114,22 @@
         <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="F6" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G6">
         <v>2708</v>
       </c>
       <c r="H6" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I6" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="J6" s="1">
         <v>46301</v>
@@ -1093,25 +1141,31 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N6" s="1">
         <v>46333</v>
       </c>
+      <c r="O6" s="1">
+        <v>46214</v>
+      </c>
       <c r="Q6">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R6">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S6" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T6" t="s">
-        <v>107</v>
+        <v>116</v>
+      </c>
+      <c r="V6" t="s">
+        <v>125</v>
       </c>
       <c r="W6" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1128,22 +1182,22 @@
         <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E7" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F7" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="G7">
         <v>2742</v>
       </c>
       <c r="H7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I7" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="J7" s="1">
         <v>46302</v>
@@ -1155,28 +1209,31 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N7" s="1">
         <v>46333</v>
       </c>
+      <c r="O7" s="1">
+        <v>46214</v>
+      </c>
       <c r="Q7">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="R7">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S7" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T7" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="V7" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="W7" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1193,22 +1250,22 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F8" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G8">
         <v>2721</v>
       </c>
       <c r="H8" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I8" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="J8" s="1">
         <v>46304</v>
@@ -1220,25 +1277,28 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N8" s="1">
         <v>46315</v>
       </c>
       <c r="Q8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S8" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T8" t="s">
-        <v>106</v>
+        <v>115</v>
+      </c>
+      <c r="V8" t="s">
+        <v>127</v>
       </c>
       <c r="W8" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1255,22 +1315,22 @@
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F9" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="G9">
         <v>2721</v>
       </c>
       <c r="H9" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I9" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J9" s="1">
         <v>46304</v>
@@ -1282,25 +1342,31 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N9" s="1">
         <v>46311</v>
       </c>
+      <c r="O9" s="1">
+        <v>46308</v>
+      </c>
       <c r="Q9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R9">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S9" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T9" t="s">
-        <v>106</v>
+        <v>115</v>
+      </c>
+      <c r="V9" t="s">
+        <v>128</v>
       </c>
       <c r="W9" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1308,31 +1374,31 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="F10" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="G10">
-        <v>2731</v>
+        <v>2729</v>
       </c>
       <c r="H10" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I10" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="J10" s="1">
         <v>46303</v>
@@ -1341,28 +1407,34 @@
         <v>46304</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M10" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N10" s="1">
+        <v>46315</v>
+      </c>
+      <c r="O10" s="1">
         <v>46311</v>
       </c>
       <c r="Q10">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="R10">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S10" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T10" t="s">
-        <v>107</v>
+        <v>116</v>
+      </c>
+      <c r="V10" t="s">
+        <v>129</v>
       </c>
       <c r="W10" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1370,31 +1442,31 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
         <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F11" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G11">
-        <v>2729</v>
+        <v>2727</v>
       </c>
       <c r="H11" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I11" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="J11" s="1">
         <v>46303</v>
@@ -1403,28 +1475,37 @@
         <v>46304</v>
       </c>
       <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>114</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46311</v>
+      </c>
+      <c r="O11" s="1">
+        <v>46311</v>
+      </c>
+      <c r="Q11">
+        <v>5</v>
+      </c>
+      <c r="R11">
         <v>12</v>
       </c>
-      <c r="M11" t="s">
-        <v>105</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46315</v>
-      </c>
-      <c r="Q11">
-        <v>0</v>
-      </c>
-      <c r="R11">
-        <v>11</v>
-      </c>
       <c r="S11" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="T11" t="s">
-        <v>107</v>
+        <v>115</v>
+      </c>
+      <c r="U11" t="s">
+        <v>119</v>
+      </c>
+      <c r="V11" t="s">
+        <v>130</v>
       </c>
       <c r="W11" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1435,28 +1516,28 @@
         <v>690</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
         <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E12" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F12" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="G12">
         <v>2727</v>
       </c>
       <c r="H12" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I12" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J12" s="1">
         <v>46303</v>
@@ -1468,25 +1549,34 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N12" s="1">
         <v>46311</v>
       </c>
+      <c r="O12" s="1">
+        <v>46309</v>
+      </c>
       <c r="Q12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R12">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="S12" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="T12" t="s">
-        <v>106</v>
+        <v>115</v>
+      </c>
+      <c r="U12" t="s">
+        <v>119</v>
+      </c>
+      <c r="V12" t="s">
+        <v>130</v>
       </c>
       <c r="W12" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1494,61 +1584,61 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>690</v>
+        <v>329</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="F13" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G13">
-        <v>2727</v>
+        <v>2721</v>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I13" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="J13" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K13" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N13" s="1">
-        <v>46311</v>
+        <v>46320</v>
       </c>
       <c r="Q13">
-        <v>4</v>
+        <v>-4</v>
       </c>
       <c r="R13">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="S13" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T13" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="W13" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1556,64 +1646,61 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>690</v>
+        <v>329</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="E14" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F14" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="G14">
-        <v>2727</v>
+        <v>2721</v>
       </c>
       <c r="H14" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I14" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="J14" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K14" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N14" s="1">
-        <v>46311</v>
+        <v>46320</v>
       </c>
       <c r="Q14">
-        <v>4</v>
+        <v>-4</v>
       </c>
       <c r="R14">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="S14" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="T14" t="s">
-        <v>106</v>
-      </c>
-      <c r="U14" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="W14" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1621,7 +1708,7 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>690</v>
+        <v>396</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
@@ -1630,52 +1717,52 @@
         <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="F15" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G15">
-        <v>2727</v>
+        <v>2731</v>
       </c>
       <c r="H15" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I15" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J15" s="1">
-        <v>46303</v>
+        <v>46309</v>
       </c>
       <c r="K15" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N15" s="1">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="Q15">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R15">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="S15" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T15" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="W15" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1683,64 +1770,61 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
         <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="E16" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F16" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G16">
-        <v>2727</v>
+        <v>2703</v>
       </c>
       <c r="H16" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I16" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="J16" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
       <c r="K16" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
       <c r="L16">
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N16" s="1">
-        <v>46311</v>
+        <v>46340</v>
       </c>
       <c r="Q16">
-        <v>4</v>
+        <v>-24</v>
       </c>
       <c r="R16">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="S16" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="T16" t="s">
-        <v>106</v>
-      </c>
-      <c r="U16" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="W16" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1748,61 +1832,61 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>690</v>
+        <v>313</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C17" t="s">
         <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="E17" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="F17" t="s">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="G17">
-        <v>2727</v>
+        <v>2730</v>
       </c>
       <c r="H17" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I17" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="J17" s="1">
-        <v>46303</v>
+        <v>46309</v>
       </c>
       <c r="K17" s="1">
-        <v>46304</v>
+        <v>46316</v>
       </c>
       <c r="L17">
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N17" s="1">
-        <v>46311</v>
+        <v>46327</v>
       </c>
       <c r="Q17">
-        <v>4</v>
+        <v>-11</v>
       </c>
       <c r="R17">
-        <v>11</v>
-      </c>
-      <c r="S17" t="s">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="T17" t="s">
-        <v>106</v>
+        <v>116</v>
+      </c>
+      <c r="U17" t="s">
+        <v>120</v>
       </c>
       <c r="W17" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1810,7 +1894,7 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>690</v>
+        <v>396</v>
       </c>
       <c r="B18" t="s">
         <v>33</v>
@@ -1819,55 +1903,52 @@
         <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="E18" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="F18" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="G18">
-        <v>2727</v>
+        <v>2731</v>
       </c>
       <c r="H18" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I18" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J18" s="1">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="K18" s="1">
-        <v>46304</v>
+        <v>46315</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M18" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N18" s="1">
-        <v>46311</v>
+        <v>46322</v>
       </c>
       <c r="Q18">
-        <v>4</v>
+        <v>-6</v>
       </c>
       <c r="R18">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="S18" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="T18" t="s">
-        <v>106</v>
-      </c>
-      <c r="U18" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="W18" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1875,7 +1956,7 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>690</v>
+        <v>396</v>
       </c>
       <c r="B19" t="s">
         <v>33</v>
@@ -1884,52 +1965,52 @@
         <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="E19" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="F19" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="G19">
-        <v>2727</v>
+        <v>2731</v>
       </c>
       <c r="H19" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I19" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J19" s="1">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="K19" s="1">
-        <v>46304</v>
+        <v>46315</v>
       </c>
       <c r="L19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M19" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N19" s="1">
-        <v>46311</v>
+        <v>46322</v>
       </c>
       <c r="Q19">
-        <v>4</v>
+        <v>-6</v>
       </c>
       <c r="R19">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="S19" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T19" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="W19" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -1937,61 +2018,61 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
         <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E20" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F20" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="G20">
-        <v>2721</v>
+        <v>2702</v>
       </c>
       <c r="H20" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I20" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="J20" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="K20" s="1">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L20">
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N20" s="1">
-        <v>46320</v>
+        <v>46346</v>
       </c>
       <c r="Q20">
-        <v>-5</v>
+        <v>-30</v>
       </c>
       <c r="R20">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="S20" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T20" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="W20" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -1999,61 +2080,61 @@
     </row>
     <row r="21" spans="1:27">
       <c r="A21">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C21" t="s">
         <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="F21" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="G21">
-        <v>2721</v>
+        <v>2719</v>
       </c>
       <c r="H21" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I21" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="J21" s="1">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="K21" s="1">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L21">
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N21" s="1">
-        <v>46320</v>
+        <v>46346</v>
       </c>
       <c r="Q21">
-        <v>-5</v>
+        <v>-30</v>
       </c>
       <c r="R21">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="S21" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T21" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="W21" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2061,61 +2142,61 @@
     </row>
     <row r="22" spans="1:27">
       <c r="A22">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C22" t="s">
         <v>54</v>
       </c>
       <c r="D22" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E22" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F22" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="G22">
-        <v>2731</v>
+        <v>2722</v>
       </c>
       <c r="H22" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I22" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="J22" s="1">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="K22" s="1">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L22">
         <v>1</v>
       </c>
       <c r="M22" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="N22" s="1">
-        <v>46316</v>
+        <v>46326</v>
       </c>
       <c r="Q22">
-        <v>-1</v>
+        <v>-10</v>
       </c>
       <c r="R22">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="S22" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="T22" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="W22" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2132,54 +2213,302 @@
         <v>55</v>
       </c>
       <c r="D23" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E23" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="F23" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="G23">
-        <v>2703</v>
+        <v>2722</v>
       </c>
       <c r="H23" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I23" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="J23" s="1">
-        <v>46308</v>
+        <v>46311</v>
       </c>
       <c r="K23" s="1">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="L23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M23" t="s">
+        <v>114</v>
+      </c>
+      <c r="N23" s="1">
+        <v>46326</v>
+      </c>
+      <c r="Q23">
+        <v>-10</v>
+      </c>
+      <c r="R23">
+        <v>1</v>
+      </c>
+      <c r="S23" t="s">
+        <v>115</v>
+      </c>
+      <c r="T23" t="s">
+        <v>116</v>
+      </c>
+      <c r="W23" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27">
+      <c r="A24">
+        <v>685</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E24" t="s">
+        <v>103</v>
+      </c>
+      <c r="F24" t="s">
+        <v>108</v>
+      </c>
+      <c r="G24">
+        <v>2722</v>
+      </c>
+      <c r="H24" t="s">
+        <v>110</v>
+      </c>
+      <c r="I24" t="s">
+        <v>111</v>
+      </c>
+      <c r="J24" s="1">
+        <v>46311</v>
+      </c>
+      <c r="K24" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L24">
+        <v>3</v>
+      </c>
+      <c r="M24" t="s">
+        <v>114</v>
+      </c>
+      <c r="N24" s="1">
+        <v>46346</v>
+      </c>
+      <c r="Q24">
+        <v>-30</v>
+      </c>
+      <c r="R24">
+        <v>1</v>
+      </c>
+      <c r="S24" t="s">
+        <v>115</v>
+      </c>
+      <c r="T24" t="s">
+        <v>116</v>
+      </c>
+      <c r="W24" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27">
+      <c r="A25">
+        <v>685</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" t="s">
+        <v>80</v>
+      </c>
+      <c r="E25" t="s">
+        <v>103</v>
+      </c>
+      <c r="F25" t="s">
+        <v>108</v>
+      </c>
+      <c r="G25">
+        <v>2719</v>
+      </c>
+      <c r="H25" t="s">
+        <v>110</v>
+      </c>
+      <c r="I25" t="s">
+        <v>111</v>
+      </c>
+      <c r="J25" s="1">
+        <v>46311</v>
+      </c>
+      <c r="K25" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L25">
+        <v>3</v>
+      </c>
+      <c r="M25" t="s">
+        <v>114</v>
+      </c>
+      <c r="N25" s="1">
+        <v>46346</v>
+      </c>
+      <c r="Q25">
+        <v>-30</v>
+      </c>
+      <c r="R25">
+        <v>1</v>
+      </c>
+      <c r="S25" t="s">
+        <v>115</v>
+      </c>
+      <c r="T25" t="s">
+        <v>116</v>
+      </c>
+      <c r="W25" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27">
+      <c r="A26">
+        <v>685</v>
+      </c>
+      <c r="B26" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" t="s">
+        <v>104</v>
+      </c>
+      <c r="F26" t="s">
+        <v>106</v>
+      </c>
+      <c r="G26">
+        <v>2722</v>
+      </c>
+      <c r="H26" t="s">
+        <v>110</v>
+      </c>
+      <c r="I26" t="s">
+        <v>112</v>
+      </c>
+      <c r="J26" s="1">
+        <v>46315</v>
+      </c>
+      <c r="K26" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L26">
+        <v>12</v>
+      </c>
+      <c r="M26" t="s">
+        <v>114</v>
+      </c>
+      <c r="N26" s="1">
+        <v>46326</v>
+      </c>
+      <c r="Q26">
+        <v>-10</v>
+      </c>
+      <c r="R26">
+        <v>1</v>
+      </c>
+      <c r="S26" t="s">
+        <v>116</v>
+      </c>
+      <c r="T26" t="s">
+        <v>116</v>
+      </c>
+      <c r="W26" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27">
+      <c r="A27">
+        <v>396</v>
+      </c>
+      <c r="B27" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" t="s">
+        <v>82</v>
+      </c>
+      <c r="E27" t="s">
         <v>105</v>
       </c>
-      <c r="N23" s="1">
-        <v>46340</v>
-      </c>
-      <c r="Q23">
-        <v>-25</v>
-      </c>
-      <c r="R23">
-        <v>6</v>
-      </c>
-      <c r="S23" t="s">
-        <v>106</v>
-      </c>
-      <c r="T23" t="s">
-        <v>107</v>
-      </c>
-      <c r="W23" t="s">
+      <c r="F27" t="s">
+        <v>108</v>
+      </c>
+      <c r="G27">
+        <v>2731</v>
+      </c>
+      <c r="H27" t="s">
+        <v>110</v>
+      </c>
+      <c r="I27" t="s">
+        <v>113</v>
+      </c>
+      <c r="J27" s="1">
+        <v>46315</v>
+      </c>
+      <c r="K27" s="1">
+        <v>46316</v>
+      </c>
+      <c r="L27">
+        <v>1</v>
+      </c>
+      <c r="M27" t="s">
+        <v>114</v>
+      </c>
+      <c r="N27" s="1">
+        <v>46323</v>
+      </c>
+      <c r="Q27">
+        <v>-7</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+      <c r="S27" t="s">
+        <v>115</v>
+      </c>
+      <c r="T27" t="s">
         <v>116</v>
       </c>
-      <c r="AA23" t="b">
+      <c r="W27" t="s">
+        <v>131</v>
+      </c>
+      <c r="AA27" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (21/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -419,8 +419,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -436,7 +444,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -444,12 +452,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -749,85 +775,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -859,10 +885,10 @@
       <c r="I2" t="s">
         <v>111</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -871,7 +897,7 @@
       <c r="M2" t="s">
         <v>114</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -927,10 +953,10 @@
       <c r="I3" t="s">
         <v>111</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46294</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -939,10 +965,10 @@
       <c r="M3" t="s">
         <v>114</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46326</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46326</v>
       </c>
       <c r="Q3">
@@ -995,10 +1021,10 @@
       <c r="I4" t="s">
         <v>111</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46294</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -1007,10 +1033,10 @@
       <c r="M4" t="s">
         <v>114</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46326</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46305</v>
       </c>
       <c r="Q4">
@@ -1063,10 +1089,10 @@
       <c r="I5" t="s">
         <v>111</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46296</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1075,7 +1101,7 @@
       <c r="M5" t="s">
         <v>114</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46327</v>
       </c>
       <c r="Q5">
@@ -1131,10 +1157,10 @@
       <c r="I6" t="s">
         <v>111</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46301</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1143,10 +1169,10 @@
       <c r="M6" t="s">
         <v>114</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46333</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46214</v>
       </c>
       <c r="Q6">
@@ -1199,10 +1225,10 @@
       <c r="I7" t="s">
         <v>111</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46302</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1211,10 +1237,10 @@
       <c r="M7" t="s">
         <v>114</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46333</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46214</v>
       </c>
       <c r="Q7">
@@ -1267,10 +1293,10 @@
       <c r="I8" t="s">
         <v>112</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46304</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1279,7 +1305,7 @@
       <c r="M8" t="s">
         <v>114</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46315</v>
       </c>
       <c r="Q8">
@@ -1332,10 +1358,10 @@
       <c r="I9" t="s">
         <v>113</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46304</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1344,10 +1370,10 @@
       <c r="M9" t="s">
         <v>114</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46311</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46308</v>
       </c>
       <c r="Q9">
@@ -1400,10 +1426,10 @@
       <c r="I10" t="s">
         <v>112</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46303</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46304</v>
       </c>
       <c r="L10">
@@ -1412,10 +1438,10 @@
       <c r="M10" t="s">
         <v>114</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46315</v>
       </c>
-      <c r="O10" s="1">
+      <c r="O10" s="2">
         <v>46311</v>
       </c>
       <c r="Q10">
@@ -1468,10 +1494,10 @@
       <c r="I11" t="s">
         <v>113</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46303</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46304</v>
       </c>
       <c r="L11">
@@ -1480,10 +1506,10 @@
       <c r="M11" t="s">
         <v>114</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46311</v>
       </c>
-      <c r="O11" s="1">
+      <c r="O11" s="2">
         <v>46311</v>
       </c>
       <c r="Q11">
@@ -1539,10 +1565,10 @@
       <c r="I12" t="s">
         <v>113</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46303</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46304</v>
       </c>
       <c r="L12">
@@ -1551,10 +1577,10 @@
       <c r="M12" t="s">
         <v>114</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46311</v>
       </c>
-      <c r="O12" s="1">
+      <c r="O12" s="2">
         <v>46309</v>
       </c>
       <c r="Q12">
@@ -1610,10 +1636,10 @@
       <c r="I13" t="s">
         <v>112</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46308</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46309</v>
       </c>
       <c r="L13">
@@ -1622,7 +1648,7 @@
       <c r="M13" t="s">
         <v>114</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46320</v>
       </c>
       <c r="Q13">
@@ -1672,10 +1698,10 @@
       <c r="I14" t="s">
         <v>112</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46308</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46309</v>
       </c>
       <c r="L14">
@@ -1684,7 +1710,7 @@
       <c r="M14" t="s">
         <v>114</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46320</v>
       </c>
       <c r="Q14">
@@ -1734,10 +1760,10 @@
       <c r="I15" t="s">
         <v>113</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46309</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46309</v>
       </c>
       <c r="L15">
@@ -1746,7 +1772,7 @@
       <c r="M15" t="s">
         <v>114</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46316</v>
       </c>
       <c r="Q15">
@@ -1796,10 +1822,10 @@
       <c r="I16" t="s">
         <v>111</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46308</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46309</v>
       </c>
       <c r="L16">
@@ -1808,7 +1834,7 @@
       <c r="M16" t="s">
         <v>114</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46340</v>
       </c>
       <c r="Q16">
@@ -1858,10 +1884,10 @@
       <c r="I17" t="s">
         <v>112</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46309</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46316</v>
       </c>
       <c r="L17">
@@ -1870,7 +1896,7 @@
       <c r="M17" t="s">
         <v>114</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46327</v>
       </c>
       <c r="Q17">
@@ -1920,10 +1946,10 @@
       <c r="I18" t="s">
         <v>113</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46310</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46315</v>
       </c>
       <c r="L18">
@@ -1932,7 +1958,7 @@
       <c r="M18" t="s">
         <v>114</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46322</v>
       </c>
       <c r="Q18">
@@ -1982,10 +2008,10 @@
       <c r="I19" t="s">
         <v>113</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46310</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46315</v>
       </c>
       <c r="L19">
@@ -1994,7 +2020,7 @@
       <c r="M19" t="s">
         <v>114</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46322</v>
       </c>
       <c r="Q19">
@@ -2044,10 +2070,10 @@
       <c r="I20" t="s">
         <v>111</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46310</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46315</v>
       </c>
       <c r="L20">
@@ -2056,7 +2082,7 @@
       <c r="M20" t="s">
         <v>114</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46346</v>
       </c>
       <c r="Q20">
@@ -2106,10 +2132,10 @@
       <c r="I21" t="s">
         <v>111</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46310</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46315</v>
       </c>
       <c r="L21">
@@ -2118,7 +2144,7 @@
       <c r="M21" t="s">
         <v>114</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46346</v>
       </c>
       <c r="Q21">
@@ -2168,10 +2194,10 @@
       <c r="I22" t="s">
         <v>112</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46311</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>46315</v>
       </c>
       <c r="L22">
@@ -2180,7 +2206,7 @@
       <c r="M22" t="s">
         <v>114</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <v>46326</v>
       </c>
       <c r="Q22">
@@ -2230,10 +2256,10 @@
       <c r="I23" t="s">
         <v>112</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46311</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>46315</v>
       </c>
       <c r="L23">
@@ -2242,7 +2268,7 @@
       <c r="M23" t="s">
         <v>114</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <v>46326</v>
       </c>
       <c r="Q23">
@@ -2292,10 +2318,10 @@
       <c r="I24" t="s">
         <v>111</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46311</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>46315</v>
       </c>
       <c r="L24">
@@ -2304,7 +2330,7 @@
       <c r="M24" t="s">
         <v>114</v>
       </c>
-      <c r="N24" s="1">
+      <c r="N24" s="2">
         <v>46346</v>
       </c>
       <c r="Q24">
@@ -2354,10 +2380,10 @@
       <c r="I25" t="s">
         <v>111</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46311</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>46315</v>
       </c>
       <c r="L25">
@@ -2366,7 +2392,7 @@
       <c r="M25" t="s">
         <v>114</v>
       </c>
-      <c r="N25" s="1">
+      <c r="N25" s="2">
         <v>46346</v>
       </c>
       <c r="Q25">
@@ -2416,10 +2442,10 @@
       <c r="I26" t="s">
         <v>112</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46315</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>46315</v>
       </c>
       <c r="L26">
@@ -2428,7 +2454,7 @@
       <c r="M26" t="s">
         <v>114</v>
       </c>
-      <c r="N26" s="1">
+      <c r="N26" s="2">
         <v>46326</v>
       </c>
       <c r="Q26">
@@ -2478,10 +2504,10 @@
       <c r="I27" t="s">
         <v>113</v>
       </c>
-      <c r="J27" s="1">
+      <c r="J27" s="2">
         <v>46315</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>46316</v>
       </c>
       <c r="L27">
@@ -2490,7 +2516,7 @@
       <c r="M27" t="s">
         <v>114</v>
       </c>
-      <c r="N27" s="1">
+      <c r="N27" s="2">
         <v>46323</v>
       </c>
       <c r="Q27">

</xml_diff>

<commit_message>
Atualização automática: emergencias (22/10/2026 12:52)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="144">
   <si>
     <t>om_emg</t>
   </si>
@@ -112,9 +112,6 @@
     <t>BABR</t>
   </si>
   <si>
-    <t>BACG</t>
-  </si>
-  <si>
     <t>BABE</t>
   </si>
   <si>
@@ -139,18 +136,9 @@
     <t>329260019312</t>
   </si>
   <si>
-    <t>329260019313</t>
-  </si>
-  <si>
     <t>685260012964</t>
   </si>
   <si>
-    <t>690260002678</t>
-  </si>
-  <si>
-    <t>690260002680</t>
-  </si>
-  <si>
     <t>329260019318</t>
   </si>
   <si>
@@ -196,6 +184,12 @@
     <t>396260016650</t>
   </si>
   <si>
+    <t>329260019334</t>
+  </si>
+  <si>
+    <t>329260019335</t>
+  </si>
+  <si>
     <t>040-0043</t>
   </si>
   <si>
@@ -217,18 +211,9 @@
     <t>9910338-6</t>
   </si>
   <si>
-    <t>MS28773-05</t>
-  </si>
-  <si>
     <t>103-20400</t>
   </si>
   <si>
-    <t>3034792</t>
-  </si>
-  <si>
-    <t>M83248/1-029</t>
-  </si>
-  <si>
     <t>9910592-2</t>
   </si>
   <si>
@@ -265,6 +250,12 @@
     <t>2643100-201</t>
   </si>
   <si>
+    <t>030-02178-0000</t>
+  </si>
+  <si>
+    <t>C660501-0102</t>
+  </si>
+  <si>
     <t>STROB TUB</t>
   </si>
   <si>
@@ -286,18 +277,9 @@
     <t>TRANSMITTER,RATE OF</t>
   </si>
   <si>
-    <t>RETAINER,PACKING</t>
-  </si>
-  <si>
     <t>BOLT,MACHINE</t>
   </si>
   <si>
-    <t>BOMBA DE COMBUSTÍVEL</t>
-  </si>
-  <si>
-    <t>ANEL-O</t>
-  </si>
-  <si>
     <t>ALTERNADOR</t>
   </si>
   <si>
@@ -334,6 +316,12 @@
     <t>NOSE GEAR STRUT ASSY</t>
   </si>
   <si>
+    <t>CONNECTOR,ELECTRICAL</t>
+  </si>
+  <si>
+    <t>COMPASS ASSY</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -349,15 +337,18 @@
     <t>Aguardando solução</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
+    <t>AIFP</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -370,43 +361,88 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
+    <t>AWB 127-6186 9835 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
+  </si>
+  <si>
     <t>O compressor passou por teste no PAMALS onde foi identificada a pane nesse item. Ramon 21/10/26.</t>
   </si>
   <si>
-    <t>Atendido com estoque local em 09/10. Ramon 09/10/26. AWB 127-6253 8910 liberado para retirada em 13/10. Ramon 14/10/26.</t>
+    <t>Recibo 887/FAB/26 AWB 127-6307 3301 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
+  </si>
+  <si>
+    <t>AWB 127-6350 4696 retirado por Jader Dantas, recebedor desconhecido. Ramon 22/10/26.</t>
+  </si>
+  <si>
+    <t>AWB 127-6350 5142 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
   </si>
   <si>
     <t>Cedeu o item para o C-98 2736. Ramon 21/10.</t>
   </si>
   <si>
+    <t>Atendido com estoque local em 21/10. Agd AWB 127-6466 1855 com previsão de entrega em 24/10. Ramon 22/10</t>
+  </si>
+  <si>
+    <t>Atendido com estoque local em 21/10. AWB 127-6465 9825 com previsão de entrega em 23/10. Ramon 22/10/26</t>
+  </si>
+  <si>
+    <t>Autorizado reparo de fones do A7 para posterior mudança para U8. Ramon 22/10</t>
+  </si>
+  <si>
+    <t>Atendido com estoque local em 21/10 TSP 18710930. AWB 127-6465 9825 com previsão de entrega em 23/10. Ramon 22/10/26</t>
+  </si>
+  <si>
+    <t>Estoque do PN superador. Ramon 22/10</t>
+  </si>
+  <si>
     <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
   </si>
   <si>
-    <t>AGD ABERTURA DE OS- REZ , email solicitando abertura de o.s. dia 30-09-26, CLA -06-10-26. Abertas OS para 05 ea dia 07/10.Material será coletado dia 09/10 fins reparo - REZ</t>
+    <t>Enviados 02 ea para reparo em 09/10/2026 - REZ - Ag orçamento</t>
   </si>
   <si>
     <t>Enviado para o Operador dia 09/10/26 - AWB 127-6186 9835 - REZ - MATERIAL ENTREGUE DIA 10/10/2026 no CAN BANT</t>
   </si>
   <si>
-    <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26</t>
-  </si>
-  <si>
-    <t>Abertas OS para 05 ea dia 07/10.Material será coletado dia 09/10 fins reparo - REZ</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17796997 - entregue em Miami 09/10</t>
-  </si>
-  <si>
-    <t>solicitado abertura de OS de 03 ea em 09/10/2026.REZ</t>
-  </si>
-  <si>
-    <t>MATERIAL EM TRANSITO - RECIBO 884/FAB/26 AWB 12762528605 RC 09/10/2026 - AWB DISPONIVEL PARA RETIRADA 13/10/2026</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron WB0003180334 - previsão de entrega no RJ 13/10 - MATERIAL RECEBIDO EM RJ 13/10 - PREPARANDO ENVIO 13/10 - recibo 887/FAB/26 AWB 12763073301 DPE 16/10/2026</t>
-  </si>
-  <si>
-    <t>ATENDIDO VIA ESTOQUE FAB, AWB A SER GERADA GOLLOG 09/10/2026. AWB 127-6253 8910</t>
+    <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26 .Segundo informações do Ten Soares do CLA não é preciso a compra do compressor no monento.(19/10/26 (SO R1 Bispo)</t>
+  </si>
+  <si>
+    <t>Abertas OS para 03 ea dia 07/10.Material coletado dia 09/10 fins reparo - AGD orçamento - REZ</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17796997 - chegada GIG 14/10 (voo 4588) em desembaraço - Material aguardando a documentação da Textron, pois não veio com o material 20/10/26. Solicitado abertura de Os para 01 ea em 07/10/2026 para fazer o envio a Textron por ser unidade como CORE -REZ</t>
+  </si>
+  <si>
+    <t>abertas OS de 03 ea em 09/10/2026.REZ</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron WB0003180334 - previsão de entrega no RJ 13/10 - MATERIAL RECEBIDO EM RJ 13/10 - PREPARANDO ENVIO 13/10 - recibo 887/FAB/26 AWB 12763073301 DPE 16/10/2026 - MATERIAL ENTREGUE DIA 15/10/2026</t>
+  </si>
+  <si>
+    <t>04 ea em reparo na William e 02 ea na Av aeronáutica. Solicitado apressamento e DPE para ambas as empresas em 15/10/26 - REZ</t>
+  </si>
+  <si>
+    <t>Há no estq V1/LS para atender. Será enviado dia 15/10/26 para o Operador - REZ - AWB 127-6350 4696</t>
+  </si>
+  <si>
+    <t>FCU enviada de Belém para RJ AWB 12763294361, disponível para retirada dia 15/10/2026 - Material enviado para a oficina, já em bancada realizando testes finais - 20/10/2026 - MATERIAL ENVIADO VIA RECIBO 911/FAB/26 - AWB A SER GERADA PELA GOLLOG RC 21-10-26</t>
+  </si>
+  <si>
+    <t>Há no estq V1/LS para atender. Será enviado dia 15/10/26 para o Operador - REZ- --AWB 127-6350 5142</t>
+  </si>
+  <si>
+    <t>Colocado pedido I837605 - entregue 02ea em Miami 21/10</t>
+  </si>
+  <si>
+    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , PELO PN ALTERNADO MS20007-70. - RC 20/10/2026</t>
+  </si>
+  <si>
+    <t>01 EA SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA".- RC 20/10/2026 01 EA ENVIADO PELO RECIBO 907/FAB/26, AWB A SER GERADA PELA GOLLOG RC 20/10/2026</t>
+  </si>
+  <si>
+    <t>SOLICITAMOS OS CORES PARA REALIZAR REPARO, TENDO EM VISTA QUE NÃO TEMOS NO TSAM PARA RECOLHIMENTO. RC 20/10/2026</t>
+  </si>
+  <si>
+    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , - RC 20/10/2026</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -419,16 +455,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -444,7 +472,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -452,30 +480,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -771,89 +781,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA27"/>
+  <dimension ref="A1:AA26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -865,61 +875,61 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I2" t="s">
-        <v>111</v>
-      </c>
-      <c r="J2" s="2">
+        <v>108</v>
+      </c>
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
         <v>2</v>
       </c>
       <c r="M2" t="s">
+        <v>111</v>
+      </c>
+      <c r="N2" s="1">
+        <v>46280</v>
+      </c>
+      <c r="Q2">
+        <v>37</v>
+      </c>
+      <c r="R2">
+        <v>68</v>
+      </c>
+      <c r="S2" t="s">
+        <v>112</v>
+      </c>
+      <c r="T2" t="s">
+        <v>113</v>
+      </c>
+      <c r="U2" t="s">
         <v>114</v>
       </c>
-      <c r="N2" s="2">
-        <v>46280</v>
-      </c>
-      <c r="Q2">
-        <v>36</v>
-      </c>
-      <c r="R2">
-        <v>67</v>
-      </c>
-      <c r="S2" t="s">
-        <v>115</v>
-      </c>
-      <c r="T2" t="s">
-        <v>116</v>
-      </c>
-      <c r="U2" t="s">
-        <v>117</v>
-      </c>
       <c r="V2" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="W2" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -933,61 +943,61 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G3">
         <v>2703</v>
       </c>
       <c r="H3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J3" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
         <v>111</v>
       </c>
-      <c r="J3" s="2">
-        <v>46294</v>
-      </c>
-      <c r="K3" s="2">
-        <v>46295</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-      <c r="M3" t="s">
-        <v>114</v>
-      </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46326</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R3">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="V3" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="W3" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -1001,61 +1011,64 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F4" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G4">
         <v>2703</v>
       </c>
       <c r="H4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I4" t="s">
+        <v>108</v>
+      </c>
+      <c r="J4" s="1">
+        <v>46294</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46295</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="s">
         <v>111</v>
       </c>
-      <c r="J4" s="2">
-        <v>46294</v>
-      </c>
-      <c r="K4" s="2">
-        <v>46295</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4" t="s">
-        <v>114</v>
-      </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46326</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46305</v>
       </c>
       <c r="Q4">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R4">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S4" t="s">
+        <v>112</v>
+      </c>
+      <c r="T4" t="s">
+        <v>113</v>
+      </c>
+      <c r="U4" t="s">
         <v>115</v>
       </c>
-      <c r="T4" t="s">
-        <v>116</v>
-      </c>
       <c r="V4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="W4" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1069,61 +1082,61 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F5" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G5">
         <v>2723</v>
       </c>
       <c r="H5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I5" t="s">
+        <v>108</v>
+      </c>
+      <c r="J5" s="1">
+        <v>46296</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46296</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
         <v>111</v>
       </c>
-      <c r="J5" s="2">
-        <v>46296</v>
-      </c>
-      <c r="K5" s="2">
-        <v>46296</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5" t="s">
-        <v>114</v>
-      </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="U5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="V5" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="W5" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1137,61 +1150,61 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G6">
         <v>2708</v>
       </c>
       <c r="H6" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I6" t="s">
+        <v>108</v>
+      </c>
+      <c r="J6" s="1">
+        <v>46301</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46302</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
         <v>111</v>
       </c>
-      <c r="J6" s="2">
-        <v>46301</v>
-      </c>
-      <c r="K6" s="2">
-        <v>46302</v>
-      </c>
-      <c r="L6">
-        <v>1</v>
-      </c>
-      <c r="M6" t="s">
-        <v>114</v>
-      </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46333</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46214</v>
       </c>
       <c r="Q6">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T6" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="V6" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="W6" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1205,61 +1218,61 @@
         <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F7" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G7">
         <v>2742</v>
       </c>
       <c r="H7" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I7" t="s">
+        <v>108</v>
+      </c>
+      <c r="J7" s="1">
+        <v>46302</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46302</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>111</v>
       </c>
-      <c r="J7" s="2">
-        <v>46302</v>
-      </c>
-      <c r="K7" s="2">
-        <v>46302</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>114</v>
-      </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46333</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46214</v>
       </c>
       <c r="Q7">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="R7">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="V7" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="W7" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1273,58 +1286,58 @@
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E8" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G8">
         <v>2721</v>
       </c>
       <c r="H8" t="s">
+        <v>105</v>
+      </c>
+      <c r="I8" t="s">
         <v>109</v>
       </c>
-      <c r="I8" t="s">
-        <v>112</v>
-      </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46304</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46304</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>114</v>
-      </c>
-      <c r="N8" s="2">
-        <v>46315</v>
+        <v>111</v>
+      </c>
+      <c r="N8" s="1">
+        <v>46311</v>
       </c>
       <c r="Q8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="R8">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="V8" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="W8" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1332,67 +1345,70 @@
     </row>
     <row r="9" spans="1:27">
       <c r="A9">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E9" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="F9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G9">
-        <v>2721</v>
+        <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I9" t="s">
+        <v>110</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46303</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46304</v>
+      </c>
+      <c r="L9">
+        <v>12</v>
+      </c>
+      <c r="M9" t="s">
+        <v>111</v>
+      </c>
+      <c r="N9" s="1">
+        <v>46315</v>
+      </c>
+      <c r="O9" s="1">
+        <v>46310</v>
+      </c>
+      <c r="Q9">
+        <v>2</v>
+      </c>
+      <c r="R9">
+        <v>13</v>
+      </c>
+      <c r="S9" t="s">
+        <v>112</v>
+      </c>
+      <c r="T9" t="s">
         <v>113</v>
       </c>
-      <c r="J9" s="2">
-        <v>46304</v>
-      </c>
-      <c r="K9" s="2">
-        <v>46304</v>
-      </c>
-      <c r="L9">
-        <v>1</v>
-      </c>
-      <c r="M9" t="s">
-        <v>114</v>
-      </c>
-      <c r="N9" s="2">
-        <v>46311</v>
-      </c>
-      <c r="O9" s="2">
-        <v>46308</v>
-      </c>
-      <c r="Q9">
-        <v>5</v>
-      </c>
-      <c r="R9">
-        <v>12</v>
-      </c>
-      <c r="S9" t="s">
-        <v>115</v>
-      </c>
-      <c r="T9" t="s">
-        <v>115</v>
+      <c r="U9" t="s">
+        <v>117</v>
       </c>
       <c r="V9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="W9" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1400,67 +1416,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G10">
-        <v>2729</v>
+        <v>2721</v>
       </c>
       <c r="H10" t="s">
+        <v>105</v>
+      </c>
+      <c r="I10" t="s">
         <v>109</v>
       </c>
-      <c r="I10" t="s">
-        <v>112</v>
-      </c>
-      <c r="J10" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K10" s="2">
-        <v>46304</v>
+      <c r="J10" s="1">
+        <v>46308</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46309</v>
       </c>
       <c r="L10">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>114</v>
-      </c>
-      <c r="N10" s="2">
-        <v>46315</v>
-      </c>
-      <c r="O10" s="2">
-        <v>46311</v>
+        <v>111</v>
+      </c>
+      <c r="N10" s="1">
+        <v>46316</v>
       </c>
       <c r="Q10">
         <v>1</v>
       </c>
       <c r="R10">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="S10" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="V10" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="W10" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1468,70 +1481,67 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>690</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E11" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F11" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G11">
-        <v>2727</v>
+        <v>2721</v>
       </c>
       <c r="H11" t="s">
+        <v>105</v>
+      </c>
+      <c r="I11" t="s">
         <v>109</v>
       </c>
-      <c r="I11" t="s">
-        <v>113</v>
-      </c>
-      <c r="J11" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K11" s="2">
-        <v>46304</v>
+      <c r="J11" s="1">
+        <v>46308</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46309</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>114</v>
-      </c>
-      <c r="N11" s="2">
-        <v>46311</v>
-      </c>
-      <c r="O11" s="2">
-        <v>46311</v>
+        <v>111</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46316</v>
       </c>
       <c r="Q11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R11">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="S11" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="T11" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="U11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="V11" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="W11" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1539,70 +1549,64 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>690</v>
+        <v>396</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F12" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G12">
-        <v>2727</v>
+        <v>2731</v>
       </c>
       <c r="H12" t="s">
+        <v>105</v>
+      </c>
+      <c r="I12" t="s">
         <v>109</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" s="1">
+        <v>46309</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46309</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>111</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46316</v>
+      </c>
+      <c r="Q12">
+        <v>1</v>
+      </c>
+      <c r="R12">
+        <v>8</v>
+      </c>
+      <c r="S12" t="s">
+        <v>112</v>
+      </c>
+      <c r="T12" t="s">
         <v>113</v>
       </c>
-      <c r="J12" s="2">
-        <v>46303</v>
-      </c>
-      <c r="K12" s="2">
-        <v>46304</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>114</v>
-      </c>
-      <c r="N12" s="2">
-        <v>46311</v>
-      </c>
-      <c r="O12" s="2">
-        <v>46309</v>
-      </c>
-      <c r="Q12">
-        <v>5</v>
-      </c>
-      <c r="R12">
-        <v>12</v>
-      </c>
-      <c r="S12" t="s">
-        <v>116</v>
-      </c>
-      <c r="T12" t="s">
-        <v>115</v>
-      </c>
-      <c r="U12" t="s">
-        <v>119</v>
-      </c>
       <c r="V12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="W12" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1610,61 +1614,67 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E13" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F13" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G13">
-        <v>2721</v>
+        <v>2703</v>
       </c>
       <c r="H13" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I13" t="s">
-        <v>112</v>
-      </c>
-      <c r="J13" s="2">
+        <v>108</v>
+      </c>
+      <c r="J13" s="1">
         <v>46308</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46309</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>114</v>
-      </c>
-      <c r="N13" s="2">
-        <v>46320</v>
+        <v>111</v>
+      </c>
+      <c r="N13" s="1">
+        <v>46340</v>
       </c>
       <c r="Q13">
-        <v>-4</v>
+        <v>-23</v>
       </c>
       <c r="R13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S13" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T13" t="s">
-        <v>115</v>
+        <v>113</v>
+      </c>
+      <c r="U13" t="s">
+        <v>119</v>
+      </c>
+      <c r="V13" t="s">
+        <v>137</v>
       </c>
       <c r="W13" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1672,61 +1682,61 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E14" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F14" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="G14">
-        <v>2721</v>
+        <v>2730</v>
       </c>
       <c r="H14" t="s">
+        <v>105</v>
+      </c>
+      <c r="I14" t="s">
         <v>110</v>
       </c>
-      <c r="I14" t="s">
-        <v>112</v>
-      </c>
-      <c r="J14" s="2">
-        <v>46308</v>
-      </c>
-      <c r="K14" s="2">
+      <c r="J14" s="1">
         <v>46309</v>
       </c>
+      <c r="K14" s="1">
+        <v>46316</v>
+      </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>114</v>
-      </c>
-      <c r="N14" s="2">
-        <v>46320</v>
+        <v>111</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46327</v>
       </c>
       <c r="Q14">
-        <v>-4</v>
+        <v>-10</v>
       </c>
       <c r="R14">
-        <v>7</v>
-      </c>
-      <c r="S14" t="s">
-        <v>115</v>
+        <v>1</v>
       </c>
       <c r="T14" t="s">
-        <v>115</v>
+        <v>113</v>
+      </c>
+      <c r="U14" t="s">
+        <v>120</v>
       </c>
       <c r="W14" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1737,58 +1747,61 @@
         <v>396</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E15" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F15" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G15">
         <v>2731</v>
       </c>
       <c r="H15" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="I15" t="s">
+        <v>109</v>
+      </c>
+      <c r="J15" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L15">
+        <v>4</v>
+      </c>
+      <c r="M15" t="s">
+        <v>111</v>
+      </c>
+      <c r="N15" s="1">
+        <v>46322</v>
+      </c>
+      <c r="Q15">
+        <v>-5</v>
+      </c>
+      <c r="R15">
+        <v>2</v>
+      </c>
+      <c r="S15" t="s">
+        <v>112</v>
+      </c>
+      <c r="T15" t="s">
         <v>113</v>
       </c>
-      <c r="J15" s="2">
-        <v>46309</v>
-      </c>
-      <c r="K15" s="2">
-        <v>46309</v>
-      </c>
-      <c r="L15">
-        <v>1</v>
-      </c>
-      <c r="M15" t="s">
-        <v>114</v>
-      </c>
-      <c r="N15" s="2">
-        <v>46316</v>
-      </c>
-      <c r="Q15">
-        <v>0</v>
-      </c>
-      <c r="R15">
-        <v>7</v>
-      </c>
-      <c r="S15" t="s">
-        <v>115</v>
-      </c>
-      <c r="T15" t="s">
-        <v>116</v>
+      <c r="V15" t="s">
+        <v>138</v>
       </c>
       <c r="W15" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1796,61 +1809,67 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E16" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F16" t="s">
+        <v>102</v>
+      </c>
+      <c r="G16">
+        <v>2731</v>
+      </c>
+      <c r="H16" t="s">
         <v>107</v>
       </c>
-      <c r="G16">
-        <v>2703</v>
-      </c>
-      <c r="H16" t="s">
-        <v>110</v>
-      </c>
       <c r="I16" t="s">
+        <v>109</v>
+      </c>
+      <c r="J16" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L16">
+        <v>2</v>
+      </c>
+      <c r="M16" t="s">
         <v>111</v>
       </c>
-      <c r="J16" s="2">
-        <v>46308</v>
-      </c>
-      <c r="K16" s="2">
-        <v>46309</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16" t="s">
-        <v>114</v>
-      </c>
-      <c r="N16" s="2">
-        <v>46340</v>
+      <c r="N16" s="1">
+        <v>46322</v>
       </c>
       <c r="Q16">
-        <v>-24</v>
+        <v>-5</v>
       </c>
       <c r="R16">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="S16" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T16" t="s">
-        <v>116</v>
+        <v>113</v>
+      </c>
+      <c r="U16" t="s">
+        <v>121</v>
+      </c>
+      <c r="V16" t="s">
+        <v>139</v>
       </c>
       <c r="W16" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1858,61 +1877,61 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="E17" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="F17" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G17">
-        <v>2730</v>
+        <v>2702</v>
       </c>
       <c r="H17" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I17" t="s">
-        <v>112</v>
-      </c>
-      <c r="J17" s="2">
-        <v>46309</v>
-      </c>
-      <c r="K17" s="2">
-        <v>46316</v>
+        <v>108</v>
+      </c>
+      <c r="J17" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46315</v>
       </c>
       <c r="L17">
         <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>114</v>
-      </c>
-      <c r="N17" s="2">
-        <v>46327</v>
+        <v>111</v>
+      </c>
+      <c r="N17" s="1">
+        <v>46346</v>
       </c>
       <c r="Q17">
-        <v>-11</v>
+        <v>-29</v>
       </c>
       <c r="R17">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="S17" t="s">
+        <v>112</v>
       </c>
       <c r="T17" t="s">
-        <v>116</v>
-      </c>
-      <c r="U17" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="W17" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1920,61 +1939,61 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="E18" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="F18" t="s">
+        <v>103</v>
+      </c>
+      <c r="G18">
+        <v>2719</v>
+      </c>
+      <c r="H18" t="s">
         <v>106</v>
       </c>
-      <c r="G18">
-        <v>2731</v>
-      </c>
-      <c r="H18" t="s">
-        <v>110</v>
-      </c>
       <c r="I18" t="s">
+        <v>108</v>
+      </c>
+      <c r="J18" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K18" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18" t="s">
+        <v>111</v>
+      </c>
+      <c r="N18" s="1">
+        <v>46346</v>
+      </c>
+      <c r="Q18">
+        <v>-29</v>
+      </c>
+      <c r="R18">
+        <v>2</v>
+      </c>
+      <c r="S18" t="s">
+        <v>112</v>
+      </c>
+      <c r="T18" t="s">
         <v>113</v>
       </c>
-      <c r="J18" s="2">
-        <v>46310</v>
-      </c>
-      <c r="K18" s="2">
-        <v>46315</v>
-      </c>
-      <c r="L18">
-        <v>4</v>
-      </c>
-      <c r="M18" t="s">
-        <v>114</v>
-      </c>
-      <c r="N18" s="2">
-        <v>46322</v>
-      </c>
-      <c r="Q18">
-        <v>-6</v>
-      </c>
-      <c r="R18">
-        <v>1</v>
-      </c>
-      <c r="S18" t="s">
-        <v>115</v>
-      </c>
-      <c r="T18" t="s">
-        <v>116</v>
-      </c>
       <c r="W18" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1982,61 +2001,61 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E19" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F19" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G19">
-        <v>2731</v>
+        <v>2722</v>
       </c>
       <c r="H19" t="s">
+        <v>105</v>
+      </c>
+      <c r="I19" t="s">
         <v>110</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" s="1">
+        <v>46311</v>
+      </c>
+      <c r="K19" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19" t="s">
+        <v>111</v>
+      </c>
+      <c r="N19" s="1">
+        <v>46326</v>
+      </c>
+      <c r="Q19">
+        <v>-9</v>
+      </c>
+      <c r="R19">
+        <v>2</v>
+      </c>
+      <c r="S19" t="s">
+        <v>112</v>
+      </c>
+      <c r="T19" t="s">
         <v>113</v>
       </c>
-      <c r="J19" s="2">
-        <v>46310</v>
-      </c>
-      <c r="K19" s="2">
-        <v>46315</v>
-      </c>
-      <c r="L19">
-        <v>2</v>
-      </c>
-      <c r="M19" t="s">
-        <v>114</v>
-      </c>
-      <c r="N19" s="2">
-        <v>46322</v>
-      </c>
-      <c r="Q19">
-        <v>-6</v>
-      </c>
-      <c r="R19">
-        <v>1</v>
-      </c>
-      <c r="S19" t="s">
-        <v>115</v>
-      </c>
-      <c r="T19" t="s">
-        <v>116</v>
-      </c>
       <c r="W19" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2050,55 +2069,61 @@
         <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="E20" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="F20" t="s">
+        <v>104</v>
+      </c>
+      <c r="G20">
+        <v>2722</v>
+      </c>
+      <c r="H20" t="s">
         <v>107</v>
       </c>
-      <c r="G20">
-        <v>2702</v>
-      </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>110</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" s="1">
+        <v>46311</v>
+      </c>
+      <c r="K20" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L20">
+        <v>2</v>
+      </c>
+      <c r="M20" t="s">
         <v>111</v>
       </c>
-      <c r="J20" s="2">
-        <v>46310</v>
-      </c>
-      <c r="K20" s="2">
-        <v>46315</v>
-      </c>
-      <c r="L20">
-        <v>1</v>
-      </c>
-      <c r="M20" t="s">
-        <v>114</v>
-      </c>
-      <c r="N20" s="2">
-        <v>46346</v>
+      <c r="N20" s="1">
+        <v>46326</v>
       </c>
       <c r="Q20">
-        <v>-30</v>
+        <v>-9</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T20" t="s">
-        <v>116</v>
+        <v>113</v>
+      </c>
+      <c r="U20" t="s">
+        <v>122</v>
+      </c>
+      <c r="V20" t="s">
+        <v>140</v>
       </c>
       <c r="W20" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2112,55 +2137,61 @@
         <v>28</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="E21" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="F21" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G21">
-        <v>2719</v>
+        <v>2722</v>
       </c>
       <c r="H21" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I21" t="s">
+        <v>108</v>
+      </c>
+      <c r="J21" s="1">
+        <v>46311</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L21">
+        <v>3</v>
+      </c>
+      <c r="M21" t="s">
         <v>111</v>
       </c>
-      <c r="J21" s="2">
-        <v>46310</v>
-      </c>
-      <c r="K21" s="2">
-        <v>46315</v>
-      </c>
-      <c r="L21">
-        <v>1</v>
-      </c>
-      <c r="M21" t="s">
-        <v>114</v>
-      </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46346</v>
       </c>
       <c r="Q21">
-        <v>-30</v>
+        <v>-29</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S21" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T21" t="s">
-        <v>116</v>
+        <v>113</v>
+      </c>
+      <c r="U21" t="s">
+        <v>123</v>
+      </c>
+      <c r="V21" t="s">
+        <v>141</v>
       </c>
       <c r="W21" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2174,55 +2205,61 @@
         <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E22" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="F22" t="s">
+        <v>104</v>
+      </c>
+      <c r="G22">
+        <v>2719</v>
+      </c>
+      <c r="H22" t="s">
+        <v>106</v>
+      </c>
+      <c r="I22" t="s">
         <v>108</v>
       </c>
-      <c r="G22">
-        <v>2722</v>
-      </c>
-      <c r="H22" t="s">
-        <v>110</v>
-      </c>
-      <c r="I22" t="s">
-        <v>112</v>
-      </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46311</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>46315</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M22" t="s">
-        <v>114</v>
-      </c>
-      <c r="N22" s="2">
-        <v>46326</v>
+        <v>111</v>
+      </c>
+      <c r="N22" s="1">
+        <v>46346</v>
       </c>
       <c r="Q22">
-        <v>-10</v>
+        <v>-29</v>
       </c>
       <c r="R22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S22" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T22" t="s">
-        <v>116</v>
+        <v>113</v>
+      </c>
+      <c r="U22" t="s">
+        <v>123</v>
+      </c>
+      <c r="V22" t="s">
+        <v>141</v>
       </c>
       <c r="W22" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2236,55 +2273,61 @@
         <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F23" t="s">
         <v>102</v>
-      </c>
-      <c r="F23" t="s">
-        <v>108</v>
       </c>
       <c r="G23">
         <v>2722</v>
       </c>
       <c r="H23" t="s">
+        <v>105</v>
+      </c>
+      <c r="I23" t="s">
         <v>110</v>
       </c>
-      <c r="I23" t="s">
-        <v>112</v>
-      </c>
-      <c r="J23" s="2">
-        <v>46311</v>
-      </c>
-      <c r="K23" s="2">
+      <c r="J23" s="1">
         <v>46315</v>
       </c>
+      <c r="K23" s="1">
+        <v>46315</v>
+      </c>
       <c r="L23">
+        <v>12</v>
+      </c>
+      <c r="M23" t="s">
+        <v>111</v>
+      </c>
+      <c r="N23" s="1">
+        <v>46326</v>
+      </c>
+      <c r="Q23">
+        <v>-9</v>
+      </c>
+      <c r="R23">
         <v>2</v>
       </c>
-      <c r="M23" t="s">
-        <v>114</v>
-      </c>
-      <c r="N23" s="2">
-        <v>46326</v>
-      </c>
-      <c r="Q23">
-        <v>-10</v>
-      </c>
-      <c r="R23">
-        <v>1</v>
-      </c>
       <c r="S23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="T23" t="s">
-        <v>116</v>
+        <v>113</v>
+      </c>
+      <c r="U23" t="s">
+        <v>124</v>
+      </c>
+      <c r="V23" t="s">
+        <v>142</v>
       </c>
       <c r="W23" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA23" t="b">
         <v>1</v>
@@ -2292,61 +2335,61 @@
     </row>
     <row r="24" spans="1:27">
       <c r="A24">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E24" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F24" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G24">
-        <v>2722</v>
+        <v>2731</v>
       </c>
       <c r="H24" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="I24" t="s">
+        <v>109</v>
+      </c>
+      <c r="J24" s="1">
+        <v>46315</v>
+      </c>
+      <c r="K24" s="1">
+        <v>46316</v>
+      </c>
+      <c r="L24">
+        <v>1</v>
+      </c>
+      <c r="M24" t="s">
         <v>111</v>
       </c>
-      <c r="J24" s="2">
-        <v>46311</v>
-      </c>
-      <c r="K24" s="2">
-        <v>46315</v>
-      </c>
-      <c r="L24">
-        <v>3</v>
-      </c>
-      <c r="M24" t="s">
-        <v>114</v>
-      </c>
-      <c r="N24" s="2">
-        <v>46346</v>
+      <c r="N24" s="1">
+        <v>46323</v>
       </c>
       <c r="Q24">
-        <v>-30</v>
+        <v>-6</v>
       </c>
       <c r="R24">
         <v>1</v>
       </c>
       <c r="S24" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T24" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="W24" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA24" t="b">
         <v>1</v>
@@ -2354,61 +2397,61 @@
     </row>
     <row r="25" spans="1:27">
       <c r="A25">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E25" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F25" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G25">
-        <v>2719</v>
+        <v>2721</v>
       </c>
       <c r="H25" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I25" t="s">
+        <v>109</v>
+      </c>
+      <c r="J25" s="1">
+        <v>46316</v>
+      </c>
+      <c r="K25" s="1">
+        <v>46317</v>
+      </c>
+      <c r="L25">
+        <v>1</v>
+      </c>
+      <c r="M25" t="s">
         <v>111</v>
       </c>
-      <c r="J25" s="2">
-        <v>46311</v>
-      </c>
-      <c r="K25" s="2">
-        <v>46315</v>
-      </c>
-      <c r="L25">
-        <v>3</v>
-      </c>
-      <c r="M25" t="s">
-        <v>114</v>
-      </c>
-      <c r="N25" s="2">
-        <v>46346</v>
+      <c r="N25" s="1">
+        <v>46324</v>
       </c>
       <c r="Q25">
-        <v>-30</v>
+        <v>-7</v>
       </c>
       <c r="R25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S25" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="T25" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="W25" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA25" t="b">
         <v>1</v>
@@ -2416,125 +2459,66 @@
     </row>
     <row r="26" spans="1:27">
       <c r="A26">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B26" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D26" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E26" t="s">
+        <v>101</v>
+      </c>
+      <c r="F26" t="s">
         <v>104</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26">
+        <v>2721</v>
+      </c>
+      <c r="H26" t="s">
         <v>106</v>
       </c>
-      <c r="G26">
-        <v>2722</v>
-      </c>
-      <c r="H26" t="s">
-        <v>110</v>
-      </c>
       <c r="I26" t="s">
-        <v>112</v>
-      </c>
-      <c r="J26" s="2">
-        <v>46315</v>
-      </c>
-      <c r="K26" s="2">
-        <v>46315</v>
+        <v>109</v>
+      </c>
+      <c r="J26" s="1">
+        <v>46316</v>
+      </c>
+      <c r="K26" s="1">
+        <v>46317</v>
       </c>
       <c r="L26">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="M26" t="s">
-        <v>114</v>
-      </c>
-      <c r="N26" s="2">
-        <v>46326</v>
+        <v>111</v>
+      </c>
+      <c r="N26" s="1">
+        <v>46324</v>
       </c>
       <c r="Q26">
-        <v>-10</v>
+        <v>-7</v>
       </c>
       <c r="R26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S26" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="T26" t="s">
-        <v>116</v>
+        <v>112</v>
+      </c>
+      <c r="U26" t="s">
+        <v>125</v>
       </c>
       <c r="W26" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="AA26" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:27">
-      <c r="A27">
-        <v>396</v>
-      </c>
-      <c r="B27" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" t="s">
-        <v>59</v>
-      </c>
-      <c r="D27" t="s">
-        <v>82</v>
-      </c>
-      <c r="E27" t="s">
-        <v>105</v>
-      </c>
-      <c r="F27" t="s">
-        <v>108</v>
-      </c>
-      <c r="G27">
-        <v>2731</v>
-      </c>
-      <c r="H27" t="s">
-        <v>110</v>
-      </c>
-      <c r="I27" t="s">
-        <v>113</v>
-      </c>
-      <c r="J27" s="2">
-        <v>46315</v>
-      </c>
-      <c r="K27" s="2">
-        <v>46316</v>
-      </c>
-      <c r="L27">
-        <v>1</v>
-      </c>
-      <c r="M27" t="s">
-        <v>114</v>
-      </c>
-      <c r="N27" s="2">
-        <v>46323</v>
-      </c>
-      <c r="Q27">
-        <v>-7</v>
-      </c>
-      <c r="R27">
-        <v>0</v>
-      </c>
-      <c r="S27" t="s">
-        <v>115</v>
-      </c>
-      <c r="T27" t="s">
-        <v>116</v>
-      </c>
-      <c r="W27" t="s">
-        <v>131</v>
-      </c>
-      <c r="AA27" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/10/2026 12:43)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -911,10 +911,10 @@
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="R2">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="S2" t="s">
         <v>112</v>
@@ -982,10 +982,10 @@
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="S3" t="s">
         <v>112</v>
@@ -1050,10 +1050,10 @@
         <v>46305</v>
       </c>
       <c r="Q4">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="S4" t="s">
         <v>112</v>
@@ -1118,10 +1118,10 @@
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R5">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S5" t="s">
         <v>112</v>
@@ -1189,10 +1189,10 @@
         <v>46214</v>
       </c>
       <c r="Q6">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S6" t="s">
         <v>112</v>
@@ -1257,10 +1257,10 @@
         <v>46214</v>
       </c>
       <c r="Q7">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="R7">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S7" t="s">
         <v>112</v>
@@ -1322,10 +1322,10 @@
         <v>46311</v>
       </c>
       <c r="Q8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R8">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S8" t="s">
         <v>112</v>
@@ -1390,10 +1390,10 @@
         <v>46310</v>
       </c>
       <c r="Q9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S9" t="s">
         <v>112</v>
@@ -1458,10 +1458,10 @@
         <v>46316</v>
       </c>
       <c r="Q10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S10" t="s">
         <v>112</v>
@@ -1523,10 +1523,10 @@
         <v>46316</v>
       </c>
       <c r="Q11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S11" t="s">
         <v>112</v>
@@ -1591,10 +1591,10 @@
         <v>46316</v>
       </c>
       <c r="Q12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S12" t="s">
         <v>112</v>
@@ -1656,10 +1656,10 @@
         <v>46340</v>
       </c>
       <c r="Q13">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="R13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S13" t="s">
         <v>112</v>
@@ -1724,10 +1724,10 @@
         <v>46327</v>
       </c>
       <c r="Q14">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="R14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T14" t="s">
         <v>113</v>
@@ -1786,10 +1786,10 @@
         <v>46322</v>
       </c>
       <c r="Q15">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S15" t="s">
         <v>112</v>
@@ -1851,10 +1851,10 @@
         <v>46322</v>
       </c>
       <c r="Q16">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S16" t="s">
         <v>112</v>
@@ -1919,10 +1919,10 @@
         <v>46346</v>
       </c>
       <c r="Q17">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S17" t="s">
         <v>112</v>
@@ -1981,10 +1981,10 @@
         <v>46346</v>
       </c>
       <c r="Q18">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S18" t="s">
         <v>112</v>
@@ -2043,10 +2043,10 @@
         <v>46326</v>
       </c>
       <c r="Q19">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S19" t="s">
         <v>112</v>
@@ -2105,10 +2105,10 @@
         <v>46326</v>
       </c>
       <c r="Q20">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R20">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S20" t="s">
         <v>112</v>
@@ -2173,10 +2173,10 @@
         <v>46346</v>
       </c>
       <c r="Q21">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S21" t="s">
         <v>112</v>
@@ -2241,10 +2241,10 @@
         <v>46346</v>
       </c>
       <c r="Q22">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="R22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S22" t="s">
         <v>112</v>
@@ -2309,10 +2309,10 @@
         <v>46326</v>
       </c>
       <c r="Q23">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S23" t="s">
         <v>113</v>
@@ -2377,10 +2377,10 @@
         <v>46323</v>
       </c>
       <c r="Q24">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S24" t="s">
         <v>112</v>
@@ -2439,10 +2439,10 @@
         <v>46324</v>
       </c>
       <c r="Q25">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S25" t="s">
         <v>112</v>
@@ -2501,10 +2501,10 @@
         <v>46324</v>
       </c>
       <c r="Q26">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S26" t="s">
         <v>113</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (23/10/2026 14:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -455,8 +455,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -472,7 +480,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -480,12 +488,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -785,85 +811,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -895,10 +921,10 @@
       <c r="I2" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="2">
         <v>46251</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -907,7 +933,7 @@
       <c r="M2" t="s">
         <v>111</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>46280</v>
       </c>
       <c r="Q2">
@@ -963,10 +989,10 @@
       <c r="I3" t="s">
         <v>108</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="2">
         <v>46294</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -975,10 +1001,10 @@
       <c r="M3" t="s">
         <v>111</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>46326</v>
       </c>
-      <c r="O3" s="1">
+      <c r="O3" s="2">
         <v>46326</v>
       </c>
       <c r="Q3">
@@ -1031,10 +1057,10 @@
       <c r="I4" t="s">
         <v>108</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>46294</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -1043,10 +1069,10 @@
       <c r="M4" t="s">
         <v>111</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>46326</v>
       </c>
-      <c r="O4" s="1">
+      <c r="O4" s="2">
         <v>46305</v>
       </c>
       <c r="Q4">
@@ -1102,10 +1128,10 @@
       <c r="I5" t="s">
         <v>108</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="2">
         <v>46296</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1114,7 +1140,7 @@
       <c r="M5" t="s">
         <v>111</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>46327</v>
       </c>
       <c r="Q5">
@@ -1170,10 +1196,10 @@
       <c r="I6" t="s">
         <v>108</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="2">
         <v>46301</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1182,10 +1208,10 @@
       <c r="M6" t="s">
         <v>111</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>46333</v>
       </c>
-      <c r="O6" s="1">
+      <c r="O6" s="2">
         <v>46214</v>
       </c>
       <c r="Q6">
@@ -1238,10 +1264,10 @@
       <c r="I7" t="s">
         <v>108</v>
       </c>
-      <c r="J7" s="1">
+      <c r="J7" s="2">
         <v>46302</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1250,10 +1276,10 @@
       <c r="M7" t="s">
         <v>111</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>46333</v>
       </c>
-      <c r="O7" s="1">
+      <c r="O7" s="2">
         <v>46214</v>
       </c>
       <c r="Q7">
@@ -1306,10 +1332,10 @@
       <c r="I8" t="s">
         <v>109</v>
       </c>
-      <c r="J8" s="1">
+      <c r="J8" s="2">
         <v>46304</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1318,7 +1344,7 @@
       <c r="M8" t="s">
         <v>111</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>46311</v>
       </c>
       <c r="Q8">
@@ -1371,10 +1397,10 @@
       <c r="I9" t="s">
         <v>110</v>
       </c>
-      <c r="J9" s="1">
+      <c r="J9" s="2">
         <v>46303</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1383,10 +1409,10 @@
       <c r="M9" t="s">
         <v>111</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>46315</v>
       </c>
-      <c r="O9" s="1">
+      <c r="O9" s="2">
         <v>46310</v>
       </c>
       <c r="Q9">
@@ -1442,10 +1468,10 @@
       <c r="I10" t="s">
         <v>109</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10" s="2">
         <v>46308</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>46309</v>
       </c>
       <c r="L10">
@@ -1454,7 +1480,7 @@
       <c r="M10" t="s">
         <v>111</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>46316</v>
       </c>
       <c r="Q10">
@@ -1507,10 +1533,10 @@
       <c r="I11" t="s">
         <v>109</v>
       </c>
-      <c r="J11" s="1">
+      <c r="J11" s="2">
         <v>46308</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>46309</v>
       </c>
       <c r="L11">
@@ -1519,7 +1545,7 @@
       <c r="M11" t="s">
         <v>111</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>46316</v>
       </c>
       <c r="Q11">
@@ -1575,10 +1601,10 @@
       <c r="I12" t="s">
         <v>109</v>
       </c>
-      <c r="J12" s="1">
+      <c r="J12" s="2">
         <v>46309</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>46309</v>
       </c>
       <c r="L12">
@@ -1587,7 +1613,7 @@
       <c r="M12" t="s">
         <v>111</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46316</v>
       </c>
       <c r="Q12">
@@ -1640,10 +1666,10 @@
       <c r="I13" t="s">
         <v>108</v>
       </c>
-      <c r="J13" s="1">
+      <c r="J13" s="2">
         <v>46308</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>46309</v>
       </c>
       <c r="L13">
@@ -1652,7 +1678,7 @@
       <c r="M13" t="s">
         <v>111</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="2">
         <v>46340</v>
       </c>
       <c r="Q13">
@@ -1708,10 +1734,10 @@
       <c r="I14" t="s">
         <v>110</v>
       </c>
-      <c r="J14" s="1">
+      <c r="J14" s="2">
         <v>46309</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>46316</v>
       </c>
       <c r="L14">
@@ -1720,7 +1746,7 @@
       <c r="M14" t="s">
         <v>111</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="2">
         <v>46327</v>
       </c>
       <c r="Q14">
@@ -1770,10 +1796,10 @@
       <c r="I15" t="s">
         <v>109</v>
       </c>
-      <c r="J15" s="1">
+      <c r="J15" s="2">
         <v>46310</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>46315</v>
       </c>
       <c r="L15">
@@ -1782,7 +1808,7 @@
       <c r="M15" t="s">
         <v>111</v>
       </c>
-      <c r="N15" s="1">
+      <c r="N15" s="2">
         <v>46322</v>
       </c>
       <c r="Q15">
@@ -1835,10 +1861,10 @@
       <c r="I16" t="s">
         <v>109</v>
       </c>
-      <c r="J16" s="1">
+      <c r="J16" s="2">
         <v>46310</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>46315</v>
       </c>
       <c r="L16">
@@ -1847,7 +1873,7 @@
       <c r="M16" t="s">
         <v>111</v>
       </c>
-      <c r="N16" s="1">
+      <c r="N16" s="2">
         <v>46322</v>
       </c>
       <c r="Q16">
@@ -1903,10 +1929,10 @@
       <c r="I17" t="s">
         <v>108</v>
       </c>
-      <c r="J17" s="1">
+      <c r="J17" s="2">
         <v>46310</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>46315</v>
       </c>
       <c r="L17">
@@ -1915,7 +1941,7 @@
       <c r="M17" t="s">
         <v>111</v>
       </c>
-      <c r="N17" s="1">
+      <c r="N17" s="2">
         <v>46346</v>
       </c>
       <c r="Q17">
@@ -1965,10 +1991,10 @@
       <c r="I18" t="s">
         <v>108</v>
       </c>
-      <c r="J18" s="1">
+      <c r="J18" s="2">
         <v>46310</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>46315</v>
       </c>
       <c r="L18">
@@ -1977,7 +2003,7 @@
       <c r="M18" t="s">
         <v>111</v>
       </c>
-      <c r="N18" s="1">
+      <c r="N18" s="2">
         <v>46346</v>
       </c>
       <c r="Q18">
@@ -2027,10 +2053,10 @@
       <c r="I19" t="s">
         <v>110</v>
       </c>
-      <c r="J19" s="1">
+      <c r="J19" s="2">
         <v>46311</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>46315</v>
       </c>
       <c r="L19">
@@ -2039,7 +2065,7 @@
       <c r="M19" t="s">
         <v>111</v>
       </c>
-      <c r="N19" s="1">
+      <c r="N19" s="2">
         <v>46326</v>
       </c>
       <c r="Q19">
@@ -2089,10 +2115,10 @@
       <c r="I20" t="s">
         <v>110</v>
       </c>
-      <c r="J20" s="1">
+      <c r="J20" s="2">
         <v>46311</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>46315</v>
       </c>
       <c r="L20">
@@ -2101,7 +2127,7 @@
       <c r="M20" t="s">
         <v>111</v>
       </c>
-      <c r="N20" s="1">
+      <c r="N20" s="2">
         <v>46326</v>
       </c>
       <c r="Q20">
@@ -2157,10 +2183,10 @@
       <c r="I21" t="s">
         <v>108</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J21" s="2">
         <v>46311</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>46315</v>
       </c>
       <c r="L21">
@@ -2169,7 +2195,7 @@
       <c r="M21" t="s">
         <v>111</v>
       </c>
-      <c r="N21" s="1">
+      <c r="N21" s="2">
         <v>46346</v>
       </c>
       <c r="Q21">
@@ -2225,10 +2251,10 @@
       <c r="I22" t="s">
         <v>108</v>
       </c>
-      <c r="J22" s="1">
+      <c r="J22" s="2">
         <v>46311</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>46315</v>
       </c>
       <c r="L22">
@@ -2237,7 +2263,7 @@
       <c r="M22" t="s">
         <v>111</v>
       </c>
-      <c r="N22" s="1">
+      <c r="N22" s="2">
         <v>46346</v>
       </c>
       <c r="Q22">
@@ -2293,10 +2319,10 @@
       <c r="I23" t="s">
         <v>110</v>
       </c>
-      <c r="J23" s="1">
+      <c r="J23" s="2">
         <v>46315</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>46315</v>
       </c>
       <c r="L23">
@@ -2305,7 +2331,7 @@
       <c r="M23" t="s">
         <v>111</v>
       </c>
-      <c r="N23" s="1">
+      <c r="N23" s="2">
         <v>46326</v>
       </c>
       <c r="Q23">
@@ -2361,10 +2387,10 @@
       <c r="I24" t="s">
         <v>109</v>
       </c>
-      <c r="J24" s="1">
+      <c r="J24" s="2">
         <v>46315</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>46316</v>
       </c>
       <c r="L24">
@@ -2373,7 +2399,7 @@
       <c r="M24" t="s">
         <v>111</v>
       </c>
-      <c r="N24" s="1">
+      <c r="N24" s="2">
         <v>46323</v>
       </c>
       <c r="Q24">
@@ -2423,10 +2449,10 @@
       <c r="I25" t="s">
         <v>109</v>
       </c>
-      <c r="J25" s="1">
+      <c r="J25" s="2">
         <v>46316</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>46317</v>
       </c>
       <c r="L25">
@@ -2435,7 +2461,7 @@
       <c r="M25" t="s">
         <v>111</v>
       </c>
-      <c r="N25" s="1">
+      <c r="N25" s="2">
         <v>46324</v>
       </c>
       <c r="Q25">
@@ -2485,10 +2511,10 @@
       <c r="I26" t="s">
         <v>109</v>
       </c>
-      <c r="J26" s="1">
+      <c r="J26" s="2">
         <v>46316</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>46317</v>
       </c>
       <c r="L26">
@@ -2497,7 +2523,7 @@
       <c r="M26" t="s">
         <v>111</v>
       </c>
-      <c r="N26" s="1">
+      <c r="N26" s="2">
         <v>46324</v>
       </c>
       <c r="Q26">

</xml_diff>

<commit_message>
Atualização automática: emergencias (26/10/2026 14:17)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -455,16 +455,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -480,7 +472,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -488,30 +480,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -811,85 +785,85 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -921,10 +895,10 @@
       <c r="I2" t="s">
         <v>108</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>46251</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>46249</v>
       </c>
       <c r="L2">
@@ -933,14 +907,14 @@
       <c r="M2" t="s">
         <v>111</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="R2">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="S2" t="s">
         <v>112</v>
@@ -989,10 +963,10 @@
       <c r="I3" t="s">
         <v>108</v>
       </c>
-      <c r="J3" s="2">
+      <c r="J3" s="1">
         <v>46294</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>46295</v>
       </c>
       <c r="L3">
@@ -1001,17 +975,17 @@
       <c r="M3" t="s">
         <v>111</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="1">
         <v>46326</v>
       </c>
-      <c r="O3" s="2">
+      <c r="O3" s="1">
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R3">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="S3" t="s">
         <v>112</v>
@@ -1057,10 +1031,10 @@
       <c r="I4" t="s">
         <v>108</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>46294</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>46295</v>
       </c>
       <c r="L4">
@@ -1069,17 +1043,17 @@
       <c r="M4" t="s">
         <v>111</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="1">
         <v>46326</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4" s="1">
         <v>46305</v>
       </c>
       <c r="Q4">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R4">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="S4" t="s">
         <v>112</v>
@@ -1128,10 +1102,10 @@
       <c r="I5" t="s">
         <v>108</v>
       </c>
-      <c r="J5" s="2">
+      <c r="J5" s="1">
         <v>46296</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>46296</v>
       </c>
       <c r="L5">
@@ -1140,14 +1114,14 @@
       <c r="M5" t="s">
         <v>111</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R5">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="S5" t="s">
         <v>112</v>
@@ -1196,10 +1170,10 @@
       <c r="I6" t="s">
         <v>108</v>
       </c>
-      <c r="J6" s="2">
+      <c r="J6" s="1">
         <v>46301</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>46302</v>
       </c>
       <c r="L6">
@@ -1208,17 +1182,17 @@
       <c r="M6" t="s">
         <v>111</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="1">
         <v>46333</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="1">
         <v>46214</v>
       </c>
       <c r="Q6">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="R6">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S6" t="s">
         <v>112</v>
@@ -1264,10 +1238,10 @@
       <c r="I7" t="s">
         <v>108</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>46302</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>46302</v>
       </c>
       <c r="L7">
@@ -1276,17 +1250,17 @@
       <c r="M7" t="s">
         <v>111</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="1">
         <v>46333</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="1">
         <v>46214</v>
       </c>
       <c r="Q7">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="R7">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="S7" t="s">
         <v>112</v>
@@ -1332,10 +1306,10 @@
       <c r="I8" t="s">
         <v>109</v>
       </c>
-      <c r="J8" s="2">
+      <c r="J8" s="1">
         <v>46304</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>46304</v>
       </c>
       <c r="L8">
@@ -1344,14 +1318,14 @@
       <c r="M8" t="s">
         <v>111</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="1">
         <v>46311</v>
       </c>
       <c r="Q8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="R8">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S8" t="s">
         <v>112</v>
@@ -1397,10 +1371,10 @@
       <c r="I9" t="s">
         <v>110</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="1">
         <v>46303</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>46304</v>
       </c>
       <c r="L9">
@@ -1409,17 +1383,17 @@
       <c r="M9" t="s">
         <v>111</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="1">
         <v>46315</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9" s="1">
         <v>46310</v>
       </c>
       <c r="Q9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R9">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S9" t="s">
         <v>112</v>
@@ -1468,10 +1442,10 @@
       <c r="I10" t="s">
         <v>109</v>
       </c>
-      <c r="J10" s="2">
+      <c r="J10" s="1">
         <v>46308</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>46309</v>
       </c>
       <c r="L10">
@@ -1480,14 +1454,14 @@
       <c r="M10" t="s">
         <v>111</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="1">
         <v>46316</v>
       </c>
       <c r="Q10">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R10">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S10" t="s">
         <v>112</v>
@@ -1533,10 +1507,10 @@
       <c r="I11" t="s">
         <v>109</v>
       </c>
-      <c r="J11" s="2">
+      <c r="J11" s="1">
         <v>46308</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>46309</v>
       </c>
       <c r="L11">
@@ -1545,14 +1519,14 @@
       <c r="M11" t="s">
         <v>111</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="1">
         <v>46316</v>
       </c>
       <c r="Q11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S11" t="s">
         <v>112</v>
@@ -1601,10 +1575,10 @@
       <c r="I12" t="s">
         <v>109</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J12" s="1">
         <v>46309</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>46309</v>
       </c>
       <c r="L12">
@@ -1613,14 +1587,14 @@
       <c r="M12" t="s">
         <v>111</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="1">
         <v>46316</v>
       </c>
       <c r="Q12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R12">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S12" t="s">
         <v>112</v>
@@ -1666,10 +1640,10 @@
       <c r="I13" t="s">
         <v>108</v>
       </c>
-      <c r="J13" s="2">
+      <c r="J13" s="1">
         <v>46308</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>46309</v>
       </c>
       <c r="L13">
@@ -1678,14 +1652,14 @@
       <c r="M13" t="s">
         <v>111</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="1">
         <v>46340</v>
       </c>
       <c r="Q13">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="R13">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="S13" t="s">
         <v>112</v>
@@ -1734,10 +1708,10 @@
       <c r="I14" t="s">
         <v>110</v>
       </c>
-      <c r="J14" s="2">
+      <c r="J14" s="1">
         <v>46309</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>46316</v>
       </c>
       <c r="L14">
@@ -1746,14 +1720,14 @@
       <c r="M14" t="s">
         <v>111</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14" s="1">
         <v>46327</v>
       </c>
       <c r="Q14">
-        <v>-9</v>
+        <v>-6</v>
       </c>
       <c r="R14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T14" t="s">
         <v>113</v>
@@ -1796,10 +1770,10 @@
       <c r="I15" t="s">
         <v>109</v>
       </c>
-      <c r="J15" s="2">
+      <c r="J15" s="1">
         <v>46310</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>46315</v>
       </c>
       <c r="L15">
@@ -1808,14 +1782,14 @@
       <c r="M15" t="s">
         <v>111</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15" s="1">
         <v>46322</v>
       </c>
       <c r="Q15">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R15">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S15" t="s">
         <v>112</v>
@@ -1861,10 +1835,10 @@
       <c r="I16" t="s">
         <v>109</v>
       </c>
-      <c r="J16" s="2">
+      <c r="J16" s="1">
         <v>46310</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>46315</v>
       </c>
       <c r="L16">
@@ -1873,14 +1847,14 @@
       <c r="M16" t="s">
         <v>111</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16" s="1">
         <v>46322</v>
       </c>
       <c r="Q16">
-        <v>-4</v>
+        <v>-1</v>
       </c>
       <c r="R16">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S16" t="s">
         <v>112</v>
@@ -1929,10 +1903,10 @@
       <c r="I17" t="s">
         <v>108</v>
       </c>
-      <c r="J17" s="2">
+      <c r="J17" s="1">
         <v>46310</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>46315</v>
       </c>
       <c r="L17">
@@ -1941,14 +1915,14 @@
       <c r="M17" t="s">
         <v>111</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17" s="1">
         <v>46346</v>
       </c>
       <c r="Q17">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R17">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S17" t="s">
         <v>112</v>
@@ -1991,10 +1965,10 @@
       <c r="I18" t="s">
         <v>108</v>
       </c>
-      <c r="J18" s="2">
+      <c r="J18" s="1">
         <v>46310</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>46315</v>
       </c>
       <c r="L18">
@@ -2003,14 +1977,14 @@
       <c r="M18" t="s">
         <v>111</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18" s="1">
         <v>46346</v>
       </c>
       <c r="Q18">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R18">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S18" t="s">
         <v>112</v>
@@ -2053,10 +2027,10 @@
       <c r="I19" t="s">
         <v>110</v>
       </c>
-      <c r="J19" s="2">
+      <c r="J19" s="1">
         <v>46311</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>46315</v>
       </c>
       <c r="L19">
@@ -2065,14 +2039,14 @@
       <c r="M19" t="s">
         <v>111</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19" s="1">
         <v>46326</v>
       </c>
       <c r="Q19">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R19">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S19" t="s">
         <v>112</v>
@@ -2115,10 +2089,10 @@
       <c r="I20" t="s">
         <v>110</v>
       </c>
-      <c r="J20" s="2">
+      <c r="J20" s="1">
         <v>46311</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>46315</v>
       </c>
       <c r="L20">
@@ -2127,14 +2101,14 @@
       <c r="M20" t="s">
         <v>111</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20" s="1">
         <v>46326</v>
       </c>
       <c r="Q20">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R20">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S20" t="s">
         <v>112</v>
@@ -2183,10 +2157,10 @@
       <c r="I21" t="s">
         <v>108</v>
       </c>
-      <c r="J21" s="2">
+      <c r="J21" s="1">
         <v>46311</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>46315</v>
       </c>
       <c r="L21">
@@ -2195,14 +2169,14 @@
       <c r="M21" t="s">
         <v>111</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21" s="1">
         <v>46346</v>
       </c>
       <c r="Q21">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R21">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S21" t="s">
         <v>112</v>
@@ -2251,10 +2225,10 @@
       <c r="I22" t="s">
         <v>108</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="1">
         <v>46311</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>46315</v>
       </c>
       <c r="L22">
@@ -2263,14 +2237,14 @@
       <c r="M22" t="s">
         <v>111</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22" s="1">
         <v>46346</v>
       </c>
       <c r="Q22">
-        <v>-28</v>
+        <v>-25</v>
       </c>
       <c r="R22">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S22" t="s">
         <v>112</v>
@@ -2319,10 +2293,10 @@
       <c r="I23" t="s">
         <v>110</v>
       </c>
-      <c r="J23" s="2">
+      <c r="J23" s="1">
         <v>46315</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>46315</v>
       </c>
       <c r="L23">
@@ -2331,14 +2305,14 @@
       <c r="M23" t="s">
         <v>111</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23" s="1">
         <v>46326</v>
       </c>
       <c r="Q23">
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="R23">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="S23" t="s">
         <v>113</v>
@@ -2387,10 +2361,10 @@
       <c r="I24" t="s">
         <v>109</v>
       </c>
-      <c r="J24" s="2">
+      <c r="J24" s="1">
         <v>46315</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>46316</v>
       </c>
       <c r="L24">
@@ -2399,14 +2373,14 @@
       <c r="M24" t="s">
         <v>111</v>
       </c>
-      <c r="N24" s="2">
+      <c r="N24" s="1">
         <v>46323</v>
       </c>
       <c r="Q24">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="R24">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S24" t="s">
         <v>112</v>
@@ -2449,10 +2423,10 @@
       <c r="I25" t="s">
         <v>109</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="1">
         <v>46316</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>46317</v>
       </c>
       <c r="L25">
@@ -2461,14 +2435,14 @@
       <c r="M25" t="s">
         <v>111</v>
       </c>
-      <c r="N25" s="2">
+      <c r="N25" s="1">
         <v>46324</v>
       </c>
       <c r="Q25">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="R25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S25" t="s">
         <v>112</v>
@@ -2511,10 +2485,10 @@
       <c r="I26" t="s">
         <v>109</v>
       </c>
-      <c r="J26" s="2">
+      <c r="J26" s="1">
         <v>46316</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>46317</v>
       </c>
       <c r="L26">
@@ -2523,14 +2497,14 @@
       <c r="M26" t="s">
         <v>111</v>
       </c>
-      <c r="N26" s="2">
+      <c r="N26" s="1">
         <v>46324</v>
       </c>
       <c r="Q26">
-        <v>-6</v>
+        <v>-3</v>
       </c>
       <c r="R26">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S26" t="s">
         <v>113</v>

</xml_diff>

<commit_message>
Atualização automática: emergencias (27/10/2026 13:26)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="137">
   <si>
     <t>om_emg</t>
   </si>
@@ -139,18 +139,6 @@
     <t>685260012964</t>
   </si>
   <si>
-    <t>329260019318</t>
-  </si>
-  <si>
-    <t>329260019319</t>
-  </si>
-  <si>
-    <t>396260016644</t>
-  </si>
-  <si>
-    <t>685260012971</t>
-  </si>
-  <si>
     <t>313260019100</t>
   </si>
   <si>
@@ -169,9 +157,6 @@
     <t>685260012993</t>
   </si>
   <si>
-    <t>685260012994</t>
-  </si>
-  <si>
     <t>685260012995</t>
   </si>
   <si>
@@ -181,15 +166,27 @@
     <t>685260012998</t>
   </si>
   <si>
-    <t>396260016650</t>
-  </si>
-  <si>
     <t>329260019334</t>
   </si>
   <si>
     <t>329260019335</t>
   </si>
   <si>
+    <t>313260019118</t>
+  </si>
+  <si>
+    <t>685260013019</t>
+  </si>
+  <si>
+    <t>685260013020</t>
+  </si>
+  <si>
+    <t>685260013035</t>
+  </si>
+  <si>
+    <t>685260013047</t>
+  </si>
+  <si>
     <t>040-0043</t>
   </si>
   <si>
@@ -214,18 +211,6 @@
     <t>103-20400</t>
   </si>
   <si>
-    <t>9910592-2</t>
-  </si>
-  <si>
-    <t>C611008-0101</t>
-  </si>
-  <si>
-    <t>3244809-4</t>
-  </si>
-  <si>
-    <t>066-3046-01</t>
-  </si>
-  <si>
     <t>011-00870-00</t>
   </si>
   <si>
@@ -238,24 +223,33 @@
     <t>2641014-9</t>
   </si>
   <si>
-    <t>2641010-7</t>
-  </si>
-  <si>
     <t>324843-W020</t>
   </si>
   <si>
     <t>MS21043-3</t>
   </si>
   <si>
-    <t>2643100-201</t>
-  </si>
-  <si>
     <t>030-02178-0000</t>
   </si>
   <si>
     <t>C660501-0102</t>
   </si>
   <si>
+    <t>2682004-1</t>
+  </si>
+  <si>
+    <t>066-4010-12</t>
+  </si>
+  <si>
+    <t>2522179-1</t>
+  </si>
+  <si>
+    <t>071-1242-06</t>
+  </si>
+  <si>
+    <t>C668050-1103</t>
+  </si>
+  <si>
     <t>STROB TUB</t>
   </si>
   <si>
@@ -280,18 +274,6 @@
     <t>BOLT,MACHINE</t>
   </si>
   <si>
-    <t>ALTERNADOR</t>
-  </si>
-  <si>
-    <t>ALTERNATOR CONTROL U</t>
-  </si>
-  <si>
-    <t>FUEL CONTROL,MAIN,TU</t>
-  </si>
-  <si>
-    <t>CONTROL,INDICATOR</t>
-  </si>
-  <si>
     <t>MAGNETOMETER GMU 44</t>
   </si>
   <si>
@@ -304,24 +286,33 @@
     <t>SPRING ASSY-MAIN GEA</t>
   </si>
   <si>
-    <t>AXLE FITTING</t>
-  </si>
-  <si>
     <t>HEADSET-MICROPHONE</t>
   </si>
   <si>
     <t>NUT,SELF-LOCKING,EXT</t>
   </si>
   <si>
-    <t>NOSE GEAR STRUT ASSY</t>
-  </si>
-  <si>
     <t>CONNECTOR,ELECTRICAL</t>
   </si>
   <si>
     <t>COMPASS ASSY</t>
   </si>
   <si>
+    <t>RESERVOIR ASSY-BRAKE</t>
+  </si>
+  <si>
+    <t>RECEIVER VOR/LOC (KN</t>
+  </si>
+  <si>
+    <t>ROD ASSEMBLY</t>
+  </si>
+  <si>
+    <t>SLAVING ACCESS,SPEC</t>
+  </si>
+  <si>
+    <t>TRANSMITER FUEL</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -334,12 +325,12 @@
     <t>Providência tomada</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
-    <t>Expedido total</t>
-  </si>
-  <si>
     <t>ANCE</t>
   </si>
   <si>
@@ -370,21 +361,12 @@
     <t>Recibo 887/FAB/26 AWB 127-6307 3301 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
   </si>
   <si>
-    <t>AWB 127-6350 4696 retirado por Jader Dantas, recebedor desconhecido. Ramon 22/10/26.</t>
-  </si>
-  <si>
-    <t>AWB 127-6350 5142 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
-  </si>
-  <si>
     <t>Cedeu o item para o C-98 2736. Ramon 21/10.</t>
   </si>
   <si>
     <t>Atendido com estoque local em 21/10. Agd AWB 127-6466 1855 com previsão de entrega em 24/10. Ramon 22/10</t>
   </si>
   <si>
-    <t>Atendido com estoque local em 21/10. AWB 127-6465 9825 com previsão de entrega em 23/10. Ramon 22/10/26</t>
-  </si>
-  <si>
     <t>Autorizado reparo de fones do A7 para posterior mudança para U8. Ramon 22/10</t>
   </si>
   <si>
@@ -394,7 +376,10 @@
     <t>Estoque do PN superador. Ramon 22/10</t>
   </si>
   <si>
-    <t>ESTE ITEM FOI ENVIADO POR ENGANO PARA BAMN. ESTAMOS RESGATANDO O ITEM PARA ENVIAR DE VOLTA AO FORNECEDOR PARA QUE ELE NOS ENVIE O ITEM CORRETO.</t>
+    <t>Cedeu o item para o 2738. Ramon 27/10/26</t>
+  </si>
+  <si>
+    <t>Colocado o pedido junto ao fornecedor AEROTECHNIC e WAGA INTERNATIONAL. Em processo de envio para a AGS Miami. ATZ 22/10</t>
   </si>
   <si>
     <t>Enviados 02 ea para reparo em 09/10/2026 - REZ - Ag orçamento</t>
@@ -406,43 +391,37 @@
     <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26 .Segundo informações do Ten Soares do CLA não é preciso a compra do compressor no monento.(19/10/26 (SO R1 Bispo)</t>
   </si>
   <si>
-    <t>Abertas OS para 03 ea dia 07/10.Material coletado dia 09/10 fins reparo - AGD orçamento - REZ</t>
+    <t>Abertas OS para 03 ea dia 07/10.Material coletado dia 09/10 fins reparo - AGD orçamento - REZ MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE</t>
   </si>
   <si>
     <t>Colocado pedido Textron IJ17796997 - chegada GIG 14/10 (voo 4588) em desembaraço - Material aguardando a documentação da Textron, pois não veio com o material 20/10/26. Solicitado abertura de Os para 01 ea em 07/10/2026 para fazer o envio a Textron por ser unidade como CORE -REZ</t>
   </si>
   <si>
-    <t>abertas OS de 03 ea em 09/10/2026.REZ</t>
+    <t>abertas OS de 03 ea em 09/10/2026.REZ - Material enviado via recibo 912/FAB/26, AWB 12764844850 DPE 23/10/26</t>
   </si>
   <si>
     <t>Colocado pedido Textron WB0003180334 - previsão de entrega no RJ 13/10 - MATERIAL RECEBIDO EM RJ 13/10 - PREPARANDO ENVIO 13/10 - recibo 887/FAB/26 AWB 12763073301 DPE 16/10/2026 - MATERIAL ENTREGUE DIA 15/10/2026</t>
   </si>
   <si>
-    <t>04 ea em reparo na William e 02 ea na Av aeronáutica. Solicitado apressamento e DPE para ambas as empresas em 15/10/26 - REZ</t>
-  </si>
-  <si>
-    <t>Há no estq V1/LS para atender. Será enviado dia 15/10/26 para o Operador - REZ - AWB 127-6350 4696</t>
-  </si>
-  <si>
-    <t>FCU enviada de Belém para RJ AWB 12763294361, disponível para retirada dia 15/10/2026 - Material enviado para a oficina, já em bancada realizando testes finais - 20/10/2026 - MATERIAL ENVIADO VIA RECIBO 911/FAB/26 - AWB A SER GERADA PELA GOLLOG RC 21-10-26</t>
-  </si>
-  <si>
-    <t>Há no estq V1/LS para atender. Será enviado dia 15/10/26 para o Operador - REZ- --AWB 127-6350 5142</t>
-  </si>
-  <si>
     <t>Colocado pedido I837605 - entregue 02ea em Miami 21/10</t>
   </si>
   <si>
-    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , PELO PN ALTERNADO MS20007-70. - RC 20/10/2026</t>
-  </si>
-  <si>
-    <t>01 EA SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA".- RC 20/10/2026 01 EA ENVIADO PELO RECIBO 907/FAB/26, AWB A SER GERADA PELA GOLLOG RC 20/10/2026</t>
+    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , PELO PN ALTERNADO MS20007-70. - RC 20/10/2026 - AWB 127-6466 1855</t>
+  </si>
+  <si>
+    <t>MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE</t>
+  </si>
+  <si>
+    <t>Foi solicitado via Email no dia 20/10/26 o core para revisão. Aguardando resposta.</t>
   </si>
   <si>
     <t>SOLICITAMOS OS CORES PARA REALIZAR REPARO, TENDO EM VISTA QUE NÃO TEMOS NO TSAM PARA RECOLHIMENTO. RC 20/10/2026</t>
   </si>
   <si>
-    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , - RC 20/10/2026</t>
+    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , - RC 20/10/2026 - AWB ENVIADA 12764659825</t>
+  </si>
+  <si>
+    <t>MATERIAL ENVIADO VIA AWB 12764891315, DISPONIVEL PARA RETIRADA DIA 23/10.</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -781,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA26"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -878,22 +857,22 @@
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
+        <v>102</v>
+      </c>
+      <c r="I2" t="s">
         <v>105</v>
-      </c>
-      <c r="I2" t="s">
-        <v>108</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -905,31 +884,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="R2">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="S2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="U2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="V2" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="W2" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -946,22 +925,22 @@
         <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G3">
         <v>2703</v>
       </c>
       <c r="H3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I3" t="s">
         <v>105</v>
-      </c>
-      <c r="I3" t="s">
-        <v>108</v>
       </c>
       <c r="J3" s="1">
         <v>46294</v>
@@ -973,7 +952,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N3" s="1">
         <v>46326</v>
@@ -982,22 +961,22 @@
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R3">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="V3" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="W3" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -1014,22 +993,22 @@
         <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G4">
         <v>2703</v>
       </c>
       <c r="H4" t="s">
+        <v>102</v>
+      </c>
+      <c r="I4" t="s">
         <v>105</v>
-      </c>
-      <c r="I4" t="s">
-        <v>108</v>
       </c>
       <c r="J4" s="1">
         <v>46294</v>
@@ -1041,7 +1020,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N4" s="1">
         <v>46326</v>
@@ -1050,25 +1029,25 @@
         <v>46305</v>
       </c>
       <c r="Q4">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R4">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S4" t="s">
+        <v>109</v>
+      </c>
+      <c r="T4" t="s">
+        <v>110</v>
+      </c>
+      <c r="U4" t="s">
         <v>112</v>
       </c>
-      <c r="T4" t="s">
-        <v>113</v>
-      </c>
-      <c r="U4" t="s">
-        <v>115</v>
-      </c>
       <c r="V4" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="W4" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1085,22 +1064,22 @@
         <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G5">
         <v>2723</v>
       </c>
       <c r="H5" t="s">
+        <v>102</v>
+      </c>
+      <c r="I5" t="s">
         <v>105</v>
-      </c>
-      <c r="I5" t="s">
-        <v>108</v>
       </c>
       <c r="J5" s="1">
         <v>46296</v>
@@ -1112,31 +1091,31 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R5">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="U5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="V5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="W5" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1153,22 +1132,22 @@
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G6">
         <v>2708</v>
       </c>
       <c r="H6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I6" t="s">
         <v>105</v>
-      </c>
-      <c r="I6" t="s">
-        <v>108</v>
       </c>
       <c r="J6" s="1">
         <v>46301</v>
@@ -1180,7 +1159,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N6" s="1">
         <v>46333</v>
@@ -1189,22 +1168,22 @@
         <v>46214</v>
       </c>
       <c r="Q6">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R6">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="V6" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="W6" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1221,22 +1200,22 @@
         <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G7">
         <v>2742</v>
       </c>
       <c r="H7" t="s">
+        <v>102</v>
+      </c>
+      <c r="I7" t="s">
         <v>105</v>
-      </c>
-      <c r="I7" t="s">
-        <v>108</v>
       </c>
       <c r="J7" s="1">
         <v>46302</v>
@@ -1248,7 +1227,7 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N7" s="1">
         <v>46333</v>
@@ -1257,22 +1236,22 @@
         <v>46214</v>
       </c>
       <c r="Q7">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="R7">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="S7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T7" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="V7" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="W7" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1289,22 +1268,22 @@
         <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G8">
         <v>2721</v>
       </c>
       <c r="H8" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I8" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="J8" s="1">
         <v>46304</v>
@@ -1316,28 +1295,31 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N8" s="1">
         <v>46311</v>
       </c>
+      <c r="O8" s="1">
+        <v>46318</v>
+      </c>
       <c r="Q8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R8">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="V8" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="W8" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1354,22 +1336,22 @@
         <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G9">
         <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I9" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="J9" s="1">
         <v>46303</v>
@@ -1381,7 +1363,7 @@
         <v>12</v>
       </c>
       <c r="M9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N9" s="1">
         <v>46315</v>
@@ -1390,25 +1372,25 @@
         <v>46310</v>
       </c>
       <c r="Q9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S9" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T9" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="U9" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="V9" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="W9" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1416,64 +1398,61 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F10" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G10">
-        <v>2721</v>
+        <v>2730</v>
       </c>
       <c r="H10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J10" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K10" s="1">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N10" s="1">
-        <v>46316</v>
+        <v>46327</v>
       </c>
       <c r="Q10">
-        <v>5</v>
+        <v>-5</v>
       </c>
       <c r="R10">
-        <v>12</v>
-      </c>
-      <c r="S10" t="s">
-        <v>112</v>
+        <v>6</v>
       </c>
       <c r="T10" t="s">
-        <v>112</v>
-      </c>
-      <c r="V10" t="s">
-        <v>134</v>
+        <v>110</v>
+      </c>
+      <c r="U10" t="s">
+        <v>115</v>
       </c>
       <c r="W10" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1481,67 +1460,64 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F11" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G11">
-        <v>2721</v>
+        <v>2731</v>
       </c>
       <c r="H11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I11" t="s">
+        <v>106</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L11">
+        <v>4</v>
+      </c>
+      <c r="M11" t="s">
+        <v>108</v>
+      </c>
+      <c r="N11" s="1">
+        <v>46322</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>7</v>
+      </c>
+      <c r="S11" t="s">
         <v>109</v>
       </c>
-      <c r="J11" s="1">
-        <v>46308</v>
-      </c>
-      <c r="K11" s="1">
-        <v>46309</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11" t="s">
-        <v>111</v>
-      </c>
-      <c r="N11" s="1">
-        <v>46316</v>
-      </c>
-      <c r="Q11">
-        <v>5</v>
-      </c>
-      <c r="R11">
-        <v>12</v>
-      </c>
-      <c r="S11" t="s">
-        <v>112</v>
-      </c>
       <c r="T11" t="s">
-        <v>112</v>
-      </c>
-      <c r="U11" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="V11" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="W11" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1558,55 +1534,58 @@
         <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F12" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="G12">
         <v>2731</v>
       </c>
       <c r="H12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I12" t="s">
+        <v>106</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L12">
+        <v>2</v>
+      </c>
+      <c r="M12" t="s">
+        <v>108</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46322</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>7</v>
+      </c>
+      <c r="S12" t="s">
         <v>109</v>
       </c>
-      <c r="J12" s="1">
-        <v>46309</v>
-      </c>
-      <c r="K12" s="1">
-        <v>46309</v>
-      </c>
-      <c r="L12">
-        <v>1</v>
-      </c>
-      <c r="M12" t="s">
-        <v>111</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46316</v>
-      </c>
-      <c r="Q12">
-        <v>5</v>
-      </c>
-      <c r="R12">
-        <v>12</v>
-      </c>
-      <c r="S12" t="s">
-        <v>112</v>
-      </c>
       <c r="T12" t="s">
-        <v>113</v>
+        <v>110</v>
+      </c>
+      <c r="U12" t="s">
+        <v>116</v>
       </c>
       <c r="V12" t="s">
+        <v>130</v>
+      </c>
+      <c r="W12" t="s">
         <v>136</v>
-      </c>
-      <c r="W12" t="s">
-        <v>143</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1623,58 +1602,55 @@
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E13" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G13">
-        <v>2703</v>
+        <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I13" t="s">
+        <v>105</v>
+      </c>
+      <c r="J13" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13" t="s">
         <v>108</v>
       </c>
-      <c r="J13" s="1">
-        <v>46308</v>
-      </c>
-      <c r="K13" s="1">
-        <v>46309</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
-      </c>
-      <c r="M13" t="s">
-        <v>111</v>
-      </c>
       <c r="N13" s="1">
-        <v>46340</v>
+        <v>46346</v>
       </c>
       <c r="Q13">
-        <v>-19</v>
+        <v>-24</v>
       </c>
       <c r="R13">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="S13" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T13" t="s">
-        <v>113</v>
-      </c>
-      <c r="U13" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="V13" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="W13" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1682,61 +1658,64 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E14" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="F14" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G14">
-        <v>2730</v>
+        <v>2719</v>
       </c>
       <c r="H14" t="s">
+        <v>104</v>
+      </c>
+      <c r="I14" t="s">
         <v>105</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>108</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46346</v>
+      </c>
+      <c r="Q14">
+        <v>-24</v>
+      </c>
+      <c r="R14">
+        <v>7</v>
+      </c>
+      <c r="S14" t="s">
+        <v>109</v>
+      </c>
+      <c r="T14" t="s">
         <v>110</v>
       </c>
-      <c r="J14" s="1">
-        <v>46309</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46316</v>
-      </c>
-      <c r="L14">
-        <v>1</v>
-      </c>
-      <c r="M14" t="s">
-        <v>111</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46327</v>
-      </c>
-      <c r="Q14">
-        <v>-6</v>
-      </c>
-      <c r="R14">
-        <v>5</v>
-      </c>
-      <c r="T14" t="s">
-        <v>113</v>
-      </c>
-      <c r="U14" t="s">
-        <v>120</v>
+      <c r="V14" t="s">
+        <v>131</v>
       </c>
       <c r="W14" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1744,64 +1723,64 @@
     </row>
     <row r="15" spans="1:27">
       <c r="A15">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
         <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E15" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
+        <v>101</v>
+      </c>
+      <c r="G15">
+        <v>2722</v>
+      </c>
+      <c r="H15" t="s">
         <v>102</v>
       </c>
-      <c r="G15">
-        <v>2731</v>
-      </c>
-      <c r="H15" t="s">
-        <v>105</v>
-      </c>
       <c r="I15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J15" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="K15" s="1">
         <v>46315</v>
       </c>
       <c r="L15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N15" s="1">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="Q15">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="R15">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S15" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T15" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="V15" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="W15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1809,67 +1788,67 @@
     </row>
     <row r="16" spans="1:27">
       <c r="A16">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
         <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G16">
-        <v>2731</v>
+        <v>2722</v>
       </c>
       <c r="H16" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="J16" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="K16" s="1">
         <v>46315</v>
       </c>
       <c r="L16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M16" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N16" s="1">
-        <v>46322</v>
+        <v>46346</v>
       </c>
       <c r="Q16">
-        <v>-1</v>
+        <v>-24</v>
       </c>
       <c r="R16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S16" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T16" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="U16" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="V16" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="W16" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1886,52 +1865,58 @@
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G17">
-        <v>2702</v>
+        <v>2719</v>
       </c>
       <c r="H17" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I17" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="J17" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="K17" s="1">
         <v>46315</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M17" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N17" s="1">
         <v>46346</v>
       </c>
       <c r="Q17">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="R17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S17" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T17" t="s">
-        <v>113</v>
+        <v>110</v>
+      </c>
+      <c r="U17" t="s">
+        <v>117</v>
+      </c>
+      <c r="V17" t="s">
+        <v>133</v>
       </c>
       <c r="W17" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1948,52 +1933,61 @@
         <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="F18" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="G18">
-        <v>2719</v>
+        <v>2722</v>
       </c>
       <c r="H18" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="I18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J18" s="1">
-        <v>46310</v>
+        <v>46315</v>
       </c>
       <c r="K18" s="1">
         <v>46315</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M18" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N18" s="1">
-        <v>46346</v>
+        <v>46326</v>
+      </c>
+      <c r="O18" s="1">
+        <v>46317</v>
       </c>
       <c r="Q18">
-        <v>-25</v>
+        <v>-4</v>
       </c>
       <c r="R18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S18" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="T18" t="s">
-        <v>113</v>
+        <v>110</v>
+      </c>
+      <c r="U18" t="s">
+        <v>118</v>
+      </c>
+      <c r="V18" t="s">
+        <v>134</v>
       </c>
       <c r="W18" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -2001,61 +1995,61 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C19" t="s">
         <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E19" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F19" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G19">
-        <v>2722</v>
+        <v>2721</v>
       </c>
       <c r="H19" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="I19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="J19" s="1">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="K19" s="1">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="L19">
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N19" s="1">
-        <v>46326</v>
+        <v>46324</v>
       </c>
       <c r="Q19">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="R19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S19" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T19" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="W19" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2063,67 +2057,67 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E20" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F20" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G20">
-        <v>2722</v>
+        <v>2721</v>
       </c>
       <c r="H20" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="I20" t="s">
+        <v>106</v>
+      </c>
+      <c r="J20" s="1">
+        <v>46316</v>
+      </c>
+      <c r="K20" s="1">
+        <v>46317</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20" t="s">
+        <v>108</v>
+      </c>
+      <c r="N20" s="1">
+        <v>46324</v>
+      </c>
+      <c r="Q20">
+        <v>-2</v>
+      </c>
+      <c r="R20">
+        <v>5</v>
+      </c>
+      <c r="S20" t="s">
         <v>110</v>
       </c>
-      <c r="J20" s="1">
-        <v>46311</v>
-      </c>
-      <c r="K20" s="1">
-        <v>46315</v>
-      </c>
-      <c r="L20">
-        <v>2</v>
-      </c>
-      <c r="M20" t="s">
-        <v>111</v>
-      </c>
-      <c r="N20" s="1">
-        <v>46326</v>
-      </c>
-      <c r="Q20">
-        <v>-5</v>
-      </c>
-      <c r="R20">
-        <v>6</v>
-      </c>
-      <c r="S20" t="s">
-        <v>112</v>
-      </c>
       <c r="T20" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="U20" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="V20" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="W20" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2131,67 +2125,64 @@
     </row>
     <row r="21" spans="1:27">
       <c r="A21">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
         <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E21" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F21" t="s">
+        <v>99</v>
+      </c>
+      <c r="G21">
+        <v>2734</v>
+      </c>
+      <c r="H21" t="s">
         <v>104</v>
       </c>
-      <c r="G21">
-        <v>2722</v>
-      </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>106</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" s="1">
+        <v>46321</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46322</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21" t="s">
         <v>108</v>
       </c>
-      <c r="J21" s="1">
-        <v>46311</v>
-      </c>
-      <c r="K21" s="1">
-        <v>46315</v>
-      </c>
-      <c r="L21">
-        <v>3</v>
-      </c>
-      <c r="M21" t="s">
-        <v>111</v>
-      </c>
       <c r="N21" s="1">
-        <v>46346</v>
+        <v>46329</v>
       </c>
       <c r="Q21">
-        <v>-25</v>
+        <v>-7</v>
       </c>
       <c r="R21">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="T21" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="U21" t="s">
-        <v>123</v>
-      </c>
-      <c r="V21" t="s">
-        <v>141</v>
+        <v>120</v>
       </c>
       <c r="W21" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2208,58 +2199,52 @@
         <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E22" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F22" t="s">
+        <v>100</v>
+      </c>
+      <c r="G22">
+        <v>2708</v>
+      </c>
+      <c r="H22" t="s">
         <v>104</v>
       </c>
-      <c r="G22">
-        <v>2719</v>
-      </c>
-      <c r="H22" t="s">
-        <v>106</v>
-      </c>
       <c r="I22" t="s">
+        <v>105</v>
+      </c>
+      <c r="J22" s="1">
+        <v>46317</v>
+      </c>
+      <c r="K22" s="1">
+        <v>46322</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22" t="s">
         <v>108</v>
       </c>
-      <c r="J22" s="1">
-        <v>46311</v>
-      </c>
-      <c r="K22" s="1">
-        <v>46315</v>
-      </c>
-      <c r="L22">
-        <v>3</v>
-      </c>
-      <c r="M22" t="s">
-        <v>111</v>
-      </c>
       <c r="N22" s="1">
-        <v>46346</v>
+        <v>46353</v>
       </c>
       <c r="Q22">
-        <v>-25</v>
+        <v>-31</v>
       </c>
       <c r="R22">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S22" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="T22" t="s">
-        <v>113</v>
-      </c>
-      <c r="U22" t="s">
-        <v>123</v>
-      </c>
-      <c r="V22" t="s">
-        <v>141</v>
+        <v>110</v>
       </c>
       <c r="W22" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2276,58 +2261,52 @@
         <v>54</v>
       </c>
       <c r="D23" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E23" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F23" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G23">
-        <v>2722</v>
+        <v>2729</v>
       </c>
       <c r="H23" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I23" t="s">
+        <v>107</v>
+      </c>
+      <c r="J23" s="1">
+        <v>46317</v>
+      </c>
+      <c r="K23" s="1">
+        <v>46322</v>
+      </c>
+      <c r="L23">
+        <v>2</v>
+      </c>
+      <c r="M23" t="s">
+        <v>108</v>
+      </c>
+      <c r="N23" s="1">
+        <v>46333</v>
+      </c>
+      <c r="Q23">
+        <v>-11</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23" t="s">
         <v>110</v>
       </c>
-      <c r="J23" s="1">
-        <v>46315</v>
-      </c>
-      <c r="K23" s="1">
-        <v>46315</v>
-      </c>
-      <c r="L23">
-        <v>12</v>
-      </c>
-      <c r="M23" t="s">
-        <v>111</v>
-      </c>
-      <c r="N23" s="1">
-        <v>46326</v>
-      </c>
-      <c r="Q23">
-        <v>-5</v>
-      </c>
-      <c r="R23">
-        <v>6</v>
-      </c>
-      <c r="S23" t="s">
-        <v>113</v>
-      </c>
       <c r="T23" t="s">
-        <v>113</v>
-      </c>
-      <c r="U23" t="s">
-        <v>124</v>
-      </c>
-      <c r="V23" t="s">
-        <v>142</v>
+        <v>110</v>
       </c>
       <c r="W23" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA23" t="b">
         <v>1</v>
@@ -2335,61 +2314,61 @@
     </row>
     <row r="24" spans="1:27">
       <c r="A24">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
         <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E24" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F24" t="s">
+        <v>100</v>
+      </c>
+      <c r="G24">
+        <v>2729</v>
+      </c>
+      <c r="H24" t="s">
         <v>104</v>
       </c>
-      <c r="G24">
-        <v>2731</v>
-      </c>
-      <c r="H24" t="s">
-        <v>105</v>
-      </c>
       <c r="I24" t="s">
+        <v>107</v>
+      </c>
+      <c r="J24" s="1">
+        <v>46321</v>
+      </c>
+      <c r="K24" s="1">
+        <v>46322</v>
+      </c>
+      <c r="L24">
+        <v>1</v>
+      </c>
+      <c r="M24" t="s">
+        <v>108</v>
+      </c>
+      <c r="N24" s="1">
+        <v>46333</v>
+      </c>
+      <c r="Q24">
+        <v>-11</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24" t="s">
         <v>109</v>
       </c>
-      <c r="J24" s="1">
-        <v>46315</v>
-      </c>
-      <c r="K24" s="1">
-        <v>46316</v>
-      </c>
-      <c r="L24">
-        <v>1</v>
-      </c>
-      <c r="M24" t="s">
-        <v>111</v>
-      </c>
-      <c r="N24" s="1">
-        <v>46323</v>
-      </c>
-      <c r="Q24">
-        <v>-2</v>
-      </c>
-      <c r="R24">
-        <v>5</v>
-      </c>
-      <c r="S24" t="s">
-        <v>112</v>
-      </c>
       <c r="T24" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="W24" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA24" t="b">
         <v>1</v>
@@ -2397,128 +2376,63 @@
     </row>
     <row r="25" spans="1:27">
       <c r="A25">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B25" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
         <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F25" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G25">
-        <v>2721</v>
+        <v>2708</v>
       </c>
       <c r="H25" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I25" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J25" s="1">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="K25" s="1">
-        <v>46317</v>
+        <v>46322</v>
       </c>
       <c r="L25">
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="N25" s="1">
-        <v>46324</v>
+        <v>46333</v>
       </c>
       <c r="Q25">
-        <v>-3</v>
+        <v>-11</v>
       </c>
       <c r="R25">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="T25" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="W25" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="AA25" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:27">
-      <c r="A26">
-        <v>329</v>
-      </c>
-      <c r="B26" t="s">
-        <v>31</v>
-      </c>
-      <c r="C26" t="s">
-        <v>57</v>
-      </c>
-      <c r="D26" t="s">
-        <v>79</v>
-      </c>
-      <c r="E26" t="s">
-        <v>101</v>
-      </c>
-      <c r="F26" t="s">
-        <v>104</v>
-      </c>
-      <c r="G26">
-        <v>2721</v>
-      </c>
-      <c r="H26" t="s">
-        <v>106</v>
-      </c>
-      <c r="I26" t="s">
-        <v>109</v>
-      </c>
-      <c r="J26" s="1">
-        <v>46316</v>
-      </c>
-      <c r="K26" s="1">
-        <v>46317</v>
-      </c>
-      <c r="L26">
-        <v>1</v>
-      </c>
-      <c r="M26" t="s">
-        <v>111</v>
-      </c>
-      <c r="N26" s="1">
-        <v>46324</v>
-      </c>
-      <c r="Q26">
-        <v>-3</v>
-      </c>
-      <c r="R26">
-        <v>4</v>
-      </c>
-      <c r="S26" t="s">
-        <v>113</v>
-      </c>
-      <c r="T26" t="s">
-        <v>112</v>
-      </c>
-      <c r="U26" t="s">
-        <v>125</v>
-      </c>
-      <c r="W26" t="s">
-        <v>143</v>
-      </c>
-      <c r="AA26" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (28/10/2026 14:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="157">
   <si>
     <t>om_emg</t>
   </si>
@@ -115,6 +115,9 @@
     <t>BABE</t>
   </si>
   <si>
+    <t>PAMA-LS</t>
+  </si>
+  <si>
     <t>313260018702</t>
   </si>
   <si>
@@ -187,6 +190,21 @@
     <t>685260013047</t>
   </si>
   <si>
+    <t>304260077166</t>
+  </si>
+  <si>
+    <t>304260077164</t>
+  </si>
+  <si>
+    <t>304260077165</t>
+  </si>
+  <si>
+    <t>329260019338</t>
+  </si>
+  <si>
+    <t>396260016657</t>
+  </si>
+  <si>
     <t>040-0043</t>
   </si>
   <si>
@@ -250,6 +268,21 @@
     <t>C668050-1103</t>
   </si>
   <si>
+    <t>PR1425B2</t>
+  </si>
+  <si>
+    <t>2613088-2</t>
+  </si>
+  <si>
+    <t>FS4291</t>
+  </si>
+  <si>
+    <t>066-3054-01</t>
+  </si>
+  <si>
+    <t>2643091-1</t>
+  </si>
+  <si>
     <t>STROB TUB</t>
   </si>
   <si>
@@ -313,6 +346,21 @@
     <t>TRANSMITER FUEL</t>
   </si>
   <si>
+    <t>SEALING COMPOUND</t>
+  </si>
+  <si>
+    <t>WINDSHIELD-RH 5/16 A</t>
+  </si>
+  <si>
+    <t>SEALANT TAPE</t>
+  </si>
+  <si>
+    <t>INDICATOR RADAR ALTI</t>
+  </si>
+  <si>
+    <t>PIN ASSY-TORQUE LINK</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -343,6 +391,12 @@
     <t>EA</t>
   </si>
   <si>
+    <t>KT</t>
+  </si>
+  <si>
+    <t>FT</t>
+  </si>
+  <si>
     <t>Não</t>
   </si>
   <si>
@@ -379,10 +433,10 @@
     <t>Cedeu o item para o 2738. Ramon 27/10/26</t>
   </si>
   <si>
-    <t>Colocado o pedido junto ao fornecedor AEROTECHNIC e WAGA INTERNATIONAL. Em processo de envio para a AGS Miami. ATZ 22/10</t>
-  </si>
-  <si>
-    <t>Enviados 02 ea para reparo em 09/10/2026 - REZ - Ag orçamento</t>
+    <t>Colocado o pedido junto ao fornecedor AEROTECHNIC - tracking 879206907443 e WAGA INTERNATIONAL - tracking 879129734726 - previsão de chegada dia 27/10 em Miami</t>
+  </si>
+  <si>
+    <t>Item recebido da William. Será enviado para o Operador em 27/10/2026- REZ</t>
   </si>
   <si>
     <t>Enviado para o Operador dia 09/10/26 - AWB 127-6186 9835 - REZ - MATERIAL ENTREGUE DIA 10/10/2026 no CAN BANT</t>
@@ -391,22 +445,25 @@
     <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26 .Segundo informações do Ten Soares do CLA não é preciso a compra do compressor no monento.(19/10/26 (SO R1 Bispo)</t>
   </si>
   <si>
-    <t>Abertas OS para 03 ea dia 07/10.Material coletado dia 09/10 fins reparo - AGD orçamento - REZ MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE</t>
-  </si>
-  <si>
-    <t>Colocado pedido Textron IJ17796997 - chegada GIG 14/10 (voo 4588) em desembaraço - Material aguardando a documentação da Textron, pois não veio com o material 20/10/26. Solicitado abertura de Os para 01 ea em 07/10/2026 para fazer o envio a Textron por ser unidade como CORE -REZ</t>
-  </si>
-  <si>
-    <t>abertas OS de 03 ea em 09/10/2026.REZ - Material enviado via recibo 912/FAB/26, AWB 12764844850 DPE 23/10/26</t>
+    <t>Abertas OS para 03 ea dia 07/10.Material coletado dia 09/10 fins reparo - AGD orçamento - REZ MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE - Chegada em Miami dia 30/10/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido Textron IJ17796997 - chegada GIG 14/10 (voo 4588) em desembaraço - Material aguardando a documentação da Textron, pois não veio com o material 20/10/26 - MATERIAL ENVIADO VIA AWB 12764403776, DPE 27/10/2026. Solicitado abertura de Os para 01 ea em 07/10/2026 para fazer o envio a Textron por ser unidade como CORE -REZ</t>
+  </si>
+  <si>
+    <t>abertas OS de 03 ea em 09/10/2026.REZ - Material enviado via recibo 912/FAB/26, AWB 12764844850 DPE 23/10/26 - AWB ENTROU EM FISCALIZAÇÃO, EM CONTATO COM A GOLLOG PARA ENTENDER O MOTIVO. - GOLLOG COLOCOU ERRONEAMENTE EM FISCALIZAÇÃO, MATERIAL LIBERADO E ENTREGUE PELA NOTA FSICAL NF 2339</t>
   </si>
   <si>
     <t>Colocado pedido Textron WB0003180334 - previsão de entrega no RJ 13/10 - MATERIAL RECEBIDO EM RJ 13/10 - PREPARANDO ENVIO 13/10 - recibo 887/FAB/26 AWB 12763073301 DPE 16/10/2026 - MATERIAL ENTREGUE DIA 15/10/2026</t>
   </si>
   <si>
-    <t>Colocado pedido I837605 - entregue 02ea em Miami 21/10</t>
-  </si>
-  <si>
-    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , PELO PN ALTERNADO MS20007-70. - RC 20/10/2026 - AWB 127-6466 1855</t>
+    <t>Material enviado via recibo 915/FAB/26, AWB 12764889333, DPE 27/10/2026</t>
+  </si>
+  <si>
+    <t>Colocado pedido I837605 (voo 4661 - em desembaraço GIG). I838606 - previsão de entrega em Miami 26/10</t>
+  </si>
+  <si>
+    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , PELO PN ALTERNADO MS20007-70. - RC 20/10/2026 - AWB 127-6466 1855 - ENTREGUE DIA 21/10/2026</t>
   </si>
   <si>
     <t>MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE</t>
@@ -421,7 +478,10 @@
     <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , - RC 20/10/2026 - AWB ENVIADA 12764659825</t>
   </si>
   <si>
-    <t>MATERIAL ENVIADO VIA AWB 12764891315, DISPONIVEL PARA RETIRADA DIA 23/10.</t>
+    <t>MATERIAL ENVIADO VIA AWB 12764891315, DISPONIVEL PARA RETIRADA DIA 23/10. - material entregue dia 23/10/2026</t>
+  </si>
+  <si>
+    <t>será atendido via estoque FAB</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -760,7 +820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AA30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -854,25 +914,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="F2" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I2" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -884,31 +944,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R2">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="S2" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T2" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U2" t="s">
-        <v>111</v>
+        <v>129</v>
       </c>
       <c r="V2" t="s">
-        <v>121</v>
+        <v>139</v>
       </c>
       <c r="W2" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -922,25 +982,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G3">
         <v>2703</v>
       </c>
       <c r="H3" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I3" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J3" s="1">
         <v>46294</v>
@@ -952,7 +1012,7 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N3" s="1">
         <v>46326</v>
@@ -961,22 +1021,22 @@
         <v>46326</v>
       </c>
       <c r="Q3">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R3">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S3" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T3" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="V3" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="W3" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -990,25 +1050,25 @@
         <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="F4" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="G4">
         <v>2703</v>
       </c>
       <c r="H4" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I4" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J4" s="1">
         <v>46294</v>
@@ -1020,7 +1080,7 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N4" s="1">
         <v>46326</v>
@@ -1029,25 +1089,25 @@
         <v>46305</v>
       </c>
       <c r="Q4">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S4" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T4" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U4" t="s">
-        <v>112</v>
+        <v>130</v>
       </c>
       <c r="V4" t="s">
-        <v>123</v>
+        <v>141</v>
       </c>
       <c r="W4" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1061,25 +1121,25 @@
         <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="F5" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G5">
         <v>2723</v>
       </c>
       <c r="H5" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I5" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J5" s="1">
         <v>46296</v>
@@ -1091,31 +1151,31 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N5" s="1">
         <v>46327</v>
       </c>
       <c r="Q5">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R5">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="S5" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T5" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="U5" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="V5" t="s">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="W5" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1129,25 +1189,25 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="F6" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G6">
         <v>2708</v>
       </c>
       <c r="H6" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I6" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J6" s="1">
         <v>46301</v>
@@ -1159,7 +1219,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N6" s="1">
         <v>46333</v>
@@ -1168,22 +1228,22 @@
         <v>46214</v>
       </c>
       <c r="Q6">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R6">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S6" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T6" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="V6" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="W6" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1197,25 +1257,25 @@
         <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="F7" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G7">
         <v>2742</v>
       </c>
       <c r="H7" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I7" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J7" s="1">
         <v>46302</v>
@@ -1227,31 +1287,31 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N7" s="1">
         <v>46333</v>
       </c>
       <c r="O7" s="1">
-        <v>46214</v>
+        <v>46322</v>
       </c>
       <c r="Q7">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R7">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S7" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T7" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="V7" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="W7" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1265,25 +1325,25 @@
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G8">
         <v>2721</v>
       </c>
       <c r="H8" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="J8" s="1">
         <v>46304</v>
@@ -1295,31 +1355,31 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N8" s="1">
         <v>46311</v>
       </c>
       <c r="O8" s="1">
-        <v>46318</v>
+        <v>46322</v>
       </c>
       <c r="Q8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S8" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T8" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="V8" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="W8" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1333,25 +1393,25 @@
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="F9" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G9">
         <v>2729</v>
       </c>
       <c r="H9" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I9" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="J9" s="1">
         <v>46303</v>
@@ -1363,7 +1423,7 @@
         <v>12</v>
       </c>
       <c r="M9" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N9" s="1">
         <v>46315</v>
@@ -1372,25 +1432,25 @@
         <v>46310</v>
       </c>
       <c r="Q9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R9">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="S9" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T9" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U9" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="V9" t="s">
-        <v>128</v>
+        <v>146</v>
       </c>
       <c r="W9" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1404,25 +1464,25 @@
         <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E10" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="F10" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G10">
         <v>2730</v>
       </c>
       <c r="H10" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I10" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="J10" s="1">
         <v>46309</v>
@@ -1434,25 +1494,31 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N10" s="1">
         <v>46327</v>
       </c>
+      <c r="O10" s="1">
+        <v>46322</v>
+      </c>
       <c r="Q10">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="R10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T10" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U10" t="s">
-        <v>115</v>
+        <v>133</v>
+      </c>
+      <c r="V10" t="s">
+        <v>147</v>
       </c>
       <c r="W10" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1466,25 +1532,25 @@
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="E11" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="F11" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G11">
         <v>2731</v>
       </c>
       <c r="H11" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I11" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="J11" s="1">
         <v>46310</v>
@@ -1496,28 +1562,28 @@
         <v>4</v>
       </c>
       <c r="M11" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N11" s="1">
         <v>46322</v>
       </c>
       <c r="Q11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R11">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S11" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T11" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="V11" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="W11" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1531,25 +1597,25 @@
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="F12" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G12">
         <v>2731</v>
       </c>
       <c r="H12" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="I12" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="J12" s="1">
         <v>46310</v>
@@ -1561,31 +1627,31 @@
         <v>2</v>
       </c>
       <c r="M12" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N12" s="1">
         <v>46322</v>
       </c>
       <c r="Q12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S12" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T12" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U12" t="s">
-        <v>116</v>
+        <v>134</v>
       </c>
       <c r="V12" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="W12" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1599,25 +1665,25 @@
         <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E13" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G13">
         <v>2702</v>
       </c>
       <c r="H13" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I13" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J13" s="1">
         <v>46310</v>
@@ -1629,28 +1695,28 @@
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N13" s="1">
         <v>46346</v>
       </c>
       <c r="Q13">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S13" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T13" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="V13" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="W13" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1664,25 +1730,25 @@
         <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E14" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="F14" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G14">
         <v>2719</v>
       </c>
       <c r="H14" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I14" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J14" s="1">
         <v>46310</v>
@@ -1694,28 +1760,28 @@
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N14" s="1">
         <v>46346</v>
       </c>
       <c r="Q14">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S14" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T14" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="V14" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="W14" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1729,25 +1795,25 @@
         <v>28</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="E15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="F15" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="G15">
         <v>2722</v>
       </c>
       <c r="H15" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I15" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="J15" s="1">
         <v>46311</v>
@@ -1759,28 +1825,28 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N15" s="1">
         <v>46326</v>
       </c>
       <c r="Q15">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R15">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S15" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T15" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="V15" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="W15" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1794,25 +1860,25 @@
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="F16" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="G16">
         <v>2722</v>
       </c>
       <c r="H16" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I16" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J16" s="1">
         <v>46311</v>
@@ -1824,31 +1890,31 @@
         <v>3</v>
       </c>
       <c r="M16" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N16" s="1">
         <v>46346</v>
       </c>
       <c r="Q16">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S16" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T16" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U16" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="V16" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="W16" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1862,25 +1928,25 @@
         <v>28</v>
       </c>
       <c r="C17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="E17" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="F17" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="G17">
         <v>2719</v>
       </c>
       <c r="H17" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I17" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J17" s="1">
         <v>46311</v>
@@ -1892,31 +1958,31 @@
         <v>3</v>
       </c>
       <c r="M17" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N17" s="1">
         <v>46346</v>
       </c>
       <c r="Q17">
-        <v>-24</v>
+        <v>-23</v>
       </c>
       <c r="R17">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S17" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T17" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U17" t="s">
-        <v>117</v>
+        <v>135</v>
       </c>
       <c r="V17" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="W17" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1930,25 +1996,25 @@
         <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="F18" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G18">
         <v>2722</v>
       </c>
       <c r="H18" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I18" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="J18" s="1">
         <v>46315</v>
@@ -1960,7 +2026,7 @@
         <v>12</v>
       </c>
       <c r="M18" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N18" s="1">
         <v>46326</v>
@@ -1969,25 +2035,25 @@
         <v>46317</v>
       </c>
       <c r="Q18">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="R18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S18" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="T18" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U18" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="V18" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="W18" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -2001,25 +2067,25 @@
         <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E19" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="F19" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G19">
         <v>2721</v>
       </c>
       <c r="H19" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="I19" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="J19" s="1">
         <v>46316</v>
@@ -2031,25 +2097,25 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N19" s="1">
         <v>46324</v>
       </c>
       <c r="Q19">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S19" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T19" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="W19" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2063,25 +2129,25 @@
         <v>31</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E20" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="F20" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="G20">
         <v>2721</v>
       </c>
       <c r="H20" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="I20" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="J20" s="1">
         <v>46316</v>
@@ -2093,31 +2159,34 @@
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N20" s="1">
         <v>46324</v>
       </c>
+      <c r="O20" s="1">
+        <v>46318</v>
+      </c>
       <c r="Q20">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="R20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="S20" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="T20" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="U20" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="V20" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="W20" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2131,25 +2200,25 @@
         <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="F21" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G21">
         <v>2734</v>
       </c>
       <c r="H21" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I21" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="J21" s="1">
         <v>46321</v>
@@ -2161,28 +2230,31 @@
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N21" s="1">
         <v>46329</v>
       </c>
       <c r="Q21">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S21" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="T21" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="U21" t="s">
-        <v>120</v>
+        <v>138</v>
+      </c>
+      <c r="V21" t="s">
+        <v>155</v>
       </c>
       <c r="W21" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2196,25 +2268,25 @@
         <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="E22" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="F22" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G22">
         <v>2708</v>
       </c>
       <c r="H22" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I22" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="J22" s="1">
         <v>46317</v>
@@ -2226,25 +2298,25 @@
         <v>1</v>
       </c>
       <c r="M22" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N22" s="1">
         <v>46353</v>
       </c>
       <c r="Q22">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T22" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="W22" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2258,25 +2330,25 @@
         <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E23" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="F23" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G23">
         <v>2729</v>
       </c>
       <c r="H23" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I23" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="J23" s="1">
         <v>46317</v>
@@ -2288,25 +2360,28 @@
         <v>2</v>
       </c>
       <c r="M23" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N23" s="1">
         <v>46333</v>
       </c>
       <c r="Q23">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="T23" t="s">
-        <v>110</v>
+        <v>128</v>
+      </c>
+      <c r="V23" t="s">
+        <v>155</v>
       </c>
       <c r="W23" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA23" t="b">
         <v>1</v>
@@ -2320,25 +2395,25 @@
         <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E24" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="F24" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="G24">
         <v>2729</v>
       </c>
       <c r="H24" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I24" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="J24" s="1">
         <v>46321</v>
@@ -2350,25 +2425,25 @@
         <v>1</v>
       </c>
       <c r="M24" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N24" s="1">
         <v>46333</v>
       </c>
       <c r="Q24">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="s">
-        <v>109</v>
+        <v>127</v>
       </c>
       <c r="T24" t="s">
-        <v>110</v>
+        <v>128</v>
       </c>
       <c r="W24" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
       <c r="AA24" t="b">
         <v>1</v>
@@ -2382,25 +2457,25 @@
         <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D25" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="E25" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="F25" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="G25">
         <v>2708</v>
       </c>
       <c r="H25" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="I25" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="J25" s="1">
         <v>46322</v>
@@ -2412,27 +2487,340 @@
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="N25" s="1">
         <v>46333</v>
       </c>
       <c r="Q25">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="R25">
+        <v>1</v>
+      </c>
+      <c r="S25" t="s">
+        <v>128</v>
+      </c>
+      <c r="T25" t="s">
+        <v>128</v>
+      </c>
+      <c r="V25" t="s">
+        <v>155</v>
+      </c>
+      <c r="W25" t="s">
+        <v>156</v>
+      </c>
+      <c r="AA25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:27">
+      <c r="A26">
+        <v>304</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" t="s">
+        <v>115</v>
+      </c>
+      <c r="G26">
+        <v>2704</v>
+      </c>
+      <c r="H26" t="s">
+        <v>120</v>
+      </c>
+      <c r="I26" t="s">
+        <v>122</v>
+      </c>
+      <c r="J26" s="1">
+        <v>46323</v>
+      </c>
+      <c r="K26" s="1">
+        <v>46323</v>
+      </c>
+      <c r="L26">
+        <v>5</v>
+      </c>
+      <c r="M26" t="s">
+        <v>125</v>
+      </c>
+      <c r="N26" s="1">
+        <v>46330</v>
+      </c>
+      <c r="Q26">
+        <v>-7</v>
+      </c>
+      <c r="R26">
         <v>0</v>
       </c>
-      <c r="S25" t="s">
-        <v>110</v>
-      </c>
-      <c r="T25" t="s">
-        <v>110</v>
-      </c>
-      <c r="W25" t="s">
-        <v>136</v>
-      </c>
-      <c r="AA25" t="b">
+      <c r="S26" t="s">
+        <v>127</v>
+      </c>
+      <c r="T26" t="s">
+        <v>128</v>
+      </c>
+      <c r="W26" t="s">
+        <v>156</v>
+      </c>
+      <c r="AA26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:27">
+      <c r="A27">
+        <v>304</v>
+      </c>
+      <c r="B27" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" t="s">
+        <v>111</v>
+      </c>
+      <c r="F27" t="s">
+        <v>115</v>
+      </c>
+      <c r="G27">
+        <v>2704</v>
+      </c>
+      <c r="H27" t="s">
+        <v>120</v>
+      </c>
+      <c r="I27" t="s">
+        <v>122</v>
+      </c>
+      <c r="J27" s="1">
+        <v>46323</v>
+      </c>
+      <c r="K27" s="1">
+        <v>46323</v>
+      </c>
+      <c r="L27">
+        <v>1</v>
+      </c>
+      <c r="M27" t="s">
+        <v>124</v>
+      </c>
+      <c r="N27" s="1">
+        <v>46330</v>
+      </c>
+      <c r="Q27">
+        <v>-7</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+      <c r="S27" t="s">
+        <v>127</v>
+      </c>
+      <c r="T27" t="s">
+        <v>128</v>
+      </c>
+      <c r="W27" t="s">
+        <v>156</v>
+      </c>
+      <c r="AA27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27">
+      <c r="A28">
+        <v>304</v>
+      </c>
+      <c r="B28" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" t="s">
+        <v>112</v>
+      </c>
+      <c r="F28" t="s">
+        <v>115</v>
+      </c>
+      <c r="G28">
+        <v>2704</v>
+      </c>
+      <c r="H28" t="s">
+        <v>120</v>
+      </c>
+      <c r="I28" t="s">
+        <v>122</v>
+      </c>
+      <c r="J28" s="1">
+        <v>46323</v>
+      </c>
+      <c r="K28" s="1">
+        <v>46323</v>
+      </c>
+      <c r="L28">
+        <v>5</v>
+      </c>
+      <c r="M28" t="s">
+        <v>126</v>
+      </c>
+      <c r="N28" s="1">
+        <v>46330</v>
+      </c>
+      <c r="Q28">
+        <v>-7</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+      <c r="S28" t="s">
+        <v>127</v>
+      </c>
+      <c r="T28" t="s">
+        <v>128</v>
+      </c>
+      <c r="W28" t="s">
+        <v>156</v>
+      </c>
+      <c r="AA28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27">
+      <c r="A29">
+        <v>329</v>
+      </c>
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" t="s">
+        <v>113</v>
+      </c>
+      <c r="F29" t="s">
+        <v>116</v>
+      </c>
+      <c r="G29">
+        <v>2721</v>
+      </c>
+      <c r="H29" t="s">
+        <v>120</v>
+      </c>
+      <c r="I29" t="s">
+        <v>122</v>
+      </c>
+      <c r="J29" s="1">
+        <v>46322</v>
+      </c>
+      <c r="K29" s="1">
+        <v>46323</v>
+      </c>
+      <c r="L29">
+        <v>1</v>
+      </c>
+      <c r="M29" t="s">
+        <v>124</v>
+      </c>
+      <c r="N29" s="1">
+        <v>46330</v>
+      </c>
+      <c r="Q29">
+        <v>-7</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+      <c r="S29" t="s">
+        <v>127</v>
+      </c>
+      <c r="T29" t="s">
+        <v>127</v>
+      </c>
+      <c r="W29" t="s">
+        <v>156</v>
+      </c>
+      <c r="AA29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:27">
+      <c r="A30">
+        <v>396</v>
+      </c>
+      <c r="B30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" t="s">
+        <v>62</v>
+      </c>
+      <c r="D30" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" t="s">
+        <v>114</v>
+      </c>
+      <c r="F30" t="s">
+        <v>115</v>
+      </c>
+      <c r="G30">
+        <v>2731</v>
+      </c>
+      <c r="H30" t="s">
+        <v>120</v>
+      </c>
+      <c r="I30" t="s">
+        <v>122</v>
+      </c>
+      <c r="J30" s="1">
+        <v>46322</v>
+      </c>
+      <c r="K30" s="1">
+        <v>46323</v>
+      </c>
+      <c r="L30">
+        <v>2</v>
+      </c>
+      <c r="M30" t="s">
+        <v>124</v>
+      </c>
+      <c r="N30" s="1">
+        <v>46330</v>
+      </c>
+      <c r="Q30">
+        <v>-7</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30" t="s">
+        <v>127</v>
+      </c>
+      <c r="T30" t="s">
+        <v>128</v>
+      </c>
+      <c r="W30" t="s">
+        <v>156</v>
+      </c>
+      <c r="AA30" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (29/10/2026 14:24)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="134">
   <si>
     <t>om_emg</t>
   </si>
@@ -106,9 +106,6 @@
     <t>CLA</t>
   </si>
   <si>
-    <t>DACTA II</t>
-  </si>
-  <si>
     <t>BABR</t>
   </si>
   <si>
@@ -121,9 +118,6 @@
     <t>313260018702</t>
   </si>
   <si>
-    <t>685260012893</t>
-  </si>
-  <si>
     <t>685260012894</t>
   </si>
   <si>
@@ -133,24 +127,12 @@
     <t>685260012943</t>
   </si>
   <si>
-    <t>384260009403</t>
-  </si>
-  <si>
-    <t>329260019312</t>
-  </si>
-  <si>
     <t>685260012964</t>
   </si>
   <si>
     <t>313260019100</t>
   </si>
   <si>
-    <t>396260016647</t>
-  </si>
-  <si>
-    <t>396260016648</t>
-  </si>
-  <si>
     <t>685260012988</t>
   </si>
   <si>
@@ -166,15 +148,9 @@
     <t>685260012996</t>
   </si>
   <si>
-    <t>685260012998</t>
-  </si>
-  <si>
     <t>329260019334</t>
   </si>
   <si>
-    <t>329260019335</t>
-  </si>
-  <si>
     <t>313260019118</t>
   </si>
   <si>
@@ -190,6 +166,15 @@
     <t>685260013047</t>
   </si>
   <si>
+    <t>396260016659</t>
+  </si>
+  <si>
+    <t>396260016657</t>
+  </si>
+  <si>
+    <t>685260013070</t>
+  </si>
+  <si>
     <t>304260077166</t>
   </si>
   <si>
@@ -202,15 +187,9 @@
     <t>329260019338</t>
   </si>
   <si>
-    <t>396260016657</t>
-  </si>
-  <si>
     <t>040-0043</t>
   </si>
   <si>
-    <t>065-0042-15</t>
-  </si>
-  <si>
     <t>065-0065-01</t>
   </si>
   <si>
@@ -220,39 +199,21 @@
     <t>065-0042-03</t>
   </si>
   <si>
-    <t>9514A-1</t>
-  </si>
-  <si>
-    <t>9910338-6</t>
-  </si>
-  <si>
     <t>103-20400</t>
   </si>
   <si>
     <t>011-00870-00</t>
   </si>
   <si>
-    <t>F2552-070</t>
-  </si>
-  <si>
-    <t>NAS147-84</t>
-  </si>
-  <si>
     <t>2641014-9</t>
   </si>
   <si>
     <t>324843-W020</t>
   </si>
   <si>
-    <t>MS21043-3</t>
-  </si>
-  <si>
     <t>030-02178-0000</t>
   </si>
   <si>
-    <t>C660501-0102</t>
-  </si>
-  <si>
     <t>2682004-1</t>
   </si>
   <si>
@@ -268,6 +229,15 @@
     <t>C668050-1103</t>
   </si>
   <si>
+    <t>011-00916-00</t>
+  </si>
+  <si>
+    <t>2643091-1</t>
+  </si>
+  <si>
+    <t>066-3038-00</t>
+  </si>
+  <si>
     <t>PR1425B2</t>
   </si>
   <si>
@@ -280,15 +250,9 @@
     <t>066-3054-01</t>
   </si>
   <si>
-    <t>2643091-1</t>
-  </si>
-  <si>
     <t>STROB TUB</t>
   </si>
   <si>
-    <t>AUTOPILOT COMPUTER</t>
-  </si>
-  <si>
     <t>SELECTOR ALT</t>
   </si>
   <si>
@@ -298,39 +262,21 @@
     <t>COMPUTER PA</t>
   </si>
   <si>
-    <t>PUMP ASSY</t>
-  </si>
-  <si>
-    <t>TRANSMITTER,RATE OF</t>
-  </si>
-  <si>
     <t>BOLT,MACHINE</t>
   </si>
   <si>
     <t>MAGNETOMETER GMU 44</t>
   </si>
   <si>
-    <t>BARREL NUT</t>
-  </si>
-  <si>
-    <t>BOLT,INTERNAL WRENCH</t>
-  </si>
-  <si>
     <t>SPRING ASSY-MAIN GEA</t>
   </si>
   <si>
     <t>HEADSET-MICROPHONE</t>
   </si>
   <si>
-    <t>NUT,SELF-LOCKING,EXT</t>
-  </si>
-  <si>
     <t>CONNECTOR,ELECTRICAL</t>
   </si>
   <si>
-    <t>COMPASS ASSY</t>
-  </si>
-  <si>
     <t>RESERVOIR ASSY-BRAKE</t>
   </si>
   <si>
@@ -346,6 +292,15 @@
     <t>TRANSMITER FUEL</t>
   </si>
   <si>
+    <t>DISPLAY UNIT GDU 104</t>
+  </si>
+  <si>
+    <t>PIN ASSY-TORQUE LINK</t>
+  </si>
+  <si>
+    <t>INDICATOR,RADIO-MAGN</t>
+  </si>
+  <si>
     <t>SEALING COMPOUND</t>
   </si>
   <si>
@@ -358,36 +313,30 @@
     <t>INDICATOR RADAR ALTI</t>
   </si>
   <si>
-    <t>PIN ASSY-TORQUE LINK</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
+    <t>T</t>
+  </si>
+  <si>
     <t>R</t>
   </si>
   <si>
-    <t>T</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
-    <t>Expedido total</t>
-  </si>
-  <si>
     <t>Aguardando solução</t>
   </si>
   <si>
     <t>ANCE</t>
   </si>
   <si>
+    <t>IPLR</t>
+  </si>
+  <si>
     <t>AIFP</t>
   </si>
   <si>
-    <t>IPLR</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -415,28 +364,19 @@
     <t>Recibo 887/FAB/26 AWB 127-6307 3301 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
   </si>
   <si>
-    <t>Cedeu o item para o C-98 2736. Ramon 21/10.</t>
-  </si>
-  <si>
-    <t>Atendido com estoque local em 21/10. Agd AWB 127-6466 1855 com previsão de entrega em 24/10. Ramon 22/10</t>
+    <t>Cedeu o item para o C-98 2736. Ramon 21/10. AWB 127-6488 9333 retirado por Francisca. Agd recibo 915/FAB/26 assinado. Ramon 29/10/26</t>
   </si>
   <si>
     <t>Autorizado reparo de fones do A7 para posterior mudança para U8. Ramon 22/10</t>
   </si>
   <si>
-    <t>Atendido com estoque local em 21/10 TSP 18710930. AWB 127-6465 9825 com previsão de entrega em 23/10. Ramon 22/10/26</t>
-  </si>
-  <si>
-    <t>Estoque do PN superador. Ramon 22/10</t>
-  </si>
-  <si>
-    <t>Cedeu o item para o 2738. Ramon 27/10/26</t>
-  </si>
-  <si>
-    <t>Colocado o pedido junto ao fornecedor AEROTECHNIC - tracking 879206907443 e WAGA INTERNATIONAL - tracking 879129734726 - previsão de chegada dia 27/10 em Miami</t>
-  </si>
-  <si>
-    <t>Item recebido da William. Será enviado para o Operador em 27/10/2026- REZ</t>
+    <t>Cedeu o item para o 2738. Ramon 27/10. Atendido com estoque local em 29/10. Ramon 29/10/26.</t>
+  </si>
+  <si>
+    <t>Atendido com estoque local em 29/10. Ramon 29/10/26.</t>
+  </si>
+  <si>
+    <t>Colocado o pedido junto ao fornecedor AEROTECHNIC previsão de chegada GIG 29/10 e WAGA INTERNATIONAL - será enviado em voo CAO</t>
   </si>
   <si>
     <t>Enviado para o Operador dia 09/10/26 - AWB 127-6186 9835 - REZ - MATERIAL ENTREGUE DIA 10/10/2026 no CAN BANT</t>
@@ -448,24 +388,12 @@
     <t>Abertas OS para 03 ea dia 07/10.Material coletado dia 09/10 fins reparo - AGD orçamento - REZ MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE - Chegada em Miami dia 30/10/2026</t>
   </si>
   <si>
-    <t>Colocado pedido Textron IJ17796997 - chegada GIG 14/10 (voo 4588) em desembaraço - Material aguardando a documentação da Textron, pois não veio com o material 20/10/26 - MATERIAL ENVIADO VIA AWB 12764403776, DPE 27/10/2026. Solicitado abertura de Os para 01 ea em 07/10/2026 para fazer o envio a Textron por ser unidade como CORE -REZ</t>
-  </si>
-  <si>
-    <t>abertas OS de 03 ea em 09/10/2026.REZ - Material enviado via recibo 912/FAB/26, AWB 12764844850 DPE 23/10/26 - AWB ENTROU EM FISCALIZAÇÃO, EM CONTATO COM A GOLLOG PARA ENTENDER O MOTIVO. - GOLLOG COLOCOU ERRONEAMENTE EM FISCALIZAÇÃO, MATERIAL LIBERADO E ENTREGUE PELA NOTA FSICAL NF 2339</t>
-  </si>
-  <si>
     <t>Colocado pedido Textron WB0003180334 - previsão de entrega no RJ 13/10 - MATERIAL RECEBIDO EM RJ 13/10 - PREPARANDO ENVIO 13/10 - recibo 887/FAB/26 AWB 12763073301 DPE 16/10/2026 - MATERIAL ENTREGUE DIA 15/10/2026</t>
   </si>
   <si>
     <t>Material enviado via recibo 915/FAB/26, AWB 12764889333, DPE 27/10/2026</t>
   </si>
   <si>
-    <t>Colocado pedido I837605 (voo 4661 - em desembaraço GIG). I838606 - previsão de entrega em Miami 26/10</t>
-  </si>
-  <si>
-    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , PELO PN ALTERNADO MS20007-70. - RC 20/10/2026 - AWB 127-6466 1855 - ENTREGUE DIA 21/10/2026</t>
-  </si>
-  <si>
     <t>MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE</t>
   </si>
   <si>
@@ -475,13 +403,16 @@
     <t>SOLICITAMOS OS CORES PARA REALIZAR REPARO, TENDO EM VISTA QUE NÃO TEMOS NO TSAM PARA RECOLHIMENTO. RC 20/10/2026</t>
   </si>
   <si>
-    <t>MATERIAL SOLICITADO VIA EMAIL "ATENDIMENTO COM ESTOQUE FAB EMERGÊNCIA" , - RC 20/10/2026 - AWB ENVIADA 12764659825</t>
-  </si>
-  <si>
-    <t>MATERIAL ENVIADO VIA AWB 12764891315, DISPONIVEL PARA RETIRADA DIA 23/10. - material entregue dia 23/10/2026</t>
-  </si>
-  <si>
     <t>será atendido via estoque FAB</t>
+  </si>
+  <si>
+    <t>validando estoque V1</t>
+  </si>
+  <si>
+    <t>MATERIAL EM TRANSITO, RECIBO 930/FAB/26</t>
+  </si>
+  <si>
+    <t>MATERIAL EM TRANSITO, SERÁ ATENDIDO O PN LP-1011GT, RECIBO 930/FAB/26</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -820,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA30"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -914,25 +845,25 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I2" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -944,31 +875,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R2">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="S2" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T2" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="U2" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="V2" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="W2" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -982,25 +913,25 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="F3" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="G3">
         <v>2703</v>
       </c>
       <c r="H3" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I3" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="J3" s="1">
         <v>46294</v>
@@ -1012,31 +943,34 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N3" s="1">
         <v>46326</v>
       </c>
       <c r="O3" s="1">
-        <v>46326</v>
+        <v>46305</v>
       </c>
       <c r="Q3">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="R3">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T3" t="s">
-        <v>128</v>
+        <v>111</v>
+      </c>
+      <c r="U3" t="s">
+        <v>113</v>
       </c>
       <c r="V3" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
       <c r="W3" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -1044,49 +978,46 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E4" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="F4" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="G4">
-        <v>2703</v>
+        <v>2723</v>
       </c>
       <c r="H4" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I4" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="J4" s="1">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K4" s="1">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N4" s="1">
-        <v>46326</v>
-      </c>
-      <c r="O4" s="1">
-        <v>46305</v>
+        <v>46327</v>
       </c>
       <c r="Q4">
         <v>-3</v>
@@ -1095,19 +1026,19 @@
         <v>28</v>
       </c>
       <c r="S4" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T4" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="U4" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="V4" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="W4" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1115,67 +1046,67 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E5" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="F5" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="G5">
-        <v>2723</v>
+        <v>2708</v>
       </c>
       <c r="H5" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I5" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="J5" s="1">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K5" s="1">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N5" s="1">
-        <v>46327</v>
+        <v>46333</v>
+      </c>
+      <c r="O5" s="1">
+        <v>46214</v>
       </c>
       <c r="Q5">
-        <v>-4</v>
+        <v>-9</v>
       </c>
       <c r="R5">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="S5" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T5" t="s">
-        <v>127</v>
-      </c>
-      <c r="U5" t="s">
-        <v>131</v>
+        <v>111</v>
       </c>
       <c r="V5" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
       <c r="W5" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1189,61 +1120,64 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="F6" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="G6">
-        <v>2708</v>
+        <v>2729</v>
       </c>
       <c r="H6" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I6" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="J6" s="1">
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="K6" s="1">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M6" t="s">
+        <v>107</v>
+      </c>
+      <c r="N6" s="1">
+        <v>46315</v>
+      </c>
+      <c r="O6" s="1">
+        <v>46310</v>
+      </c>
+      <c r="Q6">
+        <v>9</v>
+      </c>
+      <c r="R6">
+        <v>20</v>
+      </c>
+      <c r="S6" t="s">
+        <v>110</v>
+      </c>
+      <c r="T6" t="s">
+        <v>111</v>
+      </c>
+      <c r="U6" t="s">
+        <v>115</v>
+      </c>
+      <c r="V6" t="s">
         <v>124</v>
       </c>
-      <c r="N6" s="1">
-        <v>46333</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46214</v>
-      </c>
-      <c r="Q6">
-        <v>-10</v>
-      </c>
-      <c r="R6">
-        <v>21</v>
-      </c>
-      <c r="S6" t="s">
-        <v>127</v>
-      </c>
-      <c r="T6" t="s">
-        <v>128</v>
-      </c>
-      <c r="V6" t="s">
-        <v>143</v>
-      </c>
       <c r="W6" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1251,67 +1185,67 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>384</v>
+        <v>313</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E7" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="F7" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="G7">
-        <v>2742</v>
+        <v>2730</v>
       </c>
       <c r="H7" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I7" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="J7" s="1">
-        <v>46302</v>
+        <v>46309</v>
       </c>
       <c r="K7" s="1">
-        <v>46302</v>
+        <v>46316</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N7" s="1">
-        <v>46333</v>
+        <v>46327</v>
       </c>
       <c r="O7" s="1">
         <v>46322</v>
       </c>
       <c r="Q7">
-        <v>-10</v>
+        <v>-3</v>
       </c>
       <c r="R7">
-        <v>21</v>
-      </c>
-      <c r="S7" t="s">
-        <v>127</v>
+        <v>8</v>
       </c>
       <c r="T7" t="s">
-        <v>127</v>
+        <v>111</v>
+      </c>
+      <c r="U7" t="s">
+        <v>116</v>
       </c>
       <c r="V7" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="W7" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1319,67 +1253,64 @@
     </row>
     <row r="8" spans="1:27">
       <c r="A8">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="F8" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="G8">
-        <v>2721</v>
+        <v>2702</v>
       </c>
       <c r="H8" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I8" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="J8" s="1">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="K8" s="1">
-        <v>46304</v>
+        <v>46315</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N8" s="1">
-        <v>46311</v>
-      </c>
-      <c r="O8" s="1">
-        <v>46322</v>
+        <v>46346</v>
       </c>
       <c r="Q8">
-        <v>12</v>
+        <v>-22</v>
       </c>
       <c r="R8">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="S8" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T8" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="V8" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="W8" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1393,64 +1324,58 @@
         <v>28</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="F9" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="G9">
-        <v>2729</v>
+        <v>2719</v>
       </c>
       <c r="H9" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I9" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="J9" s="1">
-        <v>46303</v>
+        <v>46310</v>
       </c>
       <c r="K9" s="1">
-        <v>46304</v>
+        <v>46315</v>
       </c>
       <c r="L9">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N9" s="1">
-        <v>46315</v>
-      </c>
-      <c r="O9" s="1">
-        <v>46310</v>
+        <v>46346</v>
       </c>
       <c r="Q9">
-        <v>8</v>
+        <v>-22</v>
       </c>
       <c r="R9">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="S9" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T9" t="s">
-        <v>128</v>
-      </c>
-      <c r="U9" t="s">
-        <v>132</v>
+        <v>111</v>
       </c>
       <c r="V9" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="W9" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1458,67 +1383,64 @@
     </row>
     <row r="10" spans="1:27">
       <c r="A10">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="F10" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="G10">
-        <v>2730</v>
+        <v>2722</v>
       </c>
       <c r="H10" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I10" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="J10" s="1">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="K10" s="1">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N10" s="1">
-        <v>46327</v>
-      </c>
-      <c r="O10" s="1">
-        <v>46322</v>
+        <v>46326</v>
       </c>
       <c r="Q10">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="R10">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="S10" t="s">
+        <v>110</v>
       </c>
       <c r="T10" t="s">
-        <v>128</v>
-      </c>
-      <c r="U10" t="s">
+        <v>111</v>
+      </c>
+      <c r="V10" t="s">
+        <v>127</v>
+      </c>
+      <c r="W10" t="s">
         <v>133</v>
-      </c>
-      <c r="V10" t="s">
-        <v>147</v>
-      </c>
-      <c r="W10" t="s">
-        <v>156</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1526,64 +1448,67 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="G11">
-        <v>2731</v>
+        <v>2722</v>
       </c>
       <c r="H11" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I11" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="J11" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="K11" s="1">
         <v>46315</v>
       </c>
       <c r="L11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M11" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N11" s="1">
-        <v>46322</v>
+        <v>46346</v>
       </c>
       <c r="Q11">
-        <v>1</v>
+        <v>-22</v>
       </c>
       <c r="R11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S11" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T11" t="s">
+        <v>111</v>
+      </c>
+      <c r="U11" t="s">
+        <v>117</v>
+      </c>
+      <c r="V11" t="s">
         <v>128</v>
       </c>
-      <c r="V11" t="s">
-        <v>148</v>
-      </c>
       <c r="W11" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1591,67 +1516,67 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E12" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="G12">
-        <v>2731</v>
+        <v>2719</v>
       </c>
       <c r="H12" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="I12" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="J12" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="K12" s="1">
         <v>46315</v>
       </c>
       <c r="L12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M12" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N12" s="1">
-        <v>46322</v>
+        <v>46346</v>
       </c>
       <c r="Q12">
-        <v>1</v>
+        <v>-22</v>
       </c>
       <c r="R12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S12" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T12" t="s">
+        <v>111</v>
+      </c>
+      <c r="U12" t="s">
+        <v>117</v>
+      </c>
+      <c r="V12" t="s">
         <v>128</v>
       </c>
-      <c r="U12" t="s">
-        <v>134</v>
-      </c>
-      <c r="V12" t="s">
-        <v>149</v>
-      </c>
       <c r="W12" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1659,64 +1584,61 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F13" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="G13">
-        <v>2702</v>
+        <v>2721</v>
       </c>
       <c r="H13" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I13" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="J13" s="1">
-        <v>46310</v>
+        <v>46316</v>
       </c>
       <c r="K13" s="1">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N13" s="1">
-        <v>46346</v>
+        <v>46324</v>
       </c>
       <c r="Q13">
-        <v>-23</v>
+        <v>0</v>
       </c>
       <c r="R13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S13" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T13" t="s">
-        <v>128</v>
-      </c>
-      <c r="V13" t="s">
-        <v>150</v>
+        <v>110</v>
       </c>
       <c r="W13" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1724,64 +1646,67 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F14" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="G14">
-        <v>2719</v>
+        <v>2734</v>
       </c>
       <c r="H14" t="s">
+        <v>102</v>
+      </c>
+      <c r="I14" t="s">
+        <v>106</v>
+      </c>
+      <c r="J14" s="1">
+        <v>46321</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46322</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14" t="s">
+        <v>107</v>
+      </c>
+      <c r="N14" s="1">
+        <v>46329</v>
+      </c>
+      <c r="Q14">
+        <v>-5</v>
+      </c>
+      <c r="R14">
+        <v>2</v>
+      </c>
+      <c r="S14" t="s">
+        <v>111</v>
+      </c>
+      <c r="T14" t="s">
+        <v>111</v>
+      </c>
+      <c r="U14" t="s">
         <v>118</v>
       </c>
-      <c r="I14" t="s">
-        <v>121</v>
-      </c>
-      <c r="J14" s="1">
-        <v>46310</v>
-      </c>
-      <c r="K14" s="1">
-        <v>46315</v>
-      </c>
-      <c r="L14">
-        <v>1</v>
-      </c>
-      <c r="M14" t="s">
-        <v>124</v>
-      </c>
-      <c r="N14" s="1">
-        <v>46346</v>
-      </c>
-      <c r="Q14">
-        <v>-23</v>
-      </c>
-      <c r="R14">
-        <v>8</v>
-      </c>
-      <c r="S14" t="s">
-        <v>127</v>
-      </c>
-      <c r="T14" t="s">
-        <v>128</v>
-      </c>
       <c r="V14" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="W14" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1795,58 +1720,55 @@
         <v>28</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E15" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="F15" t="s">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="G15">
-        <v>2722</v>
+        <v>2708</v>
       </c>
       <c r="H15" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I15" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="J15" s="1">
-        <v>46311</v>
+        <v>46317</v>
       </c>
       <c r="K15" s="1">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="L15">
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N15" s="1">
-        <v>46326</v>
+        <v>46353</v>
       </c>
       <c r="Q15">
-        <v>-3</v>
+        <v>-29</v>
       </c>
       <c r="R15">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="S15" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T15" t="s">
-        <v>128</v>
-      </c>
-      <c r="V15" t="s">
-        <v>151</v>
+        <v>111</v>
       </c>
       <c r="W15" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1860,61 +1782,61 @@
         <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E16" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F16" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="G16">
-        <v>2722</v>
+        <v>2729</v>
       </c>
       <c r="H16" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I16" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="J16" s="1">
-        <v>46311</v>
+        <v>46317</v>
       </c>
       <c r="K16" s="1">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="L16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M16" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N16" s="1">
-        <v>46346</v>
+        <v>46333</v>
       </c>
       <c r="Q16">
-        <v>-23</v>
+        <v>-9</v>
       </c>
       <c r="R16">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="S16" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="T16" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="U16" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="V16" t="s">
-        <v>152</v>
+        <v>129</v>
       </c>
       <c r="W16" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1928,61 +1850,55 @@
         <v>28</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" t="s">
         <v>101</v>
       </c>
-      <c r="F17" t="s">
-        <v>117</v>
-      </c>
       <c r="G17">
-        <v>2719</v>
+        <v>2729</v>
       </c>
       <c r="H17" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I17" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="J17" s="1">
-        <v>46311</v>
+        <v>46321</v>
       </c>
       <c r="K17" s="1">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="L17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M17" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N17" s="1">
-        <v>46346</v>
+        <v>46333</v>
       </c>
       <c r="Q17">
-        <v>-23</v>
+        <v>-9</v>
       </c>
       <c r="R17">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="S17" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T17" t="s">
-        <v>128</v>
-      </c>
-      <c r="U17" t="s">
-        <v>135</v>
-      </c>
-      <c r="V17" t="s">
-        <v>152</v>
+        <v>111</v>
       </c>
       <c r="W17" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1996,64 +1912,61 @@
         <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E18" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" t="s">
+        <v>99</v>
+      </c>
+      <c r="G18">
+        <v>2708</v>
+      </c>
+      <c r="H18" t="s">
         <v>102</v>
       </c>
-      <c r="F18" t="s">
-        <v>115</v>
-      </c>
-      <c r="G18">
-        <v>2722</v>
-      </c>
-      <c r="H18" t="s">
-        <v>118</v>
-      </c>
       <c r="I18" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="J18" s="1">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="K18" s="1">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="L18">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N18" s="1">
-        <v>46326</v>
-      </c>
-      <c r="O18" s="1">
-        <v>46317</v>
+        <v>46333</v>
       </c>
       <c r="Q18">
-        <v>-3</v>
+        <v>-9</v>
       </c>
       <c r="R18">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="S18" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="T18" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="U18" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="V18" t="s">
-        <v>153</v>
+        <v>129</v>
       </c>
       <c r="W18" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -2061,61 +1974,61 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B19" t="s">
         <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="E19" t="s">
+        <v>92</v>
+      </c>
+      <c r="F19" t="s">
+        <v>101</v>
+      </c>
+      <c r="G19">
+        <v>2733</v>
+      </c>
+      <c r="H19" t="s">
         <v>103</v>
       </c>
-      <c r="F19" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19">
-        <v>2721</v>
-      </c>
-      <c r="H19" t="s">
-        <v>118</v>
-      </c>
       <c r="I19" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="J19" s="1">
-        <v>46316</v>
+        <v>46324</v>
       </c>
       <c r="K19" s="1">
-        <v>46317</v>
+        <v>46324</v>
       </c>
       <c r="L19">
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N19" s="1">
-        <v>46324</v>
+        <v>46355</v>
       </c>
       <c r="Q19">
-        <v>-1</v>
+        <v>-31</v>
       </c>
       <c r="R19">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="S19" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="T19" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="W19" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2123,70 +2036,64 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20">
-        <v>329</v>
+        <v>396</v>
       </c>
       <c r="B20" t="s">
         <v>31</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="E20" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="F20" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="G20">
-        <v>2721</v>
+        <v>2731</v>
       </c>
       <c r="H20" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="I20" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="J20" s="1">
-        <v>46316</v>
+        <v>46322</v>
       </c>
       <c r="K20" s="1">
-        <v>46317</v>
+        <v>46323</v>
       </c>
       <c r="L20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M20" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N20" s="1">
-        <v>46324</v>
-      </c>
-      <c r="O20" s="1">
-        <v>46318</v>
+        <v>46330</v>
       </c>
       <c r="Q20">
-        <v>-1</v>
+        <v>-6</v>
       </c>
       <c r="R20">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="S20" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="T20" t="s">
-        <v>127</v>
-      </c>
-      <c r="U20" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="V20" t="s">
-        <v>154</v>
+        <v>130</v>
       </c>
       <c r="W20" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2194,67 +2101,64 @@
     </row>
     <row r="21" spans="1:27">
       <c r="A21">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E21" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="F21" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="G21">
-        <v>2734</v>
+        <v>2708</v>
       </c>
       <c r="H21" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="I21" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="J21" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="K21" s="1">
-        <v>46322</v>
+        <v>46324</v>
       </c>
       <c r="L21">
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N21" s="1">
-        <v>46329</v>
+        <v>46355</v>
       </c>
       <c r="Q21">
-        <v>-6</v>
+        <v>-31</v>
       </c>
       <c r="R21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="T21" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="U21" t="s">
-        <v>138</v>
-      </c>
-      <c r="V21" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
       <c r="W21" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2262,61 +2166,64 @@
     </row>
     <row r="22" spans="1:27">
       <c r="A22">
-        <v>685</v>
+        <v>304</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E22" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G22">
+        <v>2704</v>
+      </c>
+      <c r="H22" t="s">
+        <v>102</v>
+      </c>
+      <c r="I22" t="s">
         <v>106</v>
       </c>
-      <c r="F22" t="s">
-        <v>116</v>
-      </c>
-      <c r="G22">
-        <v>2708</v>
-      </c>
-      <c r="H22" t="s">
-        <v>118</v>
-      </c>
-      <c r="I22" t="s">
-        <v>121</v>
-      </c>
       <c r="J22" s="1">
-        <v>46317</v>
+        <v>46323</v>
       </c>
       <c r="K22" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="L22">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M22" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="N22" s="1">
-        <v>46353</v>
+        <v>46330</v>
       </c>
       <c r="Q22">
-        <v>-30</v>
+        <v>-6</v>
       </c>
       <c r="R22">
         <v>1</v>
       </c>
       <c r="S22" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T22" t="s">
-        <v>128</v>
+        <v>111</v>
+      </c>
+      <c r="V22" t="s">
+        <v>131</v>
       </c>
       <c r="W22" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2324,64 +2231,64 @@
     </row>
     <row r="23" spans="1:27">
       <c r="A23">
-        <v>685</v>
+        <v>304</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E23" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23">
+        <v>2704</v>
+      </c>
+      <c r="H23" t="s">
+        <v>102</v>
+      </c>
+      <c r="I23" t="s">
+        <v>106</v>
+      </c>
+      <c r="J23" s="1">
+        <v>46323</v>
+      </c>
+      <c r="K23" s="1">
+        <v>46323</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23" t="s">
         <v>107</v>
       </c>
-      <c r="F23" t="s">
-        <v>115</v>
-      </c>
-      <c r="G23">
-        <v>2729</v>
-      </c>
-      <c r="H23" t="s">
-        <v>118</v>
-      </c>
-      <c r="I23" t="s">
-        <v>123</v>
-      </c>
-      <c r="J23" s="1">
-        <v>46317</v>
-      </c>
-      <c r="K23" s="1">
-        <v>46322</v>
-      </c>
-      <c r="L23">
-        <v>2</v>
-      </c>
-      <c r="M23" t="s">
-        <v>124</v>
-      </c>
       <c r="N23" s="1">
-        <v>46333</v>
+        <v>46330</v>
       </c>
       <c r="Q23">
-        <v>-10</v>
+        <v>-6</v>
       </c>
       <c r="R23">
         <v>1</v>
       </c>
       <c r="S23" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="T23" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="V23" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="W23" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA23" t="b">
         <v>1</v>
@@ -2389,61 +2296,64 @@
     </row>
     <row r="24" spans="1:27">
       <c r="A24">
-        <v>685</v>
+        <v>304</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E24" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="F24" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="G24">
-        <v>2729</v>
+        <v>2704</v>
       </c>
       <c r="H24" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I24" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="J24" s="1">
-        <v>46321</v>
+        <v>46323</v>
       </c>
       <c r="K24" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="L24">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M24" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="N24" s="1">
-        <v>46333</v>
+        <v>46330</v>
       </c>
       <c r="Q24">
-        <v>-10</v>
+        <v>-6</v>
       </c>
       <c r="R24">
         <v>1</v>
       </c>
       <c r="S24" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="T24" t="s">
-        <v>128</v>
+        <v>111</v>
+      </c>
+      <c r="V24" t="s">
+        <v>131</v>
       </c>
       <c r="W24" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA24" t="b">
         <v>1</v>
@@ -2451,376 +2361,63 @@
     </row>
     <row r="25" spans="1:27">
       <c r="A25">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D25" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="E25" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="F25" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="G25">
-        <v>2708</v>
+        <v>2721</v>
       </c>
       <c r="H25" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="I25" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="J25" s="1">
         <v>46322</v>
       </c>
       <c r="K25" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="L25">
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="N25" s="1">
-        <v>46333</v>
+        <v>46330</v>
       </c>
       <c r="Q25">
-        <v>-10</v>
+        <v>-6</v>
       </c>
       <c r="R25">
         <v>1</v>
       </c>
       <c r="S25" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="T25" t="s">
-        <v>128</v>
-      </c>
-      <c r="V25" t="s">
-        <v>155</v>
+        <v>110</v>
       </c>
       <c r="W25" t="s">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="AA25" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:27">
-      <c r="A26">
-        <v>304</v>
-      </c>
-      <c r="B26" t="s">
-        <v>33</v>
-      </c>
-      <c r="C26" t="s">
-        <v>58</v>
-      </c>
-      <c r="D26" t="s">
-        <v>84</v>
-      </c>
-      <c r="E26" t="s">
-        <v>110</v>
-      </c>
-      <c r="F26" t="s">
-        <v>115</v>
-      </c>
-      <c r="G26">
-        <v>2704</v>
-      </c>
-      <c r="H26" t="s">
-        <v>120</v>
-      </c>
-      <c r="I26" t="s">
-        <v>122</v>
-      </c>
-      <c r="J26" s="1">
-        <v>46323</v>
-      </c>
-      <c r="K26" s="1">
-        <v>46323</v>
-      </c>
-      <c r="L26">
-        <v>5</v>
-      </c>
-      <c r="M26" t="s">
-        <v>125</v>
-      </c>
-      <c r="N26" s="1">
-        <v>46330</v>
-      </c>
-      <c r="Q26">
-        <v>-7</v>
-      </c>
-      <c r="R26">
-        <v>0</v>
-      </c>
-      <c r="S26" t="s">
-        <v>127</v>
-      </c>
-      <c r="T26" t="s">
-        <v>128</v>
-      </c>
-      <c r="W26" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA26" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:27">
-      <c r="A27">
-        <v>304</v>
-      </c>
-      <c r="B27" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" t="s">
-        <v>59</v>
-      </c>
-      <c r="D27" t="s">
-        <v>85</v>
-      </c>
-      <c r="E27" t="s">
-        <v>111</v>
-      </c>
-      <c r="F27" t="s">
-        <v>115</v>
-      </c>
-      <c r="G27">
-        <v>2704</v>
-      </c>
-      <c r="H27" t="s">
-        <v>120</v>
-      </c>
-      <c r="I27" t="s">
-        <v>122</v>
-      </c>
-      <c r="J27" s="1">
-        <v>46323</v>
-      </c>
-      <c r="K27" s="1">
-        <v>46323</v>
-      </c>
-      <c r="L27">
-        <v>1</v>
-      </c>
-      <c r="M27" t="s">
-        <v>124</v>
-      </c>
-      <c r="N27" s="1">
-        <v>46330</v>
-      </c>
-      <c r="Q27">
-        <v>-7</v>
-      </c>
-      <c r="R27">
-        <v>0</v>
-      </c>
-      <c r="S27" t="s">
-        <v>127</v>
-      </c>
-      <c r="T27" t="s">
-        <v>128</v>
-      </c>
-      <c r="W27" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA27" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:27">
-      <c r="A28">
-        <v>304</v>
-      </c>
-      <c r="B28" t="s">
-        <v>33</v>
-      </c>
-      <c r="C28" t="s">
-        <v>60</v>
-      </c>
-      <c r="D28" t="s">
-        <v>86</v>
-      </c>
-      <c r="E28" t="s">
-        <v>112</v>
-      </c>
-      <c r="F28" t="s">
-        <v>115</v>
-      </c>
-      <c r="G28">
-        <v>2704</v>
-      </c>
-      <c r="H28" t="s">
-        <v>120</v>
-      </c>
-      <c r="I28" t="s">
-        <v>122</v>
-      </c>
-      <c r="J28" s="1">
-        <v>46323</v>
-      </c>
-      <c r="K28" s="1">
-        <v>46323</v>
-      </c>
-      <c r="L28">
-        <v>5</v>
-      </c>
-      <c r="M28" t="s">
-        <v>126</v>
-      </c>
-      <c r="N28" s="1">
-        <v>46330</v>
-      </c>
-      <c r="Q28">
-        <v>-7</v>
-      </c>
-      <c r="R28">
-        <v>0</v>
-      </c>
-      <c r="S28" t="s">
-        <v>127</v>
-      </c>
-      <c r="T28" t="s">
-        <v>128</v>
-      </c>
-      <c r="W28" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA28" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:27">
-      <c r="A29">
-        <v>329</v>
-      </c>
-      <c r="B29" t="s">
-        <v>31</v>
-      </c>
-      <c r="C29" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" t="s">
-        <v>87</v>
-      </c>
-      <c r="E29" t="s">
-        <v>113</v>
-      </c>
-      <c r="F29" t="s">
-        <v>116</v>
-      </c>
-      <c r="G29">
-        <v>2721</v>
-      </c>
-      <c r="H29" t="s">
-        <v>120</v>
-      </c>
-      <c r="I29" t="s">
-        <v>122</v>
-      </c>
-      <c r="J29" s="1">
-        <v>46322</v>
-      </c>
-      <c r="K29" s="1">
-        <v>46323</v>
-      </c>
-      <c r="L29">
-        <v>1</v>
-      </c>
-      <c r="M29" t="s">
-        <v>124</v>
-      </c>
-      <c r="N29" s="1">
-        <v>46330</v>
-      </c>
-      <c r="Q29">
-        <v>-7</v>
-      </c>
-      <c r="R29">
-        <v>0</v>
-      </c>
-      <c r="S29" t="s">
-        <v>127</v>
-      </c>
-      <c r="T29" t="s">
-        <v>127</v>
-      </c>
-      <c r="W29" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA29" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:27">
-      <c r="A30">
-        <v>396</v>
-      </c>
-      <c r="B30" t="s">
-        <v>32</v>
-      </c>
-      <c r="C30" t="s">
-        <v>62</v>
-      </c>
-      <c r="D30" t="s">
-        <v>88</v>
-      </c>
-      <c r="E30" t="s">
-        <v>114</v>
-      </c>
-      <c r="F30" t="s">
-        <v>115</v>
-      </c>
-      <c r="G30">
-        <v>2731</v>
-      </c>
-      <c r="H30" t="s">
-        <v>120</v>
-      </c>
-      <c r="I30" t="s">
-        <v>122</v>
-      </c>
-      <c r="J30" s="1">
-        <v>46322</v>
-      </c>
-      <c r="K30" s="1">
-        <v>46323</v>
-      </c>
-      <c r="L30">
-        <v>2</v>
-      </c>
-      <c r="M30" t="s">
-        <v>124</v>
-      </c>
-      <c r="N30" s="1">
-        <v>46330</v>
-      </c>
-      <c r="Q30">
-        <v>-7</v>
-      </c>
-      <c r="R30">
-        <v>0</v>
-      </c>
-      <c r="S30" t="s">
-        <v>127</v>
-      </c>
-      <c r="T30" t="s">
-        <v>128</v>
-      </c>
-      <c r="W30" t="s">
-        <v>156</v>
-      </c>
-      <c r="AA30" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: emergencias (30/10/2026 14:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_emergencias_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="129">
   <si>
     <t>om_emg</t>
   </si>
@@ -100,37 +100,31 @@
     <t>BAMN</t>
   </si>
   <si>
+    <t>CLA</t>
+  </si>
+  <si>
     <t>BANT</t>
   </si>
   <si>
-    <t>CLA</t>
+    <t>BABE</t>
   </si>
   <si>
     <t>BABR</t>
   </si>
   <si>
-    <t>BABE</t>
-  </si>
-  <si>
     <t>PAMA-LS</t>
   </si>
   <si>
     <t>313260018702</t>
   </si>
   <si>
-    <t>685260012894</t>
-  </si>
-  <si>
     <t>419260000561</t>
   </si>
   <si>
     <t>685260012943</t>
   </si>
   <si>
-    <t>685260012964</t>
-  </si>
-  <si>
-    <t>313260019100</t>
+    <t>396260016645</t>
   </si>
   <si>
     <t>685260012988</t>
@@ -187,22 +181,19 @@
     <t>329260019338</t>
   </si>
   <si>
+    <t>685260013074</t>
+  </si>
+  <si>
     <t>040-0043</t>
   </si>
   <si>
-    <t>065-0065-01</t>
-  </si>
-  <si>
     <t>SD5H14C4527</t>
   </si>
   <si>
     <t>065-0042-03</t>
   </si>
   <si>
-    <t>103-20400</t>
-  </si>
-  <si>
-    <t>011-00870-00</t>
+    <t>2643100-201</t>
   </si>
   <si>
     <t>2641014-9</t>
@@ -250,22 +241,19 @@
     <t>066-3054-01</t>
   </si>
   <si>
+    <t>066-1069-00</t>
+  </si>
+  <si>
     <t>STROB TUB</t>
   </si>
   <si>
-    <t>SELECTOR ALT</t>
-  </si>
-  <si>
     <t>AIR COMPRESSOR</t>
   </si>
   <si>
     <t>COMPUTER PA</t>
   </si>
   <si>
-    <t>BOLT,MACHINE</t>
-  </si>
-  <si>
-    <t>MAGNETOMETER GMU 44</t>
+    <t>NOSE GEAR STRUT ASSY</t>
   </si>
   <si>
     <t>SPRING ASSY-MAIN GEA</t>
@@ -313,30 +301,36 @@
     <t>INDICATOR RADAR ALTI</t>
   </si>
   <si>
+    <t>INDICATOR,BEARING-DI</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
+    <t>R</t>
+  </si>
+  <si>
     <t>T</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
     <t>Providência tomada</t>
   </si>
   <si>
     <t>Aguardando solução</t>
   </si>
   <si>
+    <t>Expedido total</t>
+  </si>
+  <si>
     <t>ANCE</t>
   </si>
   <si>
+    <t>AIFP</t>
+  </si>
+  <si>
     <t>IPLR</t>
   </si>
   <si>
-    <t>AIFP</t>
-  </si>
-  <si>
     <t>EA</t>
   </si>
   <si>
@@ -355,16 +349,10 @@
     <t>AWB 12759015025 - volume retirado na loja GOLLOG - QMA por kleyton Pena em 24/09. Godoy 28/09/26. Informado Recibo 814/FAB/26 assinado em 24/09, porém o item atendido nesse recibo não é alternado. Emg segue aguardando atendimento. Ramon 28/09/26</t>
   </si>
   <si>
-    <t>AWB 127-6186 9835 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
-  </si>
-  <si>
     <t>O compressor passou por teste no PAMALS onde foi identificada a pane nesse item. Ramon 21/10/26.</t>
   </si>
   <si>
-    <t>Recibo 887/FAB/26 AWB 127-6307 3301 retirado por Teodoro Silva. Agd recibo assinado. Ramon 22/10</t>
-  </si>
-  <si>
-    <t>Cedeu o item para o C-98 2736. Ramon 21/10. AWB 127-6488 9333 retirado por Francisca. Agd recibo 915/FAB/26 assinado. Ramon 29/10/26</t>
+    <t>Cedeu o item para o 2731. Ramon 30/10/26.</t>
   </si>
   <si>
     <t>Autorizado reparo de fones do A7 para posterior mudança para U8. Ramon 22/10</t>
@@ -376,10 +364,7 @@
     <t>Atendido com estoque local em 29/10. Ramon 29/10/26.</t>
   </si>
   <si>
-    <t>Colocado o pedido junto ao fornecedor AEROTECHNIC previsão de chegada GIG 29/10 e WAGA INTERNATIONAL - será enviado em voo CAO</t>
-  </si>
-  <si>
-    <t>Enviado para o Operador dia 09/10/26 - AWB 127-6186 9835 - REZ - MATERIAL ENTREGUE DIA 10/10/2026 no CAN BANT</t>
+    <t>Colocado o pedido junto ao fornecedor AEROTECHNIC previsão de chegada GIG 29/10 - voo 4704 em desembaraço - e WAGA INTERNATIONAL - será enviado em voo CAO</t>
   </si>
   <si>
     <t>Item ainda em pesquisa de pane pelo CLA. Não confirmaram a pane como COMPRESSOR. SO R1 BISPO 07/10/26 .Segundo informações do Ten Soares do CLA não é preciso a compra do compressor no monento.(19/10/26 (SO R1 Bispo)</t>
@@ -388,31 +373,31 @@
     <t>Abertas OS para 03 ea dia 07/10.Material coletado dia 09/10 fins reparo - AGD orçamento - REZ MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE - Chegada em Miami dia 30/10/2026</t>
   </si>
   <si>
-    <t>Colocado pedido Textron WB0003180334 - previsão de entrega no RJ 13/10 - MATERIAL RECEBIDO EM RJ 13/10 - PREPARANDO ENVIO 13/10 - recibo 887/FAB/26 AWB 12763073301 DPE 16/10/2026 - MATERIAL ENTREGUE DIA 15/10/2026</t>
-  </si>
-  <si>
-    <t>Material enviado via recibo 915/FAB/26, AWB 12764889333, DPE 27/10/2026</t>
-  </si>
-  <si>
     <t>MATERIAL EM PROCESSO DE AQUISIÇÃO, SERÁ FEITO EXCHANGE</t>
   </si>
   <si>
     <t>Foi solicitado via Email no dia 20/10/26 o core para revisão. Aguardando resposta.</t>
   </si>
   <si>
-    <t>SOLICITAMOS OS CORES PARA REALIZAR REPARO, TENDO EM VISTA QUE NÃO TEMOS NO TSAM PARA RECOLHIMENTO. RC 20/10/2026</t>
-  </si>
-  <si>
-    <t>será atendido via estoque FAB</t>
-  </si>
-  <si>
-    <t>validando estoque V1</t>
-  </si>
-  <si>
-    <t>MATERIAL EM TRANSITO, RECIBO 930/FAB/26</t>
-  </si>
-  <si>
-    <t>MATERIAL EM TRANSITO, SERÁ ATENDIDO O PN LP-1011GT, RECIBO 930/FAB/26</t>
+    <t>SOLICITAMOS OS CORES PARA REALIZAR REPARO, TENDO EM VISTA QUE NÃO TEMOS NO TSAM PARA RECOLHIMENTO. RC 20/10/2026 - Aguardando o recolhimento do fone cadastrado no projeto A7 para realizar reparo.</t>
+  </si>
+  <si>
+    <t>será atendido via estoque FAB, foi solicitado a atendimento via email CLA-29-10</t>
+  </si>
+  <si>
+    <t>Recebido 01 ea da empresa William, reparado, em 29/10/2026- Será atd este emerg - REZ</t>
+  </si>
+  <si>
+    <t>Solicitado abertura de OS para 03 ea em 27/10/26- REZ - Pago hoje enviado Swift para fornecer e regar hoje em Miami</t>
+  </si>
+  <si>
+    <t>Material em transito, RECIBO 931/FAB/26 - AWB A SER GERADA NA GOLLOG - RC DIA 29/10/2026</t>
+  </si>
+  <si>
+    <t>MATERIAL EM TRANSITO, RECIBO 930/FAB/26 - rc 29/10/26</t>
+  </si>
+  <si>
+    <t>MATERIAL EM TRANSITO, SERÁ ATENDIDO O PN LP-1011GT, RECIBO 930/FAB/26 - rc 29/10/26</t>
   </si>
   <si>
     <t>VEE ONE</t>
@@ -751,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -848,22 +833,22 @@
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G2">
         <v>2741</v>
       </c>
       <c r="H2" t="s">
+        <v>99</v>
+      </c>
+      <c r="I2" t="s">
         <v>102</v>
-      </c>
-      <c r="I2" t="s">
-        <v>104</v>
       </c>
       <c r="J2" s="1">
         <v>46251</v>
@@ -875,31 +860,31 @@
         <v>2</v>
       </c>
       <c r="M2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N2" s="1">
         <v>46280</v>
       </c>
       <c r="Q2">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R2">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S2" t="s">
+        <v>108</v>
+      </c>
+      <c r="T2" t="s">
+        <v>109</v>
+      </c>
+      <c r="U2" t="s">
         <v>110</v>
       </c>
-      <c r="T2" t="s">
-        <v>111</v>
-      </c>
-      <c r="U2" t="s">
-        <v>112</v>
-      </c>
       <c r="V2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="W2" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA2" t="b">
         <v>1</v>
@@ -907,7 +892,7 @@
     </row>
     <row r="3" spans="1:27">
       <c r="A3">
-        <v>685</v>
+        <v>419</v>
       </c>
       <c r="B3" t="s">
         <v>28</v>
@@ -916,40 +901,37 @@
         <v>34</v>
       </c>
       <c r="D3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G3">
-        <v>2703</v>
+        <v>2723</v>
       </c>
       <c r="H3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I3" t="s">
         <v>102</v>
       </c>
-      <c r="I3" t="s">
-        <v>104</v>
-      </c>
       <c r="J3" s="1">
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="K3" s="1">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L3">
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N3" s="1">
-        <v>46326</v>
-      </c>
-      <c r="O3" s="1">
-        <v>46305</v>
+        <v>46327</v>
       </c>
       <c r="Q3">
         <v>-2</v>
@@ -958,19 +940,19 @@
         <v>29</v>
       </c>
       <c r="S3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T3" t="s">
+        <v>108</v>
+      </c>
+      <c r="U3" t="s">
         <v>111</v>
       </c>
-      <c r="U3" t="s">
-        <v>113</v>
-      </c>
       <c r="V3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="W3" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA3" t="b">
         <v>1</v>
@@ -978,7 +960,7 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4">
-        <v>419</v>
+        <v>685</v>
       </c>
       <c r="B4" t="s">
         <v>29</v>
@@ -987,58 +969,58 @@
         <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G4">
-        <v>2723</v>
+        <v>2708</v>
       </c>
       <c r="H4" t="s">
+        <v>99</v>
+      </c>
+      <c r="I4" t="s">
         <v>102</v>
       </c>
-      <c r="I4" t="s">
-        <v>104</v>
-      </c>
       <c r="J4" s="1">
-        <v>46296</v>
+        <v>46301</v>
       </c>
       <c r="K4" s="1">
-        <v>46296</v>
+        <v>46302</v>
       </c>
       <c r="L4">
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N4" s="1">
-        <v>46327</v>
+        <v>46333</v>
+      </c>
+      <c r="O4" s="1">
+        <v>46333</v>
       </c>
       <c r="Q4">
-        <v>-3</v>
+        <v>-8</v>
       </c>
       <c r="R4">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="S4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T4" t="s">
-        <v>110</v>
-      </c>
-      <c r="U4" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="V4" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="W4" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA4" t="b">
         <v>1</v>
@@ -1046,67 +1028,64 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
         <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G5">
-        <v>2708</v>
+        <v>2726</v>
       </c>
       <c r="H5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J5" s="1">
-        <v>46301</v>
+        <v>46310</v>
       </c>
       <c r="K5" s="1">
-        <v>46302</v>
+        <v>46329</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N5" s="1">
-        <v>46333</v>
-      </c>
-      <c r="O5" s="1">
-        <v>46214</v>
+        <v>46336</v>
       </c>
       <c r="Q5">
-        <v>-9</v>
+        <v>-11</v>
       </c>
       <c r="R5">
-        <v>22</v>
+        <v>-4</v>
       </c>
       <c r="S5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T5" t="s">
-        <v>111</v>
-      </c>
-      <c r="V5" t="s">
-        <v>123</v>
+        <v>109</v>
+      </c>
+      <c r="U5" t="s">
+        <v>112</v>
       </c>
       <c r="W5" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA5" t="b">
         <v>1</v>
@@ -1117,67 +1096,61 @@
         <v>685</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G6">
+        <v>2702</v>
+      </c>
+      <c r="H6" t="s">
         <v>99</v>
       </c>
-      <c r="G6">
-        <v>2729</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>102</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
         <v>105</v>
       </c>
-      <c r="J6" s="1">
-        <v>46303</v>
-      </c>
-      <c r="K6" s="1">
-        <v>46304</v>
-      </c>
-      <c r="L6">
-        <v>12</v>
-      </c>
-      <c r="M6" t="s">
-        <v>107</v>
-      </c>
       <c r="N6" s="1">
-        <v>46315</v>
-      </c>
-      <c r="O6" s="1">
-        <v>46310</v>
+        <v>46346</v>
       </c>
       <c r="Q6">
-        <v>9</v>
+        <v>-21</v>
       </c>
       <c r="R6">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="S6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T6" t="s">
-        <v>111</v>
-      </c>
-      <c r="U6" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="V6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="W6" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA6" t="b">
         <v>1</v>
@@ -1185,67 +1158,64 @@
     </row>
     <row r="7" spans="1:27">
       <c r="A7">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
         <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G7">
-        <v>2730</v>
+        <v>2719</v>
       </c>
       <c r="H7" t="s">
+        <v>99</v>
+      </c>
+      <c r="I7" t="s">
         <v>102</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" s="1">
+        <v>46310</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46315</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
         <v>105</v>
       </c>
-      <c r="J7" s="1">
-        <v>46309</v>
-      </c>
-      <c r="K7" s="1">
-        <v>46316</v>
-      </c>
-      <c r="L7">
-        <v>1</v>
-      </c>
-      <c r="M7" t="s">
-        <v>107</v>
-      </c>
       <c r="N7" s="1">
-        <v>46327</v>
-      </c>
-      <c r="O7" s="1">
-        <v>46322</v>
+        <v>46346</v>
       </c>
       <c r="Q7">
-        <v>-3</v>
+        <v>-21</v>
       </c>
       <c r="R7">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="S7" t="s">
+        <v>108</v>
       </c>
       <c r="T7" t="s">
-        <v>111</v>
-      </c>
-      <c r="U7" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="V7" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="W7" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA7" t="b">
         <v>1</v>
@@ -1256,7 +1226,7 @@
         <v>685</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
         <v>39</v>
@@ -1265,22 +1235,22 @@
         <v>60</v>
       </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G8">
-        <v>2702</v>
+        <v>2722</v>
       </c>
       <c r="H8" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I8" t="s">
         <v>104</v>
       </c>
       <c r="J8" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="K8" s="1">
         <v>46315</v>
@@ -1289,28 +1259,28 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N8" s="1">
-        <v>46346</v>
+        <v>46326</v>
       </c>
       <c r="Q8">
-        <v>-22</v>
+        <v>-1</v>
       </c>
       <c r="R8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V8" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="W8" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA8" t="b">
         <v>1</v>
@@ -1321,61 +1291,64 @@
         <v>685</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>40</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
         <v>81</v>
       </c>
       <c r="F9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G9">
-        <v>2719</v>
+        <v>2722</v>
       </c>
       <c r="H9" t="s">
+        <v>99</v>
+      </c>
+      <c r="I9" t="s">
         <v>102</v>
       </c>
-      <c r="I9" t="s">
-        <v>104</v>
-      </c>
       <c r="J9" s="1">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="K9" s="1">
         <v>46315</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N9" s="1">
         <v>46346</v>
       </c>
       <c r="Q9">
-        <v>-22</v>
+        <v>-21</v>
       </c>
       <c r="R9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T9" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="U9" t="s">
+        <v>113</v>
       </c>
       <c r="V9" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="W9" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA9" t="b">
         <v>1</v>
@@ -1386,28 +1359,28 @@
         <v>685</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G10">
-        <v>2722</v>
+        <v>2719</v>
       </c>
       <c r="H10" t="s">
+        <v>99</v>
+      </c>
+      <c r="I10" t="s">
         <v>102</v>
-      </c>
-      <c r="I10" t="s">
-        <v>105</v>
       </c>
       <c r="J10" s="1">
         <v>46311</v>
@@ -1416,31 +1389,34 @@
         <v>46315</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N10" s="1">
-        <v>46326</v>
+        <v>46346</v>
       </c>
       <c r="Q10">
-        <v>-2</v>
+        <v>-21</v>
       </c>
       <c r="R10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="S10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T10" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="U10" t="s">
+        <v>113</v>
       </c>
       <c r="V10" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="W10" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA10" t="b">
         <v>1</v>
@@ -1448,67 +1424,61 @@
     </row>
     <row r="11" spans="1:27">
       <c r="A11">
-        <v>685</v>
+        <v>329</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G11">
-        <v>2722</v>
+        <v>2721</v>
       </c>
       <c r="H11" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J11" s="1">
-        <v>46311</v>
+        <v>46316</v>
       </c>
       <c r="K11" s="1">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="L11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N11" s="1">
-        <v>46346</v>
+        <v>46324</v>
       </c>
       <c r="Q11">
-        <v>-22</v>
+        <v>1</v>
       </c>
       <c r="R11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="S11" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T11" t="s">
-        <v>111</v>
-      </c>
-      <c r="U11" t="s">
-        <v>117</v>
-      </c>
-      <c r="V11" t="s">
+        <v>108</v>
+      </c>
+      <c r="W11" t="s">
         <v>128</v>
-      </c>
-      <c r="W11" t="s">
-        <v>133</v>
       </c>
       <c r="AA11" t="b">
         <v>1</v>
@@ -1516,67 +1486,67 @@
     </row>
     <row r="12" spans="1:27">
       <c r="A12">
-        <v>685</v>
+        <v>313</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
         <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G12">
-        <v>2719</v>
+        <v>2734</v>
       </c>
       <c r="H12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J12" s="1">
-        <v>46311</v>
+        <v>46321</v>
       </c>
       <c r="K12" s="1">
-        <v>46315</v>
+        <v>46322</v>
       </c>
       <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>105</v>
+      </c>
+      <c r="N12" s="1">
+        <v>46329</v>
+      </c>
+      <c r="Q12">
+        <v>-4</v>
+      </c>
+      <c r="R12">
         <v>3</v>
       </c>
-      <c r="M12" t="s">
-        <v>107</v>
-      </c>
-      <c r="N12" s="1">
-        <v>46346</v>
-      </c>
-      <c r="Q12">
-        <v>-22</v>
-      </c>
-      <c r="R12">
-        <v>9</v>
-      </c>
       <c r="S12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="T12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="U12" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="V12" t="s">
+        <v>122</v>
+      </c>
+      <c r="W12" t="s">
         <v>128</v>
-      </c>
-      <c r="W12" t="s">
-        <v>133</v>
       </c>
       <c r="AA12" t="b">
         <v>1</v>
@@ -1584,61 +1554,64 @@
     </row>
     <row r="13" spans="1:27">
       <c r="A13">
-        <v>329</v>
+        <v>685</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
         <v>44</v>
       </c>
       <c r="D13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
+        <v>97</v>
+      </c>
+      <c r="G13">
+        <v>2708</v>
+      </c>
+      <c r="H13" t="s">
         <v>99</v>
       </c>
-      <c r="G13">
-        <v>2721</v>
-      </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>102</v>
       </c>
-      <c r="I13" t="s">
-        <v>106</v>
-      </c>
       <c r="J13" s="1">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="K13" s="1">
-        <v>46317</v>
+        <v>46322</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N13" s="1">
-        <v>46324</v>
+        <v>46353</v>
       </c>
       <c r="Q13">
-        <v>0</v>
+        <v>-28</v>
       </c>
       <c r="R13">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="S13" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T13" t="s">
-        <v>110</v>
+        <v>109</v>
+      </c>
+      <c r="V13" t="s">
+        <v>123</v>
       </c>
       <c r="W13" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA13" t="b">
         <v>1</v>
@@ -1646,67 +1619,67 @@
     </row>
     <row r="14" spans="1:27">
       <c r="A14">
-        <v>313</v>
+        <v>685</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G14">
-        <v>2734</v>
+        <v>2729</v>
       </c>
       <c r="H14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="J14" s="1">
-        <v>46321</v>
+        <v>46317</v>
       </c>
       <c r="K14" s="1">
         <v>46322</v>
       </c>
       <c r="L14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N14" s="1">
-        <v>46329</v>
+        <v>46333</v>
       </c>
       <c r="Q14">
-        <v>-5</v>
+        <v>-8</v>
       </c>
       <c r="R14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="T14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="U14" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="V14" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="W14" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA14" t="b">
         <v>1</v>
@@ -1717,31 +1690,31 @@
         <v>685</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
         <v>46</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G15">
-        <v>2708</v>
+        <v>2729</v>
       </c>
       <c r="H15" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I15" t="s">
         <v>104</v>
       </c>
       <c r="J15" s="1">
-        <v>46317</v>
+        <v>46321</v>
       </c>
       <c r="K15" s="1">
         <v>46322</v>
@@ -1750,25 +1723,28 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N15" s="1">
-        <v>46353</v>
+        <v>46333</v>
       </c>
       <c r="Q15">
-        <v>-29</v>
+        <v>-8</v>
       </c>
       <c r="R15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S15" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T15" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="V15" t="s">
+        <v>124</v>
       </c>
       <c r="W15" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA15" t="b">
         <v>1</v>
@@ -1779,64 +1755,64 @@
         <v>685</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
         <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G16">
-        <v>2729</v>
+        <v>2708</v>
       </c>
       <c r="H16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J16" s="1">
-        <v>46317</v>
+        <v>46322</v>
       </c>
       <c r="K16" s="1">
         <v>46322</v>
       </c>
       <c r="L16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N16" s="1">
         <v>46333</v>
       </c>
       <c r="Q16">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="R16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="T16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="U16" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="V16" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="W16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA16" t="b">
         <v>1</v>
@@ -1844,61 +1820,61 @@
     </row>
     <row r="17" spans="1:27">
       <c r="A17">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F17" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G17">
-        <v>2729</v>
+        <v>2733</v>
       </c>
       <c r="H17" t="s">
+        <v>100</v>
+      </c>
+      <c r="I17" t="s">
         <v>102</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" s="1">
+        <v>46324</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46324</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17" t="s">
         <v>105</v>
       </c>
-      <c r="J17" s="1">
-        <v>46321</v>
-      </c>
-      <c r="K17" s="1">
-        <v>46322</v>
-      </c>
-      <c r="L17">
-        <v>1</v>
-      </c>
-      <c r="M17" t="s">
-        <v>107</v>
-      </c>
       <c r="N17" s="1">
-        <v>46333</v>
+        <v>46355</v>
       </c>
       <c r="Q17">
-        <v>-9</v>
+        <v>-30</v>
       </c>
       <c r="R17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S17" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="T17" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="W17" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA17" t="b">
         <v>1</v>
@@ -1906,67 +1882,67 @@
     </row>
     <row r="18" spans="1:27">
       <c r="A18">
-        <v>685</v>
+        <v>396</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F18" t="s">
+        <v>96</v>
+      </c>
+      <c r="G18">
+        <v>2731</v>
+      </c>
+      <c r="H18" t="s">
         <v>99</v>
       </c>
-      <c r="G18">
-        <v>2708</v>
-      </c>
-      <c r="H18" t="s">
-        <v>102</v>
-      </c>
       <c r="I18" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="J18" s="1">
         <v>46322</v>
       </c>
       <c r="K18" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="L18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M18" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N18" s="1">
-        <v>46333</v>
+        <v>46330</v>
+      </c>
+      <c r="O18" s="1">
+        <v>46325</v>
       </c>
       <c r="Q18">
-        <v>-9</v>
+        <v>-5</v>
       </c>
       <c r="R18">
         <v>2</v>
       </c>
       <c r="S18" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="T18" t="s">
-        <v>111</v>
-      </c>
-      <c r="U18" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="V18" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="W18" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA18" t="b">
         <v>1</v>
@@ -1974,34 +1950,34 @@
     </row>
     <row r="19" spans="1:27">
       <c r="A19">
-        <v>396</v>
+        <v>685</v>
       </c>
       <c r="B19" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
         <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E19" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
+        <v>97</v>
+      </c>
+      <c r="G19">
+        <v>2708</v>
+      </c>
+      <c r="H19" t="s">
         <v>101</v>
       </c>
-      <c r="G19">
-        <v>2733</v>
-      </c>
-      <c r="H19" t="s">
-        <v>103</v>
-      </c>
       <c r="I19" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J19" s="1">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="K19" s="1">
         <v>46324</v>
@@ -2010,25 +1986,28 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N19" s="1">
         <v>46355</v>
       </c>
       <c r="Q19">
-        <v>-31</v>
+        <v>-30</v>
       </c>
       <c r="R19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S19" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="T19" t="s">
-        <v>111</v>
+        <v>109</v>
+      </c>
+      <c r="U19" t="s">
+        <v>115</v>
       </c>
       <c r="W19" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA19" t="b">
         <v>1</v>
@@ -2036,64 +2015,67 @@
     </row>
     <row r="20" spans="1:27">
       <c r="A20">
-        <v>396</v>
+        <v>304</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C20" t="s">
         <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E20" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
+        <v>96</v>
+      </c>
+      <c r="G20">
+        <v>2704</v>
+      </c>
+      <c r="H20" t="s">
         <v>99</v>
       </c>
-      <c r="G20">
-        <v>2731</v>
-      </c>
-      <c r="H20" t="s">
-        <v>102</v>
-      </c>
       <c r="I20" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J20" s="1">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="K20" s="1">
         <v>46323</v>
       </c>
       <c r="L20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="N20" s="1">
         <v>46330</v>
       </c>
+      <c r="O20" s="1">
+        <v>46325</v>
+      </c>
       <c r="Q20">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S20" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T20" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V20" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="W20" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA20" t="b">
         <v>1</v>
@@ -2101,64 +2083,67 @@
     </row>
     <row r="21" spans="1:27">
       <c r="A21">
-        <v>685</v>
+        <v>304</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
         <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F21" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="G21">
-        <v>2708</v>
+        <v>2704</v>
       </c>
       <c r="H21" t="s">
+        <v>99</v>
+      </c>
+      <c r="I21" t="s">
         <v>103</v>
-      </c>
-      <c r="I21" t="s">
-        <v>104</v>
       </c>
       <c r="J21" s="1">
         <v>46323</v>
       </c>
       <c r="K21" s="1">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="L21">
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N21" s="1">
-        <v>46355</v>
+        <v>46330</v>
+      </c>
+      <c r="O21" s="1">
+        <v>46325</v>
       </c>
       <c r="Q21">
-        <v>-31</v>
+        <v>-5</v>
       </c>
       <c r="R21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S21" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="T21" t="s">
-        <v>111</v>
-      </c>
-      <c r="U21" t="s">
-        <v>119</v>
+        <v>109</v>
+      </c>
+      <c r="V21" t="s">
+        <v>127</v>
       </c>
       <c r="W21" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA21" t="b">
         <v>1</v>
@@ -2175,22 +2160,22 @@
         <v>53</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F22" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G22">
         <v>2704</v>
       </c>
       <c r="H22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J22" s="1">
         <v>46323</v>
@@ -2202,28 +2187,31 @@
         <v>5</v>
       </c>
       <c r="M22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N22" s="1">
         <v>46330</v>
       </c>
+      <c r="O22" s="1">
+        <v>46325</v>
+      </c>
       <c r="Q22">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T22" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="V22" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="W22" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA22" t="b">
         <v>1</v>
@@ -2231,34 +2219,34 @@
     </row>
     <row r="23" spans="1:27">
       <c r="A23">
-        <v>304</v>
+        <v>329</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23" t="s">
         <v>54</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F23" t="s">
+        <v>97</v>
+      </c>
+      <c r="G23">
+        <v>2721</v>
+      </c>
+      <c r="H23" t="s">
         <v>99</v>
       </c>
-      <c r="G23">
-        <v>2704</v>
-      </c>
-      <c r="H23" t="s">
-        <v>102</v>
-      </c>
       <c r="I23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J23" s="1">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="K23" s="1">
         <v>46323</v>
@@ -2267,28 +2255,28 @@
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N23" s="1">
         <v>46330</v>
       </c>
       <c r="Q23">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="R23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S23" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="T23" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="V23" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="W23" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA23" t="b">
         <v>1</v>
@@ -2296,128 +2284,63 @@
     </row>
     <row r="24" spans="1:27">
       <c r="A24">
-        <v>304</v>
+        <v>685</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C24" t="s">
         <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E24" t="s">
+        <v>95</v>
+      </c>
+      <c r="F24" t="s">
         <v>97</v>
       </c>
-      <c r="F24" t="s">
-        <v>99</v>
-      </c>
       <c r="G24">
-        <v>2704</v>
+        <v>2708</v>
       </c>
       <c r="H24" t="s">
+        <v>100</v>
+      </c>
+      <c r="I24" t="s">
         <v>102</v>
       </c>
-      <c r="I24" t="s">
-        <v>106</v>
-      </c>
       <c r="J24" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="K24" s="1">
-        <v>46323</v>
+        <v>46325</v>
       </c>
       <c r="L24">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="N24" s="1">
-        <v>46330</v>
+        <v>46356</v>
       </c>
       <c r="Q24">
-        <v>-6</v>
+        <v>-31</v>
       </c>
       <c r="R24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="T24" t="s">
-        <v>111</v>
-      </c>
-      <c r="V24" t="s">
-        <v>131</v>
+        <v>109</v>
       </c>
       <c r="W24" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="AA24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:27">
-      <c r="A25">
-        <v>329</v>
-      </c>
-      <c r="B25" t="s">
-        <v>30</v>
-      </c>
-      <c r="C25" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" t="s">
-        <v>98</v>
-      </c>
-      <c r="F25" t="s">
-        <v>101</v>
-      </c>
-      <c r="G25">
-        <v>2721</v>
-      </c>
-      <c r="H25" t="s">
-        <v>102</v>
-      </c>
-      <c r="I25" t="s">
-        <v>106</v>
-      </c>
-      <c r="J25" s="1">
-        <v>46322</v>
-      </c>
-      <c r="K25" s="1">
-        <v>46323</v>
-      </c>
-      <c r="L25">
-        <v>1</v>
-      </c>
-      <c r="M25" t="s">
-        <v>107</v>
-      </c>
-      <c r="N25" s="1">
-        <v>46330</v>
-      </c>
-      <c r="Q25">
-        <v>-6</v>
-      </c>
-      <c r="R25">
-        <v>1</v>
-      </c>
-      <c r="S25" t="s">
-        <v>110</v>
-      </c>
-      <c r="T25" t="s">
-        <v>110</v>
-      </c>
-      <c r="W25" t="s">
-        <v>133</v>
-      </c>
-      <c r="AA25" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>